<commit_message>
nouveau ajout derniere fonction chcab att j
</commit_message>
<xml_diff>
--- a/front/src/assets/template4CA.xlsx
+++ b/front/src/assets/template4CA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1B5D026-C468-7F42-9B0D-D9A7E658636E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16270FC1-9EC2-CA4B-96B5-AFC4D23B2327}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -27,7 +27,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ETPT A-JUST'!$A$2:$DN$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ETPT Format DDG'!$A$2:$DT$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Table_Fonctions!$A$1:$F$78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Table_Fonctions!$A$1:$F$80</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="810" uniqueCount="374">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="823" uniqueCount="378">
   <si>
     <t>#! END_ROW</t>
   </si>
@@ -2494,6 +2494,18 @@
   </si>
   <si>
     <t>ajouter ? JA Pôle Social,JA Parquet,JA JP,JA VIF</t>
+  </si>
+  <si>
+    <t>A GREFFIER</t>
+  </si>
+  <si>
+    <t>à valider</t>
+  </si>
+  <si>
+    <t>Att. J</t>
+  </si>
+  <si>
+    <t>ATTACHÉ DE JUSTICE</t>
   </si>
 </sst>
 </file>
@@ -2847,7 +2859,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="25">
+  <fills count="26">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2989,6 +3001,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -3389,7 +3407,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="181">
+  <cellXfs count="186">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -3926,6 +3944,21 @@
     </xf>
     <xf numFmtId="0" fontId="36" fillId="10" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="25" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="25" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -6818,7 +6851,7 @@
   <sheetPr codeName="Feuil14">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G78"/>
+  <dimension ref="A1:G80"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.83203125" style="35" bestFit="1" customWidth="1"/>
@@ -7149,7 +7182,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="137" t="s">
         <v>79</v>
       </c>
@@ -7169,7 +7202,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="137" t="s">
         <v>79</v>
       </c>
@@ -7189,35 +7222,38 @@
         <v>46</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A19" s="137" t="s">
+    <row r="19" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A19" s="181" t="s">
         <v>79</v>
       </c>
-      <c r="B19" s="132" t="s">
-        <v>44</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D19" s="2" t="s">
+      <c r="B19" s="182" t="s">
+        <v>374</v>
+      </c>
+      <c r="C19" s="183" t="s">
+        <v>374</v>
+      </c>
+      <c r="D19" s="183" t="s">
         <v>88</v>
       </c>
-      <c r="E19" s="136" t="s">
+      <c r="E19" s="184" t="s">
         <v>45</v>
       </c>
-      <c r="F19" s="134" t="s">
+      <c r="F19" s="185" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G19" s="35" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="137" t="s">
         <v>79</v>
       </c>
       <c r="B20" s="132" t="s">
-        <v>89</v>
+        <v>44</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>88</v>
@@ -7229,15 +7265,15 @@
         <v>46</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" s="137" t="s">
         <v>79</v>
       </c>
       <c r="B21" s="132" t="s">
-        <v>49</v>
+        <v>89</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>88</v>
@@ -7249,15 +7285,15 @@
         <v>46</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" s="137" t="s">
         <v>79</v>
       </c>
       <c r="B22" s="132" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>88</v>
@@ -7269,15 +7305,15 @@
         <v>46</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="137" t="s">
         <v>79</v>
       </c>
       <c r="B23" s="132" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>88</v>
@@ -7286,30 +7322,30 @@
         <v>45</v>
       </c>
       <c r="F23" s="134" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="137" t="s">
         <v>79</v>
       </c>
       <c r="B24" s="132" t="s">
-        <v>327</v>
+        <v>51</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>327</v>
+        <v>51</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="E24" s="138" t="s">
-        <v>53</v>
+        <v>88</v>
+      </c>
+      <c r="E24" s="136" t="s">
+        <v>45</v>
       </c>
       <c r="F24" s="134" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="137" t="s">
         <v>79</v>
       </c>
@@ -7317,7 +7353,7 @@
         <v>327</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>358</v>
+        <v>327</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>87</v>
@@ -7329,7 +7365,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" s="137" t="s">
         <v>79</v>
       </c>
@@ -7337,39 +7373,39 @@
         <v>327</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>87</v>
       </c>
       <c r="E26" s="138" t="s">
-        <v>360</v>
+        <v>53</v>
       </c>
       <c r="F26" s="134" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="137" t="s">
         <v>79</v>
       </c>
       <c r="B27" s="132" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>329</v>
+        <v>359</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>87</v>
       </c>
       <c r="E27" s="138" t="s">
-        <v>53</v>
+        <v>360</v>
       </c>
       <c r="F27" s="134" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="137" t="s">
         <v>79</v>
       </c>
@@ -7377,7 +7413,7 @@
         <v>328</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>362</v>
+        <v>329</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>87</v>
@@ -7389,7 +7425,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="137" t="s">
         <v>79</v>
       </c>
@@ -7397,39 +7433,39 @@
         <v>328</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>87</v>
       </c>
       <c r="E29" s="138" t="s">
-        <v>360</v>
+        <v>53</v>
       </c>
       <c r="F29" s="134" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" s="137" t="s">
         <v>79</v>
       </c>
       <c r="B30" s="132" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>330</v>
+        <v>363</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>87</v>
       </c>
       <c r="E30" s="138" t="s">
-        <v>53</v>
+        <v>360</v>
       </c>
       <c r="F30" s="134" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A31" s="137" t="s">
         <v>79</v>
       </c>
@@ -7437,7 +7473,7 @@
         <v>330</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>364</v>
+        <v>330</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>87</v>
@@ -7449,7 +7485,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" s="137" t="s">
         <v>79</v>
       </c>
@@ -7457,16 +7493,16 @@
         <v>330</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>87</v>
       </c>
       <c r="E32" s="138" t="s">
-        <v>360</v>
+        <v>53</v>
       </c>
       <c r="F32" s="134" t="s">
-        <v>361</v>
+        <v>54</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -7474,19 +7510,19 @@
         <v>79</v>
       </c>
       <c r="B33" s="132" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>331</v>
+        <v>365</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>87</v>
       </c>
       <c r="E33" s="138" t="s">
-        <v>53</v>
+        <v>360</v>
       </c>
       <c r="F33" s="134" t="s">
-        <v>54</v>
+        <v>361</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -7497,7 +7533,7 @@
         <v>331</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>366</v>
+        <v>331</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>87</v>
@@ -7517,16 +7553,16 @@
         <v>331</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>87</v>
       </c>
       <c r="E35" s="138" t="s">
-        <v>360</v>
+        <v>53</v>
       </c>
       <c r="F35" s="134" t="s">
-        <v>361</v>
+        <v>54</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -7534,19 +7570,19 @@
         <v>79</v>
       </c>
       <c r="B36" s="132" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>332</v>
+        <v>367</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>87</v>
       </c>
       <c r="E36" s="138" t="s">
-        <v>53</v>
+        <v>360</v>
       </c>
       <c r="F36" s="134" t="s">
-        <v>55</v>
+        <v>361</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -7557,7 +7593,7 @@
         <v>332</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>368</v>
+        <v>332</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>87</v>
@@ -7577,16 +7613,16 @@
         <v>332</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>87</v>
       </c>
       <c r="E38" s="138" t="s">
-        <v>360</v>
+        <v>53</v>
       </c>
       <c r="F38" s="134" t="s">
-        <v>370</v>
+        <v>55</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -7594,28 +7630,30 @@
         <v>79</v>
       </c>
       <c r="B39" s="132" t="s">
-        <v>86</v>
+        <v>332</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>56</v>
+        <v>369</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="E39" s="136" t="s">
-        <v>57</v>
-      </c>
-      <c r="F39" s="134"/>
+        <v>87</v>
+      </c>
+      <c r="E39" s="138" t="s">
+        <v>360</v>
+      </c>
+      <c r="F39" s="134" t="s">
+        <v>370</v>
+      </c>
     </row>
     <row r="40" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="137" t="s">
         <v>79</v>
       </c>
       <c r="B40" s="132" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>73</v>
@@ -7630,10 +7668,10 @@
         <v>79</v>
       </c>
       <c r="B41" s="132" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>73</v>
@@ -7648,10 +7686,10 @@
         <v>79</v>
       </c>
       <c r="B42" s="132" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>73</v>
@@ -7666,10 +7704,10 @@
         <v>79</v>
       </c>
       <c r="B43" s="132" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>73</v>
@@ -7684,10 +7722,10 @@
         <v>79</v>
       </c>
       <c r="B44" s="132" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>73</v>
@@ -7702,10 +7740,10 @@
         <v>79</v>
       </c>
       <c r="B45" s="132" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>73</v>
@@ -7720,10 +7758,10 @@
         <v>79</v>
       </c>
       <c r="B46" s="132" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>73</v>
@@ -7738,10 +7776,10 @@
         <v>79</v>
       </c>
       <c r="B47" s="132" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>73</v>
@@ -7756,10 +7794,10 @@
         <v>79</v>
       </c>
       <c r="B48" s="132" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>73</v>
@@ -7771,16 +7809,16 @@
     </row>
     <row r="49" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A49" s="137" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B49" s="132" t="s">
-        <v>333</v>
+        <v>80</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="D49" s="139" t="s">
-        <v>334</v>
+        <v>63</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>73</v>
       </c>
       <c r="E49" s="136" t="s">
         <v>57</v>
@@ -7788,26 +7826,24 @@
       <c r="F49" s="134"/>
     </row>
     <row r="50" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A50" s="137" t="s">
+      <c r="A50" s="181" t="s">
         <v>75</v>
       </c>
-      <c r="B50" s="132" t="s">
-        <v>335</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>336</v>
-      </c>
-      <c r="D50" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="E50" s="136" t="s">
+      <c r="B50" s="182" t="s">
+        <v>377</v>
+      </c>
+      <c r="C50" s="183" t="s">
+        <v>376</v>
+      </c>
+      <c r="D50" s="183" t="s">
+        <v>73</v>
+      </c>
+      <c r="E50" s="184" t="s">
         <v>57</v>
       </c>
-      <c r="F50" s="134" t="s">
-        <v>69</v>
-      </c>
+      <c r="F50" s="185"/>
       <c r="G50" s="35" t="s">
-        <v>353</v>
+        <v>375</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="16" x14ac:dyDescent="0.2">
@@ -7815,72 +7851,74 @@
         <v>75</v>
       </c>
       <c r="B51" s="132" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>372</v>
-      </c>
-      <c r="D51" s="2" t="s">
-        <v>88</v>
+        <v>67</v>
+      </c>
+      <c r="D51" s="139" t="s">
+        <v>334</v>
       </c>
       <c r="E51" s="136" t="s">
         <v>57</v>
       </c>
-      <c r="F51" s="134" t="s">
-        <v>69</v>
-      </c>
-      <c r="G51" s="35" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F51" s="134"/>
+    </row>
+    <row r="52" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A52" s="137" t="s">
         <v>75</v>
       </c>
       <c r="B52" s="132" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="D52" s="139" t="s">
-        <v>73</v>
+        <v>336</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>88</v>
       </c>
       <c r="E52" s="136" t="s">
         <v>57</v>
       </c>
-      <c r="F52" s="134"/>
+      <c r="F52" s="134" t="s">
+        <v>69</v>
+      </c>
       <c r="G52" s="35" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A53" s="137" t="s">
         <v>75</v>
       </c>
       <c r="B53" s="132" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D53" s="139" t="s">
-        <v>73</v>
+        <v>372</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>88</v>
       </c>
       <c r="E53" s="136" t="s">
         <v>57</v>
       </c>
-      <c r="F53" s="134"/>
+      <c r="F53" s="134" t="s">
+        <v>69</v>
+      </c>
+      <c r="G53" s="35" t="s">
+        <v>373</v>
+      </c>
     </row>
     <row r="54" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="137" t="s">
         <v>75</v>
       </c>
       <c r="B54" s="132" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="D54" s="139" t="s">
         <v>73</v>
@@ -7889,16 +7927,19 @@
         <v>57</v>
       </c>
       <c r="F54" s="134"/>
+      <c r="G54" s="35" t="s">
+        <v>354</v>
+      </c>
     </row>
     <row r="55" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="137" t="s">
         <v>75</v>
       </c>
       <c r="B55" s="132" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D55" s="139" t="s">
         <v>73</v>
@@ -7909,37 +7950,58 @@
       <c r="F55" s="134"/>
     </row>
     <row r="56" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="140" t="s">
+      <c r="A56" s="137" t="s">
         <v>75</v>
       </c>
-      <c r="B56" s="141" t="s">
-        <v>341</v>
-      </c>
-      <c r="C56" s="142" t="s">
-        <v>70</v>
+      <c r="B56" s="132" t="s">
+        <v>339</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>65</v>
       </c>
       <c r="D56" s="139" t="s">
         <v>73</v>
       </c>
-      <c r="E56" s="143" t="s">
+      <c r="E56" s="136" t="s">
         <v>57</v>
       </c>
-      <c r="F56" s="144"/>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A57" s="43"/>
-      <c r="B57" s="42"/>
-      <c r="C57" s="42"/>
-      <c r="D57" s="42"/>
-      <c r="E57" s="42"/>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A58" s="43"/>
-      <c r="B58" s="42"/>
-      <c r="C58" s="42"/>
-      <c r="D58" s="42"/>
-      <c r="E58" s="42"/>
-      <c r="F58" s="40"/>
+      <c r="F56" s="134"/>
+    </row>
+    <row r="57" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A57" s="137" t="s">
+        <v>75</v>
+      </c>
+      <c r="B57" s="132" t="s">
+        <v>340</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D57" s="139" t="s">
+        <v>73</v>
+      </c>
+      <c r="E57" s="136" t="s">
+        <v>57</v>
+      </c>
+      <c r="F57" s="134"/>
+    </row>
+    <row r="58" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A58" s="140" t="s">
+        <v>75</v>
+      </c>
+      <c r="B58" s="141" t="s">
+        <v>341</v>
+      </c>
+      <c r="C58" s="142" t="s">
+        <v>70</v>
+      </c>
+      <c r="D58" s="139" t="s">
+        <v>73</v>
+      </c>
+      <c r="E58" s="143" t="s">
+        <v>57</v>
+      </c>
+      <c r="F58" s="144"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A59" s="43"/>
@@ -7947,7 +8009,6 @@
       <c r="C59" s="42"/>
       <c r="D59" s="42"/>
       <c r="E59" s="42"/>
-      <c r="F59" s="40"/>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A60" s="43"/>
@@ -7974,60 +8035,58 @@
       <c r="F62" s="40"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A63" s="44"/>
+      <c r="A63" s="43"/>
+      <c r="B63" s="42"/>
+      <c r="C63" s="42"/>
       <c r="D63" s="42"/>
       <c r="E63" s="42"/>
+      <c r="F63" s="40"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A64" s="44"/>
+      <c r="A64" s="43"/>
+      <c r="B64" s="42"/>
+      <c r="C64" s="42"/>
       <c r="D64" s="42"/>
       <c r="E64" s="42"/>
-      <c r="F64" s="36"/>
+      <c r="F64" s="40"/>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A65" s="44"/>
       <c r="D65" s="42"/>
       <c r="E65" s="42"/>
-      <c r="F65" s="40"/>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A66" s="49"/>
-      <c r="B66" s="48"/>
-      <c r="C66" s="48"/>
-      <c r="D66" s="48"/>
-      <c r="E66" s="47"/>
-      <c r="F66" s="37"/>
-    </row>
-    <row r="67" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A67" s="46"/>
-      <c r="B67" s="45"/>
-      <c r="C67" s="45"/>
-      <c r="D67" s="45"/>
-      <c r="G67" s="36"/>
-    </row>
-    <row r="68" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A68" s="44"/>
-    </row>
-    <row r="69" spans="1:7" s="36" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="41"/>
+      <c r="A66" s="44"/>
+      <c r="D66" s="42"/>
+      <c r="E66" s="42"/>
+      <c r="F66" s="36"/>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A67" s="44"/>
+      <c r="D67" s="42"/>
+      <c r="E67" s="42"/>
+      <c r="F67" s="40"/>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A68" s="49"/>
+      <c r="B68" s="48"/>
+      <c r="C68" s="48"/>
+      <c r="D68" s="48"/>
+      <c r="E68" s="47"/>
+      <c r="F68" s="37"/>
+    </row>
+    <row r="69" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A69" s="46"/>
+      <c r="B69" s="45"/>
+      <c r="C69" s="45"/>
+      <c r="D69" s="45"/>
+      <c r="G69" s="36"/>
     </row>
     <row r="70" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A70" s="43"/>
-      <c r="B70" s="42"/>
-      <c r="C70" s="42"/>
-      <c r="D70" s="42"/>
-      <c r="E70" s="42"/>
-      <c r="F70" s="42"/>
-      <c r="G70" s="36"/>
-    </row>
-    <row r="71" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="43"/>
-      <c r="B71" s="42"/>
-      <c r="C71" s="42"/>
-      <c r="D71" s="42"/>
-      <c r="E71" s="42"/>
-      <c r="F71" s="42"/>
-      <c r="G71" s="36"/>
+      <c r="A70" s="44"/>
+    </row>
+    <row r="71" spans="1:7" s="36" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A71" s="41"/>
     </row>
     <row r="72" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="43"/>
@@ -8039,11 +8098,11 @@
       <c r="G72" s="36"/>
     </row>
     <row r="73" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A73" s="91"/>
-      <c r="B73" s="92"/>
-      <c r="C73" s="92"/>
-      <c r="D73" s="92"/>
-      <c r="E73" s="92"/>
+      <c r="A73" s="43"/>
+      <c r="B73" s="42"/>
+      <c r="C73" s="42"/>
+      <c r="D73" s="42"/>
+      <c r="E73" s="42"/>
       <c r="F73" s="42"/>
       <c r="G73" s="36"/>
     </row>
@@ -8053,15 +8112,17 @@
       <c r="C74" s="42"/>
       <c r="D74" s="42"/>
       <c r="E74" s="42"/>
+      <c r="F74" s="42"/>
       <c r="G74" s="36"/>
     </row>
     <row r="75" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A75" s="43"/>
-      <c r="B75" s="42"/>
-      <c r="C75" s="42"/>
-      <c r="D75" s="42"/>
-      <c r="E75" s="42"/>
+      <c r="A75" s="91"/>
+      <c r="B75" s="92"/>
+      <c r="C75" s="92"/>
+      <c r="D75" s="92"/>
+      <c r="E75" s="92"/>
       <c r="F75" s="42"/>
+      <c r="G75" s="36"/>
     </row>
     <row r="76" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="43"/>
@@ -8069,25 +8130,41 @@
       <c r="C76" s="42"/>
       <c r="D76" s="42"/>
       <c r="E76" s="42"/>
-      <c r="F76" s="42"/>
+      <c r="G76" s="36"/>
     </row>
     <row r="77" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A77" s="41"/>
-      <c r="B77" s="36"/>
-      <c r="C77" s="36"/>
-      <c r="D77" s="36"/>
-      <c r="E77" s="36"/>
-      <c r="F77" s="40"/>
-      <c r="G77" s="36"/>
+      <c r="A77" s="43"/>
+      <c r="B77" s="42"/>
+      <c r="C77" s="42"/>
+      <c r="D77" s="42"/>
+      <c r="E77" s="42"/>
+      <c r="F77" s="42"/>
     </row>
     <row r="78" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A78" s="39"/>
-      <c r="B78" s="38"/>
-      <c r="C78" s="38"/>
-      <c r="D78" s="38"/>
-      <c r="E78" s="38"/>
-      <c r="F78" s="37"/>
-      <c r="G78" s="36"/>
+      <c r="A78" s="43"/>
+      <c r="B78" s="42"/>
+      <c r="C78" s="42"/>
+      <c r="D78" s="42"/>
+      <c r="E78" s="42"/>
+      <c r="F78" s="42"/>
+    </row>
+    <row r="79" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A79" s="41"/>
+      <c r="B79" s="36"/>
+      <c r="C79" s="36"/>
+      <c r="D79" s="36"/>
+      <c r="E79" s="36"/>
+      <c r="F79" s="40"/>
+      <c r="G79" s="36"/>
+    </row>
+    <row r="80" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A80" s="39"/>
+      <c r="B80" s="38"/>
+      <c r="C80" s="38"/>
+      <c r="D80" s="38"/>
+      <c r="E80" s="38"/>
+      <c r="F80" s="37"/>
+      <c r="G80" s="36"/>
     </row>
   </sheetData>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>

<commit_message>
hide tab extractor CA
</commit_message>
<xml_diff>
--- a/front/src/assets/template4CA.xlsx
+++ b/front/src/assets/template4CA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC82489D-FECF-8F41-BD85-8DA2F8E9FD60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{896F4498-4BDF-2249-9C96-9F745064010A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
   <sheets>
     <sheet name="ACCUEIL" sheetId="33" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <sheet name="codage tribunal" sheetId="12" state="hidden" r:id="rId5"/>
     <sheet name="Juridictions" sheetId="17" state="hidden" r:id="rId6"/>
     <sheet name="Table_Fonctions" sheetId="19" state="hidden" r:id="rId7"/>
-    <sheet name="ETPT_CA_JUR" sheetId="30" r:id="rId8"/>
+    <sheet name="ETPT_CA_JUR" sheetId="30" state="hidden" r:id="rId8"/>
     <sheet name="ETPT_CA_JUR_DDG" sheetId="25" r:id="rId9"/>
     <sheet name="ETPT_CA_JUR Corresp" sheetId="38" state="hidden" r:id="rId10"/>
   </sheets>

</xml_diff>

<commit_message>
update menu déroulant JA
</commit_message>
<xml_diff>
--- a/front/src/assets/template4CA.xlsx
+++ b/front/src/assets/template4CA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAF39370-4BCF-7C41-BDA0-61B4BDD022F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15666CDA-98BA-8C4E-9634-66219B71164B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -27,7 +27,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ETPT A-JUST'!$A$2:$DN$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ETPT Format DDG'!$A$2:$DT$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Table_Fonctions!$A$1:$F$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Table_Fonctions!$A$1:$F$83</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="824" uniqueCount="380">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="838" uniqueCount="381">
   <si>
     <t>#! END_ROW</t>
   </si>
@@ -2433,15 +2433,6 @@
     <t>Indisponibilité des placés à reporter sur le SAR, ligne "Etpt placés absents non affectés", colonne ABC-BUR</t>
   </si>
   <si>
-    <t>manque : JURISTE AS chambres sociales</t>
-  </si>
-  <si>
-    <t>manque : JURISTE AS parquet général</t>
-  </si>
-  <si>
-    <t>manque : Magistrat placé SUB</t>
-  </si>
-  <si>
     <t xml:space="preserve">                Déclaration des ETPT CA</t>
   </si>
   <si>
@@ -2487,21 +2478,12 @@
     <t>Fonctionnaire CTECH placé SUB</t>
   </si>
   <si>
-    <t>manque : VPP add / sub et JP add / sub</t>
-  </si>
-  <si>
     <t>JA Siège autres</t>
   </si>
   <si>
-    <t>ajouter ? JA Pôle Social,JA Parquet,JA JP,JA VIF</t>
-  </si>
-  <si>
     <t>A GREFFIER</t>
   </si>
   <si>
-    <t>à valider</t>
-  </si>
-  <si>
     <t>Att. J</t>
   </si>
   <si>
@@ -2512,6 +2494,27 @@
   </si>
   <si>
     <t>Pas encore appelé dans la matrice DDG, à voir lors de la publication de la prochaine circulaire 2025/2026</t>
+  </si>
+  <si>
+    <t>JURISTE AS chambres sociales</t>
+  </si>
+  <si>
+    <t>JURISTE AS parquet général</t>
+  </si>
+  <si>
+    <t>JA Chambres Sociales</t>
+  </si>
+  <si>
+    <t>JA Siège Autres</t>
+  </si>
+  <si>
+    <t>JA Parquet Général</t>
+  </si>
+  <si>
+    <t>manque : Magistrat placé SUB en attente de retour d'Aurélie</t>
+  </si>
+  <si>
+    <t>manque : VPP add / sub et JP add / sub en attente de retour d'Aurélie</t>
   </si>
 </sst>
 </file>
@@ -4265,8 +4268,8 @@
       <xdr:rowOff>28222</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>1326444</xdr:colOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1086556</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>976232</xdr:rowOff>
     </xdr:to>
@@ -6463,7 +6466,7 @@
   <dimension ref="A1:X7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="32.5" customWidth="1"/>
+    <col min="1" max="1" width="32.5" hidden="1" customWidth="1"/>
     <col min="2" max="2" width="4.6640625" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="38.33203125" hidden="1" customWidth="1"/>
     <col min="4" max="4" width="51.83203125" customWidth="1"/>
@@ -6857,7 +6860,7 @@
   <sheetPr codeName="Feuil14">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G80"/>
+  <dimension ref="A1:G83"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.83203125" style="35" bestFit="1" customWidth="1"/>
@@ -7030,7 +7033,7 @@
         <v>38</v>
       </c>
       <c r="G8" s="35" t="s">
-        <v>355</v>
+        <v>379</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="16" x14ac:dyDescent="0.2">
@@ -7053,7 +7056,7 @@
         <v>38</v>
       </c>
       <c r="G9" s="35" t="s">
-        <v>371</v>
+        <v>380</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="16" x14ac:dyDescent="0.2">
@@ -7188,7 +7191,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="137" t="s">
         <v>79</v>
       </c>
@@ -7208,7 +7211,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="137" t="s">
         <v>79</v>
       </c>
@@ -7228,15 +7231,15 @@
         <v>46</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="153" t="s">
         <v>79</v>
       </c>
       <c r="B19" s="154" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="C19" s="155" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="D19" s="155" t="s">
         <v>88</v>
@@ -7247,11 +7250,8 @@
       <c r="F19" s="157" t="s">
         <v>46</v>
       </c>
-      <c r="G19" s="35" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    </row>
+    <row r="20" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="137" t="s">
         <v>79</v>
       </c>
@@ -7271,7 +7271,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" s="137" t="s">
         <v>79</v>
       </c>
@@ -7291,7 +7291,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" s="137" t="s">
         <v>79</v>
       </c>
@@ -7311,7 +7311,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="137" t="s">
         <v>79</v>
       </c>
@@ -7331,7 +7331,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="137" t="s">
         <v>79</v>
       </c>
@@ -7351,7 +7351,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="137" t="s">
         <v>79</v>
       </c>
@@ -7371,7 +7371,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" s="137" t="s">
         <v>79</v>
       </c>
@@ -7379,7 +7379,7 @@
         <v>327</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>87</v>
@@ -7391,7 +7391,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="137" t="s">
         <v>79</v>
       </c>
@@ -7399,19 +7399,19 @@
         <v>327</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>87</v>
       </c>
       <c r="E27" s="138" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="F27" s="134" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="137" t="s">
         <v>79</v>
       </c>
@@ -7431,7 +7431,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="137" t="s">
         <v>79</v>
       </c>
@@ -7439,7 +7439,7 @@
         <v>328</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>87</v>
@@ -7451,7 +7451,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" s="137" t="s">
         <v>79</v>
       </c>
@@ -7459,19 +7459,19 @@
         <v>328</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>87</v>
       </c>
       <c r="E30" s="138" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="F30" s="134" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A31" s="137" t="s">
         <v>79</v>
       </c>
@@ -7491,7 +7491,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" s="137" t="s">
         <v>79</v>
       </c>
@@ -7499,7 +7499,7 @@
         <v>330</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>87</v>
@@ -7519,16 +7519,16 @@
         <v>330</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>87</v>
       </c>
       <c r="E33" s="138" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="F33" s="134" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -7559,7 +7559,7 @@
         <v>331</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>87</v>
@@ -7579,16 +7579,16 @@
         <v>331</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>87</v>
       </c>
       <c r="E36" s="138" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="F36" s="134" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -7619,7 +7619,7 @@
         <v>332</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>87</v>
@@ -7639,16 +7639,16 @@
         <v>332</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>87</v>
       </c>
       <c r="E39" s="138" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="F39" s="134" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -7836,10 +7836,10 @@
         <v>75</v>
       </c>
       <c r="B50" s="154" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="C50" s="155" t="s">
-        <v>376</v>
+        <v>370</v>
       </c>
       <c r="D50" s="155" t="s">
         <v>73</v>
@@ -7848,10 +7848,10 @@
         <v>57</v>
       </c>
       <c r="F50" s="157" t="s">
-        <v>378</v>
+        <v>372</v>
       </c>
       <c r="G50" s="35" t="s">
-        <v>379</v>
+        <v>373</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="16" x14ac:dyDescent="0.2">
@@ -7880,7 +7880,7 @@
         <v>335</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>336</v>
+        <v>376</v>
       </c>
       <c r="D52" s="2" t="s">
         <v>88</v>
@@ -7889,10 +7889,7 @@
         <v>57</v>
       </c>
       <c r="F52" s="134" t="s">
-        <v>69</v>
-      </c>
-      <c r="G52" s="35" t="s">
-        <v>353</v>
+        <v>374</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="16" x14ac:dyDescent="0.2">
@@ -7903,7 +7900,7 @@
         <v>335</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>372</v>
+        <v>377</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>88</v>
@@ -7914,76 +7911,76 @@
       <c r="F53" s="134" t="s">
         <v>69</v>
       </c>
-      <c r="G53" s="35" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="54" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A54" s="137" t="s">
         <v>75</v>
       </c>
       <c r="B54" s="132" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="D54" s="139" t="s">
-        <v>73</v>
+        <v>378</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>88</v>
       </c>
       <c r="E54" s="136" t="s">
         <v>57</v>
       </c>
-      <c r="F54" s="134"/>
-      <c r="G54" s="35" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F54" s="134" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A55" s="137" t="s">
         <v>75</v>
       </c>
       <c r="B55" s="132" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D55" s="139" t="s">
-        <v>73</v>
+        <v>336</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>88</v>
       </c>
       <c r="E55" s="136" t="s">
         <v>57</v>
       </c>
-      <c r="F55" s="134"/>
-    </row>
-    <row r="56" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F55" s="134" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A56" s="137" t="s">
         <v>75</v>
       </c>
       <c r="B56" s="132" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D56" s="139" t="s">
-        <v>73</v>
+        <v>368</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>88</v>
       </c>
       <c r="E56" s="136" t="s">
         <v>57</v>
       </c>
-      <c r="F56" s="134"/>
+      <c r="F56" s="134" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="57" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="137" t="s">
         <v>75</v>
       </c>
       <c r="B57" s="132" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D57" s="139" t="s">
         <v>73</v>
@@ -7994,45 +7991,76 @@
       <c r="F57" s="134"/>
     </row>
     <row r="58" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="140" t="s">
+      <c r="A58" s="137" t="s">
         <v>75</v>
       </c>
-      <c r="B58" s="141" t="s">
-        <v>341</v>
-      </c>
-      <c r="C58" s="142" t="s">
-        <v>70</v>
+      <c r="B58" s="132" t="s">
+        <v>338</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>64</v>
       </c>
       <c r="D58" s="139" t="s">
         <v>73</v>
       </c>
-      <c r="E58" s="143" t="s">
+      <c r="E58" s="136" t="s">
         <v>57</v>
       </c>
-      <c r="F58" s="144"/>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A59" s="43"/>
-      <c r="B59" s="42"/>
-      <c r="C59" s="42"/>
-      <c r="D59" s="42"/>
-      <c r="E59" s="42"/>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A60" s="43"/>
-      <c r="B60" s="42"/>
-      <c r="C60" s="42"/>
-      <c r="D60" s="42"/>
-      <c r="E60" s="42"/>
-      <c r="F60" s="40"/>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A61" s="43"/>
-      <c r="B61" s="42"/>
-      <c r="C61" s="42"/>
-      <c r="D61" s="42"/>
-      <c r="E61" s="42"/>
-      <c r="F61" s="40"/>
+      <c r="F58" s="134"/>
+    </row>
+    <row r="59" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A59" s="137" t="s">
+        <v>75</v>
+      </c>
+      <c r="B59" s="132" t="s">
+        <v>339</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D59" s="139" t="s">
+        <v>73</v>
+      </c>
+      <c r="E59" s="136" t="s">
+        <v>57</v>
+      </c>
+      <c r="F59" s="134"/>
+    </row>
+    <row r="60" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A60" s="137" t="s">
+        <v>75</v>
+      </c>
+      <c r="B60" s="132" t="s">
+        <v>340</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D60" s="139" t="s">
+        <v>73</v>
+      </c>
+      <c r="E60" s="136" t="s">
+        <v>57</v>
+      </c>
+      <c r="F60" s="134"/>
+    </row>
+    <row r="61" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A61" s="140" t="s">
+        <v>75</v>
+      </c>
+      <c r="B61" s="141" t="s">
+        <v>341</v>
+      </c>
+      <c r="C61" s="142" t="s">
+        <v>70</v>
+      </c>
+      <c r="D61" s="139" t="s">
+        <v>73</v>
+      </c>
+      <c r="E61" s="143" t="s">
+        <v>57</v>
+      </c>
+      <c r="F61" s="144"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A62" s="43"/>
@@ -8040,7 +8068,6 @@
       <c r="C62" s="42"/>
       <c r="D62" s="42"/>
       <c r="E62" s="42"/>
-      <c r="F62" s="40"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A63" s="43"/>
@@ -8059,76 +8086,73 @@
       <c r="F64" s="40"/>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A65" s="44"/>
+      <c r="A65" s="43"/>
+      <c r="B65" s="42"/>
+      <c r="C65" s="42"/>
       <c r="D65" s="42"/>
       <c r="E65" s="42"/>
+      <c r="F65" s="40"/>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A66" s="44"/>
+      <c r="A66" s="43"/>
+      <c r="B66" s="42"/>
+      <c r="C66" s="42"/>
       <c r="D66" s="42"/>
       <c r="E66" s="42"/>
-      <c r="F66" s="36"/>
+      <c r="F66" s="40"/>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A67" s="44"/>
+      <c r="A67" s="43"/>
+      <c r="B67" s="42"/>
+      <c r="C67" s="42"/>
       <c r="D67" s="42"/>
       <c r="E67" s="42"/>
       <c r="F67" s="40"/>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A68" s="49"/>
-      <c r="B68" s="48"/>
-      <c r="C68" s="48"/>
-      <c r="D68" s="48"/>
-      <c r="E68" s="47"/>
-      <c r="F68" s="37"/>
-    </row>
-    <row r="69" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="46"/>
-      <c r="B69" s="45"/>
-      <c r="C69" s="45"/>
-      <c r="D69" s="45"/>
-      <c r="G69" s="36"/>
-    </row>
-    <row r="70" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A68" s="44"/>
+      <c r="D68" s="42"/>
+      <c r="E68" s="42"/>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A69" s="44"/>
+      <c r="D69" s="42"/>
+      <c r="E69" s="42"/>
+      <c r="F69" s="36"/>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A70" s="44"/>
-    </row>
-    <row r="71" spans="1:7" s="36" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="41"/>
+      <c r="D70" s="42"/>
+      <c r="E70" s="42"/>
+      <c r="F70" s="40"/>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A71" s="49"/>
+      <c r="B71" s="48"/>
+      <c r="C71" s="48"/>
+      <c r="D71" s="48"/>
+      <c r="E71" s="47"/>
+      <c r="F71" s="37"/>
     </row>
     <row r="72" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A72" s="43"/>
-      <c r="B72" s="42"/>
-      <c r="C72" s="42"/>
-      <c r="D72" s="42"/>
-      <c r="E72" s="42"/>
-      <c r="F72" s="42"/>
+      <c r="A72" s="46"/>
+      <c r="B72" s="45"/>
+      <c r="C72" s="45"/>
+      <c r="D72" s="45"/>
       <c r="G72" s="36"/>
     </row>
     <row r="73" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A73" s="43"/>
-      <c r="B73" s="42"/>
-      <c r="C73" s="42"/>
-      <c r="D73" s="42"/>
-      <c r="E73" s="42"/>
-      <c r="F73" s="42"/>
-      <c r="G73" s="36"/>
-    </row>
-    <row r="74" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A74" s="43"/>
-      <c r="B74" s="42"/>
-      <c r="C74" s="42"/>
-      <c r="D74" s="42"/>
-      <c r="E74" s="42"/>
-      <c r="F74" s="42"/>
-      <c r="G74" s="36"/>
+      <c r="A73" s="44"/>
+    </row>
+    <row r="74" spans="1:7" s="36" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A74" s="41"/>
     </row>
     <row r="75" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A75" s="91"/>
-      <c r="B75" s="92"/>
-      <c r="C75" s="92"/>
-      <c r="D75" s="92"/>
-      <c r="E75" s="92"/>
+      <c r="A75" s="43"/>
+      <c r="B75" s="42"/>
+      <c r="C75" s="42"/>
+      <c r="D75" s="42"/>
+      <c r="E75" s="42"/>
       <c r="F75" s="42"/>
       <c r="G75" s="36"/>
     </row>
@@ -8138,6 +8162,7 @@
       <c r="C76" s="42"/>
       <c r="D76" s="42"/>
       <c r="E76" s="42"/>
+      <c r="F76" s="42"/>
       <c r="G76" s="36"/>
     </row>
     <row r="77" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -8147,32 +8172,58 @@
       <c r="D77" s="42"/>
       <c r="E77" s="42"/>
       <c r="F77" s="42"/>
+      <c r="G77" s="36"/>
     </row>
     <row r="78" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A78" s="43"/>
-      <c r="B78" s="42"/>
-      <c r="C78" s="42"/>
-      <c r="D78" s="42"/>
-      <c r="E78" s="42"/>
+      <c r="A78" s="91"/>
+      <c r="B78" s="92"/>
+      <c r="C78" s="92"/>
+      <c r="D78" s="92"/>
+      <c r="E78" s="92"/>
       <c r="F78" s="42"/>
+      <c r="G78" s="36"/>
     </row>
     <row r="79" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A79" s="41"/>
-      <c r="B79" s="36"/>
-      <c r="C79" s="36"/>
-      <c r="D79" s="36"/>
-      <c r="E79" s="36"/>
-      <c r="F79" s="40"/>
+      <c r="A79" s="43"/>
+      <c r="B79" s="42"/>
+      <c r="C79" s="42"/>
+      <c r="D79" s="42"/>
+      <c r="E79" s="42"/>
       <c r="G79" s="36"/>
     </row>
     <row r="80" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A80" s="39"/>
-      <c r="B80" s="38"/>
-      <c r="C80" s="38"/>
-      <c r="D80" s="38"/>
-      <c r="E80" s="38"/>
-      <c r="F80" s="37"/>
-      <c r="G80" s="36"/>
+      <c r="A80" s="43"/>
+      <c r="B80" s="42"/>
+      <c r="C80" s="42"/>
+      <c r="D80" s="42"/>
+      <c r="E80" s="42"/>
+      <c r="F80" s="42"/>
+    </row>
+    <row r="81" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A81" s="43"/>
+      <c r="B81" s="42"/>
+      <c r="C81" s="42"/>
+      <c r="D81" s="42"/>
+      <c r="E81" s="42"/>
+      <c r="F81" s="42"/>
+    </row>
+    <row r="82" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A82" s="41"/>
+      <c r="B82" s="36"/>
+      <c r="C82" s="36"/>
+      <c r="D82" s="36"/>
+      <c r="E82" s="36"/>
+      <c r="F82" s="40"/>
+      <c r="G82" s="36"/>
+    </row>
+    <row r="83" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A83" s="39"/>
+      <c r="B83" s="38"/>
+      <c r="C83" s="38"/>
+      <c r="D83" s="38"/>
+      <c r="E83" s="38"/>
+      <c r="F83" s="37"/>
+      <c r="G83" s="36"/>
     </row>
   </sheetData>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -8507,7 +8558,7 @@
       <c r="B5" s="54"/>
       <c r="C5" s="54"/>
       <c r="D5" s="60" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="E5" s="146" t="s">
         <v>117</v>
@@ -9694,12 +9745,12 @@
   <sheetData>
     <row r="1" spans="1:31" ht="87" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
       <c r="D1" s="3" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="E1" s="7"/>
       <c r="F1" s="6"/>

</xml_diff>

<commit_message>
add fix agregat placé CA
</commit_message>
<xml_diff>
--- a/front/src/assets/template4CA.xlsx
+++ b/front/src/assets/template4CA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBB0B10B-3D41-0E43-BFAB-7C7A4C31C851}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DEB85F7-B5BB-F443-95DF-E2870479884F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -6152,7 +6152,7 @@
         <v>138</v>
       </c>
       <c r="G6" s="19" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FF,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"M-TIT",'ETPT Format DDG'!$C:$C,$A$3)</f>
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FF,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"M-TIT",'ETPT Format DDG'!$C:$C,$A$3)</f>
         <v>#N/A</v>
       </c>
       <c r="H6" s="91" t="str">
@@ -6160,11 +6160,11 @@
         <v/>
       </c>
       <c r="I6" s="18" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FF,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"M-PLAC-ADD",'ETPT Format DDG'!$C:$C,$A$3)</f>
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FF,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"M-PLAC-ADD",'ETPT Format DDG'!$C:$C,$A$3)</f>
         <v>#N/A</v>
       </c>
       <c r="J6" s="18" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FF,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"M-PLAC-SUB",'ETPT Format DDG'!$C:$C,$A$3)</f>
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FF,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"M-PLAC-SUB",'ETPT Format DDG'!$C:$C,$A$3)</f>
         <v>#N/A</v>
       </c>
       <c r="K6" s="18" t="e">
@@ -6172,7 +6172,7 @@
 INDEX('ETPT Format DDG'!$A:$FF,
 ,
 IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))
-),'ETPT Format DDG'!$I:$I,"C",
+),'ETPT Format DDG'!$FG:$FG,"C",
 'ETPT Format DDG'!$C:$C,$A$3,
 'ETPT Format DDG'!$G:$G,"Magistrat")</f>
         <v>#N/A</v>
@@ -6192,7 +6192,7 @@
         <v/>
       </c>
       <c r="N6" s="18" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FF,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"F-TIT",'ETPT Format DDG'!$C:$C,$A$3)</f>
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FF,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"F-TIT",'ETPT Format DDG'!$C:$C,$A$3)</f>
         <v>#N/A</v>
       </c>
       <c r="O6" s="91" t="str">
@@ -6200,15 +6200,15 @@
         <v/>
       </c>
       <c r="P6" s="18" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FF,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"F-PLAC-ADD",'ETPT Format DDG'!$C:$C,$A$3)</f>
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FF,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"F-PLAC-ADD",'ETPT Format DDG'!$C:$C,$A$3)</f>
         <v>#N/A</v>
       </c>
       <c r="Q6" s="18" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FF,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"F-PLAC-SUB",'ETPT Format DDG'!$C:$C,$A$3)</f>
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FF,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"F-PLAC-SUB",'ETPT Format DDG'!$C:$C,$A$3)</f>
         <v>#N/A</v>
       </c>
       <c r="R6" s="18" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FF,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"C",'ETPT Format DDG'!$C:$C,$A$3,'ETPT Format DDG'!$G:$G,"Greffe")</f>
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FF,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"C",'ETPT Format DDG'!$C:$C,$A$3,'ETPT Format DDG'!$G:$G,"Greffe")</f>
         <v>#N/A</v>
       </c>
       <c r="S6" s="19" t="e">
@@ -6230,7 +6230,7 @@
 INDEX('ETPT Format DDG'!$A:$FF,
 ,
 IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))
-),'ETPT Format DDG'!$I:$I,"C",
+),'ETPT Format DDG'!$FG:$FG,"C",
 'ETPT Format DDG'!$C:$C,$A$3,
 'ETPT Format DDG'!$G:$G,"Autour du magistrat")</f>
         <v>#N/A</v>

</xml_diff>

<commit_message>
add contentieux mineur ca gap
</commit_message>
<xml_diff>
--- a/front/src/assets/template4CA.xlsx
+++ b/front/src/assets/template4CA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0860825-BB90-D143-A29B-F00B6CED0756}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2A27792-112A-FB4A-829B-B40BB5EEDBF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="40" yWindow="760" windowWidth="23880" windowHeight="17780" activeTab="2" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -3494,27 +3494,7 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{6FC886D6-2077-B34D-B1DF-739B068A66D1}"/>
     <cellStyle name="Normal 3" xfId="4" xr:uid="{6BD57324-3FD5-D341-A299-730D14794802}"/>
   </cellStyles>
-  <dxfs count="16">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="15">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -3654,6 +3634,16 @@
       <font>
         <color theme="0"/>
       </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -6027,7 +6017,7 @@
   <cols>
     <col min="1" max="1" width="18.6640625" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="16" max="16" width="0" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="10.83203125" customWidth="1"/>
     <col min="126" max="126" width="13.5" customWidth="1"/>
     <col min="127" max="127" width="15.83203125" customWidth="1"/>
     <col min="128" max="128" width="36.1640625" customWidth="1"/>
@@ -6110,7 +6100,7 @@
     <mergeCell ref="FA1:FF1"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:FF1048576">
-    <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
+    <cfRule type="expression" dxfId="14" priority="1" stopIfTrue="1">
       <formula>AND(OR($N1&lt;&gt;"-",$O1&lt;&gt;0,$P1&lt;&gt;0),ROW()&gt;2,$A1&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6420,64 +6410,64 @@
     <mergeCell ref="U4:V4"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:F4">
-    <cfRule type="expression" dxfId="15" priority="13">
+    <cfRule type="expression" dxfId="13" priority="13">
       <formula>IF(LEFT($A$3,2)&lt;&gt;"TJ",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:V151">
-    <cfRule type="expression" dxfId="14" priority="15">
+    <cfRule type="expression" dxfId="12" priority="15">
       <formula>AND(ISBLANK($C6)=FALSE,ISBLANK($E6)=TRUE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:F1048576">
-    <cfRule type="expression" dxfId="13" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="11" priority="11" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)+_xlfn.NUMBERVALUE($L4)-_xlfn.NUMBERVALUE($L5)+_xlfn.NUMBERVALUE($L6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="12">
+    <cfRule type="expression" dxfId="10" priority="12">
       <formula>AND($D1="7. TOTAL CONTENTIEUX DES MINEURS",OR(_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3))&lt;&gt;0,_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3))&lt;&gt;0,_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3))&lt;&gt;0))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D7:F7">
-    <cfRule type="expression" dxfId="11" priority="10" stopIfTrue="1">
+    <cfRule type="expression" dxfId="9" priority="10" stopIfTrue="1">
       <formula>OR(_xlfn.NUMBERVALUE($L6)&lt;&gt;_xlfn.NUMBERVALUE($L7),_xlfn.NUMBERVALUE($S6)&lt;&gt;_xlfn.NUMBERVALUE($S7),_xlfn.NUMBERVALUE($U6)&lt;&gt;_xlfn.NUMBERVALUE($U7))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:M1048576">
-    <cfRule type="expression" dxfId="10" priority="8" stopIfTrue="1">
+    <cfRule type="expression" dxfId="8" priority="8" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)+_xlfn.NUMBERVALUE($L4)+_xlfn.NUMBERVALUE($L5)+_xlfn.NUMBERVALUE($L6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="9">
+    <cfRule type="expression" dxfId="7" priority="9">
       <formula>AND($D1="7. TOTAL CONTENTIEUX DES MINEURS",_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3))&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G7:M7">
-    <cfRule type="expression" dxfId="8" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="6" priority="7" stopIfTrue="1">
       <formula>_xlfn.NUMBERVALUE($L7)&lt;&gt;_xlfn.NUMBERVALUE($L6)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1:T1048576">
-    <cfRule type="expression" dxfId="7" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="5" priority="5" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3)+_xlfn.NUMBERVALUE($S4)+_xlfn.NUMBERVALUE($S5)+_xlfn.NUMBERVALUE($S6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="4" priority="6" stopIfTrue="1">
       <formula>AND($D1="7. TOTAL CONTENTIEUX DES MINEURS",_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3))&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N7:T7">
-    <cfRule type="expression" dxfId="5" priority="4" stopIfTrue="1">
+    <cfRule type="expression" dxfId="3" priority="4" stopIfTrue="1">
       <formula>_xlfn.NUMBERVALUE($S7)&lt;&gt;_xlfn.NUMBERVALUE($S6)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U1:V1048576">
-    <cfRule type="expression" dxfId="4" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="2" priority="2" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3)+_xlfn.NUMBERVALUE($U4)+_xlfn.NUMBERVALUE($U5)+_xlfn.NUMBERVALUE($U6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="3">
+    <cfRule type="expression" dxfId="1" priority="3">
       <formula>AND($D1="7. TOTAL CONTENTIEUX DES MINEURS",_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3))&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U7:V7">
-    <cfRule type="expression" dxfId="2" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>_xlfn.NUMBERVALUE($U7)&lt;&gt;_xlfn.NUMBERVALUE($U6)</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
update extractors with automation
</commit_message>
<xml_diff>
--- a/front/src/assets/template4CA.xlsx
+++ b/front/src/assets/template4CA.xlsx
@@ -8,21 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2A27792-112A-FB4A-829B-B40BB5EEDBF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DE02AFD-3461-0B4A-A860-F79A1F0EC7C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="40" yWindow="760" windowWidth="23880" windowHeight="17780" activeTab="2" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
+    <workbookView xWindow="40" yWindow="760" windowWidth="23880" windowHeight="17780" firstSheet="2" activeTab="2" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
   <sheets>
     <sheet name="ACCUEIL" sheetId="33" r:id="rId1"/>
     <sheet name="ETPT A-JUST" sheetId="1" r:id="rId2"/>
     <sheet name="ETPT Format DDG" sheetId="9" r:id="rId3"/>
     <sheet name="Agrégats DDG" sheetId="10" r:id="rId4"/>
-    <sheet name="codage tribunal" sheetId="12" state="hidden" r:id="rId5"/>
-    <sheet name="Juridictions" sheetId="17" state="hidden" r:id="rId6"/>
-    <sheet name="Table_Fonctions" sheetId="19" state="hidden" r:id="rId7"/>
-    <sheet name="ETPT_CA_JUR" sheetId="30" state="hidden" r:id="rId8"/>
+    <sheet name="codage tribunal" sheetId="12" r:id="rId5"/>
+    <sheet name="Juridictions" sheetId="17" r:id="rId6"/>
+    <sheet name="Table_Fonctions" sheetId="19" r:id="rId7"/>
+    <sheet name="ETPT_CA_JUR" sheetId="30" r:id="rId8"/>
     <sheet name="ETPT_CA_JUR_DDG" sheetId="25" r:id="rId9"/>
-    <sheet name="ETPT_CA_JUR Corresp" sheetId="38" state="hidden" r:id="rId10"/>
+    <sheet name="ETPT_CA_JUR Corresp" sheetId="38" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ETPT A-JUST'!$A$2:$DN$2</definedName>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="263">
   <si>
     <t>#! END_ROW</t>
   </si>
@@ -380,9 +380,6 @@
   </si>
   <si>
     <t xml:space="preserve">                  Extracteur de données d'effectifs</t>
-  </si>
-  <si>
-    <t>RECAPITULATIF</t>
   </si>
   <si>
     <t>CPH détachés</t>
@@ -2115,21 +2112,6 @@
     <t>Correspondance</t>
   </si>
   <si>
-    <t>Temps ventilés sur la période (contentieux sociaux civils et commerciaux)</t>
-  </si>
-  <si>
-    <t>Temps ventilés sur la période (service pénal)</t>
-  </si>
-  <si>
-    <t>Temps ventilés sur la période (hors indisponibilité)</t>
-  </si>
-  <si>
-    <t>Temps ventilés sur la période (y.c. indisponibilité)</t>
-  </si>
-  <si>
-    <t>Soutien (Hors accueil du justiciable)</t>
-  </si>
-  <si>
     <t>PARQUET_JIRS</t>
   </si>
   <si>
@@ -2173,6 +2155,12 @@
   </si>
   <si>
     <t>#! FOR_EACH f fonctions</t>
+  </si>
+  <si>
+    <t>=ETPT_CA_JUR!D5</t>
+  </si>
+  <si>
+    <t>Fonction agrégats</t>
   </si>
 </sst>
 </file>
@@ -2188,7 +2176,7 @@
     <numFmt numFmtId="169" formatCode="#,##0.00_ ;[Red]\-#,##0.00\ "/>
     <numFmt numFmtId="170" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="47" x14ac:knownFonts="1">
+  <fonts count="46" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2366,14 +2354,6 @@
     </font>
     <font>
       <b/>
-      <sz val="20"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -2520,7 +2500,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="23">
+  <fills count="22">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2554,12 +2534,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF002060"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -3028,7 +3002,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="154">
+  <cellXfs count="153">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -3141,67 +3115,67 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="4" applyProtection="1">
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="11" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="11" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="11" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="11" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="9" borderId="11" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="19" fillId="8" borderId="11" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="9" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="19" fillId="8" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="9" borderId="11" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="20" fillId="8" borderId="11" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="9" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="22" fillId="8" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="49" fontId="24" fillId="13" borderId="11" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="24" fillId="12" borderId="11" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="28" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="27" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -3210,22 +3184,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="15" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="15" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
@@ -3237,7 +3211,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
@@ -3249,49 +3223,49 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="15" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="17" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="16" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="18" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="17" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="18" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="19" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="20" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="20" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="21" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="169" fontId="17" fillId="10" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="34" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="17" fillId="9" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="33" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="37" fillId="12" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="36" fillId="11" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="37" fillId="11" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="36" fillId="10" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="38" fillId="11" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="37" fillId="10" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="38" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="36" fillId="9" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="169" fontId="37" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="169" fontId="35" fillId="8" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="36" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="40" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3301,65 +3275,65 @@
     <xf numFmtId="166" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="39" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="38" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="170" fontId="39" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="38" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="39" fillId="0" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="38" fillId="0" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="39" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="38" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="41" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="40" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="39" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="40" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="39" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="40" fillId="9" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="39" fillId="8" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="42" fillId="9" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="41" fillId="8" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="42" fillId="9" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="41" fillId="8" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="42" fillId="9" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="41" fillId="8" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="19" fillId="9" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="37" fillId="8" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="19" fillId="8" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="36" fillId="7" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="44" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="43" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="34" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="33" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="34" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="33" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="169" fontId="19" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="42" fillId="9" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="41" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="45" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="44" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="44" fillId="8" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="45" fillId="9" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="46" fillId="10" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3368,22 +3342,22 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="22" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="21" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="9" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="20" fillId="8" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="9" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="8" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="10" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="9" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -3392,7 +3366,7 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -3401,10 +3375,10 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -3413,53 +3387,50 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="15" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="15" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3479,10 +3450,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="40" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="39" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3494,7 +3465,17 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{6FC886D6-2077-B34D-B1DF-739B068A66D1}"/>
     <cellStyle name="Normal 3" xfId="4" xr:uid="{6BD57324-3FD5-D341-A299-730D14794802}"/>
   </cellStyles>
-  <dxfs count="15">
+  <dxfs count="16">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -4411,10 +4392,10 @@
     <row r="1" spans="1:8" s="26" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="50"/>
       <c r="B1" s="51" t="s">
+        <v>111</v>
+      </c>
+      <c r="C1" s="126" t="s">
         <v>112</v>
-      </c>
-      <c r="C1" s="126" t="s">
-        <v>113</v>
       </c>
       <c r="D1" s="126"/>
       <c r="E1" s="126"/>
@@ -4427,7 +4408,7 @@
       <c r="A2" s="53"/>
       <c r="B2" s="54"/>
       <c r="C2" s="127" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D2" s="127"/>
       <c r="E2" s="127"/>
@@ -4446,16 +4427,16 @@
     <row r="4" spans="1:8" s="62" customFormat="1" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="59"/>
       <c r="B4" s="60" t="s">
+        <v>113</v>
+      </c>
+      <c r="C4" s="61" t="s">
         <v>114</v>
       </c>
-      <c r="C4" s="61" t="s">
+      <c r="D4" s="61" t="s">
         <v>115</v>
       </c>
-      <c r="D4" s="61" t="s">
+      <c r="E4" s="133" t="s">
         <v>116</v>
-      </c>
-      <c r="E4" s="133" t="s">
-        <v>117</v>
       </c>
       <c r="F4" s="134"/>
       <c r="G4" s="68"/>
@@ -4466,16 +4447,16 @@
     <row r="5" spans="1:8" s="26" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="57"/>
       <c r="B5" s="72" t="s">
+        <v>117</v>
+      </c>
+      <c r="C5" s="65" t="s">
         <v>118</v>
       </c>
-      <c r="C5" s="65" t="s">
+      <c r="D5" s="65" t="s">
         <v>119</v>
       </c>
-      <c r="D5" s="65" t="s">
-        <v>120</v>
-      </c>
       <c r="E5" s="135" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F5" s="136"/>
       <c r="G5" s="67"/>
@@ -4486,16 +4467,16 @@
     <row r="6" spans="1:8" s="26" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="57"/>
       <c r="B6" s="73" t="s">
+        <v>120</v>
+      </c>
+      <c r="C6" s="66" t="s">
         <v>121</v>
       </c>
-      <c r="C6" s="66" t="s">
+      <c r="D6" s="66" t="s">
         <v>122</v>
       </c>
-      <c r="D6" s="66" t="s">
-        <v>123</v>
-      </c>
       <c r="E6" s="137" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F6" s="138"/>
       <c r="G6" s="67"/>
@@ -4506,16 +4487,16 @@
     <row r="7" spans="1:8" s="26" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="57"/>
       <c r="B7" s="74" t="s">
+        <v>123</v>
+      </c>
+      <c r="C7" s="66" t="s">
         <v>124</v>
       </c>
-      <c r="C7" s="66" t="s">
+      <c r="D7" s="66" t="s">
         <v>125</v>
       </c>
-      <c r="D7" s="66" t="s">
-        <v>126</v>
-      </c>
       <c r="E7" s="137" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F7" s="138"/>
       <c r="G7" s="67"/>
@@ -4526,16 +4507,16 @@
     <row r="8" spans="1:8" s="26" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="57"/>
       <c r="B8" s="75" t="s">
+        <v>126</v>
+      </c>
+      <c r="C8" s="128" t="s">
         <v>127</v>
       </c>
-      <c r="C8" s="128" t="s">
+      <c r="D8" s="128" t="s">
         <v>128</v>
       </c>
-      <c r="D8" s="128" t="s">
-        <v>129</v>
-      </c>
       <c r="E8" s="139" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F8" s="140"/>
       <c r="G8" s="67"/>
@@ -4546,7 +4527,7 @@
     <row r="9" spans="1:8" s="26" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="57"/>
       <c r="B9" s="76" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C9" s="128"/>
       <c r="D9" s="128"/>
@@ -4560,7 +4541,7 @@
     <row r="10" spans="1:8" s="26" customFormat="1" ht="23" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="57"/>
       <c r="B10" s="77" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C10" s="129"/>
       <c r="D10" s="129"/>
@@ -4586,7 +4567,7 @@
       <c r="A12" s="57"/>
       <c r="B12" s="69"/>
       <c r="C12" s="132" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D12" s="132"/>
       <c r="E12" s="132"/>
@@ -4649,13 +4630,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A1" s="152" t="s">
-        <v>140</v>
-      </c>
-      <c r="B1" s="152"/>
-      <c r="C1" s="152"/>
-      <c r="D1" s="152"/>
-      <c r="E1" s="152"/>
+      <c r="A1" s="151" t="s">
+        <v>139</v>
+      </c>
+      <c r="B1" s="151"/>
+      <c r="C1" s="151"/>
+      <c r="D1" s="151"/>
+      <c r="E1" s="151"/>
       <c r="F1" s="96"/>
       <c r="G1" s="78"/>
       <c r="H1" s="78"/>
@@ -4687,7 +4668,7 @@
       <c r="G2" s="80" t="s">
         <v>106</v>
       </c>
-      <c r="H2" s="153" t="s">
+      <c r="H2" s="152" t="s">
         <v>105</v>
       </c>
       <c r="I2" s="80" t="s">
@@ -4708,7 +4689,7 @@
       <c r="N2" s="80" t="s">
         <v>104</v>
       </c>
-      <c r="O2" s="153" t="s">
+      <c r="O2" s="152" t="s">
         <v>103</v>
       </c>
       <c r="P2" s="80" t="s">
@@ -4720,7 +4701,7 @@
       <c r="R2" s="80" t="s">
         <v>38</v>
       </c>
-      <c r="S2" s="153" t="s">
+      <c r="S2" s="152" t="s">
         <v>102</v>
       </c>
       <c r="T2" s="80" t="s">
@@ -4738,7 +4719,7 @@
       <c r="X2" s="80" t="s">
         <v>101</v>
       </c>
-      <c r="Y2" s="153" t="s">
+      <c r="Y2" s="152" t="s">
         <v>100</v>
       </c>
     </row>
@@ -4752,7 +4733,7 @@
       <c r="G3" s="80" t="s">
         <v>97</v>
       </c>
-      <c r="H3" s="153"/>
+      <c r="H3" s="152"/>
       <c r="I3" s="80" t="s">
         <v>96</v>
       </c>
@@ -4763,17 +4744,17 @@
         <v>94</v>
       </c>
       <c r="L3" s="80" t="s">
+        <v>140</v>
+      </c>
+      <c r="M3" s="80" t="s">
         <v>141</v>
-      </c>
-      <c r="M3" s="80" t="s">
-        <v>142</v>
       </c>
       <c r="N3" s="80" t="s">
         <v>93</v>
       </c>
-      <c r="O3" s="153"/>
+      <c r="O3" s="152"/>
       <c r="P3" s="80" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="Q3" s="80" t="s">
         <v>91</v>
@@ -4781,7 +4762,7 @@
       <c r="R3" s="80" t="s">
         <v>92</v>
       </c>
-      <c r="S3" s="153"/>
+      <c r="S3" s="152"/>
       <c r="T3" s="80" t="s">
         <v>90</v>
       </c>
@@ -4789,15 +4770,15 @@
         <v>89</v>
       </c>
       <c r="V3" s="80" t="s">
+        <v>143</v>
+      </c>
+      <c r="W3" s="80" t="s">
         <v>144</v>
-      </c>
-      <c r="W3" s="80" t="s">
-        <v>145</v>
       </c>
       <c r="X3" s="80" t="s">
         <v>88</v>
       </c>
-      <c r="Y3" s="153"/>
+      <c r="Y3" s="152"/>
     </row>
     <row r="4" spans="1:25" ht="84" x14ac:dyDescent="0.2">
       <c r="A4" s="98"/>
@@ -4819,7 +4800,7 @@
       <c r="G4" s="80" t="s">
         <v>79</v>
       </c>
-      <c r="H4" s="153"/>
+      <c r="H4" s="152"/>
       <c r="I4" s="80" t="s">
         <v>78</v>
       </c>
@@ -4830,17 +4811,17 @@
         <v>76</v>
       </c>
       <c r="L4" s="80" t="s">
+        <v>145</v>
+      </c>
+      <c r="M4" s="80" t="s">
         <v>146</v>
-      </c>
-      <c r="M4" s="80" t="s">
-        <v>147</v>
       </c>
       <c r="N4" s="80" t="s">
         <v>75</v>
       </c>
-      <c r="O4" s="153"/>
+      <c r="O4" s="152"/>
       <c r="P4" s="80" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="Q4" s="80" t="s">
         <v>73</v>
@@ -4848,7 +4829,7 @@
       <c r="R4" s="80" t="s">
         <v>74</v>
       </c>
-      <c r="S4" s="153"/>
+      <c r="S4" s="152"/>
       <c r="T4" s="80" t="s">
         <v>72</v>
       </c>
@@ -4856,19 +4837,19 @@
         <v>71</v>
       </c>
       <c r="V4" s="80" t="s">
+        <v>148</v>
+      </c>
+      <c r="W4" s="80" t="s">
         <v>149</v>
-      </c>
-      <c r="W4" s="80" t="s">
-        <v>150</v>
       </c>
       <c r="X4" s="80" t="s">
         <v>70</v>
       </c>
-      <c r="Y4" s="153"/>
+      <c r="Y4" s="152"/>
     </row>
     <row r="5" spans="1:25" ht="332" x14ac:dyDescent="0.2">
       <c r="A5" s="100" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B5" s="101"/>
       <c r="C5" s="101"/>
@@ -4880,36 +4861,36 @@
         <v>64</v>
       </c>
       <c r="G5" s="81" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="H5" s="79">
         <f>SUMIF($G$2:G$2,G$2,$G5:G5)</f>
         <v>0</v>
       </c>
       <c r="I5" s="81" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="J5" s="83"/>
       <c r="K5" s="83"/>
       <c r="L5" s="83"/>
       <c r="M5" s="81" t="s">
+        <v>153</v>
+      </c>
+      <c r="N5" s="81" t="s">
         <v>154</v>
-      </c>
-      <c r="N5" s="81" t="s">
-        <v>155</v>
       </c>
       <c r="O5" s="79">
         <f>SUMIF($G$2:N$2,N$2,$G5:N5)</f>
         <v>0</v>
       </c>
       <c r="P5" s="81" t="s">
+        <v>155</v>
+      </c>
+      <c r="Q5" s="81" t="s">
         <v>156</v>
       </c>
-      <c r="Q5" s="81" t="s">
+      <c r="R5" s="81" t="s">
         <v>157</v>
-      </c>
-      <c r="R5" s="81" t="s">
-        <v>158</v>
       </c>
       <c r="S5" s="79">
         <f>SUMIF($G$2:R$2,R$2,$G5:R5)</f>
@@ -4919,10 +4900,10 @@
       <c r="U5" s="83"/>
       <c r="V5" s="83"/>
       <c r="W5" s="81" t="s">
+        <v>158</v>
+      </c>
+      <c r="X5" s="81" t="s">
         <v>159</v>
-      </c>
-      <c r="X5" s="81" t="s">
-        <v>160</v>
       </c>
       <c r="Y5" s="79">
         <f>SUMIF($G$2:X$2,X$2,$G5:X5)</f>
@@ -4931,7 +4912,7 @@
     </row>
     <row r="6" spans="1:25" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A6" s="100" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B6" s="101"/>
       <c r="C6" s="101"/>
@@ -4943,7 +4924,7 @@
         <v>62</v>
       </c>
       <c r="G6" s="81" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="H6" s="79">
         <f>SUMIF($G$2:G$2,G$2,$G6:G6)</f>
@@ -4951,47 +4932,47 @@
       </c>
       <c r="I6" s="82"/>
       <c r="J6" s="81" t="s">
+        <v>161</v>
+      </c>
+      <c r="K6" s="81" t="s">
         <v>162</v>
       </c>
-      <c r="K6" s="81" t="s">
+      <c r="L6" s="81" t="s">
         <v>163</v>
-      </c>
-      <c r="L6" s="81" t="s">
-        <v>164</v>
       </c>
       <c r="M6" s="83"/>
       <c r="N6" s="81" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="O6" s="79">
         <f>SUMIF($G$2:N$2,N$2,$G6:N6)</f>
         <v>0</v>
       </c>
       <c r="P6" s="81" t="s">
+        <v>165</v>
+      </c>
+      <c r="Q6" s="81" t="s">
         <v>166</v>
       </c>
-      <c r="Q6" s="81" t="s">
+      <c r="R6" s="81" t="s">
         <v>167</v>
-      </c>
-      <c r="R6" s="81" t="s">
-        <v>168</v>
       </c>
       <c r="S6" s="79">
         <f>SUMIF($G$2:R$2,R$2,$G6:R6)</f>
         <v>0</v>
       </c>
       <c r="T6" s="81" t="s">
+        <v>168</v>
+      </c>
+      <c r="U6" s="81" t="s">
         <v>169</v>
       </c>
-      <c r="U6" s="81" t="s">
+      <c r="V6" s="81" t="s">
         <v>170</v>
-      </c>
-      <c r="V6" s="81" t="s">
-        <v>171</v>
       </c>
       <c r="W6" s="83"/>
       <c r="X6" s="81" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="Y6" s="79">
         <f>SUMIF($G$2:X$2,X$2,$G6:X6)</f>
@@ -5000,7 +4981,7 @@
     </row>
     <row r="7" spans="1:25" ht="90" x14ac:dyDescent="0.2">
       <c r="A7" s="100" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B7" s="101"/>
       <c r="C7" s="101"/>
@@ -5038,7 +5019,7 @@
       <c r="V7" s="103"/>
       <c r="W7" s="103"/>
       <c r="X7" s="104" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="Y7" s="79">
         <f>SUMIF($G$2:X$2,X$2,$G7:X7)</f>
@@ -5047,7 +5028,7 @@
     </row>
     <row r="8" spans="1:25" ht="140" x14ac:dyDescent="0.2">
       <c r="A8" s="100" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B8" s="101"/>
       <c r="C8" s="101"/>
@@ -5059,7 +5040,7 @@
         <v>58</v>
       </c>
       <c r="G8" s="81" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="H8" s="79">
         <f>SUMIF($G$2:G$2,G$2,$G8:G8)</f>
@@ -5071,20 +5052,20 @@
       <c r="L8" s="85"/>
       <c r="M8" s="85"/>
       <c r="N8" s="81" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="O8" s="79">
         <f>SUMIF($G$2:N$2,N$2,$G8:N8)</f>
         <v>0</v>
       </c>
       <c r="P8" s="81" t="s">
+        <v>175</v>
+      </c>
+      <c r="Q8" s="81" t="s">
         <v>176</v>
       </c>
-      <c r="Q8" s="81" t="s">
+      <c r="R8" s="81" t="s">
         <v>177</v>
-      </c>
-      <c r="R8" s="81" t="s">
-        <v>178</v>
       </c>
       <c r="S8" s="79">
         <f>SUMIF($G$2:R$2,R$2,$G8:R8)</f>
@@ -5095,7 +5076,7 @@
       <c r="V8" s="103"/>
       <c r="W8" s="103"/>
       <c r="X8" s="81" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="Y8" s="79">
         <f>SUMIF($G$2:X$2,X$2,$G8:X8)</f>
@@ -5104,7 +5085,7 @@
     </row>
     <row r="9" spans="1:25" ht="154" x14ac:dyDescent="0.2">
       <c r="A9" s="100" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B9" s="101"/>
       <c r="C9" s="101"/>
@@ -5116,7 +5097,7 @@
         <v>56</v>
       </c>
       <c r="G9" s="81" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="H9" s="79">
         <f>SUMIF($G$2:G$2,G$2,$G9:G9)</f>
@@ -5128,20 +5109,20 @@
       <c r="L9" s="85"/>
       <c r="M9" s="85"/>
       <c r="N9" s="81" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="O9" s="79">
         <f>SUMIF($G$2:N$2,N$2,$G9:N9)</f>
         <v>0</v>
       </c>
       <c r="P9" s="81" t="s">
+        <v>181</v>
+      </c>
+      <c r="Q9" s="81" t="s">
         <v>182</v>
       </c>
-      <c r="Q9" s="81" t="s">
+      <c r="R9" s="81" t="s">
         <v>183</v>
-      </c>
-      <c r="R9" s="81" t="s">
-        <v>184</v>
       </c>
       <c r="S9" s="79">
         <f>SUMIF($G$2:R$2,R$2,$G9:R9)</f>
@@ -5152,7 +5133,7 @@
       <c r="V9" s="103"/>
       <c r="W9" s="103"/>
       <c r="X9" s="81" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="Y9" s="79">
         <f>SUMIF($G$2:X$2,X$2,$G9:X9)</f>
@@ -5161,7 +5142,7 @@
     </row>
     <row r="10" spans="1:25" ht="140" x14ac:dyDescent="0.2">
       <c r="A10" s="100" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B10" s="101"/>
       <c r="C10" s="101"/>
@@ -5173,7 +5154,7 @@
         <v>54</v>
       </c>
       <c r="G10" s="81" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="H10" s="79">
         <f>SUMIF($G$2:G$2,G$2,$G10:G10)</f>
@@ -5185,20 +5166,20 @@
       <c r="L10" s="85"/>
       <c r="M10" s="85"/>
       <c r="N10" s="81" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="O10" s="79">
         <f>SUMIF($G$2:N$2,N$2,$G10:N10)</f>
         <v>0</v>
       </c>
       <c r="P10" s="81" t="s">
+        <v>187</v>
+      </c>
+      <c r="Q10" s="81" t="s">
         <v>188</v>
       </c>
-      <c r="Q10" s="81" t="s">
+      <c r="R10" s="81" t="s">
         <v>189</v>
-      </c>
-      <c r="R10" s="81" t="s">
-        <v>190</v>
       </c>
       <c r="S10" s="79">
         <f>SUMIF($G$2:R$2,R$2,$G10:R10)</f>
@@ -5209,7 +5190,7 @@
       <c r="V10" s="103"/>
       <c r="W10" s="103"/>
       <c r="X10" s="81" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="Y10" s="79">
         <f>SUMIF($G$2:X$2,X$2,$G10:X10)</f>
@@ -5218,7 +5199,7 @@
     </row>
     <row r="11" spans="1:25" ht="140" x14ac:dyDescent="0.2">
       <c r="A11" s="100" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B11" s="101"/>
       <c r="C11" s="101"/>
@@ -5230,7 +5211,7 @@
         <v>52</v>
       </c>
       <c r="G11" s="81" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="H11" s="79">
         <f>SUMIF($G$2:G$2,G$2,$G11:G11)</f>
@@ -5242,20 +5223,20 @@
       <c r="L11" s="85"/>
       <c r="M11" s="85"/>
       <c r="N11" s="81" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="O11" s="79">
         <f>SUMIF($G$2:N$2,N$2,$G11:N11)</f>
         <v>0</v>
       </c>
       <c r="P11" s="81" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q11" s="81" t="s">
         <v>194</v>
       </c>
-      <c r="Q11" s="81" t="s">
+      <c r="R11" s="81" t="s">
         <v>195</v>
-      </c>
-      <c r="R11" s="81" t="s">
-        <v>196</v>
       </c>
       <c r="S11" s="79">
         <f>SUMIF($G$2:R$2,R$2,$G11:R11)</f>
@@ -5266,7 +5247,7 @@
       <c r="V11" s="103"/>
       <c r="W11" s="103"/>
       <c r="X11" s="81" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="Y11" s="79">
         <f>SUMIF($G$2:X$2,X$2,$G11:X11)</f>
@@ -5275,7 +5256,7 @@
     </row>
     <row r="12" spans="1:25" ht="168" x14ac:dyDescent="0.2">
       <c r="A12" s="100" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B12" s="101"/>
       <c r="C12" s="101"/>
@@ -5287,7 +5268,7 @@
         <v>50</v>
       </c>
       <c r="G12" s="81" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="H12" s="79">
         <f>SUMIF($G$2:G$2,G$2,$G12:G12)</f>
@@ -5299,20 +5280,20 @@
       <c r="L12" s="85"/>
       <c r="M12" s="85"/>
       <c r="N12" s="81" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="O12" s="79">
         <f>SUMIF($G$2:N$2,N$2,$G12:N12)</f>
         <v>0</v>
       </c>
       <c r="P12" s="81" t="s">
+        <v>199</v>
+      </c>
+      <c r="Q12" s="81" t="s">
         <v>200</v>
       </c>
-      <c r="Q12" s="81" t="s">
+      <c r="R12" s="81" t="s">
         <v>201</v>
-      </c>
-      <c r="R12" s="81" t="s">
-        <v>202</v>
       </c>
       <c r="S12" s="79">
         <f>SUMIF($G$2:R$2,R$2,$G12:R12)</f>
@@ -5323,7 +5304,7 @@
       <c r="V12" s="103"/>
       <c r="W12" s="103"/>
       <c r="X12" s="81" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="Y12" s="79">
         <f>SUMIF($G$2:X$2,X$2,$G12:X12)</f>
@@ -5332,7 +5313,7 @@
     </row>
     <row r="13" spans="1:25" ht="126" x14ac:dyDescent="0.2">
       <c r="A13" s="100" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B13" s="101"/>
       <c r="C13" s="101"/>
@@ -5344,7 +5325,7 @@
         <v>48</v>
       </c>
       <c r="G13" s="81" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="H13" s="79">
         <f>SUMIF($G$2:G$2,G$2,$G13:G13)</f>
@@ -5356,20 +5337,20 @@
       <c r="L13" s="85"/>
       <c r="M13" s="85"/>
       <c r="N13" s="81" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="O13" s="79">
         <f>SUMIF($G$2:N$2,N$2,$G13:N13)</f>
         <v>0</v>
       </c>
       <c r="P13" s="81" t="s">
+        <v>205</v>
+      </c>
+      <c r="Q13" s="81" t="s">
         <v>206</v>
       </c>
-      <c r="Q13" s="81" t="s">
+      <c r="R13" s="81" t="s">
         <v>207</v>
-      </c>
-      <c r="R13" s="81" t="s">
-        <v>208</v>
       </c>
       <c r="S13" s="79">
         <f>SUMIF($G$2:R$2,R$2,$G13:R13)</f>
@@ -5380,7 +5361,7 @@
       <c r="V13" s="103"/>
       <c r="W13" s="103"/>
       <c r="X13" s="81" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="Y13" s="79">
         <f>SUMIF($G$2:X$2,X$2,$G13:X13)</f>
@@ -5389,7 +5370,7 @@
     </row>
     <row r="14" spans="1:25" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A14" s="100" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B14" s="101"/>
       <c r="C14" s="101"/>
@@ -5401,61 +5382,61 @@
         <v>46</v>
       </c>
       <c r="G14" s="81" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H14" s="79">
         <f>SUMIF($G$2:G$2,G$2,$G14:G14)</f>
         <v>0</v>
       </c>
       <c r="I14" s="81" t="s">
+        <v>210</v>
+      </c>
+      <c r="J14" s="81" t="s">
         <v>211</v>
       </c>
-      <c r="J14" s="81" t="s">
+      <c r="K14" s="81" t="s">
         <v>212</v>
       </c>
-      <c r="K14" s="81" t="s">
+      <c r="L14" s="81" t="s">
         <v>213</v>
       </c>
-      <c r="L14" s="81" t="s">
+      <c r="M14" s="81" t="s">
         <v>214</v>
       </c>
-      <c r="M14" s="81" t="s">
+      <c r="N14" s="81" t="s">
         <v>215</v>
-      </c>
-      <c r="N14" s="81" t="s">
-        <v>216</v>
       </c>
       <c r="O14" s="79">
         <f>SUMIF($G$2:N$2,N$2,$G14:N14)</f>
         <v>0</v>
       </c>
       <c r="P14" s="81" t="s">
+        <v>216</v>
+      </c>
+      <c r="Q14" s="81" t="s">
         <v>217</v>
       </c>
-      <c r="Q14" s="81" t="s">
+      <c r="R14" s="81" t="s">
         <v>218</v>
-      </c>
-      <c r="R14" s="81" t="s">
-        <v>219</v>
       </c>
       <c r="S14" s="79">
         <f>SUMIF($G$2:R$2,R$2,$G14:R14)</f>
         <v>0</v>
       </c>
       <c r="T14" s="81" t="s">
+        <v>219</v>
+      </c>
+      <c r="U14" s="81" t="s">
         <v>220</v>
       </c>
-      <c r="U14" s="81" t="s">
+      <c r="V14" s="81" t="s">
         <v>221</v>
       </c>
-      <c r="V14" s="81" t="s">
+      <c r="W14" s="81" t="s">
         <v>222</v>
       </c>
-      <c r="W14" s="81" t="s">
+      <c r="X14" s="81" t="s">
         <v>223</v>
-      </c>
-      <c r="X14" s="81" t="s">
-        <v>224</v>
       </c>
       <c r="Y14" s="79">
         <f>SUMIF($G$2:X$2,X$2,$G14:X14)</f>
@@ -5464,16 +5445,16 @@
     </row>
     <row r="15" spans="1:25" ht="224" x14ac:dyDescent="0.2">
       <c r="A15" s="100" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B15" s="101"/>
       <c r="C15" s="101"/>
       <c r="D15" s="101"/>
       <c r="E15" s="101" t="s">
+        <v>224</v>
+      </c>
+      <c r="F15" s="105" t="s">
         <v>225</v>
-      </c>
-      <c r="F15" s="105" t="s">
-        <v>226</v>
       </c>
       <c r="G15" s="106"/>
       <c r="H15" s="79">
@@ -5491,13 +5472,13 @@
         <v>0</v>
       </c>
       <c r="P15" s="81" t="s">
+        <v>226</v>
+      </c>
+      <c r="Q15" s="81" t="s">
         <v>227</v>
       </c>
-      <c r="Q15" s="81" t="s">
+      <c r="R15" s="81" t="s">
         <v>228</v>
-      </c>
-      <c r="R15" s="81" t="s">
-        <v>229</v>
       </c>
       <c r="S15" s="79">
         <f>SUMIF($G$2:R$2,R$2,$G15:R15)</f>
@@ -5508,7 +5489,7 @@
       <c r="V15" s="108"/>
       <c r="W15" s="108"/>
       <c r="X15" s="81" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="Y15" s="79">
         <f>SUMIF($G$2:X$2,X$2,$G15:X15)</f>
@@ -5517,7 +5498,7 @@
     </row>
     <row r="16" spans="1:25" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A16" s="100" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B16" s="101"/>
       <c r="C16" s="101"/>
@@ -5529,61 +5510,61 @@
         <v>44</v>
       </c>
       <c r="G16" s="81" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H16" s="79">
         <f>SUMIF($G$2:G$2,G$2,$G16:G16)</f>
         <v>0</v>
       </c>
       <c r="I16" s="81" t="s">
+        <v>231</v>
+      </c>
+      <c r="J16" s="81" t="s">
         <v>232</v>
       </c>
-      <c r="J16" s="81" t="s">
+      <c r="K16" s="81" t="s">
         <v>233</v>
       </c>
-      <c r="K16" s="81" t="s">
+      <c r="L16" s="81" t="s">
         <v>234</v>
       </c>
-      <c r="L16" s="81" t="s">
+      <c r="M16" s="81" t="s">
         <v>235</v>
       </c>
-      <c r="M16" s="81" t="s">
+      <c r="N16" s="81" t="s">
         <v>236</v>
-      </c>
-      <c r="N16" s="81" t="s">
-        <v>237</v>
       </c>
       <c r="O16" s="79">
         <f>SUMIF($G$2:N$2,N$2,$G16:N16)</f>
         <v>0</v>
       </c>
       <c r="P16" s="81" t="s">
+        <v>237</v>
+      </c>
+      <c r="Q16" s="81" t="s">
         <v>238</v>
       </c>
-      <c r="Q16" s="81" t="s">
+      <c r="R16" s="81" t="s">
         <v>239</v>
-      </c>
-      <c r="R16" s="81" t="s">
-        <v>240</v>
       </c>
       <c r="S16" s="79">
         <f>SUMIF($G$2:R$2,R$2,$G16:R16)</f>
         <v>0</v>
       </c>
       <c r="T16" s="81" t="s">
+        <v>240</v>
+      </c>
+      <c r="U16" s="81" t="s">
         <v>241</v>
       </c>
-      <c r="U16" s="81" t="s">
+      <c r="V16" s="81" t="s">
         <v>242</v>
       </c>
-      <c r="V16" s="81" t="s">
+      <c r="W16" s="81" t="s">
         <v>243</v>
       </c>
-      <c r="W16" s="81" t="s">
+      <c r="X16" s="81" t="s">
         <v>244</v>
-      </c>
-      <c r="X16" s="81" t="s">
-        <v>245</v>
       </c>
       <c r="Y16" s="79">
         <f>SUMIF($G$2:X$2,X$2,$G16:X16)</f>
@@ -6012,7 +5993,7 @@
   <sheetPr codeName="Feuil13">
     <tabColor rgb="FF2C45E0"/>
   </sheetPr>
-  <dimension ref="A1:FG4"/>
+  <dimension ref="A1:FB4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.6640625" customWidth="1"/>
@@ -6024,13 +6005,11 @@
     <col min="129" max="155" width="16.83203125" customWidth="1"/>
     <col min="156" max="156" width="20" customWidth="1"/>
     <col min="157" max="157" width="17" customWidth="1"/>
-    <col min="161" max="161" width="17.33203125" customWidth="1"/>
-    <col min="162" max="162" width="17.1640625" bestFit="1" customWidth="1"/>
-    <col min="169" max="169" width="45.1640625" bestFit="1" customWidth="1"/>
-    <col min="170" max="170" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="164" max="164" width="45.1640625" bestFit="1" customWidth="1"/>
+    <col min="165" max="165" width="15.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:163" s="4" customFormat="1" ht="80" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:158" s="4" customFormat="1" ht="80" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>108</v>
       </c>
@@ -6042,19 +6021,14 @@
       <c r="G1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="FA1" s="145" t="s">
-        <v>110</v>
-      </c>
-      <c r="FB1" s="145"/>
-      <c r="FC1" s="145"/>
-      <c r="FD1" s="145"/>
-      <c r="FE1" s="145"/>
-      <c r="FF1" s="145"/>
-      <c r="FG1" s="8" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:163" ht="66" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="FA1" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="FB1" s="8" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:158" ht="66" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="22" t="s">
         <v>8</v>
       </c>
@@ -6065,22 +6039,10 @@
         <v>34</v>
       </c>
       <c r="FB2" s="48" t="s">
-        <v>247</v>
-      </c>
-      <c r="FC2" s="48" t="s">
-        <v>248</v>
-      </c>
-      <c r="FD2" s="48" t="s">
-        <v>249</v>
-      </c>
-      <c r="FE2" s="48" t="s">
-        <v>250</v>
-      </c>
-      <c r="FF2" s="48" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="3" spans="1:163" x14ac:dyDescent="0.2">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="3" spans="1:158" x14ac:dyDescent="0.2">
       <c r="A3" s="25" t="s">
         <v>11</v>
       </c>
@@ -6088,7 +6050,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:163" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:158" x14ac:dyDescent="0.2">
       <c r="B4" s="27" t="s">
         <v>7</v>
       </c>
@@ -6096,12 +6058,14 @@
     </row>
   </sheetData>
   <autoFilter ref="A2:DT2" xr:uid="{3B89445B-6ECC-4440-B85C-E593AE209933}"/>
-  <mergeCells count="1">
-    <mergeCell ref="FA1:FF1"/>
-  </mergeCells>
-  <conditionalFormatting sqref="A1:FF1048576">
-    <cfRule type="expression" dxfId="14" priority="1" stopIfTrue="1">
+  <conditionalFormatting sqref="A2:FA1048576 A1:EZ1">
+    <cfRule type="expression" dxfId="15" priority="2" stopIfTrue="1">
       <formula>AND(OR($N1&lt;&gt;"-",$O1&lt;&gt;0,$P1&lt;&gt;0),ROW()&gt;2,$A1&lt;&gt;"")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="FB2">
+    <cfRule type="expression" dxfId="0" priority="1" stopIfTrue="1">
+      <formula>AND(OR($N2&lt;&gt;"-",$O2&lt;&gt;0,$P2&lt;&gt;0),ROW()&gt;2,$A2&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6137,7 +6101,7 @@
       <c r="A1" s="3"/>
       <c r="B1" s="5"/>
       <c r="C1" s="64" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D1" s="64"/>
       <c r="E1" s="7"/>
@@ -6192,28 +6156,28 @@
       <c r="D4" s="87"/>
       <c r="E4" s="87"/>
       <c r="F4" s="87"/>
-      <c r="G4" s="146" t="s">
+      <c r="G4" s="145" t="s">
         <v>26</v>
       </c>
-      <c r="H4" s="147"/>
-      <c r="I4" s="147"/>
-      <c r="J4" s="147"/>
-      <c r="K4" s="147"/>
-      <c r="L4" s="148"/>
-      <c r="M4" s="149"/>
-      <c r="N4" s="150" t="s">
+      <c r="H4" s="146"/>
+      <c r="I4" s="146"/>
+      <c r="J4" s="146"/>
+      <c r="K4" s="146"/>
+      <c r="L4" s="147"/>
+      <c r="M4" s="148"/>
+      <c r="N4" s="149" t="s">
         <v>27</v>
       </c>
-      <c r="O4" s="148"/>
-      <c r="P4" s="148"/>
-      <c r="Q4" s="148"/>
-      <c r="R4" s="148"/>
-      <c r="S4" s="148"/>
-      <c r="T4" s="151"/>
-      <c r="U4" s="146" t="s">
+      <c r="O4" s="147"/>
+      <c r="P4" s="147"/>
+      <c r="Q4" s="147"/>
+      <c r="R4" s="147"/>
+      <c r="S4" s="147"/>
+      <c r="T4" s="150"/>
+      <c r="U4" s="145" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="149"/>
+      <c r="V4" s="148"/>
       <c r="W4" s="94"/>
       <c r="X4" t="s">
         <v>0</v>
@@ -6228,7 +6192,7 @@
         <v>13</v>
       </c>
       <c r="H5" s="93" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I5" s="12" t="s">
         <v>14</v>
@@ -6243,13 +6207,13 @@
         <v>30</v>
       </c>
       <c r="M5" s="90" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="N5" s="12" t="s">
         <v>16</v>
       </c>
       <c r="O5" s="93" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="P5" s="12" t="s">
         <v>17</v>
@@ -6264,13 +6228,13 @@
         <v>31</v>
       </c>
       <c r="T5" s="93" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="U5" s="89" t="s">
         <v>29</v>
       </c>
       <c r="V5" s="90" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="W5" t="s">
         <v>20</v>
@@ -6282,16 +6246,16 @@
         <v>23</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E6" s="16" t="s">
         <v>22</v>
       </c>
       <c r="F6" s="125" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G6" s="19" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FF,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"M-TIT",'ETPT Format DDG'!$C:$C,$A$3)</f>
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FA,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FB:$FB,"M-TIT",'ETPT Format DDG'!$C:$C,$A$3)</f>
         <v>#N/A</v>
       </c>
       <c r="H6" s="91" t="str">
@@ -6299,26 +6263,26 @@
         <v/>
       </c>
       <c r="I6" s="18" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FF,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"M-PLAC-ADD",'ETPT Format DDG'!$C:$C,$A$3)</f>
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FA,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FB:$FB,"M-PLAC-ADD",'ETPT Format DDG'!$C:$C,$A$3)</f>
         <v>#N/A</v>
       </c>
       <c r="J6" s="18" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FF,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"M-PLAC-SUB",'ETPT Format DDG'!$C:$C,$A$3)</f>
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FA,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FB:$FB,"M-PLAC-SUB",'ETPT Format DDG'!$C:$C,$A$3)</f>
         <v>#N/A</v>
       </c>
       <c r="K6" s="18" t="e">
         <f>SUMIFS(
-INDEX('ETPT Format DDG'!$A:$FF,
+INDEX('ETPT Format DDG'!$A:$FA,
 ,
 IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))
-),'ETPT Format DDG'!$FG:$FG,"C",
+),'ETPT Format DDG'!$FB:$FB,"C",
 'ETPT Format DDG'!$C:$C,$A$3,
 'ETPT Format DDG'!$G:$G,"Magistrat")</f>
         <v>#N/A</v>
       </c>
       <c r="L6" s="19" t="e">
         <f>SUMIFS(
-INDEX('ETPT Format DDG'!$A:$FF,
+INDEX('ETPT Format DDG'!$A:$FA,
 ,
 IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))
 ),
@@ -6331,7 +6295,7 @@
         <v/>
       </c>
       <c r="N6" s="18" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FF,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"F-TIT",'ETPT Format DDG'!$C:$C,$A$3)</f>
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FA,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FB:$FB,"F-TIT",'ETPT Format DDG'!$C:$C,$A$3)</f>
         <v>#N/A</v>
       </c>
       <c r="O6" s="91" t="str">
@@ -6339,20 +6303,20 @@
         <v/>
       </c>
       <c r="P6" s="18" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FF,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"F-PLAC-ADD",'ETPT Format DDG'!$C:$C,$A$3)</f>
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FA,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FB:$FB,"F-PLAC-ADD",'ETPT Format DDG'!$C:$C,$A$3)</f>
         <v>#N/A</v>
       </c>
       <c r="Q6" s="18" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FF,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"F-PLAC-SUB",'ETPT Format DDG'!$C:$C,$A$3)</f>
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FA,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FB:$FB,"F-PLAC-SUB",'ETPT Format DDG'!$C:$C,$A$3)</f>
         <v>#N/A</v>
       </c>
       <c r="R6" s="18" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FF,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"C",'ETPT Format DDG'!$C:$C,$A$3,'ETPT Format DDG'!$G:$G,"Greffe")</f>
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FA,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FB:$FB,"C",'ETPT Format DDG'!$C:$C,$A$3,'ETPT Format DDG'!$G:$G,"Greffe")</f>
         <v>#N/A</v>
       </c>
       <c r="S6" s="19" t="e">
         <f>SUMIFS(
-INDEX('ETPT Format DDG'!$A:$FF,
+INDEX('ETPT Format DDG'!$A:$FA,
 ,
 IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))
 ),
@@ -6366,10 +6330,10 @@
       </c>
       <c r="U6" s="19" t="e">
         <f>SUMIFS(
-INDEX('ETPT Format DDG'!$A:$FF,
+INDEX('ETPT Format DDG'!$A:$FA,
 ,
 IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))
-),'ETPT Format DDG'!$FG:$FG,"C",
+),'ETPT Format DDG'!$FB:$FB,"C",
 'ETPT Format DDG'!$C:$C,$A$3,
 'ETPT Format DDG'!$G:$G,"Autour du magistrat")</f>
         <v>#N/A</v>
@@ -6410,64 +6374,64 @@
     <mergeCell ref="U4:V4"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:F4">
-    <cfRule type="expression" dxfId="13" priority="13">
+    <cfRule type="expression" dxfId="14" priority="13">
       <formula>IF(LEFT($A$3,2)&lt;&gt;"TJ",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:V151">
-    <cfRule type="expression" dxfId="12" priority="15">
+    <cfRule type="expression" dxfId="13" priority="15">
       <formula>AND(ISBLANK($C6)=FALSE,ISBLANK($E6)=TRUE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:F1048576">
-    <cfRule type="expression" dxfId="11" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="12" priority="11" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)+_xlfn.NUMBERVALUE($L4)-_xlfn.NUMBERVALUE($L5)+_xlfn.NUMBERVALUE($L6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="12">
+    <cfRule type="expression" dxfId="11" priority="12">
       <formula>AND($D1="7. TOTAL CONTENTIEUX DES MINEURS",OR(_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3))&lt;&gt;0,_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3))&lt;&gt;0,_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3))&lt;&gt;0))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D7:F7">
-    <cfRule type="expression" dxfId="9" priority="10" stopIfTrue="1">
+    <cfRule type="expression" dxfId="10" priority="10" stopIfTrue="1">
       <formula>OR(_xlfn.NUMBERVALUE($L6)&lt;&gt;_xlfn.NUMBERVALUE($L7),_xlfn.NUMBERVALUE($S6)&lt;&gt;_xlfn.NUMBERVALUE($S7),_xlfn.NUMBERVALUE($U6)&lt;&gt;_xlfn.NUMBERVALUE($U7))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:M1048576">
-    <cfRule type="expression" dxfId="8" priority="8" stopIfTrue="1">
+    <cfRule type="expression" dxfId="9" priority="8" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)+_xlfn.NUMBERVALUE($L4)+_xlfn.NUMBERVALUE($L5)+_xlfn.NUMBERVALUE($L6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="9">
+    <cfRule type="expression" dxfId="8" priority="9">
       <formula>AND($D1="7. TOTAL CONTENTIEUX DES MINEURS",_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3))&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G7:M7">
-    <cfRule type="expression" dxfId="6" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="7" priority="7" stopIfTrue="1">
       <formula>_xlfn.NUMBERVALUE($L7)&lt;&gt;_xlfn.NUMBERVALUE($L6)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1:T1048576">
-    <cfRule type="expression" dxfId="5" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="6" priority="5" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3)+_xlfn.NUMBERVALUE($S4)+_xlfn.NUMBERVALUE($S5)+_xlfn.NUMBERVALUE($S6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="5" priority="6" stopIfTrue="1">
       <formula>AND($D1="7. TOTAL CONTENTIEUX DES MINEURS",_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3))&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N7:T7">
-    <cfRule type="expression" dxfId="3" priority="4" stopIfTrue="1">
+    <cfRule type="expression" dxfId="4" priority="4" stopIfTrue="1">
       <formula>_xlfn.NUMBERVALUE($S7)&lt;&gt;_xlfn.NUMBERVALUE($S6)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U1:V1048576">
-    <cfRule type="expression" dxfId="2" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="3" priority="2" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3)+_xlfn.NUMBERVALUE($U4)+_xlfn.NUMBERVALUE($U5)+_xlfn.NUMBERVALUE($U6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="3">
+    <cfRule type="expression" dxfId="2" priority="3">
       <formula>AND($D1="7. TOTAL CONTENTIEUX DES MINEURS",_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3))&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U7:V7">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="1" priority="1">
       <formula>_xlfn.NUMBERVALUE($U7)&lt;&gt;_xlfn.NUMBERVALUE($U6)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6615,7 +6579,7 @@
       </c>
       <c r="H1"/>
       <c r="I1" s="49" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="M1" s="26" t="s">
         <v>0</v>
@@ -6775,33 +6739,33 @@
         <v>39</v>
       </c>
       <c r="F1" s="115" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="G1" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="35" t="s">
+        <v>253</v>
+      </c>
+      <c r="B2" s="35" t="s">
+        <v>254</v>
+      </c>
+      <c r="C2" s="35" t="s">
+        <v>255</v>
+      </c>
+      <c r="D2" s="124" t="s">
+        <v>256</v>
+      </c>
+      <c r="E2" s="124" t="s">
+        <v>257</v>
+      </c>
+      <c r="F2" s="124" t="s">
+        <v>258</v>
+      </c>
+      <c r="G2" t="s">
         <v>259</v>
-      </c>
-      <c r="B2" s="35" t="s">
-        <v>260</v>
-      </c>
-      <c r="C2" s="35" t="s">
-        <v>261</v>
-      </c>
-      <c r="D2" s="124" t="s">
-        <v>262</v>
-      </c>
-      <c r="E2" s="124" t="s">
-        <v>263</v>
-      </c>
-      <c r="F2" s="124" t="s">
-        <v>264</v>
-      </c>
-      <c r="G2" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -6863,7 +6827,7 @@
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
       <c r="D1" s="3" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="E1" s="7"/>
       <c r="F1" s="6"/>
@@ -7028,17 +6992,17 @@
         <v>94</v>
       </c>
       <c r="L3" s="120" t="s">
+        <v>140</v>
+      </c>
+      <c r="M3" s="120" t="s">
         <v>141</v>
-      </c>
-      <c r="M3" s="120" t="s">
-        <v>142</v>
       </c>
       <c r="N3" s="120" t="s">
         <v>93</v>
       </c>
       <c r="O3" s="123"/>
       <c r="P3" s="120" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="Q3" s="120" t="s">
         <v>91</v>
@@ -7054,10 +7018,10 @@
         <v>89</v>
       </c>
       <c r="V3" s="120" t="s">
+        <v>143</v>
+      </c>
+      <c r="W3" s="120" t="s">
         <v>144</v>
-      </c>
-      <c r="W3" s="120" t="s">
-        <v>145</v>
       </c>
       <c r="X3" s="120" t="s">
         <v>88</v>
@@ -7067,7 +7031,7 @@
         <v>87</v>
       </c>
       <c r="AA3" s="120" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="AB3" s="120" t="s">
         <v>86</v>
@@ -7111,17 +7075,17 @@
         <v>76</v>
       </c>
       <c r="L4" s="120" t="s">
+        <v>145</v>
+      </c>
+      <c r="M4" s="120" t="s">
         <v>146</v>
-      </c>
-      <c r="M4" s="120" t="s">
-        <v>147</v>
       </c>
       <c r="N4" s="120" t="s">
         <v>75</v>
       </c>
       <c r="O4" s="123"/>
       <c r="P4" s="120" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="Q4" s="120" t="s">
         <v>73</v>
@@ -7137,10 +7101,10 @@
         <v>71</v>
       </c>
       <c r="V4" s="120" t="s">
+        <v>148</v>
+      </c>
+      <c r="W4" s="120" t="s">
         <v>149</v>
-      </c>
-      <c r="W4" s="120" t="s">
-        <v>150</v>
       </c>
       <c r="X4" s="120" t="s">
         <v>70</v>
@@ -7150,7 +7114,7 @@
         <v>69</v>
       </c>
       <c r="AA4" s="120" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="AB4" s="120" t="s">
         <v>68</v>
@@ -7168,7 +7132,7 @@
       <c r="B5" s="41"/>
       <c r="C5" s="41"/>
       <c r="D5" s="47" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="E5" s="117" t="s">
         <v>65</v>
@@ -7177,8 +7141,8 @@
         <v>64</v>
       </c>
       <c r="G5" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilés sur la période (contentieux sociaux civils et commerciaux)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.9. FONCTIONNAIRES / JA AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Temps ventilés sur la période (contentieux sociaux civils et commerciaux)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.9. FONCTIONNAIRES / JA AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH")</f>
         <v>#N/A</v>
       </c>
       <c r="H5" s="79" t="e">
@@ -7186,19 +7150,19 @@
         <v>#N/A</v>
       </c>
       <c r="I5" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.9. FONCTIONNAIRES / JA AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.9. FONCTIONNAIRES / JA AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")</f>
         <v>#N/A</v>
       </c>
       <c r="J5" s="103"/>
       <c r="K5" s="103"/>
       <c r="L5" s="103"/>
       <c r="M5" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")</f>
         <v>#N/A</v>
       </c>
       <c r="N5" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilés sur la période (contentieux sociaux civils et commerciaux)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR") -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Temps ventilés sur la période (contentieux sociaux civils et commerciaux)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR") -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")</f>
         <v>#N/A</v>
       </c>
       <c r="O5" s="79" t="e">
@@ -7206,18 +7170,18 @@
         <v>#N/A</v>
       </c>
       <c r="P5" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilés sur la période (contentieux sociaux civils et commerciaux)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS chambres sociales") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.9. FONCTIONNAIRES / JA AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS chambres sociales")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Temps ventilés sur la période (contentieux sociaux civils et commerciaux)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS chambres sociales") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.9. FONCTIONNAIRES / JA AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS chambres sociales")</f>
         <v>#N/A</v>
       </c>
       <c r="Q5" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilés sur la période (contentieux sociaux civils et commerciaux)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS siège Autres") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.9. FONCTIONNAIRES / JA AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS siège Autres")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Temps ventilés sur la période (contentieux sociaux civils et commerciaux)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS siège Autres") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.9. FONCTIONNAIRES / JA AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS siège Autres")</f>
         <v>#N/A</v>
       </c>
       <c r="R5" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilés sur la période (contentieux sociaux civils et commerciaux)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS parquet général") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.9. FONCTIONNAIRES / JA AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS parquet général")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Temps ventilés sur la période (contentieux sociaux civils et commerciaux)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS parquet général") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.9. FONCTIONNAIRES / JA AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS parquet général")</f>
         <v>#N/A</v>
       </c>
       <c r="S5" s="79" t="e">
@@ -7228,12 +7192,12 @@
       <c r="U5" s="103"/>
       <c r="V5" s="103"/>
       <c r="W5" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")</f>
         <v>#N/A</v>
       </c>
       <c r="X5" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilés sur la période (contentieux sociaux civils et commerciaux)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE") -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Temps ventilés sur la période (contentieux sociaux civils et commerciaux)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE") -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")</f>
         <v>#N/A</v>
       </c>
       <c r="Y5" s="79" t="e">
@@ -7255,7 +7219,7 @@
       <c r="B6" s="41"/>
       <c r="C6" s="41"/>
       <c r="D6" s="38" t="str">
-        <f t="shared" ref="D6:D15" si="0">IF(ISBLANK($D$5),"",$D$5)</f>
+        <f>IF(ISBLANK($D$5),"",$D$5)</f>
         <v>=ETPT_CA_JUR_DDG!D5</v>
       </c>
       <c r="E6" s="117" t="s">
@@ -7265,8 +7229,8 @@
         <v>62</v>
       </c>
       <c r="G6" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilés sur la période (service pénal)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.10. AUTRES FONCTIONNAIRES / JA AFFECTÉS AU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Temps ventilés sur la période (service pénal)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.10. AUTRES FONCTIONNAIRES / JA AFFECTÉS AU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH")</f>
         <v>#N/A</v>
       </c>
       <c r="H6" s="79" t="e">
@@ -7275,91 +7239,91 @@
       </c>
       <c r="I6" s="103"/>
       <c r="J6" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.1. ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.2 ASSISES JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.1. ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.2 ASSISES JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")</f>
         <v>#N/A</v>
       </c>
       <c r="K6" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.3. COUR CRIMINELLE DÉPARTEMENTALE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.3. COUR CRIMINELLE DÉPARTEMENTALE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")</f>
         <v>#N/A</v>
       </c>
       <c r="L6" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("8.4. CONTENTIEUX JIRS CRIM-ORG",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("8.7. CONTENTIEUX JIRS ÉCO-FI",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.3. CONTENTIEUX DE LA DÉTENTION JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")+
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.5. CONTENTIEUX DU CONTRÔLE JUDICIAIRE JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")+
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.7. CONTENTIEUX DE FOND JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("8.4. CONTENTIEUX JIRS CRIM-ORG",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("8.7. CONTENTIEUX JIRS ÉCO-FI",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.3. CONTENTIEUX DE LA DÉTENTION JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.5. CONTENTIEUX DU CONTRÔLE JUDICIAIRE JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.7. CONTENTIEUX DE FOND JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")</f>
         <v>#N/A</v>
       </c>
       <c r="M6" s="103"/>
       <c r="N6" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilés sur la période (service pénal)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR") -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.1. ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.2 ASSISES JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.3. COUR CRIMINELLE DÉPARTEMENTALE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("8.4. CONTENTIEUX JIRS CRIM-ORG",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("8.7. CONTENTIEUX JIRS ÉCO-FI",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.3. CONTENTIEUX DE LA DÉTENTION JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.5. CONTENTIEUX DU CONTRÔLE JUDICIAIRE JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.7. CONTENTIEUX DE FOND JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")  +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.10. AUTRES FONCTIONNAIRES / JA AFFECTÉS AU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Temps ventilés sur la période (service pénal)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR") -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.1. ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.2 ASSISES JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.3. COUR CRIMINELLE DÉPARTEMENTALE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("8.4. CONTENTIEUX JIRS CRIM-ORG",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("8.7. CONTENTIEUX JIRS ÉCO-FI",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.3. CONTENTIEUX DE LA DÉTENTION JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.5. CONTENTIEUX DU CONTRÔLE JUDICIAIRE JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.7. CONTENTIEUX DE FOND JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")  +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.10. AUTRES FONCTIONNAIRES / JA AFFECTÉS AU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")</f>
         <v>#N/A</v>
       </c>
       <c r="O6" s="79" t="e">
-        <f t="shared" ref="O6:O15" si="1">SUM(I6:N6)</f>
+        <f t="shared" ref="O6:O15" si="0">SUM(I6:N6)</f>
         <v>#N/A</v>
       </c>
       <c r="P6" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilés sur la période (service pénal)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS chambres sociales") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.10. AUTRES FONCTIONNAIRES / JA AFFECTÉS AU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS chambres sociales")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Temps ventilés sur la période (service pénal)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS chambres sociales") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.10. AUTRES FONCTIONNAIRES / JA AFFECTÉS AU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS chambres sociales")</f>
         <v>#N/A</v>
       </c>
       <c r="Q6" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilés sur la période (service pénal)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS siège Autres") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.10. AUTRES FONCTIONNAIRES / JA AFFECTÉS AU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS siège Autres")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Temps ventilés sur la période (service pénal)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS siège Autres") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.10. AUTRES FONCTIONNAIRES / JA AFFECTÉS AU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS siège Autres")</f>
         <v>#N/A</v>
       </c>
       <c r="R6" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilés sur la période (service pénal)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS parquet général") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.10. AUTRES FONCTIONNAIRES / JA AFFECTÉS AU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS parquet général")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Temps ventilés sur la période (service pénal)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS parquet général") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.10. AUTRES FONCTIONNAIRES / JA AFFECTÉS AU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS parquet général")</f>
         <v>#N/A</v>
       </c>
       <c r="S6" s="79" t="e">
-        <f t="shared" ref="S6:S16" si="2">SUM(P6:R6)</f>
+        <f t="shared" ref="S6:S16" si="1">SUM(P6:R6)</f>
         <v>#N/A</v>
       </c>
       <c r="T6" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.1. ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.2 ASSISES JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.1. ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.2 ASSISES JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")</f>
         <v>#N/A</v>
       </c>
       <c r="U6" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.3. COUR CRIMINELLE DÉPARTEMENTALE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.3. COUR CRIMINELLE DÉPARTEMENTALE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")</f>
         <v>#N/A</v>
       </c>
       <c r="V6" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("8.4. CONTENTIEUX JIRS CRIM-ORG",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("8.7. CONTENTIEUX JIRS ÉCO-FI",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.3. CONTENTIEUX DE LA DÉTENTION JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")+
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.5. CONTENTIEUX DU CONTRÔLE JUDICIAIRE JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")+
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.7. CONTENTIEUX DE FOND JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("8.4. CONTENTIEUX JIRS CRIM-ORG",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("8.7. CONTENTIEUX JIRS ÉCO-FI",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.3. CONTENTIEUX DE LA DÉTENTION JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.5. CONTENTIEUX DU CONTRÔLE JUDICIAIRE JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.7. CONTENTIEUX DE FOND JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")</f>
         <v>#N/A</v>
       </c>
       <c r="W6" s="103"/>
       <c r="X6" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilés sur la période (service pénal)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE") -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.1. ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.2 ASSISES JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.3. COUR CRIMINELLE DÉPARTEMENTALE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("8.4. CONTENTIEUX JIRS CRIM-ORG",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("8.7. CONTENTIEUX JIRS ÉCO-FI",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.3. CONTENTIEUX DE LA DÉTENTION JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.5. CONTENTIEUX DU CONTRÔLE JUDICIAIRE JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.7. CONTENTIEUX DE FOND JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Temps ventilés sur la période (service pénal)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE") -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.1. ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.2 ASSISES JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.3. COUR CRIMINELLE DÉPARTEMENTALE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("8.4. CONTENTIEUX JIRS CRIM-ORG",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("8.7. CONTENTIEUX JIRS ÉCO-FI",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.3. CONTENTIEUX DE LA DÉTENTION JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.5. CONTENTIEUX DU CONTRÔLE JUDICIAIRE JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.7. CONTENTIEUX DE FOND JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")</f>
         <v>#N/A</v>
       </c>
       <c r="Y6" s="79" t="e">
-        <f t="shared" ref="Y6:Y16" si="3">SUM(T6:X6)</f>
+        <f t="shared" ref="Y6:Y16" si="2">SUM(T6:X6)</f>
         <v>#N/A</v>
       </c>
       <c r="Z6" s="103"/>
@@ -7368,7 +7332,7 @@
       <c r="AC6" s="103"/>
       <c r="AD6" s="103"/>
       <c r="AE6" s="79">
-        <f t="shared" ref="AE6:AE15" si="4">SUM(Z6:AD6)</f>
+        <f t="shared" ref="AE6:AE15" si="3">SUM(Z6:AD6)</f>
         <v>0</v>
       </c>
     </row>
@@ -7377,7 +7341,7 @@
       <c r="B7" s="41"/>
       <c r="C7" s="41"/>
       <c r="D7" s="38" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="D7:D15" si="4">IF(ISBLANK($D$5),"",$D$5)</f>
         <v>=ETPT_CA_JUR_DDG!D5</v>
       </c>
       <c r="E7" s="117" t="s">
@@ -7398,14 +7362,14 @@
       <c r="M7" s="103"/>
       <c r="N7" s="103"/>
       <c r="O7" s="79">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="P7" s="103"/>
       <c r="Q7" s="103"/>
       <c r="R7" s="103"/>
       <c r="S7" s="79">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="T7" s="103"/>
@@ -7413,11 +7377,11 @@
       <c r="V7" s="103"/>
       <c r="W7" s="103"/>
       <c r="X7" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.4 CSM",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.4 CSM",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")</f>
         <v>#N/A</v>
       </c>
       <c r="Y7" s="79" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
       <c r="Z7" s="103"/>
@@ -7426,7 +7390,7 @@
       <c r="AC7" s="103"/>
       <c r="AD7" s="103"/>
       <c r="AE7" s="79">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -7435,7 +7399,7 @@
       <c r="B8" s="41"/>
       <c r="C8" s="41"/>
       <c r="D8" s="38" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>=ETPT_CA_JUR_DDG!D5</v>
       </c>
       <c r="E8" s="117" t="s">
@@ -7445,7 +7409,7 @@
         <v>58</v>
       </c>
       <c r="G8" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.8. ACCUEIL DU JUSTICIABLE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.8. ACCUEIL DU JUSTICIABLE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH")</f>
         <v>#N/A</v>
       </c>
       <c r="H8" s="79" t="e">
@@ -7458,27 +7422,27 @@
       <c r="L8" s="103"/>
       <c r="M8" s="103"/>
       <c r="N8" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.8. ACCUEIL DU JUSTICIABLE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.8. ACCUEIL DU JUSTICIABLE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")</f>
         <v>#N/A</v>
       </c>
       <c r="O8" s="79" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P8" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.8. ACCUEIL DU JUSTICIABLE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS chambres sociales")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="Q8" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.8. ACCUEIL DU JUSTICIABLE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS siège Autres")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="R8" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.8. ACCUEIL DU JUSTICIABLE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS parquet général")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="S8" s="79" t="e">
         <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="P8" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.8. ACCUEIL DU JUSTICIABLE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS chambres sociales")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="Q8" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.8. ACCUEIL DU JUSTICIABLE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS siège Autres")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="R8" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.8. ACCUEIL DU JUSTICIABLE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS parquet général")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="S8" s="79" t="e">
-        <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
       <c r="T8" s="103"/>
@@ -7486,11 +7450,11 @@
       <c r="V8" s="103"/>
       <c r="W8" s="103"/>
       <c r="X8" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.8. ACCUEIL DU JUSTICIABLE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.8. ACCUEIL DU JUSTICIABLE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")</f>
         <v>#N/A</v>
       </c>
       <c r="Y8" s="79" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
       <c r="Z8" s="103"/>
@@ -7499,7 +7463,7 @@
       <c r="AC8" s="103"/>
       <c r="AD8" s="103"/>
       <c r="AE8" s="79">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -7508,7 +7472,7 @@
       <c r="B9" s="41"/>
       <c r="C9" s="41"/>
       <c r="D9" s="38" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>=ETPT_CA_JUR_DDG!D5</v>
       </c>
       <c r="E9" s="117" t="s">
@@ -7517,54 +7481,54 @@
       <c r="F9" s="117" t="s">
         <v>56</v>
       </c>
-      <c r="G9" s="103">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Soutien (Hors accueil du justiciable)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH")</f>
-        <v>0</v>
-      </c>
-      <c r="H9" s="79">
+      <c r="G9" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Soutien (Hors accueil du justiciable)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H9" s="79" t="e">
         <f>SUM(G9)</f>
-        <v>0</v>
+        <v>#N/A</v>
       </c>
       <c r="I9" s="103"/>
       <c r="J9" s="103"/>
       <c r="K9" s="103"/>
       <c r="L9" s="103"/>
       <c r="M9" s="103"/>
-      <c r="N9" s="103">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Soutien (Hors accueil du justiciable)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")</f>
-        <v>0</v>
-      </c>
-      <c r="O9" s="79">
+      <c r="N9" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Soutien (Hors accueil du justiciable)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="O9" s="79" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P9" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Soutien (Hors accueil du justiciable)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS chambres sociales")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="Q9" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Soutien (Hors accueil du justiciable)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS siège Autres")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="R9" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Soutien (Hors accueil du justiciable)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS parquet général")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="S9" s="79" t="e">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="P9" s="103">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Soutien (Hors accueil du justiciable)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS chambres sociales")</f>
-        <v>0</v>
-      </c>
-      <c r="Q9" s="103">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Soutien (Hors accueil du justiciable)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS siège Autres")</f>
-        <v>0</v>
-      </c>
-      <c r="R9" s="103">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Soutien (Hors accueil du justiciable)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS parquet général")</f>
-        <v>0</v>
-      </c>
-      <c r="S9" s="79">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <v>#N/A</v>
       </c>
       <c r="T9" s="103"/>
       <c r="U9" s="103"/>
       <c r="V9" s="103"/>
       <c r="W9" s="103"/>
-      <c r="X9" s="103">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Soutien (Hors accueil du justiciable)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")</f>
-        <v>0</v>
-      </c>
-      <c r="Y9" s="79">
-        <f t="shared" si="3"/>
-        <v>0</v>
+      <c r="X9" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Soutien (Hors accueil du justiciable)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="Y9" s="79" t="e">
+        <f t="shared" si="2"/>
+        <v>#N/A</v>
       </c>
       <c r="Z9" s="103"/>
       <c r="AA9" s="103"/>
@@ -7572,7 +7536,7 @@
       <c r="AC9" s="103"/>
       <c r="AD9" s="103"/>
       <c r="AE9" s="79">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -7581,7 +7545,7 @@
       <c r="B10" s="41"/>
       <c r="C10" s="41"/>
       <c r="D10" s="38" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>=ETPT_CA_JUR_DDG!D5</v>
       </c>
       <c r="E10" s="117" t="s">
@@ -7591,7 +7555,7 @@
         <v>54</v>
       </c>
       <c r="G10" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.3. FORMATIONS DISPENSÉES",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.3. FORMATIONS DISPENSÉES",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH")</f>
         <v>#N/A</v>
       </c>
       <c r="H10" s="79" t="e">
@@ -7604,27 +7568,27 @@
       <c r="L10" s="103"/>
       <c r="M10" s="103"/>
       <c r="N10" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.3. FORMATIONS DISPENSÉES",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.3. FORMATIONS DISPENSÉES",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")</f>
         <v>#N/A</v>
       </c>
       <c r="O10" s="79" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P10" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.3. FORMATIONS DISPENSÉES",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS chambres sociales")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="Q10" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.3. FORMATIONS DISPENSÉES",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS siège Autres")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="R10" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.3. FORMATIONS DISPENSÉES",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS parquet général")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="S10" s="79" t="e">
         <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="P10" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.3. FORMATIONS DISPENSÉES",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS chambres sociales")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="Q10" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.3. FORMATIONS DISPENSÉES",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS siège Autres")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="R10" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.3. FORMATIONS DISPENSÉES",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS parquet général")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="S10" s="79" t="e">
-        <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
       <c r="T10" s="103"/>
@@ -7632,11 +7596,11 @@
       <c r="V10" s="103"/>
       <c r="W10" s="103"/>
       <c r="X10" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.3. FORMATIONS DISPENSÉES",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.3. FORMATIONS DISPENSÉES",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")</f>
         <v>#N/A</v>
       </c>
       <c r="Y10" s="79" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
       <c r="Z10" s="103"/>
@@ -7645,7 +7609,7 @@
       <c r="AC10" s="103"/>
       <c r="AD10" s="103"/>
       <c r="AE10" s="79">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -7654,7 +7618,7 @@
       <c r="B11" s="41"/>
       <c r="C11" s="41"/>
       <c r="D11" s="38" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>=ETPT_CA_JUR_DDG!D5</v>
       </c>
       <c r="E11" s="117" t="s">
@@ -7664,7 +7628,7 @@
         <v>52</v>
       </c>
       <c r="G11" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.7. ACCÈS AU DROIT ET À LA JUSTICE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.7. ACCÈS AU DROIT ET À LA JUSTICE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH")</f>
         <v>#N/A</v>
       </c>
       <c r="H11" s="79" t="e">
@@ -7677,27 +7641,27 @@
       <c r="L11" s="103"/>
       <c r="M11" s="103"/>
       <c r="N11" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.7. ACCÈS AU DROIT ET À LA JUSTICE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.7. ACCÈS AU DROIT ET À LA JUSTICE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")</f>
         <v>#N/A</v>
       </c>
       <c r="O11" s="79" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P11" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.7. ACCÈS AU DROIT ET À LA JUSTICE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS chambres sociales")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="Q11" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.7. ACCÈS AU DROIT ET À LA JUSTICE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS siège Autres")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="R11" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.7. ACCÈS AU DROIT ET À LA JUSTICE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS parquet général")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="S11" s="79" t="e">
         <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="P11" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.7. ACCÈS AU DROIT ET À LA JUSTICE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS chambres sociales")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="Q11" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.7. ACCÈS AU DROIT ET À LA JUSTICE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS siège Autres")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="R11" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.7. ACCÈS AU DROIT ET À LA JUSTICE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS parquet général")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="S11" s="79" t="e">
-        <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
       <c r="T11" s="103"/>
@@ -7705,11 +7669,11 @@
       <c r="V11" s="103"/>
       <c r="W11" s="103"/>
       <c r="X11" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.7. ACCÈS AU DROIT ET À LA JUSTICE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.7. ACCÈS AU DROIT ET À LA JUSTICE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")</f>
         <v>#N/A</v>
       </c>
       <c r="Y11" s="79" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
       <c r="Z11" s="103"/>
@@ -7718,7 +7682,7 @@
       <c r="AC11" s="103"/>
       <c r="AD11" s="103"/>
       <c r="AE11" s="79">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -7727,7 +7691,7 @@
       <c r="B12" s="41"/>
       <c r="C12" s="41"/>
       <c r="D12" s="38" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>=ETPT_CA_JUR_DDG!D5</v>
       </c>
       <c r="E12" s="117" t="s">
@@ -7737,8 +7701,8 @@
         <v>50</v>
       </c>
       <c r="G12" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH") -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14.9. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH") -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14.9. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH")</f>
         <v>#N/A</v>
       </c>
       <c r="H12" s="79" t="e">
@@ -7751,31 +7715,31 @@
       <c r="L12" s="103"/>
       <c r="M12" s="103"/>
       <c r="N12" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR") -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14.9. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR") -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14.9. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")</f>
         <v>#N/A</v>
       </c>
       <c r="O12" s="79" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P12" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS chambres sociales") -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14.9. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS chambres sociales")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="Q12" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS siège Autres") -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14.9. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS siège Autres")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="R12" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS parquet général") -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14.9. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS parquet général")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="S12" s="79" t="e">
         <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="P12" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS chambres sociales") -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14.9. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS chambres sociales")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="Q12" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS siège Autres") -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14.9. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS siège Autres")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="R12" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS parquet général") -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14.9. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS parquet général")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="S12" s="79" t="e">
-        <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
       <c r="T12" s="103"/>
@@ -7783,12 +7747,12 @@
       <c r="V12" s="103"/>
       <c r="W12" s="103"/>
       <c r="X12" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE") -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14.9. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE") -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14.9. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")</f>
         <v>#N/A</v>
       </c>
       <c r="Y12" s="79" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
       <c r="Z12" s="103"/>
@@ -7797,7 +7761,7 @@
       <c r="AC12" s="103"/>
       <c r="AD12" s="103"/>
       <c r="AE12" s="79">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -7816,7 +7780,7 @@
         <v>48</v>
       </c>
       <c r="G13" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14.9. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14.9. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH")</f>
         <v>#N/A</v>
       </c>
       <c r="H13" s="79" t="e">
@@ -7829,27 +7793,27 @@
       <c r="L13" s="103"/>
       <c r="M13" s="103"/>
       <c r="N13" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14.9. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14.9. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR")</f>
         <v>#N/A</v>
       </c>
       <c r="O13" s="79" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P13" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14.9. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS chambres sociales")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="Q13" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14.9. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS siège Autres")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="R13" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14.9. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS parquet général")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="S13" s="79" t="e">
         <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="P13" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14.9. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS chambres sociales")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="Q13" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14.9. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS siège Autres")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="R13" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14.9. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS parquet général")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="S13" s="79" t="e">
-        <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
       <c r="T13" s="103"/>
@@ -7857,11 +7821,11 @@
       <c r="V13" s="103"/>
       <c r="W13" s="103"/>
       <c r="X13" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14.9. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14.9. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE")</f>
         <v>#N/A</v>
       </c>
       <c r="Y13" s="79" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
       <c r="Z13" s="103"/>
@@ -7870,7 +7834,7 @@
       <c r="AC13" s="103"/>
       <c r="AD13" s="103"/>
       <c r="AE13" s="79">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -7888,109 +7852,109 @@
       <c r="F14" s="117" t="s">
         <v>46</v>
       </c>
-      <c r="G14" s="103">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilés sur la période (hors indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé ADD")</f>
-        <v>0</v>
-      </c>
-      <c r="H14" s="79">
+      <c r="G14" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Temps ventilés sur la période (hors indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé ADD")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H14" s="79" t="e">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>#N/A</v>
       </c>
       <c r="I14" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.9. FONCTIONNAIRES / JA AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.9. FONCTIONNAIRES / JA AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")</f>
         <v>#N/A</v>
       </c>
       <c r="J14" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.1. ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.2 ASSISES JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.1. ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.2 ASSISES JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")</f>
         <v>#N/A</v>
       </c>
       <c r="K14" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.3. COUR CRIMINELLE DÉPARTEMENTALE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.3. COUR CRIMINELLE DÉPARTEMENTALE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")</f>
         <v>#N/A</v>
       </c>
       <c r="L14" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("8.4. CONTENTIEUX JIRS CRIM-ORG",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("8.7. CONTENTIEUX JIRS ÉCO-FI",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.3. CONTENTIEUX DE LA DÉTENTION JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")+
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.5. CONTENTIEUX DU CONTRÔLE JUDICIAIRE JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")+
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.7. CONTENTIEUX DE FOND JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("8.4. CONTENTIEUX JIRS CRIM-ORG",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("8.7. CONTENTIEUX JIRS ÉCO-FI",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.3. CONTENTIEUX DE LA DÉTENTION JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.5. CONTENTIEUX DU CONTRÔLE JUDICIAIRE JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.7. CONTENTIEUX DE FOND JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")</f>
         <v>#N/A</v>
       </c>
       <c r="M14" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")</f>
         <v>#N/A</v>
       </c>
       <c r="N14" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilés sur la période (hors indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD") -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.9. FONCTIONNAIRES / JA AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.1. ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.2 ASSISES JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.3. COUR CRIMINELLE DÉPARTEMENTALE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("8.4. CONTENTIEUX JIRS CRIM-ORG",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("8.7. CONTENTIEUX JIRS ÉCO-FI",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.3. CONTENTIEUX DE LA DÉTENTION JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.5. CONTENTIEUX DU CONTRÔLE JUDICIAIRE JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.7. CONTENTIEUX DE FOND JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Temps ventilés sur la période (hors indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD") -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.9. FONCTIONNAIRES / JA AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.1. ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.2 ASSISES JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.3. COUR CRIMINELLE DÉPARTEMENTALE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("8.4. CONTENTIEUX JIRS CRIM-ORG",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("8.7. CONTENTIEUX JIRS ÉCO-FI",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.3. CONTENTIEUX DE LA DÉTENTION JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.5. CONTENTIEUX DU CONTRÔLE JUDICIAIRE JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.7. CONTENTIEUX DE FOND JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")</f>
         <v>#N/A</v>
       </c>
       <c r="O14" s="79" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="P14" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Temps ventilés sur la période (hors indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS chambres sociales placé ADD")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="Q14" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Temps ventilés sur la période (hors indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS siège Autres placé ADD")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="R14" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Temps ventilés sur la période (hors indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS parquet général placé ADD")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="S14" s="79" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
-      <c r="P14" s="103">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilés sur la période (hors indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS chambres sociales placé ADD")</f>
-        <v>0</v>
-      </c>
-      <c r="Q14" s="103">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilés sur la période (hors indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS siège Autres placé ADD")</f>
-        <v>0</v>
-      </c>
-      <c r="R14" s="103">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilés sur la période (hors indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS parquet général placé ADD")</f>
-        <v>0</v>
-      </c>
-      <c r="S14" s="79">
+      <c r="T14" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.1. ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé ADD") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.2 ASSISES JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé ADD")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="U14" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.3. COUR CRIMINELLE DÉPARTEMENTALE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé ADD")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="V14" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("8.4. CONTENTIEUX JIRS CRIM-ORG",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé ADD") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("8.7. CONTENTIEUX JIRS ÉCO-FI",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé ADD") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.3. CONTENTIEUX DE LA DÉTENTION JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé ADD")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.5. CONTENTIEUX DU CONTRÔLE JUDICIAIRE JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé ADD")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.7. CONTENTIEUX DE FOND JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé ADD")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="W14" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé ADD")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="X14" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Temps ventilés sur la période (hors indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé ADD") -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.1. ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé ADD")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.2 ASSISES JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé ADD")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.3. COUR CRIMINELLE DÉPARTEMENTALE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé ADD")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("8.4. CONTENTIEUX JIRS CRIM-ORG",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé ADD")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("8.7. CONTENTIEUX JIRS ÉCO-FI",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé ADD")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.3. CONTENTIEUX DE LA DÉTENTION JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé ADD")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.5. CONTENTIEUX DU CONTRÔLE JUDICIAIRE JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé ADD")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.7. CONTENTIEUX DE FOND JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé ADD")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé ADD")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="Y14" s="79" t="e">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="T14" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.1. ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé ADD") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.2 ASSISES JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé ADD")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="U14" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.3. COUR CRIMINELLE DÉPARTEMENTALE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé ADD")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="V14" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("8.4. CONTENTIEUX JIRS CRIM-ORG",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé ADD") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("8.7. CONTENTIEUX JIRS ÉCO-FI",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé ADD") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.3. CONTENTIEUX DE LA DÉTENTION JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé ADD")+
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.5. CONTENTIEUX DU CONTRÔLE JUDICIAIRE JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé ADD")+
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.7. CONTENTIEUX DE FOND JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé ADD")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W14" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé ADD")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="X14" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilés sur la période (hors indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé ADD") -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.1. ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé ADD")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.2 ASSISES JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé ADD")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.3. COUR CRIMINELLE DÉPARTEMENTALE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé ADD")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("8.4. CONTENTIEUX JIRS CRIM-ORG",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé ADD")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("8.7. CONTENTIEUX JIRS ÉCO-FI",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé ADD")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.3. CONTENTIEUX DE LA DÉTENTION JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé ADD")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.5. CONTENTIEUX DU CONTRÔLE JUDICIAIRE JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé ADD")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.7. CONTENTIEUX DE FOND JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé ADD")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé ADD")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="Y14" s="79" t="e">
-        <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="Z14" s="103"/>
@@ -7999,20 +7963,20 @@
       <c r="AC14" s="103"/>
       <c r="AD14" s="103"/>
       <c r="AE14" s="79">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:62" x14ac:dyDescent="0.2">
       <c r="D15" s="38" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>=ETPT_CA_JUR_DDG!D5</v>
       </c>
       <c r="E15" s="117" t="s">
+        <v>224</v>
+      </c>
+      <c r="F15" s="117" t="s">
         <v>225</v>
-      </c>
-      <c r="F15" s="117" t="s">
-        <v>226</v>
       </c>
       <c r="G15" s="103"/>
       <c r="H15" s="79">
@@ -8026,26 +7990,26 @@
       <c r="M15" s="103"/>
       <c r="N15" s="103"/>
       <c r="O15" s="79">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="P15" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="Q15" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS siège Autres placé ADD") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS siège Autres placé SUB")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="R15" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS parquet général placé ADD") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS parquet général placé SUB")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="S15" s="79" t="e">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="P15" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="Q15" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS siège Autres placé ADD") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS siège Autres placé SUB")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="R15" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS parquet général placé ADD") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS parquet général placé SUB")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="S15" s="79" t="e">
-        <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
       <c r="T15" s="103"/>
@@ -8053,12 +8017,12 @@
       <c r="V15" s="103"/>
       <c r="W15" s="103"/>
       <c r="X15" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé ADD") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé SUB")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé ADD") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé SUB")</f>
         <v>#N/A</v>
       </c>
       <c r="Y15" s="79" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
       <c r="Z15" s="103"/>
@@ -8067,7 +8031,7 @@
       <c r="AC15" s="103"/>
       <c r="AD15" s="103"/>
       <c r="AE15" s="79">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -8079,109 +8043,109 @@
       <c r="F16" s="117" t="s">
         <v>44</v>
       </c>
-      <c r="G16" s="103">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilés sur la période (hors indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé SUB")</f>
-        <v>0</v>
-      </c>
-      <c r="H16" s="79">
+      <c r="G16" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Temps ventilés sur la période (hors indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé SUB")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H16" s="79" t="e">
         <f>SUM(G16)</f>
-        <v>0</v>
+        <v>#N/A</v>
       </c>
       <c r="I16" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.9. FONCTIONNAIRES / JA AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.9. FONCTIONNAIRES / JA AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")</f>
         <v>#N/A</v>
       </c>
       <c r="J16" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.1. ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.2 ASSISES JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.1. ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.2 ASSISES JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")</f>
         <v>#N/A</v>
       </c>
       <c r="K16" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.3. COUR CRIMINELLE DÉPARTEMENTALE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.3. COUR CRIMINELLE DÉPARTEMENTALE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")</f>
         <v>#N/A</v>
       </c>
       <c r="L16" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("8.4. CONTENTIEUX JIRS CRIM-ORG",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("8.7. CONTENTIEUX JIRS ÉCO-FI",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.3. CONTENTIEUX DE LA DÉTENTION JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")+
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.5. CONTENTIEUX DU CONTRÔLE JUDICIAIRE JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")+
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.7. CONTENTIEUX DE FOND JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("8.4. CONTENTIEUX JIRS CRIM-ORG",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("8.7. CONTENTIEUX JIRS ÉCO-FI",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.3. CONTENTIEUX DE LA DÉTENTION JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.5. CONTENTIEUX DU CONTRÔLE JUDICIAIRE JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.7. CONTENTIEUX DE FOND JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")</f>
         <v>#N/A</v>
       </c>
       <c r="M16" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")</f>
         <v>#N/A</v>
       </c>
       <c r="N16" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilés sur la période (hors indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB") -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("13.9. FONCTIONNAIRES / JA AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.1. ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.2 ASSISES JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.3. COUR CRIMINELLE DÉPARTEMENTALE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("8.4. CONTENTIEUX JIRS CRIM-ORG",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("8.7. CONTENTIEUX JIRS ÉCO-FI",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.3. CONTENTIEUX DE LA DÉTENTION JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.5. CONTENTIEUX DU CONTRÔLE JUDICIAIRE JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.7. CONTENTIEUX DE FOND JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Temps ventilés sur la période (hors indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB") -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.9. FONCTIONNAIRES / JA AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.1. ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.2 ASSISES JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.3. COUR CRIMINELLE DÉPARTEMENTALE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("8.4. CONTENTIEUX JIRS CRIM-ORG",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("8.7. CONTENTIEUX JIRS ÉCO-FI",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.3. CONTENTIEUX DE LA DÉTENTION JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.5. CONTENTIEUX DU CONTRÔLE JUDICIAIRE JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.7. CONTENTIEUX DE FOND JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")</f>
         <v>#N/A</v>
       </c>
       <c r="O16" s="79" t="e">
         <f>SUM(I16:N16)</f>
         <v>#N/A</v>
       </c>
-      <c r="P16" s="103">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilés sur la période (hors indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS chambres sociales placé SUB")</f>
-        <v>0</v>
-      </c>
-      <c r="Q16" s="103">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilés sur la période (hors indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS siège Autres placé SUB")</f>
-        <v>0</v>
-      </c>
-      <c r="R16" s="103">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilés sur la période (hors indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS parquet général placé SUB")</f>
-        <v>0</v>
-      </c>
-      <c r="S16" s="79">
+      <c r="P16" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Temps ventilés sur la période (hors indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS chambres sociales placé SUB")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="Q16" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Temps ventilés sur la période (hors indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS siège Autres placé SUB")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="R16" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Temps ventilés sur la période (hors indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"JURISTE AS parquet général placé SUB")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="S16" s="79" t="e">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="T16" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.1. ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé SUB") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.2 ASSISES JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé SUB")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="U16" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.3. COUR CRIMINELLE DÉPARTEMENTALE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé SUB")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="V16" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("8.4. CONTENTIEUX JIRS CRIM-ORG",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé SUB") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("8.7. CONTENTIEUX JIRS ÉCO-FI",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé SUB") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.3. CONTENTIEUX DE LA DÉTENTION JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé SUB")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.5. CONTENTIEUX DU CONTRÔLE JUDICIAIRE JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé SUB")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.7. CONTENTIEUX DE FOND JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé SUB")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="W16" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé SUB")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="X16" s="103" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Temps ventilés sur la période (hors indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé SUB")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.1. ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé SUB")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.2 ASSISES JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé SUB")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("11.3. COUR CRIMINELLE DÉPARTEMENTALE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé SUB")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("8.4. CONTENTIEUX JIRS CRIM-ORG",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé SUB")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("8.7. CONTENTIEUX JIRS ÉCO-FI",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé SUB")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.3. CONTENTIEUX DE LA DÉTENTION JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé SUB")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.5. CONTENTIEUX DU CONTRÔLE JUDICIAIRE JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé SUB")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("9.7. CONTENTIEUX DE FOND JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé SUB")  -
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé SUB")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="Y16" s="79" t="e">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="T16" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.1. ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé SUB") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.2 ASSISES JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé SUB")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="U16" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.3. COUR CRIMINELLE DÉPARTEMENTALE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé SUB")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="V16" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("8.4. CONTENTIEUX JIRS CRIM-ORG",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé SUB") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("8.7. CONTENTIEUX JIRS ÉCO-FI",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé SUB") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.3. CONTENTIEUX DE LA DÉTENTION JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé SUB")+
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.5. CONTENTIEUX DU CONTRÔLE JUDICIAIRE JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé SUB")+
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.7. CONTENTIEUX DE FOND JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé SUB")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W16" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE placé SUB")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="X16" s="103" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilés sur la période (hors indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé SUB")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.1. ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé SUB")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.2 ASSISES JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé SUB")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.3. COUR CRIMINELLE DÉPARTEMENTALE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé SUB")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("8.4. CONTENTIEUX JIRS CRIM-ORG",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé SUB")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("8.7. CONTENTIEUX JIRS ÉCO-FI",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé SUB")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.3. CONTENTIEUX DE LA DÉTENTION JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé SUB")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.5. CONTENTIEUX DU CONTRÔLE JUDICIAIRE JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé SUB")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9.7. CONTENTIEUX DE FOND JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé SUB")  -
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé SUB")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="Y16" s="79" t="e">
-        <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="Z16" s="103"/>
@@ -8304,19 +8268,19 @@
     <row r="19" spans="1:31" customFormat="1" ht="102.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="4"/>
       <c r="F19" s="121" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="G19" s="81" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé ADD") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé SUB")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé ADD") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé SUB")</f>
         <v>#N/A</v>
       </c>
       <c r="M19" s="122" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="N19" s="81" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -8355,12 +8319,12 @@
   <sheetData>
     <row r="1" spans="1:31" ht="87" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
       <c r="D1" s="3" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="E1" s="7"/>
       <c r="F1" s="6"/>
@@ -8494,17 +8458,17 @@
         <v>94</v>
       </c>
       <c r="L3" s="120" t="s">
+        <v>140</v>
+      </c>
+      <c r="M3" s="120" t="s">
         <v>141</v>
-      </c>
-      <c r="M3" s="120" t="s">
-        <v>142</v>
       </c>
       <c r="N3" s="120" t="s">
         <v>93</v>
       </c>
       <c r="O3" s="123"/>
       <c r="P3" s="120" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="Q3" s="120" t="s">
         <v>91</v>
@@ -8520,10 +8484,10 @@
         <v>89</v>
       </c>
       <c r="V3" s="120" t="s">
+        <v>143</v>
+      </c>
+      <c r="W3" s="120" t="s">
         <v>144</v>
-      </c>
-      <c r="W3" s="120" t="s">
-        <v>145</v>
       </c>
       <c r="X3" s="120" t="s">
         <v>88</v>
@@ -8533,7 +8497,7 @@
         <v>87</v>
       </c>
       <c r="AA3" s="120" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="AB3" s="120" t="s">
         <v>86</v>
@@ -8577,17 +8541,17 @@
         <v>76</v>
       </c>
       <c r="L4" s="120" t="s">
+        <v>145</v>
+      </c>
+      <c r="M4" s="120" t="s">
         <v>146</v>
-      </c>
-      <c r="M4" s="120" t="s">
-        <v>147</v>
       </c>
       <c r="N4" s="120" t="s">
         <v>75</v>
       </c>
       <c r="O4" s="123"/>
       <c r="P4" s="120" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="Q4" s="120" t="s">
         <v>73</v>
@@ -8603,10 +8567,10 @@
         <v>71</v>
       </c>
       <c r="V4" s="120" t="s">
+        <v>148</v>
+      </c>
+      <c r="W4" s="120" t="s">
         <v>149</v>
-      </c>
-      <c r="W4" s="120" t="s">
-        <v>150</v>
       </c>
       <c r="X4" s="120" t="s">
         <v>70</v>
@@ -8616,7 +8580,7 @@
         <v>69</v>
       </c>
       <c r="AA4" s="120" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="AB4" s="120" t="s">
         <v>68</v>
@@ -8633,7 +8597,9 @@
       <c r="A5" s="42"/>
       <c r="B5" s="41"/>
       <c r="C5" s="41"/>
-      <c r="D5" s="47"/>
+      <c r="D5" s="47" t="s">
+        <v>261</v>
+      </c>
       <c r="E5" s="117" t="s">
         <v>65</v>
       </c>
@@ -8746,8 +8712,8 @@
       <c r="B6" s="41"/>
       <c r="C6" s="41"/>
       <c r="D6" s="38" t="str">
-        <f t="shared" ref="D6:D15" si="0">IF(ISBLANK($D$5),"",$D$5)</f>
-        <v/>
+        <f>IF(ISBLANK($D$5),"",$D$5)</f>
+        <v>=ETPT_CA_JUR!D5</v>
       </c>
       <c r="E6" s="117" t="s">
         <v>63</v>
@@ -8788,7 +8754,7 @@
         <v/>
       </c>
       <c r="O6" s="79">
-        <f t="shared" ref="O6:O15" si="1">SUM(I6:N6)</f>
+        <f t="shared" ref="O6:O15" si="0">SUM(I6:N6)</f>
         <v>0</v>
       </c>
       <c r="P6" s="103" t="str">
@@ -8804,7 +8770,7 @@
         <v/>
       </c>
       <c r="S6" s="79">
-        <f t="shared" ref="S6:S16" si="2">SUM(P6:R6)</f>
+        <f t="shared" ref="S6:S16" si="1">SUM(P6:R6)</f>
         <v>0</v>
       </c>
       <c r="T6" s="103" t="str">
@@ -8828,7 +8794,7 @@
         <v/>
       </c>
       <c r="Y6" s="79">
-        <f t="shared" ref="Y6:Y16" si="3">SUM(T6:X6)</f>
+        <f t="shared" ref="Y6:Y16" si="2">SUM(T6:X6)</f>
         <v>0</v>
       </c>
       <c r="Z6" s="103" t="str">
@@ -8852,7 +8818,7 @@
         <v/>
       </c>
       <c r="AE6" s="79">
-        <f t="shared" ref="AE6:AE15" si="4">SUM(Z6:AD6)</f>
+        <f t="shared" ref="AE6:AE15" si="3">SUM(Z6:AD6)</f>
         <v>0</v>
       </c>
     </row>
@@ -8861,8 +8827,8 @@
       <c r="B7" s="41"/>
       <c r="C7" s="41"/>
       <c r="D7" s="38" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+        <f t="shared" ref="D7:D15" si="4">IF(ISBLANK($D$5),"",$D$5)</f>
+        <v>=ETPT_CA_JUR!D5</v>
       </c>
       <c r="E7" s="117" t="s">
         <v>61</v>
@@ -8903,7 +8869,7 @@
         <v/>
       </c>
       <c r="O7" s="79">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="P7" s="103" t="str">
@@ -8919,7 +8885,7 @@
         <v/>
       </c>
       <c r="S7" s="79">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="T7" s="103" t="str">
@@ -8943,7 +8909,7 @@
         <v/>
       </c>
       <c r="Y7" s="79">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="Z7" s="103" t="str">
@@ -8967,7 +8933,7 @@
         <v/>
       </c>
       <c r="AE7" s="79">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -8976,8 +8942,8 @@
       <c r="B8" s="41"/>
       <c r="C8" s="41"/>
       <c r="D8" s="38" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+        <f t="shared" si="4"/>
+        <v>=ETPT_CA_JUR!D5</v>
       </c>
       <c r="E8" s="117" t="s">
         <v>59</v>
@@ -9018,7 +8984,7 @@
         <v/>
       </c>
       <c r="O8" s="79">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="P8" s="103" t="str">
@@ -9034,7 +9000,7 @@
         <v/>
       </c>
       <c r="S8" s="79">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="T8" s="103" t="str">
@@ -9058,7 +9024,7 @@
         <v/>
       </c>
       <c r="Y8" s="79">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="Z8" s="103" t="str">
@@ -9082,7 +9048,7 @@
         <v/>
       </c>
       <c r="AE8" s="79">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -9091,8 +9057,8 @@
       <c r="B9" s="41"/>
       <c r="C9" s="41"/>
       <c r="D9" s="38" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+        <f t="shared" si="4"/>
+        <v>=ETPT_CA_JUR!D5</v>
       </c>
       <c r="E9" s="117" t="s">
         <v>57</v>
@@ -9133,7 +9099,7 @@
         <v/>
       </c>
       <c r="O9" s="79">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="P9" s="103" t="str">
@@ -9149,7 +9115,7 @@
         <v/>
       </c>
       <c r="S9" s="79">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="T9" s="103" t="str">
@@ -9173,7 +9139,7 @@
         <v/>
       </c>
       <c r="Y9" s="79">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="Z9" s="103" t="str">
@@ -9197,7 +9163,7 @@
         <v/>
       </c>
       <c r="AE9" s="79">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -9206,8 +9172,8 @@
       <c r="B10" s="41"/>
       <c r="C10" s="41"/>
       <c r="D10" s="38" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+        <f t="shared" si="4"/>
+        <v>=ETPT_CA_JUR!D5</v>
       </c>
       <c r="E10" s="117" t="s">
         <v>55</v>
@@ -9248,7 +9214,7 @@
         <v/>
       </c>
       <c r="O10" s="79">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="P10" s="103" t="str">
@@ -9264,7 +9230,7 @@
         <v/>
       </c>
       <c r="S10" s="79">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="T10" s="103" t="str">
@@ -9288,7 +9254,7 @@
         <v/>
       </c>
       <c r="Y10" s="79">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="Z10" s="103" t="str">
@@ -9312,7 +9278,7 @@
         <v/>
       </c>
       <c r="AE10" s="79">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -9321,8 +9287,8 @@
       <c r="B11" s="41"/>
       <c r="C11" s="41"/>
       <c r="D11" s="38" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+        <f t="shared" si="4"/>
+        <v>=ETPT_CA_JUR!D5</v>
       </c>
       <c r="E11" s="117" t="s">
         <v>53</v>
@@ -9363,7 +9329,7 @@
         <v/>
       </c>
       <c r="O11" s="79">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="P11" s="103" t="str">
@@ -9379,7 +9345,7 @@
         <v/>
       </c>
       <c r="S11" s="79">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="T11" s="103" t="str">
@@ -9403,7 +9369,7 @@
         <v/>
       </c>
       <c r="Y11" s="79">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="Z11" s="103" t="str">
@@ -9427,7 +9393,7 @@
         <v/>
       </c>
       <c r="AE11" s="79">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -9436,8 +9402,8 @@
       <c r="B12" s="41"/>
       <c r="C12" s="41"/>
       <c r="D12" s="38" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+        <f t="shared" si="4"/>
+        <v>=ETPT_CA_JUR!D5</v>
       </c>
       <c r="E12" s="117" t="s">
         <v>51</v>
@@ -9478,7 +9444,7 @@
         <v/>
       </c>
       <c r="O12" s="79">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="P12" s="103" t="str">
@@ -9494,7 +9460,7 @@
         <v/>
       </c>
       <c r="S12" s="79">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="T12" s="103" t="str">
@@ -9518,7 +9484,7 @@
         <v/>
       </c>
       <c r="Y12" s="79">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="Z12" s="103" t="str">
@@ -9542,7 +9508,7 @@
         <v/>
       </c>
       <c r="AE12" s="79">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -9551,8 +9517,8 @@
       <c r="B13" s="41"/>
       <c r="C13" s="41"/>
       <c r="D13" s="38" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+        <f t="shared" si="4"/>
+        <v>=ETPT_CA_JUR!D5</v>
       </c>
       <c r="E13" s="117" t="s">
         <v>49</v>
@@ -9593,7 +9559,7 @@
         <v/>
       </c>
       <c r="O13" s="79">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="P13" s="103" t="str">
@@ -9609,7 +9575,7 @@
         <v/>
       </c>
       <c r="S13" s="79">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="T13" s="103" t="str">
@@ -9633,7 +9599,7 @@
         <v/>
       </c>
       <c r="Y13" s="79">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="Z13" s="103" t="str">
@@ -9657,7 +9623,7 @@
         <v/>
       </c>
       <c r="AE13" s="79">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -9666,8 +9632,8 @@
       <c r="B14" s="39"/>
       <c r="C14" s="39"/>
       <c r="D14" s="38" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+        <f t="shared" si="4"/>
+        <v>=ETPT_CA_JUR!D5</v>
       </c>
       <c r="E14" s="117" t="s">
         <v>47</v>
@@ -9708,7 +9674,7 @@
         <v/>
       </c>
       <c r="O14" s="79">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="P14" s="103" t="str">
@@ -9724,7 +9690,7 @@
         <v/>
       </c>
       <c r="S14" s="79">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="T14" s="103" t="str">
@@ -9748,7 +9714,7 @@
         <v/>
       </c>
       <c r="Y14" s="79">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="Z14" s="103" t="str">
@@ -9772,20 +9738,20 @@
         <v/>
       </c>
       <c r="AE14" s="79">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:31" x14ac:dyDescent="0.2">
       <c r="D15" s="38" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+        <f t="shared" si="4"/>
+        <v>=ETPT_CA_JUR!D5</v>
       </c>
       <c r="E15" s="117" t="s">
+        <v>224</v>
+      </c>
+      <c r="F15" s="117" t="s">
         <v>225</v>
-      </c>
-      <c r="F15" s="117" t="s">
-        <v>226</v>
       </c>
       <c r="G15" s="103" t="str">
         <f>IF(ISBLANK($D$5),"",IF(ISERROR(ETPT_CA_JUR!G15),"",IF(ETPT_CA_JUR!G15=0,"",ETPT_CA_JUR!G15)))</f>
@@ -9820,7 +9786,7 @@
         <v/>
       </c>
       <c r="O15" s="79">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="P15" s="103" t="str">
@@ -9836,7 +9802,7 @@
         <v/>
       </c>
       <c r="S15" s="79">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="T15" s="103" t="str">
@@ -9860,7 +9826,7 @@
         <v/>
       </c>
       <c r="Y15" s="79">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="Z15" s="103" t="str">
@@ -9884,7 +9850,7 @@
         <v/>
       </c>
       <c r="AE15" s="79">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -9945,7 +9911,7 @@
         <v/>
       </c>
       <c r="S16" s="79">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="T16" s="103" t="str">
@@ -9969,7 +9935,7 @@
         <v/>
       </c>
       <c r="Y16" s="79">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="Z16" s="103" t="str">
@@ -10111,11 +10077,11 @@
       <c r="D19"/>
       <c r="E19"/>
       <c r="F19" s="121" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="G19" s="81" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé ADD") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé SUB")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé ADD") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé SUB")</f>
         <v>#N/A</v>
       </c>
       <c r="H19"/>
@@ -10124,11 +10090,11 @@
       <c r="K19"/>
       <c r="L19"/>
       <c r="M19" s="122" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="N19" s="81" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD") +
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("14. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD") +
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")</f>
         <v>#N/A</v>
       </c>
       <c r="O19"/>

</xml_diff>

<commit_message>
update tj formulas and ca formulas for red flags
</commit_message>
<xml_diff>
--- a/front/src/assets/template4CA.xlsx
+++ b/front/src/assets/template4CA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E59FE00-0DE0-B74A-85D2-839147B6F581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC2295E3-2210-BD4B-8397-364EAA6F4CCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" activeTab="3" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" activeTab="2" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
   <sheets>
     <sheet name="ACCUEIL" sheetId="33" r:id="rId1"/>
@@ -3468,7 +3468,47 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{6FC886D6-2077-B34D-B1DF-739B068A66D1}"/>
     <cellStyle name="Normal 3" xfId="4" xr:uid="{6BD57324-3FD5-D341-A299-730D14794802}"/>
   </cellStyles>
-  <dxfs count="16">
+  <dxfs count="18">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -3608,26 +3648,6 @@
       <font>
         <color theme="0"/>
       </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -6062,13 +6082,13 @@
   </sheetData>
   <autoFilter ref="A2:DT2" xr:uid="{3B89445B-6ECC-4440-B85C-E593AE209933}"/>
   <conditionalFormatting sqref="A1:EZ1 A2:FB1048576">
-    <cfRule type="expression" dxfId="15" priority="2" stopIfTrue="1">
-      <formula>AND(OR($N1&lt;&gt;"-",$O1&lt;&gt;0,$P1&lt;&gt;0),ROW()&gt;2,$A1&lt;&gt;"")</formula>
+    <cfRule type="expression" dxfId="3" priority="2" stopIfTrue="1">
+      <formula>AND(OR($Q1&lt;&gt;"-",$R1&lt;&gt;0,$S1&lt;&gt;0),ROW()&gt;2,$A1&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="FB2">
-    <cfRule type="expression" dxfId="14" priority="1" stopIfTrue="1">
-      <formula>AND(OR($N2&lt;&gt;"-",$O2&lt;&gt;0,$P2&lt;&gt;0),ROW()&gt;2,$A2&lt;&gt;"")</formula>
+    <cfRule type="expression" dxfId="2" priority="1" stopIfTrue="1">
+      <formula>AND(OR($Q2&lt;&gt;"-",$R2&lt;&gt;0,$S2&lt;&gt;0),ROW()&gt;2,$A2&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6377,64 +6397,64 @@
     <mergeCell ref="U4:V4"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:F4">
-    <cfRule type="expression" dxfId="13" priority="13">
+    <cfRule type="expression" dxfId="17" priority="13">
       <formula>IF(LEFT($A$3,2)&lt;&gt;"TJ",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:V151">
-    <cfRule type="expression" dxfId="12" priority="15">
+    <cfRule type="expression" dxfId="16" priority="15">
       <formula>AND(ISBLANK($C6)=FALSE,ISBLANK($E6)=TRUE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:F1048576">
-    <cfRule type="expression" dxfId="11" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="15" priority="11" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)+_xlfn.NUMBERVALUE($L4)-_xlfn.NUMBERVALUE($L5)+_xlfn.NUMBERVALUE($L6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="12">
+    <cfRule type="expression" dxfId="14" priority="12">
       <formula>AND($D1="7. TOTAL CONTENTIEUX DES MINEURS",OR(_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3))&lt;&gt;0,_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3))&lt;&gt;0,_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3))&lt;&gt;0))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D7:F7">
-    <cfRule type="expression" dxfId="9" priority="10" stopIfTrue="1">
+    <cfRule type="expression" dxfId="13" priority="10" stopIfTrue="1">
       <formula>OR(_xlfn.NUMBERVALUE($L6)&lt;&gt;_xlfn.NUMBERVALUE($L7),_xlfn.NUMBERVALUE($S6)&lt;&gt;_xlfn.NUMBERVALUE($S7),_xlfn.NUMBERVALUE($U6)&lt;&gt;_xlfn.NUMBERVALUE($U7))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:M1048576">
-    <cfRule type="expression" dxfId="8" priority="8" stopIfTrue="1">
+    <cfRule type="expression" dxfId="12" priority="8" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)+_xlfn.NUMBERVALUE($L4)+_xlfn.NUMBERVALUE($L5)+_xlfn.NUMBERVALUE($L6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="9">
+    <cfRule type="expression" dxfId="11" priority="9">
       <formula>AND($D1="7. TOTAL CONTENTIEUX DES MINEURS",_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3))&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G7:M7">
-    <cfRule type="expression" dxfId="6" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="10" priority="7" stopIfTrue="1">
       <formula>_xlfn.NUMBERVALUE($L7)&lt;&gt;_xlfn.NUMBERVALUE($L6)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1:T1048576">
-    <cfRule type="expression" dxfId="5" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="9" priority="5" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3)+_xlfn.NUMBERVALUE($S4)+_xlfn.NUMBERVALUE($S5)+_xlfn.NUMBERVALUE($S6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="8" priority="6" stopIfTrue="1">
       <formula>AND($D1="7. TOTAL CONTENTIEUX DES MINEURS",_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3))&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N7:T7">
-    <cfRule type="expression" dxfId="3" priority="4" stopIfTrue="1">
+    <cfRule type="expression" dxfId="7" priority="4" stopIfTrue="1">
       <formula>_xlfn.NUMBERVALUE($S7)&lt;&gt;_xlfn.NUMBERVALUE($S6)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U1:V1048576">
-    <cfRule type="expression" dxfId="2" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="6" priority="2" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3)+_xlfn.NUMBERVALUE($U4)+_xlfn.NUMBERVALUE($U5)+_xlfn.NUMBERVALUE($U6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="3">
+    <cfRule type="expression" dxfId="5" priority="3">
       <formula>AND($D1="7. TOTAL CONTENTIEUX DES MINEURS",_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3))&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U7:V7">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="4" priority="1">
       <formula>_xlfn.NUMBERVALUE($U7)&lt;&gt;_xlfn.NUMBERVALUE($U6)</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
update ca fct extractor
</commit_message>
<xml_diff>
--- a/front/src/assets/template4CA.xlsx
+++ b/front/src/assets/template4CA.xlsx
@@ -8,21 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC2295E3-2210-BD4B-8397-364EAA6F4CCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B912543D-DB11-D549-B65C-628E6050E5AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" activeTab="2" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" activeTab="6" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
   <sheets>
     <sheet name="ACCUEIL" sheetId="33" r:id="rId1"/>
     <sheet name="ETPT A-JUST" sheetId="1" r:id="rId2"/>
     <sheet name="ETPT Format DDG" sheetId="9" r:id="rId3"/>
     <sheet name="Agrégats DDG" sheetId="10" r:id="rId4"/>
-    <sheet name="codage tribunal" sheetId="12" state="hidden" r:id="rId5"/>
-    <sheet name="Juridictions" sheetId="17" state="hidden" r:id="rId6"/>
-    <sheet name="Table_Fonctions" sheetId="19" state="hidden" r:id="rId7"/>
-    <sheet name="ETPT_CA_JUR" sheetId="30" state="hidden" r:id="rId8"/>
+    <sheet name="codage tribunal" sheetId="12" r:id="rId5"/>
+    <sheet name="Juridictions" sheetId="17" r:id="rId6"/>
+    <sheet name="Table_Fonctions" sheetId="19" r:id="rId7"/>
+    <sheet name="ETPT_CA_JUR" sheetId="30" r:id="rId8"/>
     <sheet name="ETPT_CA_JUR_DDG" sheetId="25" r:id="rId9"/>
-    <sheet name="ETPT_CA_JUR Corresp" sheetId="38" state="hidden" r:id="rId10"/>
+    <sheet name="ETPT_CA_JUR Corresp" sheetId="38" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ETPT A-JUST'!$A$2:$DN$2</definedName>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="541" uniqueCount="265">
   <si>
     <t>#! END_ROW</t>
   </si>
@@ -151,9 +151,6 @@
     <t>Juridiction</t>
   </si>
   <si>
-    <t>Fonction</t>
-  </si>
-  <si>
     <t>Fonction recodée</t>
   </si>
   <si>
@@ -167,18 +164,6 @@
   </si>
   <si>
     <t>JURISTE AS</t>
-  </si>
-  <si>
-    <t>CODE EXTRACTEUR</t>
-  </si>
-  <si>
-    <t>Titulaire / Placé / Contractuel</t>
-  </si>
-  <si>
-    <t>Raccourci</t>
-  </si>
-  <si>
-    <t>Catégorie(s)</t>
   </si>
   <si>
     <t>TOTAL ETPT</t>
@@ -2109,9 +2094,6 @@
     </r>
   </si>
   <si>
-    <t>Correspondance</t>
-  </si>
-  <si>
     <t>PARQUET_JIRS</t>
   </si>
   <si>
@@ -2164,6 +2146,27 @@
   </si>
   <si>
     <t>#! DUMP_COLS subtitles1</t>
+  </si>
+  <si>
+    <t>CONCAT</t>
+  </si>
+  <si>
+    <t>Catégorie</t>
+  </si>
+  <si>
+    <t>Label</t>
+  </si>
+  <si>
+    <t>Position</t>
+  </si>
+  <si>
+    <t>Fonction recodée DDG</t>
+  </si>
+  <si>
+    <t>Fonction onglet agrégat</t>
+  </si>
+  <si>
+    <t>## f.CONCAT</t>
   </si>
 </sst>
 </file>
@@ -2503,7 +2506,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="22">
+  <fills count="21">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2621,12 +2624,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF00B252"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -3005,7 +3002,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="153">
+  <cellXfs count="152">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -3339,15 +3336,6 @@
     <xf numFmtId="49" fontId="45" fillId="9" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="21" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="20" fillId="8" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3457,6 +3445,12 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3468,47 +3462,7 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{6FC886D6-2077-B34D-B1DF-739B068A66D1}"/>
     <cellStyle name="Normal 3" xfId="4" xr:uid="{6BD57324-3FD5-D341-A299-730D14794802}"/>
   </cellStyles>
-  <dxfs count="18">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="16">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -3648,6 +3602,26 @@
       <font>
         <color theme="0"/>
       </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -4415,13 +4389,13 @@
     <row r="1" spans="1:8" s="26" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="50"/>
       <c r="B1" s="51" t="s">
-        <v>111</v>
-      </c>
-      <c r="C1" s="126" t="s">
-        <v>112</v>
-      </c>
-      <c r="D1" s="126"/>
-      <c r="E1" s="126"/>
+        <v>106</v>
+      </c>
+      <c r="C1" s="123" t="s">
+        <v>107</v>
+      </c>
+      <c r="D1" s="123"/>
+      <c r="E1" s="123"/>
       <c r="F1" s="52"/>
       <c r="H1" s="26" t="s">
         <v>0</v>
@@ -4430,11 +4404,11 @@
     <row r="2" spans="1:8" s="56" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="53"/>
       <c r="B2" s="54"/>
-      <c r="C2" s="127" t="s">
-        <v>138</v>
-      </c>
-      <c r="D2" s="127"/>
-      <c r="E2" s="127"/>
+      <c r="C2" s="124" t="s">
+        <v>133</v>
+      </c>
+      <c r="D2" s="124"/>
+      <c r="E2" s="124"/>
       <c r="F2" s="55"/>
       <c r="H2" s="26" t="s">
         <v>0</v>
@@ -4450,18 +4424,18 @@
     <row r="4" spans="1:8" s="62" customFormat="1" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="59"/>
       <c r="B4" s="60" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="C4" s="61" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="D4" s="61" t="s">
-        <v>115</v>
-      </c>
-      <c r="E4" s="133" t="s">
-        <v>116</v>
-      </c>
-      <c r="F4" s="134"/>
+        <v>110</v>
+      </c>
+      <c r="E4" s="130" t="s">
+        <v>111</v>
+      </c>
+      <c r="F4" s="131"/>
       <c r="G4" s="68"/>
       <c r="H4" s="26" t="s">
         <v>0</v>
@@ -4470,18 +4444,18 @@
     <row r="5" spans="1:8" s="26" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="57"/>
       <c r="B5" s="72" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="C5" s="65" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="D5" s="65" t="s">
-        <v>119</v>
-      </c>
-      <c r="E5" s="135" t="s">
-        <v>132</v>
-      </c>
-      <c r="F5" s="136"/>
+        <v>114</v>
+      </c>
+      <c r="E5" s="132" t="s">
+        <v>127</v>
+      </c>
+      <c r="F5" s="133"/>
       <c r="G5" s="67"/>
       <c r="H5" s="26" t="s">
         <v>0</v>
@@ -4490,18 +4464,18 @@
     <row r="6" spans="1:8" s="26" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="57"/>
       <c r="B6" s="73" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="C6" s="66" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="D6" s="66" t="s">
-        <v>122</v>
-      </c>
-      <c r="E6" s="137" t="s">
-        <v>133</v>
-      </c>
-      <c r="F6" s="138"/>
+        <v>117</v>
+      </c>
+      <c r="E6" s="134" t="s">
+        <v>128</v>
+      </c>
+      <c r="F6" s="135"/>
       <c r="G6" s="67"/>
       <c r="H6" s="26" t="s">
         <v>0</v>
@@ -4510,18 +4484,18 @@
     <row r="7" spans="1:8" s="26" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="57"/>
       <c r="B7" s="74" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="C7" s="66" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="D7" s="66" t="s">
-        <v>125</v>
-      </c>
-      <c r="E7" s="137" t="s">
-        <v>132</v>
-      </c>
-      <c r="F7" s="138"/>
+        <v>120</v>
+      </c>
+      <c r="E7" s="134" t="s">
+        <v>127</v>
+      </c>
+      <c r="F7" s="135"/>
       <c r="G7" s="67"/>
       <c r="H7" s="26" t="s">
         <v>0</v>
@@ -4530,18 +4504,18 @@
     <row r="8" spans="1:8" s="26" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="57"/>
       <c r="B8" s="75" t="s">
-        <v>126</v>
-      </c>
-      <c r="C8" s="128" t="s">
-        <v>127</v>
-      </c>
-      <c r="D8" s="128" t="s">
-        <v>128</v>
-      </c>
-      <c r="E8" s="139" t="s">
-        <v>134</v>
-      </c>
-      <c r="F8" s="140"/>
+        <v>121</v>
+      </c>
+      <c r="C8" s="125" t="s">
+        <v>122</v>
+      </c>
+      <c r="D8" s="125" t="s">
+        <v>123</v>
+      </c>
+      <c r="E8" s="136" t="s">
+        <v>129</v>
+      </c>
+      <c r="F8" s="137"/>
       <c r="G8" s="67"/>
       <c r="H8" s="26" t="s">
         <v>0</v>
@@ -4550,12 +4524,12 @@
     <row r="9" spans="1:8" s="26" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="57"/>
       <c r="B9" s="76" t="s">
-        <v>129</v>
-      </c>
-      <c r="C9" s="128"/>
-      <c r="D9" s="128"/>
-      <c r="E9" s="141"/>
-      <c r="F9" s="142"/>
+        <v>124</v>
+      </c>
+      <c r="C9" s="125"/>
+      <c r="D9" s="125"/>
+      <c r="E9" s="138"/>
+      <c r="F9" s="139"/>
       <c r="G9" s="67"/>
       <c r="H9" s="26" t="s">
         <v>0</v>
@@ -4564,12 +4538,12 @@
     <row r="10" spans="1:8" s="26" customFormat="1" ht="23" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="57"/>
       <c r="B10" s="77" t="s">
-        <v>130</v>
-      </c>
-      <c r="C10" s="129"/>
-      <c r="D10" s="129"/>
-      <c r="E10" s="143"/>
-      <c r="F10" s="144"/>
+        <v>125</v>
+      </c>
+      <c r="C10" s="126"/>
+      <c r="D10" s="126"/>
+      <c r="E10" s="140"/>
+      <c r="F10" s="141"/>
       <c r="G10" s="67"/>
       <c r="H10" s="26" t="s">
         <v>0</v>
@@ -4589,11 +4563,11 @@
     <row r="12" spans="1:8" s="26" customFormat="1" ht="72" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="57"/>
       <c r="B12" s="69"/>
-      <c r="C12" s="132" t="s">
-        <v>131</v>
-      </c>
-      <c r="D12" s="132"/>
-      <c r="E12" s="132"/>
+      <c r="C12" s="129" t="s">
+        <v>126</v>
+      </c>
+      <c r="D12" s="129"/>
+      <c r="E12" s="129"/>
       <c r="F12" s="70"/>
       <c r="H12" s="26" t="s">
         <v>0</v>
@@ -4607,14 +4581,14 @@
       </c>
     </row>
     <row r="14" spans="1:8" s="26" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="130" t="s">
+      <c r="A14" s="127" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="130"/>
-      <c r="C14" s="130"/>
-      <c r="D14" s="130"/>
-      <c r="E14" s="130"/>
-      <c r="F14" s="131"/>
+      <c r="B14" s="127"/>
+      <c r="C14" s="127"/>
+      <c r="D14" s="127"/>
+      <c r="E14" s="127"/>
+      <c r="F14" s="128"/>
       <c r="H14" s="26" t="s">
         <v>0</v>
       </c>
@@ -4653,13 +4627,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A1" s="151" t="s">
-        <v>139</v>
-      </c>
-      <c r="B1" s="151"/>
-      <c r="C1" s="151"/>
-      <c r="D1" s="151"/>
-      <c r="E1" s="151"/>
+      <c r="A1" s="148" t="s">
+        <v>134</v>
+      </c>
+      <c r="B1" s="148"/>
+      <c r="C1" s="148"/>
+      <c r="D1" s="148"/>
+      <c r="E1" s="148"/>
       <c r="F1" s="96"/>
       <c r="G1" s="78"/>
       <c r="H1" s="78"/>
@@ -4689,61 +4663,61 @@
       <c r="E2" s="97"/>
       <c r="F2" s="97"/>
       <c r="G2" s="80" t="s">
-        <v>106</v>
-      </c>
-      <c r="H2" s="152" t="s">
-        <v>105</v>
+        <v>101</v>
+      </c>
+      <c r="H2" s="149" t="s">
+        <v>100</v>
       </c>
       <c r="I2" s="80" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="J2" s="80" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="K2" s="80" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="L2" s="80" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="M2" s="80" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="N2" s="80" t="s">
-        <v>104</v>
-      </c>
-      <c r="O2" s="152" t="s">
-        <v>103</v>
+        <v>99</v>
+      </c>
+      <c r="O2" s="149" t="s">
+        <v>98</v>
       </c>
       <c r="P2" s="80" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="Q2" s="80" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="R2" s="80" t="s">
-        <v>38</v>
-      </c>
-      <c r="S2" s="152" t="s">
-        <v>102</v>
+        <v>37</v>
+      </c>
+      <c r="S2" s="149" t="s">
+        <v>97</v>
       </c>
       <c r="T2" s="80" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="U2" s="80" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="V2" s="80" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="W2" s="80" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="X2" s="80" t="s">
-        <v>101</v>
-      </c>
-      <c r="Y2" s="152" t="s">
-        <v>100</v>
+        <v>96</v>
+      </c>
+      <c r="Y2" s="149" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="3" spans="1:25" ht="56" x14ac:dyDescent="0.2">
@@ -4754,166 +4728,166 @@
       <c r="E3" s="97"/>
       <c r="F3" s="97"/>
       <c r="G3" s="80" t="s">
-        <v>97</v>
-      </c>
-      <c r="H3" s="152"/>
+        <v>92</v>
+      </c>
+      <c r="H3" s="149"/>
       <c r="I3" s="80" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="J3" s="80" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="K3" s="80" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="L3" s="80" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="M3" s="80" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="N3" s="80" t="s">
-        <v>93</v>
-      </c>
-      <c r="O3" s="152"/>
+        <v>88</v>
+      </c>
+      <c r="O3" s="149"/>
       <c r="P3" s="80" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="Q3" s="80" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="R3" s="80" t="s">
-        <v>92</v>
-      </c>
-      <c r="S3" s="152"/>
+        <v>87</v>
+      </c>
+      <c r="S3" s="149"/>
       <c r="T3" s="80" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="U3" s="80" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="V3" s="80" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="W3" s="80" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="X3" s="80" t="s">
-        <v>88</v>
-      </c>
-      <c r="Y3" s="152"/>
+        <v>83</v>
+      </c>
+      <c r="Y3" s="149"/>
     </row>
     <row r="4" spans="1:25" ht="84" x14ac:dyDescent="0.2">
       <c r="A4" s="98"/>
       <c r="B4" s="99" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="C4" s="99" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="D4" s="99" t="s">
         <v>32</v>
       </c>
       <c r="E4" s="99" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F4" s="99" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="G4" s="80" t="s">
-        <v>79</v>
-      </c>
-      <c r="H4" s="152"/>
+        <v>74</v>
+      </c>
+      <c r="H4" s="149"/>
       <c r="I4" s="80" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J4" s="80" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="K4" s="80" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="L4" s="80" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="M4" s="80" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="N4" s="80" t="s">
-        <v>75</v>
-      </c>
-      <c r="O4" s="152"/>
+        <v>70</v>
+      </c>
+      <c r="O4" s="149"/>
       <c r="P4" s="80" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="Q4" s="80" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="R4" s="80" t="s">
-        <v>74</v>
-      </c>
-      <c r="S4" s="152"/>
+        <v>69</v>
+      </c>
+      <c r="S4" s="149"/>
       <c r="T4" s="80" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="U4" s="80" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="V4" s="80" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="W4" s="80" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="X4" s="80" t="s">
-        <v>70</v>
-      </c>
-      <c r="Y4" s="152"/>
+        <v>65</v>
+      </c>
+      <c r="Y4" s="149"/>
     </row>
     <row r="5" spans="1:25" ht="332" x14ac:dyDescent="0.2">
       <c r="A5" s="100" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="B5" s="101"/>
       <c r="C5" s="101"/>
       <c r="D5" s="101"/>
       <c r="E5" s="101" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="F5" s="102" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="G5" s="81" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="H5" s="79">
         <f>SUMIF($G$2:G$2,G$2,$G5:G5)</f>
         <v>0</v>
       </c>
       <c r="I5" s="81" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="J5" s="83"/>
       <c r="K5" s="83"/>
       <c r="L5" s="83"/>
       <c r="M5" s="81" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="N5" s="81" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="O5" s="79">
         <f>SUMIF($G$2:N$2,N$2,$G5:N5)</f>
         <v>0</v>
       </c>
       <c r="P5" s="81" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="Q5" s="81" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="R5" s="81" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="S5" s="79">
         <f>SUMIF($G$2:R$2,R$2,$G5:R5)</f>
@@ -4923,10 +4897,10 @@
       <c r="U5" s="83"/>
       <c r="V5" s="83"/>
       <c r="W5" s="81" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="X5" s="81" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="Y5" s="79">
         <f>SUMIF($G$2:X$2,X$2,$G5:X5)</f>
@@ -4935,19 +4909,19 @@
     </row>
     <row r="6" spans="1:25" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A6" s="100" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="B6" s="101"/>
       <c r="C6" s="101"/>
       <c r="D6" s="101"/>
       <c r="E6" s="101" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="F6" s="102" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="G6" s="81" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="H6" s="79">
         <f>SUMIF($G$2:G$2,G$2,$G6:G6)</f>
@@ -4955,47 +4929,47 @@
       </c>
       <c r="I6" s="82"/>
       <c r="J6" s="81" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="K6" s="81" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="L6" s="81" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="M6" s="83"/>
       <c r="N6" s="81" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="O6" s="79">
         <f>SUMIF($G$2:N$2,N$2,$G6:N6)</f>
         <v>0</v>
       </c>
       <c r="P6" s="81" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="Q6" s="81" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="R6" s="81" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="S6" s="79">
         <f>SUMIF($G$2:R$2,R$2,$G6:R6)</f>
         <v>0</v>
       </c>
       <c r="T6" s="81" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="U6" s="81" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="V6" s="81" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="W6" s="83"/>
       <c r="X6" s="81" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="Y6" s="79">
         <f>SUMIF($G$2:X$2,X$2,$G6:X6)</f>
@@ -5004,16 +4978,16 @@
     </row>
     <row r="7" spans="1:25" ht="90" x14ac:dyDescent="0.2">
       <c r="A7" s="100" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="B7" s="101"/>
       <c r="C7" s="101"/>
       <c r="D7" s="101"/>
       <c r="E7" s="101" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="F7" s="102" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="G7" s="86"/>
       <c r="H7" s="79">
@@ -5042,7 +5016,7 @@
       <c r="V7" s="103"/>
       <c r="W7" s="103"/>
       <c r="X7" s="104" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="Y7" s="79">
         <f>SUMIF($G$2:X$2,X$2,$G7:X7)</f>
@@ -5051,19 +5025,19 @@
     </row>
     <row r="8" spans="1:25" ht="140" x14ac:dyDescent="0.2">
       <c r="A8" s="100" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="B8" s="101"/>
       <c r="C8" s="101"/>
       <c r="D8" s="101"/>
       <c r="E8" s="101" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="F8" s="102" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="G8" s="81" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="H8" s="79">
         <f>SUMIF($G$2:G$2,G$2,$G8:G8)</f>
@@ -5075,20 +5049,20 @@
       <c r="L8" s="85"/>
       <c r="M8" s="85"/>
       <c r="N8" s="81" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="O8" s="79">
         <f>SUMIF($G$2:N$2,N$2,$G8:N8)</f>
         <v>0</v>
       </c>
       <c r="P8" s="81" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="Q8" s="81" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="R8" s="81" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="S8" s="79">
         <f>SUMIF($G$2:R$2,R$2,$G8:R8)</f>
@@ -5099,7 +5073,7 @@
       <c r="V8" s="103"/>
       <c r="W8" s="103"/>
       <c r="X8" s="81" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="Y8" s="79">
         <f>SUMIF($G$2:X$2,X$2,$G8:X8)</f>
@@ -5108,19 +5082,19 @@
     </row>
     <row r="9" spans="1:25" ht="154" x14ac:dyDescent="0.2">
       <c r="A9" s="100" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="B9" s="101"/>
       <c r="C9" s="101"/>
       <c r="D9" s="101"/>
       <c r="E9" s="101" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F9" s="102" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="G9" s="81" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="H9" s="79">
         <f>SUMIF($G$2:G$2,G$2,$G9:G9)</f>
@@ -5132,20 +5106,20 @@
       <c r="L9" s="85"/>
       <c r="M9" s="85"/>
       <c r="N9" s="81" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="O9" s="79">
         <f>SUMIF($G$2:N$2,N$2,$G9:N9)</f>
         <v>0</v>
       </c>
       <c r="P9" s="81" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="Q9" s="81" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="R9" s="81" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="S9" s="79">
         <f>SUMIF($G$2:R$2,R$2,$G9:R9)</f>
@@ -5156,7 +5130,7 @@
       <c r="V9" s="103"/>
       <c r="W9" s="103"/>
       <c r="X9" s="81" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="Y9" s="79">
         <f>SUMIF($G$2:X$2,X$2,$G9:X9)</f>
@@ -5165,19 +5139,19 @@
     </row>
     <row r="10" spans="1:25" ht="140" x14ac:dyDescent="0.2">
       <c r="A10" s="100" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="B10" s="101"/>
       <c r="C10" s="101"/>
       <c r="D10" s="101"/>
       <c r="E10" s="101" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F10" s="102" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="G10" s="81" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="H10" s="79">
         <f>SUMIF($G$2:G$2,G$2,$G10:G10)</f>
@@ -5189,20 +5163,20 @@
       <c r="L10" s="85"/>
       <c r="M10" s="85"/>
       <c r="N10" s="81" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="O10" s="79">
         <f>SUMIF($G$2:N$2,N$2,$G10:N10)</f>
         <v>0</v>
       </c>
       <c r="P10" s="81" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="Q10" s="81" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="R10" s="81" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="S10" s="79">
         <f>SUMIF($G$2:R$2,R$2,$G10:R10)</f>
@@ -5213,7 +5187,7 @@
       <c r="V10" s="103"/>
       <c r="W10" s="103"/>
       <c r="X10" s="81" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="Y10" s="79">
         <f>SUMIF($G$2:X$2,X$2,$G10:X10)</f>
@@ -5222,19 +5196,19 @@
     </row>
     <row r="11" spans="1:25" ht="140" x14ac:dyDescent="0.2">
       <c r="A11" s="100" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="B11" s="101"/>
       <c r="C11" s="101"/>
       <c r="D11" s="101"/>
       <c r="E11" s="101" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="F11" s="102" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="G11" s="81" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="H11" s="79">
         <f>SUMIF($G$2:G$2,G$2,$G11:G11)</f>
@@ -5246,20 +5220,20 @@
       <c r="L11" s="85"/>
       <c r="M11" s="85"/>
       <c r="N11" s="81" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="O11" s="79">
         <f>SUMIF($G$2:N$2,N$2,$G11:N11)</f>
         <v>0</v>
       </c>
       <c r="P11" s="81" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="Q11" s="81" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="R11" s="81" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="S11" s="79">
         <f>SUMIF($G$2:R$2,R$2,$G11:R11)</f>
@@ -5270,7 +5244,7 @@
       <c r="V11" s="103"/>
       <c r="W11" s="103"/>
       <c r="X11" s="81" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="Y11" s="79">
         <f>SUMIF($G$2:X$2,X$2,$G11:X11)</f>
@@ -5279,19 +5253,19 @@
     </row>
     <row r="12" spans="1:25" ht="168" x14ac:dyDescent="0.2">
       <c r="A12" s="100" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="B12" s="101"/>
       <c r="C12" s="101"/>
       <c r="D12" s="101"/>
       <c r="E12" s="101" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="F12" s="102" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="G12" s="81" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="H12" s="79">
         <f>SUMIF($G$2:G$2,G$2,$G12:G12)</f>
@@ -5303,20 +5277,20 @@
       <c r="L12" s="85"/>
       <c r="M12" s="85"/>
       <c r="N12" s="81" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="O12" s="79">
         <f>SUMIF($G$2:N$2,N$2,$G12:N12)</f>
         <v>0</v>
       </c>
       <c r="P12" s="81" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="Q12" s="81" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="R12" s="81" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="S12" s="79">
         <f>SUMIF($G$2:R$2,R$2,$G12:R12)</f>
@@ -5327,7 +5301,7 @@
       <c r="V12" s="103"/>
       <c r="W12" s="103"/>
       <c r="X12" s="81" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="Y12" s="79">
         <f>SUMIF($G$2:X$2,X$2,$G12:X12)</f>
@@ -5336,19 +5310,19 @@
     </row>
     <row r="13" spans="1:25" ht="126" x14ac:dyDescent="0.2">
       <c r="A13" s="100" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="B13" s="101"/>
       <c r="C13" s="101"/>
       <c r="D13" s="101"/>
       <c r="E13" s="101" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="F13" s="102" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="G13" s="81" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="H13" s="79">
         <f>SUMIF($G$2:G$2,G$2,$G13:G13)</f>
@@ -5360,20 +5334,20 @@
       <c r="L13" s="85"/>
       <c r="M13" s="85"/>
       <c r="N13" s="81" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="O13" s="79">
         <f>SUMIF($G$2:N$2,N$2,$G13:N13)</f>
         <v>0</v>
       </c>
       <c r="P13" s="81" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="Q13" s="81" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="R13" s="81" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="S13" s="79">
         <f>SUMIF($G$2:R$2,R$2,$G13:R13)</f>
@@ -5384,7 +5358,7 @@
       <c r="V13" s="103"/>
       <c r="W13" s="103"/>
       <c r="X13" s="81" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="Y13" s="79">
         <f>SUMIF($G$2:X$2,X$2,$G13:X13)</f>
@@ -5393,73 +5367,73 @@
     </row>
     <row r="14" spans="1:25" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A14" s="100" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="B14" s="101"/>
       <c r="C14" s="101"/>
       <c r="D14" s="101"/>
       <c r="E14" s="101" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="F14" s="102" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="G14" s="81" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="H14" s="79">
         <f>SUMIF($G$2:G$2,G$2,$G14:G14)</f>
         <v>0</v>
       </c>
       <c r="I14" s="81" t="s">
+        <v>205</v>
+      </c>
+      <c r="J14" s="81" t="s">
+        <v>206</v>
+      </c>
+      <c r="K14" s="81" t="s">
+        <v>207</v>
+      </c>
+      <c r="L14" s="81" t="s">
+        <v>208</v>
+      </c>
+      <c r="M14" s="81" t="s">
+        <v>209</v>
+      </c>
+      <c r="N14" s="81" t="s">
         <v>210</v>
-      </c>
-      <c r="J14" s="81" t="s">
-        <v>211</v>
-      </c>
-      <c r="K14" s="81" t="s">
-        <v>212</v>
-      </c>
-      <c r="L14" s="81" t="s">
-        <v>213</v>
-      </c>
-      <c r="M14" s="81" t="s">
-        <v>214</v>
-      </c>
-      <c r="N14" s="81" t="s">
-        <v>215</v>
       </c>
       <c r="O14" s="79">
         <f>SUMIF($G$2:N$2,N$2,$G14:N14)</f>
         <v>0</v>
       </c>
       <c r="P14" s="81" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="Q14" s="81" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="R14" s="81" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="S14" s="79">
         <f>SUMIF($G$2:R$2,R$2,$G14:R14)</f>
         <v>0</v>
       </c>
       <c r="T14" s="81" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="U14" s="81" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="V14" s="81" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="W14" s="81" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="X14" s="81" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="Y14" s="79">
         <f>SUMIF($G$2:X$2,X$2,$G14:X14)</f>
@@ -5468,16 +5442,16 @@
     </row>
     <row r="15" spans="1:25" ht="224" x14ac:dyDescent="0.2">
       <c r="A15" s="100" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="B15" s="101"/>
       <c r="C15" s="101"/>
       <c r="D15" s="101"/>
       <c r="E15" s="101" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="F15" s="105" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="G15" s="106"/>
       <c r="H15" s="79">
@@ -5495,13 +5469,13 @@
         <v>0</v>
       </c>
       <c r="P15" s="81" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="Q15" s="81" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="R15" s="81" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="S15" s="79">
         <f>SUMIF($G$2:R$2,R$2,$G15:R15)</f>
@@ -5512,7 +5486,7 @@
       <c r="V15" s="108"/>
       <c r="W15" s="108"/>
       <c r="X15" s="81" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="Y15" s="79">
         <f>SUMIF($G$2:X$2,X$2,$G15:X15)</f>
@@ -5521,73 +5495,73 @@
     </row>
     <row r="16" spans="1:25" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A16" s="100" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="B16" s="101"/>
       <c r="C16" s="101"/>
       <c r="D16" s="101"/>
       <c r="E16" s="101" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F16" s="102" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="G16" s="81" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="H16" s="79">
         <f>SUMIF($G$2:G$2,G$2,$G16:G16)</f>
         <v>0</v>
       </c>
       <c r="I16" s="81" t="s">
+        <v>226</v>
+      </c>
+      <c r="J16" s="81" t="s">
+        <v>227</v>
+      </c>
+      <c r="K16" s="81" t="s">
+        <v>228</v>
+      </c>
+      <c r="L16" s="81" t="s">
+        <v>229</v>
+      </c>
+      <c r="M16" s="81" t="s">
+        <v>230</v>
+      </c>
+      <c r="N16" s="81" t="s">
         <v>231</v>
-      </c>
-      <c r="J16" s="81" t="s">
-        <v>232</v>
-      </c>
-      <c r="K16" s="81" t="s">
-        <v>233</v>
-      </c>
-      <c r="L16" s="81" t="s">
-        <v>234</v>
-      </c>
-      <c r="M16" s="81" t="s">
-        <v>235</v>
-      </c>
-      <c r="N16" s="81" t="s">
-        <v>236</v>
       </c>
       <c r="O16" s="79">
         <f>SUMIF($G$2:N$2,N$2,$G16:N16)</f>
         <v>0</v>
       </c>
       <c r="P16" s="81" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="Q16" s="81" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="R16" s="81" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="S16" s="79">
         <f>SUMIF($G$2:R$2,R$2,$G16:R16)</f>
         <v>0</v>
       </c>
       <c r="T16" s="81" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="U16" s="81" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="V16" s="81" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="W16" s="81" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="X16" s="81" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="Y16" s="79">
         <f>SUMIF($G$2:X$2,X$2,$G16:X16)</f>
@@ -5601,7 +5575,7 @@
       <c r="D17" s="110"/>
       <c r="E17" s="110"/>
       <c r="F17" s="112" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="G17" s="79">
         <f>SUMIF($C$5:$C16,$C16,G$5:G16)</f>
@@ -5712,7 +5686,7 @@
   <sheetData>
     <row r="1" spans="1:118" s="4" customFormat="1" ht="80" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -6034,7 +6008,7 @@
   <sheetData>
     <row r="1" spans="1:158" s="4" customFormat="1" ht="80" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -6042,7 +6016,7 @@
       <c r="E1" s="7"/>
       <c r="F1" s="6"/>
       <c r="G1" s="6" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="FA1" s="8" t="s">
         <v>0</v>
@@ -6059,10 +6033,10 @@
         <v>9</v>
       </c>
       <c r="FA2" s="48" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="FB2" s="48" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
     </row>
     <row r="3" spans="1:158" x14ac:dyDescent="0.2">
@@ -6082,12 +6056,12 @@
   </sheetData>
   <autoFilter ref="A2:DT2" xr:uid="{3B89445B-6ECC-4440-B85C-E593AE209933}"/>
   <conditionalFormatting sqref="A1:EZ1 A2:FB1048576">
-    <cfRule type="expression" dxfId="3" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="15" priority="2" stopIfTrue="1">
       <formula>AND(OR($Q1&lt;&gt;"-",$R1&lt;&gt;0,$S1&lt;&gt;0),ROW()&gt;2,$A1&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="FB2">
-    <cfRule type="expression" dxfId="2" priority="1" stopIfTrue="1">
+    <cfRule type="expression" dxfId="14" priority="1" stopIfTrue="1">
       <formula>AND(OR($Q2&lt;&gt;"-",$R2&lt;&gt;0,$S2&lt;&gt;0),ROW()&gt;2,$A2&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6124,7 +6098,7 @@
       <c r="A1" s="3"/>
       <c r="B1" s="5"/>
       <c r="C1" s="64" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="D1" s="64"/>
       <c r="E1" s="7"/>
@@ -6179,28 +6153,28 @@
       <c r="D4" s="87"/>
       <c r="E4" s="87"/>
       <c r="F4" s="87"/>
-      <c r="G4" s="145" t="s">
+      <c r="G4" s="142" t="s">
         <v>26</v>
       </c>
-      <c r="H4" s="146"/>
-      <c r="I4" s="146"/>
-      <c r="J4" s="146"/>
-      <c r="K4" s="146"/>
-      <c r="L4" s="147"/>
-      <c r="M4" s="148"/>
-      <c r="N4" s="149" t="s">
+      <c r="H4" s="143"/>
+      <c r="I4" s="143"/>
+      <c r="J4" s="143"/>
+      <c r="K4" s="143"/>
+      <c r="L4" s="144"/>
+      <c r="M4" s="145"/>
+      <c r="N4" s="146" t="s">
         <v>27</v>
       </c>
-      <c r="O4" s="147"/>
-      <c r="P4" s="147"/>
-      <c r="Q4" s="147"/>
-      <c r="R4" s="147"/>
-      <c r="S4" s="147"/>
-      <c r="T4" s="150"/>
-      <c r="U4" s="145" t="s">
+      <c r="O4" s="144"/>
+      <c r="P4" s="144"/>
+      <c r="Q4" s="144"/>
+      <c r="R4" s="144"/>
+      <c r="S4" s="144"/>
+      <c r="T4" s="147"/>
+      <c r="U4" s="142" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="148"/>
+      <c r="V4" s="145"/>
       <c r="W4" s="94"/>
       <c r="X4" t="s">
         <v>0</v>
@@ -6215,7 +6189,7 @@
         <v>13</v>
       </c>
       <c r="H5" s="93" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="I5" s="12" t="s">
         <v>14</v>
@@ -6230,13 +6204,13 @@
         <v>30</v>
       </c>
       <c r="M5" s="90" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="N5" s="12" t="s">
         <v>16</v>
       </c>
       <c r="O5" s="93" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="P5" s="12" t="s">
         <v>17</v>
@@ -6251,13 +6225,13 @@
         <v>31</v>
       </c>
       <c r="T5" s="93" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="U5" s="89" t="s">
         <v>29</v>
       </c>
       <c r="V5" s="90" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="W5" t="s">
         <v>20</v>
@@ -6269,13 +6243,13 @@
         <v>23</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="E6" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="F6" s="125" t="s">
-        <v>137</v>
+      <c r="F6" s="122" t="s">
+        <v>132</v>
       </c>
       <c r="G6" s="19" t="e">
         <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FA,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FB:$FB,"M-TIT",'ETPT Format DDG'!$C:$C,$A$3)</f>
@@ -6397,64 +6371,64 @@
     <mergeCell ref="U4:V4"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:F4">
-    <cfRule type="expression" dxfId="17" priority="13">
+    <cfRule type="expression" dxfId="13" priority="13">
       <formula>IF(LEFT($A$3,2)&lt;&gt;"TJ",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:V151">
-    <cfRule type="expression" dxfId="16" priority="15">
+    <cfRule type="expression" dxfId="12" priority="15">
       <formula>AND(ISBLANK($C6)=FALSE,ISBLANK($E6)=TRUE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:F1048576">
-    <cfRule type="expression" dxfId="15" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="11" priority="11" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)+_xlfn.NUMBERVALUE($L4)-_xlfn.NUMBERVALUE($L5)+_xlfn.NUMBERVALUE($L6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="14" priority="12">
+    <cfRule type="expression" dxfId="10" priority="12">
       <formula>AND($D1="7. TOTAL CONTENTIEUX DES MINEURS",OR(_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3))&lt;&gt;0,_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3))&lt;&gt;0,_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3))&lt;&gt;0))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D7:F7">
-    <cfRule type="expression" dxfId="13" priority="10" stopIfTrue="1">
+    <cfRule type="expression" dxfId="9" priority="10" stopIfTrue="1">
       <formula>OR(_xlfn.NUMBERVALUE($L6)&lt;&gt;_xlfn.NUMBERVALUE($L7),_xlfn.NUMBERVALUE($S6)&lt;&gt;_xlfn.NUMBERVALUE($S7),_xlfn.NUMBERVALUE($U6)&lt;&gt;_xlfn.NUMBERVALUE($U7))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:M1048576">
-    <cfRule type="expression" dxfId="12" priority="8" stopIfTrue="1">
+    <cfRule type="expression" dxfId="8" priority="8" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)+_xlfn.NUMBERVALUE($L4)+_xlfn.NUMBERVALUE($L5)+_xlfn.NUMBERVALUE($L6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="9">
+    <cfRule type="expression" dxfId="7" priority="9">
       <formula>AND($D1="7. TOTAL CONTENTIEUX DES MINEURS",_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3))&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G7:M7">
-    <cfRule type="expression" dxfId="10" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="6" priority="7" stopIfTrue="1">
       <formula>_xlfn.NUMBERVALUE($L7)&lt;&gt;_xlfn.NUMBERVALUE($L6)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1:T1048576">
-    <cfRule type="expression" dxfId="9" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="5" priority="5" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3)+_xlfn.NUMBERVALUE($S4)+_xlfn.NUMBERVALUE($S5)+_xlfn.NUMBERVALUE($S6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="4" priority="6" stopIfTrue="1">
       <formula>AND($D1="7. TOTAL CONTENTIEUX DES MINEURS",_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3))&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N7:T7">
-    <cfRule type="expression" dxfId="7" priority="4" stopIfTrue="1">
+    <cfRule type="expression" dxfId="3" priority="4" stopIfTrue="1">
       <formula>_xlfn.NUMBERVALUE($S7)&lt;&gt;_xlfn.NUMBERVALUE($S6)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U1:V1048576">
-    <cfRule type="expression" dxfId="6" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="2" priority="2" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3)+_xlfn.NUMBERVALUE($U4)+_xlfn.NUMBERVALUE($U5)+_xlfn.NUMBERVALUE($U6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="3">
+    <cfRule type="expression" dxfId="1" priority="3">
       <formula>AND($D1="7. TOTAL CONTENTIEUX DES MINEURS",_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3))&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U7:V7">
-    <cfRule type="expression" dxfId="4" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>_xlfn.NUMBERVALUE($U7)&lt;&gt;_xlfn.NUMBERVALUE($U6)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6590,19 +6564,19 @@
   <sheetData>
     <row r="1" spans="1:13" s="33" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="34" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B1"/>
       <c r="D1" s="34" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E1"/>
       <c r="G1" s="34" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H1"/>
       <c r="I1" s="49" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="M1" s="26" t="s">
         <v>0</v>
@@ -6732,7 +6706,7 @@
   <sheetPr codeName="Feuil14">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G83"/>
+  <dimension ref="A1:H83"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.83203125" style="35" bestFit="1" customWidth="1"/>
@@ -6745,54 +6719,60 @@
     <col min="8" max="16384" width="11" style="35"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="76" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="113" t="s">
-        <v>42</v>
-      </c>
-      <c r="B1" s="114" t="s">
-        <v>33</v>
-      </c>
-      <c r="C1" s="114" t="s">
-        <v>41</v>
-      </c>
-      <c r="D1" s="114" t="s">
-        <v>40</v>
-      </c>
-      <c r="E1" s="114" t="s">
-        <v>39</v>
-      </c>
-      <c r="F1" s="115" t="s">
-        <v>245</v>
-      </c>
-      <c r="G1" t="s">
+    <row r="1" spans="1:8" ht="76" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="150" t="s">
+        <v>258</v>
+      </c>
+      <c r="B1" s="151" t="s">
+        <v>259</v>
+      </c>
+      <c r="C1" s="151" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" ht="32" x14ac:dyDescent="0.2">
+      <c r="D1" s="151" t="s">
+        <v>261</v>
+      </c>
+      <c r="E1" s="151" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1" s="151" t="s">
+        <v>262</v>
+      </c>
+      <c r="G1" s="151" t="s">
+        <v>263</v>
+      </c>
+      <c r="H1" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="35" t="s">
+        <v>264</v>
+      </c>
+      <c r="B2" s="35" t="s">
+        <v>247</v>
+      </c>
+      <c r="C2" s="35" t="s">
+        <v>248</v>
+      </c>
+      <c r="D2" s="121" t="s">
+        <v>250</v>
+      </c>
+      <c r="E2" s="35" t="s">
+        <v>249</v>
+      </c>
+      <c r="F2" s="121" t="s">
+        <v>252</v>
+      </c>
+      <c r="G2" s="121" t="s">
+        <v>251</v>
+      </c>
+      <c r="H2" t="s">
         <v>253</v>
       </c>
-      <c r="B2" s="35" t="s">
-        <v>254</v>
-      </c>
-      <c r="C2" s="35" t="s">
-        <v>255</v>
-      </c>
-      <c r="D2" s="124" t="s">
-        <v>256</v>
-      </c>
-      <c r="E2" s="124" t="s">
-        <v>257</v>
-      </c>
-      <c r="F2" s="124" t="s">
-        <v>258</v>
-      </c>
-      <c r="G2" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="G3" t="s">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -6845,12 +6825,12 @@
   <sheetData>
     <row r="1" spans="1:62" s="4" customFormat="1" ht="80" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
       <c r="D1" s="3" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="E1" s="7"/>
       <c r="F1" s="6"/>
@@ -6918,80 +6898,80 @@
       <c r="D2" s="45"/>
       <c r="E2" s="45"/>
       <c r="F2" s="45"/>
-      <c r="G2" s="120" t="s">
-        <v>106</v>
-      </c>
-      <c r="H2" s="123" t="s">
-        <v>105</v>
-      </c>
-      <c r="I2" s="120" t="s">
-        <v>104</v>
-      </c>
-      <c r="J2" s="120" t="s">
-        <v>104</v>
-      </c>
-      <c r="K2" s="120" t="s">
-        <v>104</v>
-      </c>
-      <c r="L2" s="120" t="s">
-        <v>104</v>
-      </c>
-      <c r="M2" s="120" t="s">
-        <v>104</v>
-      </c>
-      <c r="N2" s="120" t="s">
-        <v>104</v>
-      </c>
-      <c r="O2" s="123" t="s">
-        <v>103</v>
-      </c>
-      <c r="P2" s="120" t="s">
-        <v>38</v>
-      </c>
-      <c r="Q2" s="120" t="s">
-        <v>38</v>
-      </c>
-      <c r="R2" s="120" t="s">
-        <v>38</v>
-      </c>
-      <c r="S2" s="123" t="s">
-        <v>102</v>
-      </c>
-      <c r="T2" s="120" t="s">
+      <c r="G2" s="117" t="s">
         <v>101</v>
       </c>
-      <c r="U2" s="120" t="s">
-        <v>101</v>
-      </c>
-      <c r="V2" s="120" t="s">
-        <v>101</v>
-      </c>
-      <c r="W2" s="120" t="s">
-        <v>101</v>
-      </c>
-      <c r="X2" s="120" t="s">
-        <v>101</v>
-      </c>
-      <c r="Y2" s="123" t="s">
+      <c r="H2" s="120" t="s">
         <v>100</v>
       </c>
-      <c r="Z2" s="120" t="s">
+      <c r="I2" s="117" t="s">
         <v>99</v>
       </c>
-      <c r="AA2" s="120" t="s">
+      <c r="J2" s="117" t="s">
         <v>99</v>
       </c>
-      <c r="AB2" s="120" t="s">
+      <c r="K2" s="117" t="s">
         <v>99</v>
       </c>
-      <c r="AC2" s="120" t="s">
+      <c r="L2" s="117" t="s">
         <v>99</v>
       </c>
-      <c r="AD2" s="120" t="s">
+      <c r="M2" s="117" t="s">
         <v>99</v>
       </c>
-      <c r="AE2" s="123" t="s">
+      <c r="N2" s="117" t="s">
+        <v>99</v>
+      </c>
+      <c r="O2" s="120" t="s">
         <v>98</v>
+      </c>
+      <c r="P2" s="117" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q2" s="117" t="s">
+        <v>37</v>
+      </c>
+      <c r="R2" s="117" t="s">
+        <v>37</v>
+      </c>
+      <c r="S2" s="120" t="s">
+        <v>97</v>
+      </c>
+      <c r="T2" s="117" t="s">
+        <v>96</v>
+      </c>
+      <c r="U2" s="117" t="s">
+        <v>96</v>
+      </c>
+      <c r="V2" s="117" t="s">
+        <v>96</v>
+      </c>
+      <c r="W2" s="117" t="s">
+        <v>96</v>
+      </c>
+      <c r="X2" s="117" t="s">
+        <v>96</v>
+      </c>
+      <c r="Y2" s="120" t="s">
+        <v>95</v>
+      </c>
+      <c r="Z2" s="117" t="s">
+        <v>94</v>
+      </c>
+      <c r="AA2" s="117" t="s">
+        <v>94</v>
+      </c>
+      <c r="AB2" s="117" t="s">
+        <v>94</v>
+      </c>
+      <c r="AC2" s="117" t="s">
+        <v>94</v>
+      </c>
+      <c r="AD2" s="117" t="s">
+        <v>94</v>
+      </c>
+      <c r="AE2" s="120" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="3" spans="1:62" ht="36" x14ac:dyDescent="0.2">
@@ -7001,167 +6981,167 @@
       <c r="D3" s="45"/>
       <c r="E3" s="45"/>
       <c r="F3" s="45"/>
-      <c r="G3" s="120" t="s">
-        <v>97</v>
-      </c>
-      <c r="H3" s="123"/>
-      <c r="I3" s="120" t="s">
-        <v>96</v>
-      </c>
-      <c r="J3" s="120" t="s">
-        <v>95</v>
-      </c>
-      <c r="K3" s="120" t="s">
-        <v>94</v>
-      </c>
-      <c r="L3" s="120" t="s">
-        <v>140</v>
-      </c>
-      <c r="M3" s="120" t="s">
-        <v>141</v>
-      </c>
-      <c r="N3" s="120" t="s">
-        <v>93</v>
-      </c>
-      <c r="O3" s="123"/>
-      <c r="P3" s="120" t="s">
-        <v>142</v>
-      </c>
-      <c r="Q3" s="120" t="s">
+      <c r="G3" s="117" t="s">
+        <v>92</v>
+      </c>
+      <c r="H3" s="120"/>
+      <c r="I3" s="117" t="s">
         <v>91</v>
       </c>
-      <c r="R3" s="120" t="s">
-        <v>92</v>
-      </c>
-      <c r="S3" s="123"/>
-      <c r="T3" s="120" t="s">
+      <c r="J3" s="117" t="s">
         <v>90</v>
       </c>
-      <c r="U3" s="120" t="s">
+      <c r="K3" s="117" t="s">
         <v>89</v>
       </c>
-      <c r="V3" s="120" t="s">
-        <v>143</v>
-      </c>
-      <c r="W3" s="120" t="s">
-        <v>144</v>
-      </c>
-      <c r="X3" s="120" t="s">
+      <c r="L3" s="117" t="s">
+        <v>135</v>
+      </c>
+      <c r="M3" s="117" t="s">
+        <v>136</v>
+      </c>
+      <c r="N3" s="117" t="s">
         <v>88</v>
       </c>
-      <c r="Y3" s="123"/>
-      <c r="Z3" s="120" t="s">
+      <c r="O3" s="120"/>
+      <c r="P3" s="117" t="s">
+        <v>137</v>
+      </c>
+      <c r="Q3" s="117" t="s">
+        <v>86</v>
+      </c>
+      <c r="R3" s="117" t="s">
         <v>87</v>
       </c>
-      <c r="AA3" s="120" t="s">
-        <v>246</v>
-      </c>
-      <c r="AB3" s="120" t="s">
-        <v>86</v>
-      </c>
-      <c r="AC3" s="120" t="s">
+      <c r="S3" s="120"/>
+      <c r="T3" s="117" t="s">
         <v>85</v>
       </c>
-      <c r="AD3" s="120" t="s">
+      <c r="U3" s="117" t="s">
         <v>84</v>
       </c>
-      <c r="AE3" s="123"/>
+      <c r="V3" s="117" t="s">
+        <v>138</v>
+      </c>
+      <c r="W3" s="117" t="s">
+        <v>139</v>
+      </c>
+      <c r="X3" s="117" t="s">
+        <v>83</v>
+      </c>
+      <c r="Y3" s="120"/>
+      <c r="Z3" s="117" t="s">
+        <v>82</v>
+      </c>
+      <c r="AA3" s="117" t="s">
+        <v>240</v>
+      </c>
+      <c r="AB3" s="117" t="s">
+        <v>81</v>
+      </c>
+      <c r="AC3" s="117" t="s">
+        <v>80</v>
+      </c>
+      <c r="AD3" s="117" t="s">
+        <v>79</v>
+      </c>
+      <c r="AE3" s="120"/>
     </row>
     <row r="4" spans="1:62" ht="48" x14ac:dyDescent="0.2">
       <c r="A4" s="44"/>
       <c r="B4" s="43" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="C4" s="43" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="D4" s="43" t="s">
         <v>32</v>
       </c>
-      <c r="E4" s="116" t="s">
-        <v>81</v>
-      </c>
-      <c r="F4" s="116" t="s">
-        <v>80</v>
-      </c>
-      <c r="G4" s="120" t="s">
-        <v>79</v>
-      </c>
-      <c r="H4" s="123"/>
-      <c r="I4" s="120" t="s">
-        <v>78</v>
-      </c>
-      <c r="J4" s="120" t="s">
-        <v>77</v>
-      </c>
-      <c r="K4" s="120" t="s">
+      <c r="E4" s="113" t="s">
         <v>76</v>
       </c>
-      <c r="L4" s="120" t="s">
-        <v>145</v>
-      </c>
-      <c r="M4" s="120" t="s">
-        <v>146</v>
-      </c>
-      <c r="N4" s="120" t="s">
+      <c r="F4" s="113" t="s">
         <v>75</v>
       </c>
-      <c r="O4" s="123"/>
-      <c r="P4" s="120" t="s">
-        <v>147</v>
-      </c>
-      <c r="Q4" s="120" t="s">
+      <c r="G4" s="117" t="s">
+        <v>74</v>
+      </c>
+      <c r="H4" s="120"/>
+      <c r="I4" s="117" t="s">
         <v>73</v>
       </c>
-      <c r="R4" s="120" t="s">
-        <v>74</v>
-      </c>
-      <c r="S4" s="123"/>
-      <c r="T4" s="120" t="s">
+      <c r="J4" s="117" t="s">
         <v>72</v>
       </c>
-      <c r="U4" s="120" t="s">
+      <c r="K4" s="117" t="s">
         <v>71</v>
       </c>
-      <c r="V4" s="120" t="s">
-        <v>148</v>
-      </c>
-      <c r="W4" s="120" t="s">
-        <v>149</v>
-      </c>
-      <c r="X4" s="120" t="s">
+      <c r="L4" s="117" t="s">
+        <v>140</v>
+      </c>
+      <c r="M4" s="117" t="s">
+        <v>141</v>
+      </c>
+      <c r="N4" s="117" t="s">
         <v>70</v>
       </c>
-      <c r="Y4" s="123"/>
-      <c r="Z4" s="120" t="s">
+      <c r="O4" s="120"/>
+      <c r="P4" s="117" t="s">
+        <v>142</v>
+      </c>
+      <c r="Q4" s="117" t="s">
+        <v>68</v>
+      </c>
+      <c r="R4" s="117" t="s">
         <v>69</v>
       </c>
-      <c r="AA4" s="120" t="s">
-        <v>247</v>
-      </c>
-      <c r="AB4" s="120" t="s">
-        <v>68</v>
-      </c>
-      <c r="AC4" s="120" t="s">
+      <c r="S4" s="120"/>
+      <c r="T4" s="117" t="s">
         <v>67</v>
       </c>
-      <c r="AD4" s="120" t="s">
+      <c r="U4" s="117" t="s">
         <v>66</v>
       </c>
-      <c r="AE4" s="123"/>
+      <c r="V4" s="117" t="s">
+        <v>143</v>
+      </c>
+      <c r="W4" s="117" t="s">
+        <v>144</v>
+      </c>
+      <c r="X4" s="117" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y4" s="120"/>
+      <c r="Z4" s="117" t="s">
+        <v>64</v>
+      </c>
+      <c r="AA4" s="117" t="s">
+        <v>241</v>
+      </c>
+      <c r="AB4" s="117" t="s">
+        <v>63</v>
+      </c>
+      <c r="AC4" s="117" t="s">
+        <v>62</v>
+      </c>
+      <c r="AD4" s="117" t="s">
+        <v>61</v>
+      </c>
+      <c r="AE4" s="120"/>
     </row>
     <row r="5" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A5" s="42"/>
       <c r="B5" s="41"/>
       <c r="C5" s="41"/>
       <c r="D5" s="47" t="s">
-        <v>252</v>
-      </c>
-      <c r="E5" s="117" t="s">
-        <v>65</v>
-      </c>
-      <c r="F5" s="117" t="s">
-        <v>64</v>
+        <v>246</v>
+      </c>
+      <c r="E5" s="114" t="s">
+        <v>60</v>
+      </c>
+      <c r="F5" s="114" t="s">
+        <v>59</v>
       </c>
       <c r="G5" s="103" t="e">
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Temps ventilés sur la période (contentieux sociaux civils et commerciaux)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH") +
@@ -7245,11 +7225,11 @@
         <f>IF(ISBLANK($D$5),"",$D$5)</f>
         <v>=ETPT_CA_JUR_DDG!D5</v>
       </c>
-      <c r="E6" s="117" t="s">
-        <v>63</v>
-      </c>
-      <c r="F6" s="117" t="s">
-        <v>62</v>
+      <c r="E6" s="114" t="s">
+        <v>58</v>
+      </c>
+      <c r="F6" s="114" t="s">
+        <v>57</v>
       </c>
       <c r="G6" s="103" t="e">
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Temps ventilés sur la période (service pénal)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH") +
@@ -7367,11 +7347,11 @@
         <f t="shared" ref="D7:D15" si="4">IF(ISBLANK($D$5),"",$D$5)</f>
         <v>=ETPT_CA_JUR_DDG!D5</v>
       </c>
-      <c r="E7" s="117" t="s">
-        <v>61</v>
-      </c>
-      <c r="F7" s="117" t="s">
-        <v>60</v>
+      <c r="E7" s="114" t="s">
+        <v>56</v>
+      </c>
+      <c r="F7" s="114" t="s">
+        <v>55</v>
       </c>
       <c r="G7" s="103"/>
       <c r="H7" s="79">
@@ -7425,11 +7405,11 @@
         <f t="shared" si="4"/>
         <v>=ETPT_CA_JUR_DDG!D5</v>
       </c>
-      <c r="E8" s="117" t="s">
-        <v>59</v>
-      </c>
-      <c r="F8" s="117" t="s">
-        <v>58</v>
+      <c r="E8" s="114" t="s">
+        <v>54</v>
+      </c>
+      <c r="F8" s="114" t="s">
+        <v>53</v>
       </c>
       <c r="G8" s="103" t="e">
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.8. ACCUEIL DU JUSTICIABLE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH")</f>
@@ -7498,11 +7478,11 @@
         <f t="shared" si="4"/>
         <v>=ETPT_CA_JUR_DDG!D5</v>
       </c>
-      <c r="E9" s="117" t="s">
-        <v>57</v>
-      </c>
-      <c r="F9" s="117" t="s">
-        <v>56</v>
+      <c r="E9" s="114" t="s">
+        <v>52</v>
+      </c>
+      <c r="F9" s="114" t="s">
+        <v>51</v>
       </c>
       <c r="G9" s="103" t="e">
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Soutien (Hors accueil du justiciable)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH")</f>
@@ -7571,11 +7551,11 @@
         <f t="shared" si="4"/>
         <v>=ETPT_CA_JUR_DDG!D5</v>
       </c>
-      <c r="E10" s="117" t="s">
-        <v>55</v>
-      </c>
-      <c r="F10" s="117" t="s">
-        <v>54</v>
+      <c r="E10" s="114" t="s">
+        <v>50</v>
+      </c>
+      <c r="F10" s="114" t="s">
+        <v>49</v>
       </c>
       <c r="G10" s="103" t="e">
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.3. FORMATIONS DISPENSÉES",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH")</f>
@@ -7644,11 +7624,11 @@
         <f t="shared" si="4"/>
         <v>=ETPT_CA_JUR_DDG!D5</v>
       </c>
-      <c r="E11" s="117" t="s">
-        <v>53</v>
-      </c>
-      <c r="F11" s="117" t="s">
-        <v>52</v>
+      <c r="E11" s="114" t="s">
+        <v>48</v>
+      </c>
+      <c r="F11" s="114" t="s">
+        <v>47</v>
       </c>
       <c r="G11" s="103" t="e">
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("13.7. ACCÈS AU DROIT ET À LA JUSTICE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH")</f>
@@ -7717,11 +7697,11 @@
         <f t="shared" si="4"/>
         <v>=ETPT_CA_JUR_DDG!D5</v>
       </c>
-      <c r="E12" s="117" t="s">
-        <v>51</v>
-      </c>
-      <c r="F12" s="117" t="s">
-        <v>50</v>
+      <c r="E12" s="114" t="s">
+        <v>46</v>
+      </c>
+      <c r="F12" s="114" t="s">
+        <v>45</v>
       </c>
       <c r="G12" s="103" t="e">
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH") -
@@ -7796,11 +7776,11 @@
         <f>IF(ISBLANK($D$5),"",$D$5)</f>
         <v>=ETPT_CA_JUR_DDG!D5</v>
       </c>
-      <c r="E13" s="117" t="s">
-        <v>49</v>
-      </c>
-      <c r="F13" s="117" t="s">
-        <v>48</v>
+      <c r="E13" s="114" t="s">
+        <v>44</v>
+      </c>
+      <c r="F13" s="114" t="s">
+        <v>43</v>
       </c>
       <c r="G13" s="103" t="e">
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14.9. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH")</f>
@@ -7869,11 +7849,11 @@
         <f>IF(ISBLANK($D$5),"",$D$5)</f>
         <v>=ETPT_CA_JUR_DDG!D5</v>
       </c>
-      <c r="E14" s="117" t="s">
-        <v>47</v>
-      </c>
-      <c r="F14" s="117" t="s">
-        <v>46</v>
+      <c r="E14" s="114" t="s">
+        <v>42</v>
+      </c>
+      <c r="F14" s="114" t="s">
+        <v>41</v>
       </c>
       <c r="G14" s="103" t="e">
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Temps ventilés sur la période (hors indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé ADD")</f>
@@ -7995,11 +7975,11 @@
         <f t="shared" si="4"/>
         <v>=ETPT_CA_JUR_DDG!D5</v>
       </c>
-      <c r="E15" s="117" t="s">
-        <v>224</v>
-      </c>
-      <c r="F15" s="117" t="s">
-        <v>225</v>
+      <c r="E15" s="114" t="s">
+        <v>219</v>
+      </c>
+      <c r="F15" s="114" t="s">
+        <v>220</v>
       </c>
       <c r="G15" s="103"/>
       <c r="H15" s="79">
@@ -8060,11 +8040,11 @@
     </row>
     <row r="16" spans="1:62" x14ac:dyDescent="0.2">
       <c r="D16" s="39"/>
-      <c r="E16" s="117" t="s">
-        <v>45</v>
-      </c>
-      <c r="F16" s="117" t="s">
-        <v>44</v>
+      <c r="E16" s="114" t="s">
+        <v>40</v>
+      </c>
+      <c r="F16" s="114" t="s">
+        <v>39</v>
       </c>
       <c r="G16" s="103" t="e">
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("Temps ventilés sur la période (hors indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé SUB")</f>
@@ -8183,9 +8163,9 @@
     </row>
     <row r="17" spans="1:31" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D17" s="39"/>
-      <c r="E17" s="118"/>
-      <c r="F17" s="119" t="s">
-        <v>43</v>
+      <c r="E17" s="115"/>
+      <c r="F17" s="116" t="s">
+        <v>38</v>
       </c>
       <c r="G17" s="79" t="e">
         <f>SUM(G5:G16)</f>
@@ -8290,16 +8270,16 @@
     </row>
     <row r="19" spans="1:31" customFormat="1" ht="102.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="4"/>
-      <c r="F19" s="121" t="s">
-        <v>249</v>
+      <c r="F19" s="118" t="s">
+        <v>243</v>
       </c>
       <c r="G19" s="81" t="e">
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé ADD") +
 SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé SUB")</f>
         <v>#N/A</v>
       </c>
-      <c r="M19" s="122" t="s">
-        <v>250</v>
+      <c r="M19" s="119" t="s">
+        <v>244</v>
       </c>
       <c r="N19" s="81" t="e">
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD") +
@@ -8342,12 +8322,12 @@
   <sheetData>
     <row r="1" spans="1:31" ht="87" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
       <c r="D1" s="3" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="E1" s="7"/>
       <c r="F1" s="6"/>
@@ -8384,80 +8364,80 @@
       <c r="D2" s="45"/>
       <c r="E2" s="45"/>
       <c r="F2" s="45"/>
-      <c r="G2" s="120" t="s">
-        <v>106</v>
-      </c>
-      <c r="H2" s="123" t="s">
-        <v>105</v>
-      </c>
-      <c r="I2" s="120" t="s">
-        <v>104</v>
-      </c>
-      <c r="J2" s="120" t="s">
-        <v>104</v>
-      </c>
-      <c r="K2" s="120" t="s">
-        <v>104</v>
-      </c>
-      <c r="L2" s="120" t="s">
-        <v>104</v>
-      </c>
-      <c r="M2" s="120" t="s">
-        <v>104</v>
-      </c>
-      <c r="N2" s="120" t="s">
-        <v>104</v>
-      </c>
-      <c r="O2" s="123" t="s">
-        <v>103</v>
-      </c>
-      <c r="P2" s="120" t="s">
-        <v>38</v>
-      </c>
-      <c r="Q2" s="120" t="s">
-        <v>38</v>
-      </c>
-      <c r="R2" s="120" t="s">
-        <v>38</v>
-      </c>
-      <c r="S2" s="123" t="s">
-        <v>102</v>
-      </c>
-      <c r="T2" s="120" t="s">
+      <c r="G2" s="117" t="s">
         <v>101</v>
       </c>
-      <c r="U2" s="120" t="s">
-        <v>101</v>
-      </c>
-      <c r="V2" s="120" t="s">
-        <v>101</v>
-      </c>
-      <c r="W2" s="120" t="s">
-        <v>101</v>
-      </c>
-      <c r="X2" s="120" t="s">
-        <v>101</v>
-      </c>
-      <c r="Y2" s="123" t="s">
+      <c r="H2" s="120" t="s">
         <v>100</v>
       </c>
-      <c r="Z2" s="120" t="s">
+      <c r="I2" s="117" t="s">
         <v>99</v>
       </c>
-      <c r="AA2" s="120" t="s">
+      <c r="J2" s="117" t="s">
         <v>99</v>
       </c>
-      <c r="AB2" s="120" t="s">
+      <c r="K2" s="117" t="s">
         <v>99</v>
       </c>
-      <c r="AC2" s="120" t="s">
+      <c r="L2" s="117" t="s">
         <v>99</v>
       </c>
-      <c r="AD2" s="120" t="s">
+      <c r="M2" s="117" t="s">
         <v>99</v>
       </c>
-      <c r="AE2" s="123" t="s">
+      <c r="N2" s="117" t="s">
+        <v>99</v>
+      </c>
+      <c r="O2" s="120" t="s">
         <v>98</v>
+      </c>
+      <c r="P2" s="117" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q2" s="117" t="s">
+        <v>37</v>
+      </c>
+      <c r="R2" s="117" t="s">
+        <v>37</v>
+      </c>
+      <c r="S2" s="120" t="s">
+        <v>97</v>
+      </c>
+      <c r="T2" s="117" t="s">
+        <v>96</v>
+      </c>
+      <c r="U2" s="117" t="s">
+        <v>96</v>
+      </c>
+      <c r="V2" s="117" t="s">
+        <v>96</v>
+      </c>
+      <c r="W2" s="117" t="s">
+        <v>96</v>
+      </c>
+      <c r="X2" s="117" t="s">
+        <v>96</v>
+      </c>
+      <c r="Y2" s="120" t="s">
+        <v>95</v>
+      </c>
+      <c r="Z2" s="117" t="s">
+        <v>94</v>
+      </c>
+      <c r="AA2" s="117" t="s">
+        <v>94</v>
+      </c>
+      <c r="AB2" s="117" t="s">
+        <v>94</v>
+      </c>
+      <c r="AC2" s="117" t="s">
+        <v>94</v>
+      </c>
+      <c r="AD2" s="117" t="s">
+        <v>94</v>
+      </c>
+      <c r="AE2" s="120" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="3" spans="1:31" ht="36" x14ac:dyDescent="0.2">
@@ -8467,167 +8447,167 @@
       <c r="D3" s="45"/>
       <c r="E3" s="45"/>
       <c r="F3" s="45"/>
-      <c r="G3" s="120" t="s">
-        <v>97</v>
-      </c>
-      <c r="H3" s="123"/>
-      <c r="I3" s="120" t="s">
-        <v>96</v>
-      </c>
-      <c r="J3" s="120" t="s">
-        <v>95</v>
-      </c>
-      <c r="K3" s="120" t="s">
-        <v>94</v>
-      </c>
-      <c r="L3" s="120" t="s">
-        <v>140</v>
-      </c>
-      <c r="M3" s="120" t="s">
-        <v>141</v>
-      </c>
-      <c r="N3" s="120" t="s">
-        <v>93</v>
-      </c>
-      <c r="O3" s="123"/>
-      <c r="P3" s="120" t="s">
-        <v>142</v>
-      </c>
-      <c r="Q3" s="120" t="s">
+      <c r="G3" s="117" t="s">
+        <v>92</v>
+      </c>
+      <c r="H3" s="120"/>
+      <c r="I3" s="117" t="s">
         <v>91</v>
       </c>
-      <c r="R3" s="120" t="s">
-        <v>92</v>
-      </c>
-      <c r="S3" s="123"/>
-      <c r="T3" s="120" t="s">
+      <c r="J3" s="117" t="s">
         <v>90</v>
       </c>
-      <c r="U3" s="120" t="s">
+      <c r="K3" s="117" t="s">
         <v>89</v>
       </c>
-      <c r="V3" s="120" t="s">
-        <v>143</v>
-      </c>
-      <c r="W3" s="120" t="s">
-        <v>144</v>
-      </c>
-      <c r="X3" s="120" t="s">
+      <c r="L3" s="117" t="s">
+        <v>135</v>
+      </c>
+      <c r="M3" s="117" t="s">
+        <v>136</v>
+      </c>
+      <c r="N3" s="117" t="s">
         <v>88</v>
       </c>
-      <c r="Y3" s="123"/>
-      <c r="Z3" s="120" t="s">
+      <c r="O3" s="120"/>
+      <c r="P3" s="117" t="s">
+        <v>137</v>
+      </c>
+      <c r="Q3" s="117" t="s">
+        <v>86</v>
+      </c>
+      <c r="R3" s="117" t="s">
         <v>87</v>
       </c>
-      <c r="AA3" s="120" t="s">
-        <v>246</v>
-      </c>
-      <c r="AB3" s="120" t="s">
-        <v>86</v>
-      </c>
-      <c r="AC3" s="120" t="s">
+      <c r="S3" s="120"/>
+      <c r="T3" s="117" t="s">
         <v>85</v>
       </c>
-      <c r="AD3" s="120" t="s">
+      <c r="U3" s="117" t="s">
         <v>84</v>
       </c>
-      <c r="AE3" s="123"/>
+      <c r="V3" s="117" t="s">
+        <v>138</v>
+      </c>
+      <c r="W3" s="117" t="s">
+        <v>139</v>
+      </c>
+      <c r="X3" s="117" t="s">
+        <v>83</v>
+      </c>
+      <c r="Y3" s="120"/>
+      <c r="Z3" s="117" t="s">
+        <v>82</v>
+      </c>
+      <c r="AA3" s="117" t="s">
+        <v>240</v>
+      </c>
+      <c r="AB3" s="117" t="s">
+        <v>81</v>
+      </c>
+      <c r="AC3" s="117" t="s">
+        <v>80</v>
+      </c>
+      <c r="AD3" s="117" t="s">
+        <v>79</v>
+      </c>
+      <c r="AE3" s="120"/>
     </row>
     <row r="4" spans="1:31" ht="48" x14ac:dyDescent="0.2">
       <c r="A4" s="44"/>
       <c r="B4" s="43" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="C4" s="43" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="D4" s="43" t="s">
         <v>32</v>
       </c>
-      <c r="E4" s="116" t="s">
-        <v>81</v>
-      </c>
-      <c r="F4" s="116" t="s">
-        <v>80</v>
-      </c>
-      <c r="G4" s="120" t="s">
-        <v>79</v>
-      </c>
-      <c r="H4" s="123"/>
-      <c r="I4" s="120" t="s">
-        <v>78</v>
-      </c>
-      <c r="J4" s="120" t="s">
-        <v>77</v>
-      </c>
-      <c r="K4" s="120" t="s">
+      <c r="E4" s="113" t="s">
         <v>76</v>
       </c>
-      <c r="L4" s="120" t="s">
-        <v>145</v>
-      </c>
-      <c r="M4" s="120" t="s">
-        <v>146</v>
-      </c>
-      <c r="N4" s="120" t="s">
+      <c r="F4" s="113" t="s">
         <v>75</v>
       </c>
-      <c r="O4" s="123"/>
-      <c r="P4" s="120" t="s">
-        <v>147</v>
-      </c>
-      <c r="Q4" s="120" t="s">
+      <c r="G4" s="117" t="s">
+        <v>74</v>
+      </c>
+      <c r="H4" s="120"/>
+      <c r="I4" s="117" t="s">
         <v>73</v>
       </c>
-      <c r="R4" s="120" t="s">
-        <v>74</v>
-      </c>
-      <c r="S4" s="123"/>
-      <c r="T4" s="120" t="s">
+      <c r="J4" s="117" t="s">
         <v>72</v>
       </c>
-      <c r="U4" s="120" t="s">
+      <c r="K4" s="117" t="s">
         <v>71</v>
       </c>
-      <c r="V4" s="120" t="s">
-        <v>148</v>
-      </c>
-      <c r="W4" s="120" t="s">
-        <v>149</v>
-      </c>
-      <c r="X4" s="120" t="s">
+      <c r="L4" s="117" t="s">
+        <v>140</v>
+      </c>
+      <c r="M4" s="117" t="s">
+        <v>141</v>
+      </c>
+      <c r="N4" s="117" t="s">
         <v>70</v>
       </c>
-      <c r="Y4" s="123"/>
-      <c r="Z4" s="120" t="s">
+      <c r="O4" s="120"/>
+      <c r="P4" s="117" t="s">
+        <v>142</v>
+      </c>
+      <c r="Q4" s="117" t="s">
+        <v>68</v>
+      </c>
+      <c r="R4" s="117" t="s">
         <v>69</v>
       </c>
-      <c r="AA4" s="120" t="s">
-        <v>247</v>
-      </c>
-      <c r="AB4" s="120" t="s">
-        <v>68</v>
-      </c>
-      <c r="AC4" s="120" t="s">
+      <c r="S4" s="120"/>
+      <c r="T4" s="117" t="s">
         <v>67</v>
       </c>
-      <c r="AD4" s="120" t="s">
+      <c r="U4" s="117" t="s">
         <v>66</v>
       </c>
-      <c r="AE4" s="123"/>
+      <c r="V4" s="117" t="s">
+        <v>143</v>
+      </c>
+      <c r="W4" s="117" t="s">
+        <v>144</v>
+      </c>
+      <c r="X4" s="117" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y4" s="120"/>
+      <c r="Z4" s="117" t="s">
+        <v>64</v>
+      </c>
+      <c r="AA4" s="117" t="s">
+        <v>241</v>
+      </c>
+      <c r="AB4" s="117" t="s">
+        <v>63</v>
+      </c>
+      <c r="AC4" s="117" t="s">
+        <v>62</v>
+      </c>
+      <c r="AD4" s="117" t="s">
+        <v>61</v>
+      </c>
+      <c r="AE4" s="120"/>
     </row>
     <row r="5" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A5" s="42"/>
       <c r="B5" s="41"/>
       <c r="C5" s="41"/>
       <c r="D5" s="47" t="s">
-        <v>261</v>
-      </c>
-      <c r="E5" s="117" t="s">
-        <v>65</v>
-      </c>
-      <c r="F5" s="117" t="s">
-        <v>64</v>
+        <v>255</v>
+      </c>
+      <c r="E5" s="114" t="s">
+        <v>60</v>
+      </c>
+      <c r="F5" s="114" t="s">
+        <v>59</v>
       </c>
       <c r="G5" s="103" t="str">
         <f>IF(ISBLANK($D$5),"",IF(ISERROR(ETPT_CA_JUR!G5),"",IF(ETPT_CA_JUR!G5=0,"",ETPT_CA_JUR!G5)))</f>
@@ -8738,11 +8718,11 @@
         <f>IF(ISBLANK($D$5),"",$D$5)</f>
         <v>=ETPT_CA_JUR!D5</v>
       </c>
-      <c r="E6" s="117" t="s">
-        <v>63</v>
-      </c>
-      <c r="F6" s="117" t="s">
-        <v>62</v>
+      <c r="E6" s="114" t="s">
+        <v>58</v>
+      </c>
+      <c r="F6" s="114" t="s">
+        <v>57</v>
       </c>
       <c r="G6" s="103" t="str">
         <f>IF(ISBLANK($D$5),"",IF(ISERROR(ETPT_CA_JUR!G6),"",IF(ETPT_CA_JUR!G6=0,"",ETPT_CA_JUR!G6)))</f>
@@ -8853,11 +8833,11 @@
         <f t="shared" ref="D7:D15" si="4">IF(ISBLANK($D$5),"",$D$5)</f>
         <v>=ETPT_CA_JUR!D5</v>
       </c>
-      <c r="E7" s="117" t="s">
-        <v>61</v>
-      </c>
-      <c r="F7" s="117" t="s">
-        <v>60</v>
+      <c r="E7" s="114" t="s">
+        <v>56</v>
+      </c>
+      <c r="F7" s="114" t="s">
+        <v>55</v>
       </c>
       <c r="G7" s="103" t="str">
         <f>IF(ISBLANK($D$5),"",IF(ISERROR(ETPT_CA_JUR!G7),"",IF(ETPT_CA_JUR!G7=0,"",ETPT_CA_JUR!G7)))</f>
@@ -8968,11 +8948,11 @@
         <f t="shared" si="4"/>
         <v>=ETPT_CA_JUR!D5</v>
       </c>
-      <c r="E8" s="117" t="s">
-        <v>59</v>
-      </c>
-      <c r="F8" s="117" t="s">
-        <v>58</v>
+      <c r="E8" s="114" t="s">
+        <v>54</v>
+      </c>
+      <c r="F8" s="114" t="s">
+        <v>53</v>
       </c>
       <c r="G8" s="103" t="str">
         <f>IF(ISBLANK($D$5),"",IF(ISERROR(ETPT_CA_JUR!G8),"",IF(ETPT_CA_JUR!G8=0,"",ETPT_CA_JUR!G8)))</f>
@@ -9083,11 +9063,11 @@
         <f t="shared" si="4"/>
         <v>=ETPT_CA_JUR!D5</v>
       </c>
-      <c r="E9" s="117" t="s">
-        <v>57</v>
-      </c>
-      <c r="F9" s="117" t="s">
-        <v>56</v>
+      <c r="E9" s="114" t="s">
+        <v>52</v>
+      </c>
+      <c r="F9" s="114" t="s">
+        <v>51</v>
       </c>
       <c r="G9" s="103" t="str">
         <f>IF(ISBLANK($D$5),"",IF(ISERROR(ETPT_CA_JUR!G9),"",IF(ETPT_CA_JUR!G9=0,"",ETPT_CA_JUR!G9)))</f>
@@ -9198,11 +9178,11 @@
         <f t="shared" si="4"/>
         <v>=ETPT_CA_JUR!D5</v>
       </c>
-      <c r="E10" s="117" t="s">
-        <v>55</v>
-      </c>
-      <c r="F10" s="117" t="s">
-        <v>54</v>
+      <c r="E10" s="114" t="s">
+        <v>50</v>
+      </c>
+      <c r="F10" s="114" t="s">
+        <v>49</v>
       </c>
       <c r="G10" s="103" t="str">
         <f>IF(ISBLANK($D$5),"",IF(ISERROR(ETPT_CA_JUR!G10),"",IF(ETPT_CA_JUR!G10=0,"",ETPT_CA_JUR!G10)))</f>
@@ -9313,11 +9293,11 @@
         <f t="shared" si="4"/>
         <v>=ETPT_CA_JUR!D5</v>
       </c>
-      <c r="E11" s="117" t="s">
-        <v>53</v>
-      </c>
-      <c r="F11" s="117" t="s">
-        <v>52</v>
+      <c r="E11" s="114" t="s">
+        <v>48</v>
+      </c>
+      <c r="F11" s="114" t="s">
+        <v>47</v>
       </c>
       <c r="G11" s="103" t="str">
         <f>IF(ISBLANK($D$5),"",IF(ISERROR(ETPT_CA_JUR!G11),"",IF(ETPT_CA_JUR!G11=0,"",ETPT_CA_JUR!G11)))</f>
@@ -9428,11 +9408,11 @@
         <f t="shared" si="4"/>
         <v>=ETPT_CA_JUR!D5</v>
       </c>
-      <c r="E12" s="117" t="s">
-        <v>51</v>
-      </c>
-      <c r="F12" s="117" t="s">
-        <v>50</v>
+      <c r="E12" s="114" t="s">
+        <v>46</v>
+      </c>
+      <c r="F12" s="114" t="s">
+        <v>45</v>
       </c>
       <c r="G12" s="103" t="str">
         <f>IF(ISBLANK($D$5),"",IF(ISERROR(ETPT_CA_JUR!G12),"",IF(ETPT_CA_JUR!G12=0,"",ETPT_CA_JUR!G12)))</f>
@@ -9543,11 +9523,11 @@
         <f t="shared" si="4"/>
         <v>=ETPT_CA_JUR!D5</v>
       </c>
-      <c r="E13" s="117" t="s">
-        <v>49</v>
-      </c>
-      <c r="F13" s="117" t="s">
-        <v>48</v>
+      <c r="E13" s="114" t="s">
+        <v>44</v>
+      </c>
+      <c r="F13" s="114" t="s">
+        <v>43</v>
       </c>
       <c r="G13" s="103" t="str">
         <f>IF(ISBLANK($D$5),"",IF(ISERROR(ETPT_CA_JUR!G13),"",IF(ETPT_CA_JUR!G13=0,"",ETPT_CA_JUR!G13)))</f>
@@ -9658,11 +9638,11 @@
         <f t="shared" si="4"/>
         <v>=ETPT_CA_JUR!D5</v>
       </c>
-      <c r="E14" s="117" t="s">
-        <v>47</v>
-      </c>
-      <c r="F14" s="117" t="s">
-        <v>46</v>
+      <c r="E14" s="114" t="s">
+        <v>42</v>
+      </c>
+      <c r="F14" s="114" t="s">
+        <v>41</v>
       </c>
       <c r="G14" s="103" t="str">
         <f>IF(ISBLANK($D$5),"",IF(ISERROR(ETPT_CA_JUR!G14),"",IF(ETPT_CA_JUR!G14=0,"",ETPT_CA_JUR!G14)))</f>
@@ -9770,11 +9750,11 @@
         <f t="shared" si="4"/>
         <v>=ETPT_CA_JUR!D5</v>
       </c>
-      <c r="E15" s="117" t="s">
-        <v>224</v>
-      </c>
-      <c r="F15" s="117" t="s">
-        <v>225</v>
+      <c r="E15" s="114" t="s">
+        <v>219</v>
+      </c>
+      <c r="F15" s="114" t="s">
+        <v>220</v>
       </c>
       <c r="G15" s="103" t="str">
         <f>IF(ISBLANK($D$5),"",IF(ISERROR(ETPT_CA_JUR!G15),"",IF(ETPT_CA_JUR!G15=0,"",ETPT_CA_JUR!G15)))</f>
@@ -9879,11 +9859,11 @@
     </row>
     <row r="16" spans="1:31" x14ac:dyDescent="0.2">
       <c r="D16" s="39"/>
-      <c r="E16" s="117" t="s">
-        <v>45</v>
-      </c>
-      <c r="F16" s="117" t="s">
-        <v>44</v>
+      <c r="E16" s="114" t="s">
+        <v>40</v>
+      </c>
+      <c r="F16" s="114" t="s">
+        <v>39</v>
       </c>
       <c r="G16" s="103" t="str">
         <f>IF(ISBLANK($D$5),"",IF(ISERROR(ETPT_CA_JUR!G16),"",IF(ETPT_CA_JUR!G16=0,"",ETPT_CA_JUR!G16)))</f>
@@ -9988,9 +9968,9 @@
     </row>
     <row r="17" spans="1:31" x14ac:dyDescent="0.2">
       <c r="D17" s="39"/>
-      <c r="E17" s="118"/>
-      <c r="F17" s="119" t="s">
-        <v>43</v>
+      <c r="E17" s="115"/>
+      <c r="F17" s="116" t="s">
+        <v>38</v>
       </c>
       <c r="G17" s="79">
         <f>SUM(G5:G16)</f>
@@ -10099,8 +10079,8 @@
       <c r="C19"/>
       <c r="D19"/>
       <c r="E19"/>
-      <c r="F19" s="121" t="s">
-        <v>249</v>
+      <c r="F19" s="118" t="s">
+        <v>243</v>
       </c>
       <c r="G19" s="81" t="e">
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé ADD") +
@@ -10112,8 +10092,8 @@
       <c r="J19"/>
       <c r="K19"/>
       <c r="L19"/>
-      <c r="M19" s="122" t="s">
-        <v>250</v>
+      <c r="M19" s="119" t="s">
+        <v>244</v>
       </c>
       <c r="N19" s="81" t="e">
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FA,,MATCH("14. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD") +

</xml_diff>

<commit_message>
Features/extractor without cache memory new (#339)
* New extractor

* update detail tab

* update rules

* add column

---------

Co-authored-by: MrJimmyChevallier <103670713+MrJimmyChevallier@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/front/src/assets/template4CA.xlsx
+++ b/front/src/assets/template4CA.xlsx
@@ -1,36 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10309"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10913"/>
   <workbookPr codeName="ThisWorkbook" hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5CF8384-ABF0-2340-89BC-06326EA5BD55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03C306BD-11FC-ED4D-AA95-190E88A83AFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
+    <workbookView xWindow="0" yWindow="700" windowWidth="27040" windowHeight="15720" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
   <sheets>
     <sheet name="ACCUEIL" sheetId="33" r:id="rId1"/>
     <sheet name="ETPT A-JUST" sheetId="1" r:id="rId2"/>
     <sheet name="ETPT Format DDG" sheetId="9" r:id="rId3"/>
-    <sheet name="Agrégats DDG" sheetId="10" r:id="rId4"/>
-    <sheet name="codage tribunal" sheetId="12" state="hidden" r:id="rId5"/>
-    <sheet name="Juridictions" sheetId="17" state="hidden" r:id="rId6"/>
-    <sheet name="Table_Fonctions" sheetId="19" state="hidden" r:id="rId7"/>
-    <sheet name="ETPT_CA_JUR" sheetId="30" state="hidden" r:id="rId8"/>
-    <sheet name="ETPT_CA_JUR_DDG" sheetId="25" r:id="rId9"/>
-    <sheet name="ETPT_ATTACHES_JUSTICE" sheetId="41" state="hidden" r:id="rId10"/>
-    <sheet name="ETPT_ATTACHES_JUSTICE_DDG" sheetId="42" r:id="rId11"/>
-    <sheet name="ETPT_CA_JUR Corresp" sheetId="38" state="hidden" r:id="rId12"/>
-    <sheet name="ETPT_ATTACHES_JUSTICE Corresp" sheetId="43" state="hidden" r:id="rId13"/>
+    <sheet name="Synthèse ETPT" sheetId="10" r:id="rId4"/>
+    <sheet name="ETPT Format DDG DETAIL" sheetId="44" state="hidden" r:id="rId5"/>
+    <sheet name="codage tribunal" sheetId="12" state="hidden" r:id="rId6"/>
+    <sheet name="Juridictions" sheetId="17" state="hidden" r:id="rId7"/>
+    <sheet name="Table_Fonctions" sheetId="19" state="hidden" r:id="rId8"/>
+    <sheet name="ETPT_CA_JUR" sheetId="30" state="hidden" r:id="rId9"/>
+    <sheet name="ETPT_CA_JUR_DDG" sheetId="25" r:id="rId10"/>
+    <sheet name="ETPT_ATTACHES_JUSTICE" sheetId="41" state="hidden" r:id="rId11"/>
+    <sheet name="ETPT_ATTACHES_JUSTICE_DDG" sheetId="42" r:id="rId12"/>
+    <sheet name="ETPT_CA_JUR Corresp" sheetId="38" state="hidden" r:id="rId13"/>
+    <sheet name="ETPT_ATTACHES_JUSTICE Corresp" sheetId="43" state="hidden" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ETPT A-JUST'!$A$2:$DN$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ETPT Format DDG'!$A$2:$DT$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Table_Fonctions!$A$1:$F$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Table_Fonctions!$A$1:$F$83</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -75,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="551" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="597" uniqueCount="337">
   <si>
     <t>#! END_ROW</t>
   </si>
@@ -3134,13 +3135,153 @@
       </rPr>
       <t>Temps ventilé sur la période A-JUST* = figurant dans l'onglet ETPT A-JUST</t>
     </r>
+  </si>
+  <si>
+    <t>Synthèse ETPT</t>
+  </si>
+  <si>
+    <t>Réf.</t>
+  </si>
+  <si>
+    <t>Nom/Prénom/Matricule</t>
+  </si>
+  <si>
+    <t>Date d'arrivée</t>
+  </si>
+  <si>
+    <t>Date de départ</t>
+  </si>
+  <si>
+    <t>Date de début du segment</t>
+  </si>
+  <si>
+    <t>Date de fin du segment</t>
+  </si>
+  <si>
+    <t>Nombre jour ouvré sur période total extaction</t>
+  </si>
+  <si>
+    <t>Nombre jour ouvré segment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ratio Jour : 
+Nb jour ouvré segment /
+Nb jour ouvré total </t>
+  </si>
+  <si>
+    <t>Temps de travail en ETPT saisie</t>
+  </si>
+  <si>
+    <t>Valeur de l'ETPT sur période total d'extraction (ETPT saisi x Ratio Jour)</t>
+  </si>
+  <si>
+    <t>Indisponibilité saisie</t>
+  </si>
+  <si>
+    <t>Valeur de l'indisponibilité sur la période total d'extraction (Indisponibilité saisie en%/100 x Ratio Jour)</t>
+  </si>
+  <si>
+    <t>Nb jour ouvré CET sur toute la période d'extraction</t>
+  </si>
+  <si>
+    <t>Valeur de l'absentéisme</t>
+  </si>
+  <si>
+    <t>Valeur de l'action 99</t>
+  </si>
+  <si>
+    <t>ETPT effectif sur la période total (ETPT- action 99 + absentéisme) x Ratio Jour</t>
+  </si>
+  <si>
+    <t>#! FOR_EACH log ongletLogs</t>
+  </si>
+  <si>
+    <t>## log.id</t>
+  </si>
+  <si>
+    <t>## log.name</t>
+  </si>
+  <si>
+    <t>## log.category</t>
+  </si>
+  <si>
+    <t>## log.humanStart</t>
+  </si>
+  <si>
+    <t>## log.humanEnd</t>
+  </si>
+  <si>
+    <t>## log.main</t>
+  </si>
+  <si>
+    <t>## log.periodStart</t>
+  </si>
+  <si>
+    <t>## log.periodEnd</t>
+  </si>
+  <si>
+    <t>## log.nbOfWorkingDaysQuery</t>
+  </si>
+  <si>
+    <t>## log.workingDays</t>
+  </si>
+  <si>
+    <t>## log.dayRate</t>
+  </si>
+  <si>
+    <t>## log.filledEtp</t>
+  </si>
+  <si>
+    <t>## log.queryEtpValue</t>
+  </si>
+  <si>
+    <t>## log.totalIndispo</t>
+  </si>
+  <si>
+    <t>## log.queryIndispoValue</t>
+  </si>
+  <si>
+    <t>## log.cetDays</t>
+  </si>
+  <si>
+    <t>## log.abs</t>
+  </si>
+  <si>
+    <t>## log.action99</t>
+  </si>
+  <si>
+    <t>## log.effectifEtp</t>
+  </si>
+  <si>
+    <t>## log.logAccVentilation</t>
+  </si>
+  <si>
+    <t>## log.ctx</t>
+  </si>
+  <si>
+    <t>#! END_LOOP log</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     Détails de la ventilation (arrondi au millième) :</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                Synthèse ETPT</t>
+  </si>
+  <si>
+    <t>ETPT global sur la période (incluant absentéisme et action 99)</t>
+  </si>
+  <si>
+    <t>## log.etptGlobal</t>
+  </si>
+  <si>
+    <t>ETPT ventilé</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="166" formatCode="_-* #,##0.000_-;\-* #,##0.000_-;_-* &quot;-&quot;??_-;_-@_-"/>
@@ -3148,6 +3289,7 @@
     <numFmt numFmtId="168" formatCode="0.###;0.###;\-"/>
     <numFmt numFmtId="169" formatCode="#,##0.00_ ;[Red]\-#,##0.00\ "/>
     <numFmt numFmtId="170" formatCode="0.0%"/>
+    <numFmt numFmtId="171" formatCode="0.###"/>
   </numFmts>
   <fonts count="57" x14ac:knownFonts="1">
     <font>
@@ -3546,7 +3688,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="20">
+  <fills count="23">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3658,6 +3800,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF7F02D"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCCB1EE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -4018,7 +4178,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="197">
+  <cellXfs count="208">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -4503,6 +4663,39 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -4603,7 +4796,87 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{6FC886D6-2077-B34D-B1DF-739B068A66D1}"/>
     <cellStyle name="Normal 3" xfId="4" xr:uid="{6BD57324-3FD5-D341-A299-730D14794802}"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="23">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCB1EE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-9.9948118533890809E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -5598,11 +5871,11 @@
       <c r="B1" s="48" t="s">
         <v>84</v>
       </c>
-      <c r="C1" s="169" t="s">
+      <c r="C1" s="180" t="s">
         <v>85</v>
       </c>
-      <c r="D1" s="169"/>
-      <c r="E1" s="169"/>
+      <c r="D1" s="180"/>
+      <c r="E1" s="180"/>
       <c r="F1" s="49"/>
       <c r="H1" s="26" t="s">
         <v>0</v>
@@ -5611,11 +5884,11 @@
     <row r="2" spans="1:8" s="53" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="50"/>
       <c r="B2" s="51"/>
-      <c r="C2" s="170" t="s">
+      <c r="C2" s="181" t="s">
         <v>106</v>
       </c>
-      <c r="D2" s="170"/>
-      <c r="E2" s="170"/>
+      <c r="D2" s="181"/>
+      <c r="E2" s="181"/>
       <c r="F2" s="52"/>
       <c r="H2" s="26" t="s">
         <v>0</v>
@@ -5639,10 +5912,10 @@
       <c r="D4" s="58" t="s">
         <v>88</v>
       </c>
-      <c r="E4" s="174" t="s">
+      <c r="E4" s="185" t="s">
         <v>89</v>
       </c>
-      <c r="F4" s="175"/>
+      <c r="F4" s="186"/>
       <c r="G4" s="65"/>
       <c r="H4" s="26" t="s">
         <v>0</v>
@@ -5659,10 +5932,10 @@
       <c r="D5" s="62" t="s">
         <v>92</v>
       </c>
-      <c r="E5" s="176" t="s">
+      <c r="E5" s="187" t="s">
         <v>100</v>
       </c>
-      <c r="F5" s="177"/>
+      <c r="F5" s="188"/>
       <c r="G5" s="64"/>
       <c r="H5" s="26" t="s">
         <v>0</v>
@@ -5679,10 +5952,10 @@
       <c r="D6" s="63" t="s">
         <v>95</v>
       </c>
-      <c r="E6" s="178" t="s">
+      <c r="E6" s="189" t="s">
         <v>101</v>
       </c>
-      <c r="F6" s="179"/>
+      <c r="F6" s="190"/>
       <c r="G6" s="64"/>
       <c r="H6" s="26" t="s">
         <v>0</v>
@@ -5691,7 +5964,7 @@
     <row r="7" spans="1:8" s="26" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="54"/>
       <c r="B7" s="164" t="s">
-        <v>96</v>
+        <v>291</v>
       </c>
       <c r="C7" s="63" t="s">
         <v>283</v>
@@ -5699,10 +5972,10 @@
       <c r="D7" s="63" t="s">
         <v>97</v>
       </c>
-      <c r="E7" s="178" t="s">
+      <c r="E7" s="189" t="s">
         <v>100</v>
       </c>
-      <c r="F7" s="179"/>
+      <c r="F7" s="190"/>
       <c r="G7" s="64"/>
       <c r="H7" s="26" t="s">
         <v>0</v>
@@ -5713,16 +5986,16 @@
       <c r="B8" s="70" t="s">
         <v>255</v>
       </c>
-      <c r="C8" s="167" t="s">
+      <c r="C8" s="178" t="s">
         <v>254</v>
       </c>
-      <c r="D8" s="167" t="s">
+      <c r="D8" s="178" t="s">
         <v>98</v>
       </c>
-      <c r="E8" s="180" t="s">
+      <c r="E8" s="191" t="s">
         <v>102</v>
       </c>
-      <c r="F8" s="181"/>
+      <c r="F8" s="192"/>
       <c r="G8" s="64"/>
       <c r="H8" s="26" t="s">
         <v>0</v>
@@ -5733,10 +6006,10 @@
       <c r="B9" s="165" t="s">
         <v>253</v>
       </c>
-      <c r="C9" s="168"/>
-      <c r="D9" s="168"/>
-      <c r="E9" s="168"/>
-      <c r="F9" s="168"/>
+      <c r="C9" s="179"/>
+      <c r="D9" s="179"/>
+      <c r="E9" s="179"/>
+      <c r="F9" s="179"/>
       <c r="G9" s="64"/>
       <c r="H9" s="26" t="s">
         <v>0</v>
@@ -5756,11 +6029,11 @@
     <row r="11" spans="1:8" s="26" customFormat="1" ht="72" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="54"/>
       <c r="B11" s="66"/>
-      <c r="C11" s="173" t="s">
+      <c r="C11" s="184" t="s">
         <v>99</v>
       </c>
-      <c r="D11" s="173"/>
-      <c r="E11" s="173"/>
+      <c r="D11" s="184"/>
+      <c r="E11" s="184"/>
       <c r="F11" s="67"/>
       <c r="H11" s="26" t="s">
         <v>0</v>
@@ -5774,14 +6047,14 @@
       </c>
     </row>
     <row r="13" spans="1:8" s="26" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="171" t="s">
+      <c r="A13" s="182" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="171"/>
-      <c r="C13" s="171"/>
-      <c r="D13" s="171"/>
-      <c r="E13" s="171"/>
-      <c r="F13" s="172"/>
+      <c r="B13" s="182"/>
+      <c r="C13" s="182"/>
+      <c r="D13" s="182"/>
+      <c r="E13" s="182"/>
+      <c r="F13" s="183"/>
       <c r="H13" s="26" t="s">
         <v>0</v>
       </c>
@@ -5812,6 +6085,1491 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{701921C7-025B-4F4F-A5C7-6D94075AC520}">
+  <sheetPr codeName="Feuil8">
+    <tabColor rgb="FFC00000"/>
+  </sheetPr>
+  <dimension ref="A1:AA17"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="6" style="37" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="17.1640625" style="37" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="6.33203125" style="37" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="14.6640625" style="37" customWidth="1"/>
+    <col min="5" max="5" width="6.5" style="37" customWidth="1"/>
+    <col min="6" max="6" width="50" style="37" customWidth="1"/>
+    <col min="7" max="27" width="14" style="37" customWidth="1"/>
+    <col min="28" max="34" width="9.33203125" style="37" customWidth="1"/>
+    <col min="35" max="35" width="8.5" style="37" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="7.33203125" style="37" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="14" style="37" customWidth="1"/>
+    <col min="38" max="58" width="9.33203125" style="37" customWidth="1"/>
+    <col min="59" max="59" width="4" style="37" customWidth="1"/>
+    <col min="60" max="16384" width="11" style="37"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:27" ht="87" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="E1" s="7"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
+      <c r="M1" s="7"/>
+      <c r="N1" s="7"/>
+      <c r="O1" s="7"/>
+      <c r="P1" s="7"/>
+      <c r="Q1" s="7"/>
+      <c r="R1" s="7"/>
+      <c r="S1" s="7"/>
+      <c r="T1" s="7"/>
+      <c r="U1" s="7"/>
+      <c r="V1" s="7"/>
+      <c r="W1" s="7"/>
+      <c r="X1" s="7"/>
+      <c r="Y1" s="7"/>
+      <c r="Z1" s="7"/>
+      <c r="AA1" s="7"/>
+    </row>
+    <row r="2" spans="1:27" ht="36" x14ac:dyDescent="0.2">
+      <c r="A2" s="44"/>
+      <c r="B2" s="43" t="s">
+        <v>75</v>
+      </c>
+      <c r="C2" s="43" t="s">
+        <v>74</v>
+      </c>
+      <c r="D2" s="43" t="s">
+        <v>32</v>
+      </c>
+      <c r="E2" s="95" t="s">
+        <v>73</v>
+      </c>
+      <c r="F2" s="95" t="s">
+        <v>72</v>
+      </c>
+      <c r="G2" s="99" t="s">
+        <v>71</v>
+      </c>
+      <c r="H2" s="100" t="s">
+        <v>81</v>
+      </c>
+      <c r="I2" s="99" t="s">
+        <v>70</v>
+      </c>
+      <c r="J2" s="99" t="s">
+        <v>273</v>
+      </c>
+      <c r="K2" s="99" t="s">
+        <v>68</v>
+      </c>
+      <c r="L2" s="99" t="s">
+        <v>274</v>
+      </c>
+      <c r="M2" s="99" t="s">
+        <v>110</v>
+      </c>
+      <c r="N2" s="99" t="s">
+        <v>67</v>
+      </c>
+      <c r="O2" s="100" t="s">
+        <v>80</v>
+      </c>
+      <c r="P2" s="99" t="s">
+        <v>275</v>
+      </c>
+      <c r="Q2" s="99" t="s">
+        <v>65</v>
+      </c>
+      <c r="R2" s="99" t="s">
+        <v>276</v>
+      </c>
+      <c r="S2" s="99" t="s">
+        <v>112</v>
+      </c>
+      <c r="T2" s="99" t="s">
+        <v>64</v>
+      </c>
+      <c r="U2" s="100" t="s">
+        <v>79</v>
+      </c>
+      <c r="V2" s="99" t="s">
+        <v>63</v>
+      </c>
+      <c r="W2" s="99" t="s">
+        <v>284</v>
+      </c>
+      <c r="X2" s="99" t="s">
+        <v>285</v>
+      </c>
+      <c r="Y2" s="99" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z2" s="99" t="s">
+        <v>60</v>
+      </c>
+      <c r="AA2" s="100" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A3" s="42"/>
+      <c r="B3" s="41"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="150" t="s">
+        <v>266</v>
+      </c>
+      <c r="E3" s="96" t="s">
+        <v>59</v>
+      </c>
+      <c r="F3" s="96" t="s">
+        <v>58</v>
+      </c>
+      <c r="G3" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!G3),"",IF(ETPT_CA_JUR!G3=0,"",ETPT_CA_JUR!G3)))</f>
+        <v/>
+      </c>
+      <c r="H3" s="137">
+        <f>ETPT_CA_JUR!H3</f>
+        <v>0</v>
+      </c>
+      <c r="I3" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!I3),"",IF(ETPT_CA_JUR!I3=0,"",ETPT_CA_JUR!I3)))</f>
+        <v/>
+      </c>
+      <c r="J3" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!J3),"",IF(ETPT_CA_JUR!J3=0,"",ETPT_CA_JUR!J3)))</f>
+        <v/>
+      </c>
+      <c r="K3" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!K3),"",IF(ETPT_CA_JUR!K3=0,"",ETPT_CA_JUR!K3)))</f>
+        <v/>
+      </c>
+      <c r="L3" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!L3),"",IF(ETPT_CA_JUR!L3=0,"",ETPT_CA_JUR!L3)))</f>
+        <v/>
+      </c>
+      <c r="M3" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!M3),"",IF(ETPT_CA_JUR!M3=0,"",ETPT_CA_JUR!M3)))</f>
+        <v/>
+      </c>
+      <c r="N3" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!N3),"",IF(ETPT_CA_JUR!N3=0,"",ETPT_CA_JUR!N3)))</f>
+        <v/>
+      </c>
+      <c r="O3" s="137">
+        <f>ETPT_CA_JUR!O3</f>
+        <v>0</v>
+      </c>
+      <c r="P3" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!P3),"",IF(ETPT_CA_JUR!P3=0,"",ETPT_CA_JUR!P3)))</f>
+        <v/>
+      </c>
+      <c r="Q3" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Q3),"",IF(ETPT_CA_JUR!Q3=0,"",ETPT_CA_JUR!Q3)))</f>
+        <v/>
+      </c>
+      <c r="R3" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!R3),"",IF(ETPT_CA_JUR!R3=0,"",ETPT_CA_JUR!R3)))</f>
+        <v/>
+      </c>
+      <c r="S3" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!S3),"",IF(ETPT_CA_JUR!S3=0,"",ETPT_CA_JUR!S3)))</f>
+        <v/>
+      </c>
+      <c r="T3" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!T3),"",IF(ETPT_CA_JUR!T3=0,"",ETPT_CA_JUR!T3)))</f>
+        <v/>
+      </c>
+      <c r="U3" s="137">
+        <f>ETPT_CA_JUR!U3</f>
+        <v>0</v>
+      </c>
+      <c r="V3" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!V3),"",IF(ETPT_CA_JUR!V3=0,"",ETPT_CA_JUR!V3)))</f>
+        <v/>
+      </c>
+      <c r="W3" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!W3),"",IF(ETPT_CA_JUR!W3=0,"",ETPT_CA_JUR!W3)))</f>
+        <v/>
+      </c>
+      <c r="X3" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!X3),"",IF(ETPT_CA_JUR!X3=0,"",ETPT_CA_JUR!X3)))</f>
+        <v/>
+      </c>
+      <c r="Y3" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Y3),"",IF(ETPT_CA_JUR!Y3=0,"",ETPT_CA_JUR!Y3)))</f>
+        <v/>
+      </c>
+      <c r="Z3" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Z3),"",IF(ETPT_CA_JUR!Z3=0,"",ETPT_CA_JUR!Z3)))</f>
+        <v/>
+      </c>
+      <c r="AA3" s="137">
+        <f>ETPT_CA_JUR!AA3</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A4" s="42"/>
+      <c r="B4" s="41"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="38" t="str">
+        <f>IF(ISBLANK($D$3),"",$D$3)</f>
+        <v>A</v>
+      </c>
+      <c r="E4" s="96" t="s">
+        <v>57</v>
+      </c>
+      <c r="F4" s="96" t="s">
+        <v>56</v>
+      </c>
+      <c r="G4" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!G4),"",IF(ETPT_CA_JUR!G4=0,"",ETPT_CA_JUR!G4)))</f>
+        <v/>
+      </c>
+      <c r="H4" s="137">
+        <f>ETPT_CA_JUR!H4</f>
+        <v>0</v>
+      </c>
+      <c r="I4" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!I4),"",IF(ETPT_CA_JUR!I4=0,"",ETPT_CA_JUR!I4)))</f>
+        <v/>
+      </c>
+      <c r="J4" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!J4),"",IF(ETPT_CA_JUR!J4=0,"",ETPT_CA_JUR!J4)))</f>
+        <v/>
+      </c>
+      <c r="K4" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!K4),"",IF(ETPT_CA_JUR!K4=0,"",ETPT_CA_JUR!K4)))</f>
+        <v/>
+      </c>
+      <c r="L4" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!L4),"",IF(ETPT_CA_JUR!L4=0,"",ETPT_CA_JUR!L4)))</f>
+        <v/>
+      </c>
+      <c r="M4" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!M4),"",IF(ETPT_CA_JUR!M4=0,"",ETPT_CA_JUR!M4)))</f>
+        <v/>
+      </c>
+      <c r="N4" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!N4),"",IF(ETPT_CA_JUR!N4=0,"",ETPT_CA_JUR!N4)))</f>
+        <v/>
+      </c>
+      <c r="O4" s="137">
+        <f>ETPT_CA_JUR!O4</f>
+        <v>0</v>
+      </c>
+      <c r="P4" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!P4),"",IF(ETPT_CA_JUR!P4=0,"",ETPT_CA_JUR!P4)))</f>
+        <v/>
+      </c>
+      <c r="Q4" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Q4),"",IF(ETPT_CA_JUR!Q4=0,"",ETPT_CA_JUR!Q4)))</f>
+        <v/>
+      </c>
+      <c r="R4" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!R4),"",IF(ETPT_CA_JUR!R4=0,"",ETPT_CA_JUR!R4)))</f>
+        <v/>
+      </c>
+      <c r="S4" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!S4),"",IF(ETPT_CA_JUR!S4=0,"",ETPT_CA_JUR!S4)))</f>
+        <v/>
+      </c>
+      <c r="T4" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!T4),"",IF(ETPT_CA_JUR!T4=0,"",ETPT_CA_JUR!T4)))</f>
+        <v/>
+      </c>
+      <c r="U4" s="137">
+        <f>ETPT_CA_JUR!U4</f>
+        <v>0</v>
+      </c>
+      <c r="V4" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!V4),"",IF(ETPT_CA_JUR!V4=0,"",ETPT_CA_JUR!V4)))</f>
+        <v/>
+      </c>
+      <c r="W4" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!W4),"",IF(ETPT_CA_JUR!W4=0,"",ETPT_CA_JUR!W4)))</f>
+        <v/>
+      </c>
+      <c r="X4" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!X4),"",IF(ETPT_CA_JUR!X4=0,"",ETPT_CA_JUR!X4)))</f>
+        <v/>
+      </c>
+      <c r="Y4" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Y4),"",IF(ETPT_CA_JUR!Y4=0,"",ETPT_CA_JUR!Y4)))</f>
+        <v/>
+      </c>
+      <c r="Z4" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Z4),"",IF(ETPT_CA_JUR!Z4=0,"",ETPT_CA_JUR!Z4)))</f>
+        <v/>
+      </c>
+      <c r="AA4" s="137">
+        <f>ETPT_CA_JUR!AA4</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A5" s="42"/>
+      <c r="B5" s="41"/>
+      <c r="C5" s="41"/>
+      <c r="D5" s="38" t="str">
+        <f t="shared" ref="D5:D13" si="0">IF(ISBLANK($D$3),"",$D$3)</f>
+        <v>A</v>
+      </c>
+      <c r="E5" s="96" t="s">
+        <v>55</v>
+      </c>
+      <c r="F5" s="96" t="s">
+        <v>54</v>
+      </c>
+      <c r="G5" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!G5),"",IF(ETPT_CA_JUR!G5=0,"",ETPT_CA_JUR!G5)))</f>
+        <v/>
+      </c>
+      <c r="H5" s="137">
+        <f>ETPT_CA_JUR!H5</f>
+        <v>0</v>
+      </c>
+      <c r="I5" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!I5),"",IF(ETPT_CA_JUR!I5=0,"",ETPT_CA_JUR!I5)))</f>
+        <v/>
+      </c>
+      <c r="J5" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!J5),"",IF(ETPT_CA_JUR!J5=0,"",ETPT_CA_JUR!J5)))</f>
+        <v/>
+      </c>
+      <c r="K5" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!K5),"",IF(ETPT_CA_JUR!K5=0,"",ETPT_CA_JUR!K5)))</f>
+        <v/>
+      </c>
+      <c r="L5" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!L5),"",IF(ETPT_CA_JUR!L5=0,"",ETPT_CA_JUR!L5)))</f>
+        <v/>
+      </c>
+      <c r="M5" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!M5),"",IF(ETPT_CA_JUR!M5=0,"",ETPT_CA_JUR!M5)))</f>
+        <v/>
+      </c>
+      <c r="N5" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!N5),"",IF(ETPT_CA_JUR!N5=0,"",ETPT_CA_JUR!N5)))</f>
+        <v/>
+      </c>
+      <c r="O5" s="137">
+        <f>ETPT_CA_JUR!O5</f>
+        <v>0</v>
+      </c>
+      <c r="P5" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!P5),"",IF(ETPT_CA_JUR!P5=0,"",ETPT_CA_JUR!P5)))</f>
+        <v/>
+      </c>
+      <c r="Q5" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Q5),"",IF(ETPT_CA_JUR!Q5=0,"",ETPT_CA_JUR!Q5)))</f>
+        <v/>
+      </c>
+      <c r="R5" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!R5),"",IF(ETPT_CA_JUR!R5=0,"",ETPT_CA_JUR!R5)))</f>
+        <v/>
+      </c>
+      <c r="S5" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!S5),"",IF(ETPT_CA_JUR!S5=0,"",ETPT_CA_JUR!S5)))</f>
+        <v/>
+      </c>
+      <c r="T5" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!T5),"",IF(ETPT_CA_JUR!T5=0,"",ETPT_CA_JUR!T5)))</f>
+        <v/>
+      </c>
+      <c r="U5" s="137">
+        <f>ETPT_CA_JUR!U5</f>
+        <v>0</v>
+      </c>
+      <c r="V5" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!V5),"",IF(ETPT_CA_JUR!V5=0,"",ETPT_CA_JUR!V5)))</f>
+        <v/>
+      </c>
+      <c r="W5" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!W5),"",IF(ETPT_CA_JUR!W5=0,"",ETPT_CA_JUR!W5)))</f>
+        <v/>
+      </c>
+      <c r="X5" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!X5),"",IF(ETPT_CA_JUR!X5=0,"",ETPT_CA_JUR!X5)))</f>
+        <v/>
+      </c>
+      <c r="Y5" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Y5),"",IF(ETPT_CA_JUR!Y5=0,"",ETPT_CA_JUR!Y5)))</f>
+        <v/>
+      </c>
+      <c r="Z5" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Z5),"",IF(ETPT_CA_JUR!Z5=0,"",ETPT_CA_JUR!Z5)))</f>
+        <v/>
+      </c>
+      <c r="AA5" s="137">
+        <f>ETPT_CA_JUR!AA5</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A6" s="42"/>
+      <c r="B6" s="41"/>
+      <c r="C6" s="41"/>
+      <c r="D6" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>A</v>
+      </c>
+      <c r="E6" s="96" t="s">
+        <v>53</v>
+      </c>
+      <c r="F6" s="96" t="s">
+        <v>52</v>
+      </c>
+      <c r="G6" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!G6),"",IF(ETPT_CA_JUR!G6=0,"",ETPT_CA_JUR!G6)))</f>
+        <v/>
+      </c>
+      <c r="H6" s="137">
+        <f>ETPT_CA_JUR!H6</f>
+        <v>0</v>
+      </c>
+      <c r="I6" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!I6),"",IF(ETPT_CA_JUR!I6=0,"",ETPT_CA_JUR!I6)))</f>
+        <v/>
+      </c>
+      <c r="J6" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!J6),"",IF(ETPT_CA_JUR!J6=0,"",ETPT_CA_JUR!J6)))</f>
+        <v/>
+      </c>
+      <c r="K6" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!K6),"",IF(ETPT_CA_JUR!K6=0,"",ETPT_CA_JUR!K6)))</f>
+        <v/>
+      </c>
+      <c r="L6" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!L6),"",IF(ETPT_CA_JUR!L6=0,"",ETPT_CA_JUR!L6)))</f>
+        <v/>
+      </c>
+      <c r="M6" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!M6),"",IF(ETPT_CA_JUR!M6=0,"",ETPT_CA_JUR!M6)))</f>
+        <v/>
+      </c>
+      <c r="N6" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!N6),"",IF(ETPT_CA_JUR!N6=0,"",ETPT_CA_JUR!N6)))</f>
+        <v/>
+      </c>
+      <c r="O6" s="137">
+        <f>ETPT_CA_JUR!O6</f>
+        <v>0</v>
+      </c>
+      <c r="P6" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!P6),"",IF(ETPT_CA_JUR!P6=0,"",ETPT_CA_JUR!P6)))</f>
+        <v/>
+      </c>
+      <c r="Q6" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Q6),"",IF(ETPT_CA_JUR!Q6=0,"",ETPT_CA_JUR!Q6)))</f>
+        <v/>
+      </c>
+      <c r="R6" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!R6),"",IF(ETPT_CA_JUR!R6=0,"",ETPT_CA_JUR!R6)))</f>
+        <v/>
+      </c>
+      <c r="S6" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!S6),"",IF(ETPT_CA_JUR!S6=0,"",ETPT_CA_JUR!S6)))</f>
+        <v/>
+      </c>
+      <c r="T6" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!T6),"",IF(ETPT_CA_JUR!T6=0,"",ETPT_CA_JUR!T6)))</f>
+        <v/>
+      </c>
+      <c r="U6" s="137">
+        <f>ETPT_CA_JUR!U6</f>
+        <v>0</v>
+      </c>
+      <c r="V6" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!V6),"",IF(ETPT_CA_JUR!V6=0,"",ETPT_CA_JUR!V6)))</f>
+        <v/>
+      </c>
+      <c r="W6" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!W6),"",IF(ETPT_CA_JUR!W6=0,"",ETPT_CA_JUR!W6)))</f>
+        <v/>
+      </c>
+      <c r="X6" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!X6),"",IF(ETPT_CA_JUR!X6=0,"",ETPT_CA_JUR!X6)))</f>
+        <v/>
+      </c>
+      <c r="Y6" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Y6),"",IF(ETPT_CA_JUR!Y6=0,"",ETPT_CA_JUR!Y6)))</f>
+        <v/>
+      </c>
+      <c r="Z6" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Z6),"",IF(ETPT_CA_JUR!Z6=0,"",ETPT_CA_JUR!Z6)))</f>
+        <v/>
+      </c>
+      <c r="AA6" s="137">
+        <f>ETPT_CA_JUR!AA6</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A7" s="42"/>
+      <c r="B7" s="41"/>
+      <c r="C7" s="41"/>
+      <c r="D7" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>A</v>
+      </c>
+      <c r="E7" s="96" t="s">
+        <v>51</v>
+      </c>
+      <c r="F7" s="96" t="s">
+        <v>50</v>
+      </c>
+      <c r="G7" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!G7),"",IF(ETPT_CA_JUR!G7=0,"",ETPT_CA_JUR!G7)))</f>
+        <v/>
+      </c>
+      <c r="H7" s="137">
+        <f>ETPT_CA_JUR!H7</f>
+        <v>0</v>
+      </c>
+      <c r="I7" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!I7),"",IF(ETPT_CA_JUR!I7=0,"",ETPT_CA_JUR!I7)))</f>
+        <v/>
+      </c>
+      <c r="J7" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!J7),"",IF(ETPT_CA_JUR!J7=0,"",ETPT_CA_JUR!J7)))</f>
+        <v/>
+      </c>
+      <c r="K7" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!K7),"",IF(ETPT_CA_JUR!K7=0,"",ETPT_CA_JUR!K7)))</f>
+        <v/>
+      </c>
+      <c r="L7" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!L7),"",IF(ETPT_CA_JUR!L7=0,"",ETPT_CA_JUR!L7)))</f>
+        <v/>
+      </c>
+      <c r="M7" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!M7),"",IF(ETPT_CA_JUR!M7=0,"",ETPT_CA_JUR!M7)))</f>
+        <v/>
+      </c>
+      <c r="N7" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!N7),"",IF(ETPT_CA_JUR!N7=0,"",ETPT_CA_JUR!N7)))</f>
+        <v/>
+      </c>
+      <c r="O7" s="137">
+        <f>ETPT_CA_JUR!O7</f>
+        <v>0</v>
+      </c>
+      <c r="P7" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!P7),"",IF(ETPT_CA_JUR!P7=0,"",ETPT_CA_JUR!P7)))</f>
+        <v/>
+      </c>
+      <c r="Q7" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Q7),"",IF(ETPT_CA_JUR!Q7=0,"",ETPT_CA_JUR!Q7)))</f>
+        <v/>
+      </c>
+      <c r="R7" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!R7),"",IF(ETPT_CA_JUR!R7=0,"",ETPT_CA_JUR!R7)))</f>
+        <v/>
+      </c>
+      <c r="S7" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!S7),"",IF(ETPT_CA_JUR!S7=0,"",ETPT_CA_JUR!S7)))</f>
+        <v/>
+      </c>
+      <c r="T7" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!T7),"",IF(ETPT_CA_JUR!T7=0,"",ETPT_CA_JUR!T7)))</f>
+        <v/>
+      </c>
+      <c r="U7" s="137">
+        <f>ETPT_CA_JUR!U7</f>
+        <v>0</v>
+      </c>
+      <c r="V7" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!V7),"",IF(ETPT_CA_JUR!V7=0,"",ETPT_CA_JUR!V7)))</f>
+        <v/>
+      </c>
+      <c r="W7" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!W7),"",IF(ETPT_CA_JUR!W7=0,"",ETPT_CA_JUR!W7)))</f>
+        <v/>
+      </c>
+      <c r="X7" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!X7),"",IF(ETPT_CA_JUR!X7=0,"",ETPT_CA_JUR!X7)))</f>
+        <v/>
+      </c>
+      <c r="Y7" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Y7),"",IF(ETPT_CA_JUR!Y7=0,"",ETPT_CA_JUR!Y7)))</f>
+        <v/>
+      </c>
+      <c r="Z7" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Z7),"",IF(ETPT_CA_JUR!Z7=0,"",ETPT_CA_JUR!Z7)))</f>
+        <v/>
+      </c>
+      <c r="AA7" s="137">
+        <f>ETPT_CA_JUR!AA7</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A8" s="42"/>
+      <c r="B8" s="41"/>
+      <c r="C8" s="41"/>
+      <c r="D8" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>A</v>
+      </c>
+      <c r="E8" s="96" t="s">
+        <v>49</v>
+      </c>
+      <c r="F8" s="96" t="s">
+        <v>48</v>
+      </c>
+      <c r="G8" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!G8),"",IF(ETPT_CA_JUR!G8=0,"",ETPT_CA_JUR!G8)))</f>
+        <v/>
+      </c>
+      <c r="H8" s="137">
+        <f>ETPT_CA_JUR!H8</f>
+        <v>0</v>
+      </c>
+      <c r="I8" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!I8),"",IF(ETPT_CA_JUR!I8=0,"",ETPT_CA_JUR!I8)))</f>
+        <v/>
+      </c>
+      <c r="J8" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!J8),"",IF(ETPT_CA_JUR!J8=0,"",ETPT_CA_JUR!J8)))</f>
+        <v/>
+      </c>
+      <c r="K8" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!K8),"",IF(ETPT_CA_JUR!K8=0,"",ETPT_CA_JUR!K8)))</f>
+        <v/>
+      </c>
+      <c r="L8" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!L8),"",IF(ETPT_CA_JUR!L8=0,"",ETPT_CA_JUR!L8)))</f>
+        <v/>
+      </c>
+      <c r="M8" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!M8),"",IF(ETPT_CA_JUR!M8=0,"",ETPT_CA_JUR!M8)))</f>
+        <v/>
+      </c>
+      <c r="N8" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!N8),"",IF(ETPT_CA_JUR!N8=0,"",ETPT_CA_JUR!N8)))</f>
+        <v/>
+      </c>
+      <c r="O8" s="137">
+        <f>ETPT_CA_JUR!O8</f>
+        <v>0</v>
+      </c>
+      <c r="P8" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!P8),"",IF(ETPT_CA_JUR!P8=0,"",ETPT_CA_JUR!P8)))</f>
+        <v/>
+      </c>
+      <c r="Q8" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Q8),"",IF(ETPT_CA_JUR!Q8=0,"",ETPT_CA_JUR!Q8)))</f>
+        <v/>
+      </c>
+      <c r="R8" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!R8),"",IF(ETPT_CA_JUR!R8=0,"",ETPT_CA_JUR!R8)))</f>
+        <v/>
+      </c>
+      <c r="S8" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!S8),"",IF(ETPT_CA_JUR!S8=0,"",ETPT_CA_JUR!S8)))</f>
+        <v/>
+      </c>
+      <c r="T8" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!T8),"",IF(ETPT_CA_JUR!T8=0,"",ETPT_CA_JUR!T8)))</f>
+        <v/>
+      </c>
+      <c r="U8" s="137">
+        <f>ETPT_CA_JUR!U8</f>
+        <v>0</v>
+      </c>
+      <c r="V8" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!V8),"",IF(ETPT_CA_JUR!V8=0,"",ETPT_CA_JUR!V8)))</f>
+        <v/>
+      </c>
+      <c r="W8" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!W8),"",IF(ETPT_CA_JUR!W8=0,"",ETPT_CA_JUR!W8)))</f>
+        <v/>
+      </c>
+      <c r="X8" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!X8),"",IF(ETPT_CA_JUR!X8=0,"",ETPT_CA_JUR!X8)))</f>
+        <v/>
+      </c>
+      <c r="Y8" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Y8),"",IF(ETPT_CA_JUR!Y8=0,"",ETPT_CA_JUR!Y8)))</f>
+        <v/>
+      </c>
+      <c r="Z8" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Z8),"",IF(ETPT_CA_JUR!Z8=0,"",ETPT_CA_JUR!Z8)))</f>
+        <v/>
+      </c>
+      <c r="AA8" s="137">
+        <f>ETPT_CA_JUR!AA8</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A9" s="42"/>
+      <c r="B9" s="41"/>
+      <c r="C9" s="41"/>
+      <c r="D9" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>A</v>
+      </c>
+      <c r="E9" s="96" t="s">
+        <v>47</v>
+      </c>
+      <c r="F9" s="96" t="s">
+        <v>46</v>
+      </c>
+      <c r="G9" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!G9),"",IF(ETPT_CA_JUR!G9=0,"",ETPT_CA_JUR!G9)))</f>
+        <v/>
+      </c>
+      <c r="H9" s="137">
+        <f>ETPT_CA_JUR!H9</f>
+        <v>0</v>
+      </c>
+      <c r="I9" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!I9),"",IF(ETPT_CA_JUR!I9=0,"",ETPT_CA_JUR!I9)))</f>
+        <v/>
+      </c>
+      <c r="J9" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!J9),"",IF(ETPT_CA_JUR!J9=0,"",ETPT_CA_JUR!J9)))</f>
+        <v/>
+      </c>
+      <c r="K9" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!K9),"",IF(ETPT_CA_JUR!K9=0,"",ETPT_CA_JUR!K9)))</f>
+        <v/>
+      </c>
+      <c r="L9" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!L9),"",IF(ETPT_CA_JUR!L9=0,"",ETPT_CA_JUR!L9)))</f>
+        <v/>
+      </c>
+      <c r="M9" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!M9),"",IF(ETPT_CA_JUR!M9=0,"",ETPT_CA_JUR!M9)))</f>
+        <v/>
+      </c>
+      <c r="N9" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!N9),"",IF(ETPT_CA_JUR!N9=0,"",ETPT_CA_JUR!N9)))</f>
+        <v/>
+      </c>
+      <c r="O9" s="137">
+        <f>ETPT_CA_JUR!O9</f>
+        <v>0</v>
+      </c>
+      <c r="P9" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!P9),"",IF(ETPT_CA_JUR!P9=0,"",ETPT_CA_JUR!P9)))</f>
+        <v/>
+      </c>
+      <c r="Q9" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Q9),"",IF(ETPT_CA_JUR!Q9=0,"",ETPT_CA_JUR!Q9)))</f>
+        <v/>
+      </c>
+      <c r="R9" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!R9),"",IF(ETPT_CA_JUR!R9=0,"",ETPT_CA_JUR!R9)))</f>
+        <v/>
+      </c>
+      <c r="S9" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!S9),"",IF(ETPT_CA_JUR!S9=0,"",ETPT_CA_JUR!S9)))</f>
+        <v/>
+      </c>
+      <c r="T9" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!T9),"",IF(ETPT_CA_JUR!T9=0,"",ETPT_CA_JUR!T9)))</f>
+        <v/>
+      </c>
+      <c r="U9" s="137">
+        <f>ETPT_CA_JUR!U9</f>
+        <v>0</v>
+      </c>
+      <c r="V9" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!V9),"",IF(ETPT_CA_JUR!V9=0,"",ETPT_CA_JUR!V9)))</f>
+        <v/>
+      </c>
+      <c r="W9" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!W9),"",IF(ETPT_CA_JUR!W9=0,"",ETPT_CA_JUR!W9)))</f>
+        <v/>
+      </c>
+      <c r="X9" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!X9),"",IF(ETPT_CA_JUR!X9=0,"",ETPT_CA_JUR!X9)))</f>
+        <v/>
+      </c>
+      <c r="Y9" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Y9),"",IF(ETPT_CA_JUR!Y9=0,"",ETPT_CA_JUR!Y9)))</f>
+        <v/>
+      </c>
+      <c r="Z9" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Z9),"",IF(ETPT_CA_JUR!Z9=0,"",ETPT_CA_JUR!Z9)))</f>
+        <v/>
+      </c>
+      <c r="AA9" s="137">
+        <f>ETPT_CA_JUR!AA9</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A10" s="42"/>
+      <c r="B10" s="41"/>
+      <c r="C10" s="41"/>
+      <c r="D10" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>A</v>
+      </c>
+      <c r="E10" s="96" t="s">
+        <v>45</v>
+      </c>
+      <c r="F10" s="96" t="s">
+        <v>44</v>
+      </c>
+      <c r="G10" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!G10),"",IF(ETPT_CA_JUR!G10=0,"",ETPT_CA_JUR!G10)))</f>
+        <v/>
+      </c>
+      <c r="H10" s="137">
+        <f>ETPT_CA_JUR!H10</f>
+        <v>0</v>
+      </c>
+      <c r="I10" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!I10),"",IF(ETPT_CA_JUR!I10=0,"",ETPT_CA_JUR!I10)))</f>
+        <v/>
+      </c>
+      <c r="J10" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!J10),"",IF(ETPT_CA_JUR!J10=0,"",ETPT_CA_JUR!J10)))</f>
+        <v/>
+      </c>
+      <c r="K10" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!K10),"",IF(ETPT_CA_JUR!K10=0,"",ETPT_CA_JUR!K10)))</f>
+        <v/>
+      </c>
+      <c r="L10" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!L10),"",IF(ETPT_CA_JUR!L10=0,"",ETPT_CA_JUR!L10)))</f>
+        <v/>
+      </c>
+      <c r="M10" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!M10),"",IF(ETPT_CA_JUR!M10=0,"",ETPT_CA_JUR!M10)))</f>
+        <v/>
+      </c>
+      <c r="N10" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!N10),"",IF(ETPT_CA_JUR!N10=0,"",ETPT_CA_JUR!N10)))</f>
+        <v/>
+      </c>
+      <c r="O10" s="137">
+        <f>ETPT_CA_JUR!O10</f>
+        <v>0</v>
+      </c>
+      <c r="P10" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!P10),"",IF(ETPT_CA_JUR!P10=0,"",ETPT_CA_JUR!P10)))</f>
+        <v/>
+      </c>
+      <c r="Q10" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Q10),"",IF(ETPT_CA_JUR!Q10=0,"",ETPT_CA_JUR!Q10)))</f>
+        <v/>
+      </c>
+      <c r="R10" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!R10),"",IF(ETPT_CA_JUR!R10=0,"",ETPT_CA_JUR!R10)))</f>
+        <v/>
+      </c>
+      <c r="S10" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!S10),"",IF(ETPT_CA_JUR!S10=0,"",ETPT_CA_JUR!S10)))</f>
+        <v/>
+      </c>
+      <c r="T10" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!T10),"",IF(ETPT_CA_JUR!T10=0,"",ETPT_CA_JUR!T10)))</f>
+        <v/>
+      </c>
+      <c r="U10" s="137">
+        <f>ETPT_CA_JUR!U10</f>
+        <v>0</v>
+      </c>
+      <c r="V10" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!V10),"",IF(ETPT_CA_JUR!V10=0,"",ETPT_CA_JUR!V10)))</f>
+        <v/>
+      </c>
+      <c r="W10" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!W10),"",IF(ETPT_CA_JUR!W10=0,"",ETPT_CA_JUR!W10)))</f>
+        <v/>
+      </c>
+      <c r="X10" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!X10),"",IF(ETPT_CA_JUR!X10=0,"",ETPT_CA_JUR!X10)))</f>
+        <v/>
+      </c>
+      <c r="Y10" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Y10),"",IF(ETPT_CA_JUR!Y10=0,"",ETPT_CA_JUR!Y10)))</f>
+        <v/>
+      </c>
+      <c r="Z10" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Z10),"",IF(ETPT_CA_JUR!Z10=0,"",ETPT_CA_JUR!Z10)))</f>
+        <v/>
+      </c>
+      <c r="AA10" s="137">
+        <f>ETPT_CA_JUR!AA10</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A11" s="42"/>
+      <c r="B11" s="41"/>
+      <c r="C11" s="41"/>
+      <c r="D11" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>A</v>
+      </c>
+      <c r="E11" s="96" t="s">
+        <v>43</v>
+      </c>
+      <c r="F11" s="96" t="s">
+        <v>42</v>
+      </c>
+      <c r="G11" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!G11),"",IF(ETPT_CA_JUR!G11=0,"",ETPT_CA_JUR!G11)))</f>
+        <v/>
+      </c>
+      <c r="H11" s="137">
+        <f>ETPT_CA_JUR!H11</f>
+        <v>0</v>
+      </c>
+      <c r="I11" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!I11),"",IF(ETPT_CA_JUR!I11=0,"",ETPT_CA_JUR!I11)))</f>
+        <v/>
+      </c>
+      <c r="J11" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!J11),"",IF(ETPT_CA_JUR!J11=0,"",ETPT_CA_JUR!J11)))</f>
+        <v/>
+      </c>
+      <c r="K11" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!K11),"",IF(ETPT_CA_JUR!K11=0,"",ETPT_CA_JUR!K11)))</f>
+        <v/>
+      </c>
+      <c r="L11" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!L11),"",IF(ETPT_CA_JUR!L11=0,"",ETPT_CA_JUR!L11)))</f>
+        <v/>
+      </c>
+      <c r="M11" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!M11),"",IF(ETPT_CA_JUR!M11=0,"",ETPT_CA_JUR!M11)))</f>
+        <v/>
+      </c>
+      <c r="N11" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!N11),"",IF(ETPT_CA_JUR!N11=0,"",ETPT_CA_JUR!N11)))</f>
+        <v/>
+      </c>
+      <c r="O11" s="137">
+        <f>ETPT_CA_JUR!O11</f>
+        <v>0</v>
+      </c>
+      <c r="P11" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!P11),"",IF(ETPT_CA_JUR!P11=0,"",ETPT_CA_JUR!P11)))</f>
+        <v/>
+      </c>
+      <c r="Q11" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Q11),"",IF(ETPT_CA_JUR!Q11=0,"",ETPT_CA_JUR!Q11)))</f>
+        <v/>
+      </c>
+      <c r="R11" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!R11),"",IF(ETPT_CA_JUR!R11=0,"",ETPT_CA_JUR!R11)))</f>
+        <v/>
+      </c>
+      <c r="S11" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!S11),"",IF(ETPT_CA_JUR!S11=0,"",ETPT_CA_JUR!S11)))</f>
+        <v/>
+      </c>
+      <c r="T11" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!T11),"",IF(ETPT_CA_JUR!T11=0,"",ETPT_CA_JUR!T11)))</f>
+        <v/>
+      </c>
+      <c r="U11" s="137">
+        <f>ETPT_CA_JUR!U11</f>
+        <v>0</v>
+      </c>
+      <c r="V11" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!V11),"",IF(ETPT_CA_JUR!V11=0,"",ETPT_CA_JUR!V11)))</f>
+        <v/>
+      </c>
+      <c r="W11" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!W11),"",IF(ETPT_CA_JUR!W11=0,"",ETPT_CA_JUR!W11)))</f>
+        <v/>
+      </c>
+      <c r="X11" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!X11),"",IF(ETPT_CA_JUR!X11=0,"",ETPT_CA_JUR!X11)))</f>
+        <v/>
+      </c>
+      <c r="Y11" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Y11),"",IF(ETPT_CA_JUR!Y11=0,"",ETPT_CA_JUR!Y11)))</f>
+        <v/>
+      </c>
+      <c r="Z11" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Z11),"",IF(ETPT_CA_JUR!Z11=0,"",ETPT_CA_JUR!Z11)))</f>
+        <v/>
+      </c>
+      <c r="AA11" s="137">
+        <f>ETPT_CA_JUR!AA11</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A12" s="40"/>
+      <c r="B12" s="39"/>
+      <c r="C12" s="39"/>
+      <c r="D12" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>A</v>
+      </c>
+      <c r="E12" s="96" t="s">
+        <v>41</v>
+      </c>
+      <c r="F12" s="96" t="s">
+        <v>40</v>
+      </c>
+      <c r="G12" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!G12),"",IF(ETPT_CA_JUR!G12=0,"",ETPT_CA_JUR!G12)))</f>
+        <v/>
+      </c>
+      <c r="H12" s="137">
+        <f>ETPT_CA_JUR!H12</f>
+        <v>0</v>
+      </c>
+      <c r="I12" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!I12),"",IF(ETPT_CA_JUR!I12=0,"",ETPT_CA_JUR!I12)))</f>
+        <v/>
+      </c>
+      <c r="J12" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!J12),"",IF(ETPT_CA_JUR!J12=0,"",ETPT_CA_JUR!J12)))</f>
+        <v/>
+      </c>
+      <c r="K12" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!K12),"",IF(ETPT_CA_JUR!K12=0,"",ETPT_CA_JUR!K12)))</f>
+        <v/>
+      </c>
+      <c r="L12" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!L12),"",IF(ETPT_CA_JUR!L12=0,"",ETPT_CA_JUR!L12)))</f>
+        <v/>
+      </c>
+      <c r="M12" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!M12),"",IF(ETPT_CA_JUR!M12=0,"",ETPT_CA_JUR!M12)))</f>
+        <v/>
+      </c>
+      <c r="N12" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!N12),"",IF(ETPT_CA_JUR!N12=0,"",ETPT_CA_JUR!N12)))</f>
+        <v/>
+      </c>
+      <c r="O12" s="137">
+        <f>ETPT_CA_JUR!O12</f>
+        <v>0</v>
+      </c>
+      <c r="P12" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!P12),"",IF(ETPT_CA_JUR!P12=0,"",ETPT_CA_JUR!P12)))</f>
+        <v/>
+      </c>
+      <c r="Q12" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Q12),"",IF(ETPT_CA_JUR!Q12=0,"",ETPT_CA_JUR!Q12)))</f>
+        <v/>
+      </c>
+      <c r="R12" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!R12),"",IF(ETPT_CA_JUR!R12=0,"",ETPT_CA_JUR!R12)))</f>
+        <v/>
+      </c>
+      <c r="S12" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!S12),"",IF(ETPT_CA_JUR!S12=0,"",ETPT_CA_JUR!S12)))</f>
+        <v/>
+      </c>
+      <c r="T12" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!T12),"",IF(ETPT_CA_JUR!T12=0,"",ETPT_CA_JUR!T12)))</f>
+        <v/>
+      </c>
+      <c r="U12" s="137">
+        <f>ETPT_CA_JUR!U12</f>
+        <v>0</v>
+      </c>
+      <c r="V12" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!V12),"",IF(ETPT_CA_JUR!V12=0,"",ETPT_CA_JUR!V12)))</f>
+        <v/>
+      </c>
+      <c r="W12" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!W12),"",IF(ETPT_CA_JUR!W12=0,"",ETPT_CA_JUR!W12)))</f>
+        <v/>
+      </c>
+      <c r="X12" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!X12),"",IF(ETPT_CA_JUR!X12=0,"",ETPT_CA_JUR!X12)))</f>
+        <v/>
+      </c>
+      <c r="Y12" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Y12),"",IF(ETPT_CA_JUR!Y12=0,"",ETPT_CA_JUR!Y12)))</f>
+        <v/>
+      </c>
+      <c r="Z12" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Z12),"",IF(ETPT_CA_JUR!Z12=0,"",ETPT_CA_JUR!Z12)))</f>
+        <v/>
+      </c>
+      <c r="AA12" s="137">
+        <f>ETPT_CA_JUR!AA12</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="D13" s="38" t="str">
+        <f t="shared" si="0"/>
+        <v>A</v>
+      </c>
+      <c r="E13" s="96" t="s">
+        <v>114</v>
+      </c>
+      <c r="F13" s="96" t="s">
+        <v>115</v>
+      </c>
+      <c r="G13" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!G13),"",IF(ETPT_CA_JUR!G13=0,"",ETPT_CA_JUR!G13)))</f>
+        <v/>
+      </c>
+      <c r="H13" s="137">
+        <f>ETPT_CA_JUR!H13</f>
+        <v>0</v>
+      </c>
+      <c r="I13" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!I13),"",IF(ETPT_CA_JUR!I13=0,"",ETPT_CA_JUR!I13)))</f>
+        <v/>
+      </c>
+      <c r="J13" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!J13),"",IF(ETPT_CA_JUR!J13=0,"",ETPT_CA_JUR!J13)))</f>
+        <v/>
+      </c>
+      <c r="K13" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!K13),"",IF(ETPT_CA_JUR!K13=0,"",ETPT_CA_JUR!K13)))</f>
+        <v/>
+      </c>
+      <c r="L13" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!L13),"",IF(ETPT_CA_JUR!L13=0,"",ETPT_CA_JUR!L13)))</f>
+        <v/>
+      </c>
+      <c r="M13" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!M13),"",IF(ETPT_CA_JUR!M13=0,"",ETPT_CA_JUR!M13)))</f>
+        <v/>
+      </c>
+      <c r="N13" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!N13),"",IF(ETPT_CA_JUR!N13=0,"",ETPT_CA_JUR!N13)))</f>
+        <v/>
+      </c>
+      <c r="O13" s="137">
+        <f>ETPT_CA_JUR!O13</f>
+        <v>0</v>
+      </c>
+      <c r="P13" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!P13),"",IF(ETPT_CA_JUR!P13=0,"",ETPT_CA_JUR!P13)))</f>
+        <v/>
+      </c>
+      <c r="Q13" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Q13),"",IF(ETPT_CA_JUR!Q13=0,"",ETPT_CA_JUR!Q13)))</f>
+        <v/>
+      </c>
+      <c r="R13" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!R13),"",IF(ETPT_CA_JUR!R13=0,"",ETPT_CA_JUR!R13)))</f>
+        <v/>
+      </c>
+      <c r="S13" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!S13),"",IF(ETPT_CA_JUR!S13=0,"",ETPT_CA_JUR!S13)))</f>
+        <v/>
+      </c>
+      <c r="T13" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!T13),"",IF(ETPT_CA_JUR!T13=0,"",ETPT_CA_JUR!T13)))</f>
+        <v/>
+      </c>
+      <c r="U13" s="137">
+        <f>ETPT_CA_JUR!U13</f>
+        <v>0</v>
+      </c>
+      <c r="V13" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!V13),"",IF(ETPT_CA_JUR!V13=0,"",ETPT_CA_JUR!V13)))</f>
+        <v/>
+      </c>
+      <c r="W13" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!W13),"",IF(ETPT_CA_JUR!W13=0,"",ETPT_CA_JUR!W13)))</f>
+        <v/>
+      </c>
+      <c r="X13" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!X13),"",IF(ETPT_CA_JUR!X13=0,"",ETPT_CA_JUR!X13)))</f>
+        <v/>
+      </c>
+      <c r="Y13" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Y13),"",IF(ETPT_CA_JUR!Y13=0,"",ETPT_CA_JUR!Y13)))</f>
+        <v/>
+      </c>
+      <c r="Z13" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Z13),"",IF(ETPT_CA_JUR!Z13=0,"",ETPT_CA_JUR!Z13)))</f>
+        <v/>
+      </c>
+      <c r="AA13" s="137">
+        <f>ETPT_CA_JUR!AA13</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="D14" s="38" t="str">
+        <f>IF(ISBLANK($D$3),"",$D$3)</f>
+        <v>A</v>
+      </c>
+      <c r="E14" s="96" t="s">
+        <v>39</v>
+      </c>
+      <c r="F14" s="96" t="s">
+        <v>38</v>
+      </c>
+      <c r="G14" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!G14),"",IF(ETPT_CA_JUR!G14=0,"",ETPT_CA_JUR!G14)))</f>
+        <v/>
+      </c>
+      <c r="H14" s="137">
+        <f>ETPT_CA_JUR!H14</f>
+        <v>0</v>
+      </c>
+      <c r="I14" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!I14),"",IF(ETPT_CA_JUR!I14=0,"",ETPT_CA_JUR!I14)))</f>
+        <v/>
+      </c>
+      <c r="J14" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!J14),"",IF(ETPT_CA_JUR!J14=0,"",ETPT_CA_JUR!J14)))</f>
+        <v/>
+      </c>
+      <c r="K14" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!K14),"",IF(ETPT_CA_JUR!K14=0,"",ETPT_CA_JUR!K14)))</f>
+        <v/>
+      </c>
+      <c r="L14" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!L14),"",IF(ETPT_CA_JUR!L14=0,"",ETPT_CA_JUR!L14)))</f>
+        <v/>
+      </c>
+      <c r="M14" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!M14),"",IF(ETPT_CA_JUR!M14=0,"",ETPT_CA_JUR!M14)))</f>
+        <v/>
+      </c>
+      <c r="N14" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!N14),"",IF(ETPT_CA_JUR!N14=0,"",ETPT_CA_JUR!N14)))</f>
+        <v/>
+      </c>
+      <c r="O14" s="137">
+        <f>ETPT_CA_JUR!O14</f>
+        <v>0</v>
+      </c>
+      <c r="P14" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!P14),"",IF(ETPT_CA_JUR!P14=0,"",ETPT_CA_JUR!P14)))</f>
+        <v/>
+      </c>
+      <c r="Q14" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Q14),"",IF(ETPT_CA_JUR!Q14=0,"",ETPT_CA_JUR!Q14)))</f>
+        <v/>
+      </c>
+      <c r="R14" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!R14),"",IF(ETPT_CA_JUR!R14=0,"",ETPT_CA_JUR!R14)))</f>
+        <v/>
+      </c>
+      <c r="S14" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!S14),"",IF(ETPT_CA_JUR!S14=0,"",ETPT_CA_JUR!S14)))</f>
+        <v/>
+      </c>
+      <c r="T14" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!T14),"",IF(ETPT_CA_JUR!T14=0,"",ETPT_CA_JUR!T14)))</f>
+        <v/>
+      </c>
+      <c r="U14" s="137">
+        <f>ETPT_CA_JUR!U14</f>
+        <v>0</v>
+      </c>
+      <c r="V14" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!V14),"",IF(ETPT_CA_JUR!V14=0,"",ETPT_CA_JUR!V14)))</f>
+        <v/>
+      </c>
+      <c r="W14" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!W14),"",IF(ETPT_CA_JUR!W14=0,"",ETPT_CA_JUR!W14)))</f>
+        <v/>
+      </c>
+      <c r="X14" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!X14),"",IF(ETPT_CA_JUR!X14=0,"",ETPT_CA_JUR!X14)))</f>
+        <v/>
+      </c>
+      <c r="Y14" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Y14),"",IF(ETPT_CA_JUR!Y14=0,"",ETPT_CA_JUR!Y14)))</f>
+        <v/>
+      </c>
+      <c r="Z14" s="136" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Z14),"",IF(ETPT_CA_JUR!Z14=0,"",ETPT_CA_JUR!Z14)))</f>
+        <v/>
+      </c>
+      <c r="AA14" s="137">
+        <f>ETPT_CA_JUR!AA14</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="D15" s="38"/>
+      <c r="E15" s="97"/>
+      <c r="F15" s="98" t="s">
+        <v>37</v>
+      </c>
+      <c r="G15" s="137">
+        <f>ETPT_CA_JUR!G15</f>
+        <v>0</v>
+      </c>
+      <c r="H15" s="137">
+        <f>ETPT_CA_JUR!H15</f>
+        <v>0</v>
+      </c>
+      <c r="I15" s="137">
+        <f>ETPT_CA_JUR!I15</f>
+        <v>0</v>
+      </c>
+      <c r="J15" s="137">
+        <f>ETPT_CA_JUR!J15</f>
+        <v>0</v>
+      </c>
+      <c r="K15" s="137">
+        <f>ETPT_CA_JUR!K15</f>
+        <v>0</v>
+      </c>
+      <c r="L15" s="137">
+        <f>ETPT_CA_JUR!L15</f>
+        <v>0</v>
+      </c>
+      <c r="M15" s="137">
+        <f>ETPT_CA_JUR!M15</f>
+        <v>0</v>
+      </c>
+      <c r="N15" s="137">
+        <f>ETPT_CA_JUR!N15</f>
+        <v>0</v>
+      </c>
+      <c r="O15" s="137">
+        <f>ETPT_CA_JUR!O15</f>
+        <v>0</v>
+      </c>
+      <c r="P15" s="137">
+        <f>ETPT_CA_JUR!P15</f>
+        <v>0</v>
+      </c>
+      <c r="Q15" s="137">
+        <f>ETPT_CA_JUR!Q15</f>
+        <v>0</v>
+      </c>
+      <c r="R15" s="137">
+        <f>ETPT_CA_JUR!R15</f>
+        <v>0</v>
+      </c>
+      <c r="S15" s="137">
+        <f>ETPT_CA_JUR!S15</f>
+        <v>0</v>
+      </c>
+      <c r="T15" s="137">
+        <f>ETPT_CA_JUR!T15</f>
+        <v>0</v>
+      </c>
+      <c r="U15" s="137">
+        <f>ETPT_CA_JUR!U15</f>
+        <v>0</v>
+      </c>
+      <c r="V15" s="137">
+        <f>ETPT_CA_JUR!V15</f>
+        <v>0</v>
+      </c>
+      <c r="W15" s="137">
+        <f>ETPT_CA_JUR!W15</f>
+        <v>0</v>
+      </c>
+      <c r="X15" s="137">
+        <f>ETPT_CA_JUR!X15</f>
+        <v>0</v>
+      </c>
+      <c r="Y15" s="137">
+        <f>ETPT_CA_JUR!Y15</f>
+        <v>0</v>
+      </c>
+      <c r="Z15" s="137">
+        <f>ETPT_CA_JUR!Z15</f>
+        <v>0</v>
+      </c>
+      <c r="AA15" s="137">
+        <f>ETPT_CA_JUR!AA15</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="D16" s="134"/>
+      <c r="E16" s="134"/>
+      <c r="F16" s="134"/>
+      <c r="G16" s="138"/>
+      <c r="H16" s="138"/>
+      <c r="I16" s="138"/>
+      <c r="J16" s="138"/>
+      <c r="K16" s="138"/>
+      <c r="L16" s="138"/>
+      <c r="M16" s="138"/>
+      <c r="N16" s="138"/>
+      <c r="O16" s="138"/>
+      <c r="P16" s="138"/>
+      <c r="Q16" s="138"/>
+      <c r="R16" s="138"/>
+      <c r="S16" s="138"/>
+      <c r="T16" s="138"/>
+      <c r="U16" s="138"/>
+      <c r="V16" s="138"/>
+      <c r="W16" s="138"/>
+      <c r="X16" s="138"/>
+      <c r="Y16" s="138"/>
+      <c r="Z16" s="138"/>
+      <c r="AA16" s="138"/>
+    </row>
+    <row r="17" spans="1:27" ht="24" x14ac:dyDescent="0.2">
+      <c r="A17" s="4"/>
+      <c r="B17"/>
+      <c r="C17"/>
+      <c r="D17" s="135"/>
+      <c r="E17" s="135"/>
+      <c r="F17" s="151" t="s">
+        <v>118</v>
+      </c>
+      <c r="G17" s="140" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!G17),"",IF(ETPT_CA_JUR!G17=0,"",ETPT_CA_JUR!G17)))</f>
+        <v/>
+      </c>
+      <c r="H17" s="139"/>
+      <c r="I17" s="202" t="s">
+        <v>119</v>
+      </c>
+      <c r="J17" s="203"/>
+      <c r="K17" s="203"/>
+      <c r="L17" s="203"/>
+      <c r="M17" s="204"/>
+      <c r="N17" s="140" t="str">
+        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!N17),"",IF(ETPT_CA_JUR!N17=0,"",ETPT_CA_JUR!N17)))</f>
+        <v/>
+      </c>
+      <c r="O17" s="139"/>
+      <c r="P17" s="139"/>
+      <c r="Q17" s="139"/>
+      <c r="R17" s="139"/>
+      <c r="S17" s="139"/>
+      <c r="T17" s="139"/>
+      <c r="U17" s="139"/>
+      <c r="V17" s="139"/>
+      <c r="W17" s="139"/>
+      <c r="X17" s="139"/>
+      <c r="Y17" s="139"/>
+      <c r="Z17" s="139"/>
+      <c r="AA17" s="139"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="I17:M17"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB554CC5-4631-9C4D-9EF1-39CD273D3537}">
   <sheetPr>
     <tabColor rgb="FF0070C0"/>
@@ -6523,7 +8281,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7AA5FE4-5D9A-904C-8E7D-D70A5B5F8254}">
   <sheetPr>
     <tabColor rgb="FF0070C0"/>
@@ -7103,7 +8861,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DA9DAE4-6E6E-634B-B61F-BD7DA00BF20E}">
   <dimension ref="A1:U17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -7113,13 +8871,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="56" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="194" t="s">
+      <c r="A1" s="205" t="s">
         <v>107</v>
       </c>
-      <c r="B1" s="194"/>
-      <c r="C1" s="194"/>
-      <c r="D1" s="194"/>
-      <c r="E1" s="194"/>
+      <c r="B1" s="205"/>
+      <c r="C1" s="205"/>
+      <c r="D1" s="205"/>
+      <c r="E1" s="205"/>
       <c r="F1" s="153"/>
       <c r="G1" s="154"/>
       <c r="H1" s="154"/>
@@ -7865,7 +9623,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A2E841C-99B1-2944-9963-E2DDCA0EE564}">
   <dimension ref="A1:Q144"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -7875,12 +9633,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="44" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="195" t="s">
+      <c r="A1" s="206" t="s">
         <v>250</v>
       </c>
-      <c r="B1" s="195"/>
-      <c r="C1" s="195"/>
-      <c r="D1" s="195"/>
+      <c r="B1" s="206"/>
+      <c r="C1" s="206"/>
+      <c r="D1" s="206"/>
       <c r="E1" s="120"/>
       <c r="F1" s="119"/>
       <c r="G1" s="119"/>
@@ -7930,7 +9688,7 @@
       <c r="O2" s="105" t="s">
         <v>36</v>
       </c>
-      <c r="P2" s="196" t="s">
+      <c r="P2" s="207" t="s">
         <v>138</v>
       </c>
     </row>
@@ -7970,7 +9728,7 @@
       <c r="O3" s="105" t="s">
         <v>145</v>
       </c>
-      <c r="P3" s="196"/>
+      <c r="P3" s="207"/>
     </row>
     <row r="4" spans="1:16" ht="28" x14ac:dyDescent="0.2">
       <c r="A4" s="106" t="s">
@@ -8018,7 +9776,7 @@
       <c r="O4" s="108" t="s">
         <v>282</v>
       </c>
-      <c r="P4" s="196"/>
+      <c r="P4" s="207"/>
     </row>
     <row r="5" spans="1:16" ht="252" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="109"/>
@@ -8888,22 +10646,22 @@
       <c r="A1" s="131"/>
       <c r="B1" s="131"/>
       <c r="C1" s="131"/>
-      <c r="D1" s="182" t="s">
+      <c r="D1" s="193" t="s">
         <v>286</v>
       </c>
-      <c r="E1" s="182"/>
-      <c r="F1" s="182"/>
-      <c r="G1" s="182"/>
-      <c r="H1" s="182"/>
-      <c r="I1" s="182"/>
-      <c r="J1" s="182"/>
-      <c r="K1" s="182"/>
-      <c r="L1" s="182"/>
-      <c r="M1" s="182"/>
-      <c r="N1" s="182"/>
-      <c r="O1" s="182"/>
-      <c r="P1" s="182"/>
-      <c r="Q1" s="182"/>
+      <c r="E1" s="193"/>
+      <c r="F1" s="193"/>
+      <c r="G1" s="193"/>
+      <c r="H1" s="193"/>
+      <c r="I1" s="193"/>
+      <c r="J1" s="193"/>
+      <c r="K1" s="193"/>
+      <c r="L1" s="193"/>
+      <c r="M1" s="193"/>
+      <c r="N1" s="193"/>
+      <c r="O1" s="193"/>
+      <c r="P1" s="193"/>
+      <c r="Q1" s="193"/>
       <c r="R1" s="132" t="s">
         <v>130</v>
       </c>
@@ -8945,8 +10703,8 @@
     <mergeCell ref="D1:Q1"/>
   </mergeCells>
   <conditionalFormatting sqref="A2:EZ2 A3:FB1048576">
-    <cfRule type="expression" dxfId="11" priority="2" stopIfTrue="1">
-      <formula>AND(OR($R1&lt;&gt;"-",$S1&lt;&gt;0,$T1&lt;&gt;0,ISBLANK($P1)),ROW()&gt;2,$A1&lt;&gt;"")</formula>
+    <cfRule type="expression" dxfId="22" priority="2">
+      <formula>AND(OR($R1&lt;&gt;0,$S1&lt;&gt;0,$T1&lt;&gt;0,ISBLANK($P1)),ROW()&gt;2,$A1&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8985,7 +10743,7 @@
         <v>96</v>
       </c>
       <c r="D1" s="61" t="s">
-        <v>82</v>
+        <v>333</v>
       </c>
       <c r="E1" s="7"/>
       <c r="F1" s="7"/>
@@ -9039,28 +10797,28 @@
       <c r="D4" s="75"/>
       <c r="E4" s="75"/>
       <c r="F4" s="75"/>
-      <c r="G4" s="183" t="s">
+      <c r="G4" s="194" t="s">
         <v>26</v>
       </c>
-      <c r="H4" s="184"/>
-      <c r="I4" s="184"/>
-      <c r="J4" s="184"/>
-      <c r="K4" s="184"/>
-      <c r="L4" s="185"/>
-      <c r="M4" s="186"/>
-      <c r="N4" s="187" t="s">
+      <c r="H4" s="195"/>
+      <c r="I4" s="195"/>
+      <c r="J4" s="195"/>
+      <c r="K4" s="195"/>
+      <c r="L4" s="196"/>
+      <c r="M4" s="197"/>
+      <c r="N4" s="198" t="s">
         <v>27</v>
       </c>
-      <c r="O4" s="185"/>
-      <c r="P4" s="185"/>
-      <c r="Q4" s="185"/>
-      <c r="R4" s="185"/>
-      <c r="S4" s="185"/>
-      <c r="T4" s="188"/>
-      <c r="U4" s="183" t="s">
+      <c r="O4" s="196"/>
+      <c r="P4" s="196"/>
+      <c r="Q4" s="196"/>
+      <c r="R4" s="196"/>
+      <c r="S4" s="196"/>
+      <c r="T4" s="199"/>
+      <c r="U4" s="194" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="186"/>
+      <c r="V4" s="197"/>
       <c r="W4" s="82"/>
       <c r="X4" t="s">
         <v>0</v>
@@ -9258,57 +11016,57 @@
     <mergeCell ref="U4:V4"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:F4">
-    <cfRule type="expression" dxfId="10" priority="20">
+    <cfRule type="expression" dxfId="21" priority="20">
       <formula>IF(LEFT($A$3,2)&lt;&gt;"TJ",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:F6 C7:V151">
-    <cfRule type="expression" dxfId="9" priority="22">
+    <cfRule type="expression" dxfId="20" priority="22">
       <formula>AND(ISBLANK($C6)=FALSE,ISBLANK($E6)=TRUE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:F1048576">
-    <cfRule type="expression" dxfId="8" priority="19" stopIfTrue="1">
+    <cfRule type="expression" dxfId="19" priority="19" stopIfTrue="1">
       <formula>AND($D1="7. TOTAL CONTENTIEUX DES MINEURS",OR(ROUND(_xlfn.NUMBERVALUE($L1)-_xlfn.NUMBERVALUE($L2)-_xlfn.NUMBERVALUE($L3),3)&lt;&gt;0,ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3),3)&lt;&gt;0,ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3),3)&lt;&gt;0))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D7:F7">
-    <cfRule type="expression" dxfId="7" priority="17" stopIfTrue="1">
+    <cfRule type="expression" dxfId="18" priority="17" stopIfTrue="1">
       <formula>OR(_xlfn.NUMBERVALUE($L6)&lt;&gt;_xlfn.NUMBERVALUE($L7),_xlfn.NUMBERVALUE($S6)&lt;&gt;_xlfn.NUMBERVALUE($S7),_xlfn.NUMBERVALUE($U6)&lt;&gt;_xlfn.NUMBERVALUE($U7))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:M1048576">
-    <cfRule type="expression" dxfId="6" priority="6">
+    <cfRule type="expression" dxfId="17" priority="6">
       <formula>AND($D1="7. TOTAL CONTENTIEUX DES MINEURS",ROUND(_xlfn.NUMBERVALUE($L1)-_xlfn.NUMBERVALUE($L2)-_xlfn.NUMBERVALUE($L3),3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G7:M7">
-    <cfRule type="expression" dxfId="5" priority="14" stopIfTrue="1">
+    <cfRule type="expression" dxfId="16" priority="14" stopIfTrue="1">
       <formula>_xlfn.NUMBERVALUE($L7)&lt;&gt;_xlfn.NUMBERVALUE($L6)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G6:V6">
-    <cfRule type="expression" dxfId="4" priority="7">
+    <cfRule type="expression" dxfId="15" priority="7">
       <formula>AND(ISBLANK($C6)=FALSE,ISBLANK($E6)=TRUE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1:T1048576">
-    <cfRule type="expression" dxfId="3" priority="5">
+    <cfRule type="expression" dxfId="14" priority="5">
       <formula>AND($D1="7. TOTAL CONTENTIEUX DES MINEURS",ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3),3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N7:T7">
-    <cfRule type="expression" dxfId="2" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="13" priority="11" stopIfTrue="1">
       <formula>_xlfn.NUMBERVALUE($S7)&lt;&gt;_xlfn.NUMBERVALUE($S6)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U1:V1048576">
-    <cfRule type="expression" dxfId="1" priority="4">
+    <cfRule type="expression" dxfId="12" priority="4">
       <formula>AND($D1="7. TOTAL CONTENTIEUX DES MINEURS",ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3),3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U7:V7">
-    <cfRule type="expression" dxfId="0" priority="8">
+    <cfRule type="expression" dxfId="11" priority="8">
       <formula>_xlfn.NUMBERVALUE($U7)&lt;&gt;_xlfn.NUMBERVALUE($U6)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9318,6 +11076,235 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6ECF8FA8-E8EA-D647-9FEC-F590B68508F3}">
+  <dimension ref="A1:W3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="26.6640625" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="15.1640625" customWidth="1"/>
+    <col min="6" max="6" width="0" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="15.1640625" customWidth="1"/>
+    <col min="9" max="9" width="13" customWidth="1"/>
+    <col min="11" max="11" width="16.6640625" customWidth="1"/>
+    <col min="12" max="12" width="14" customWidth="1"/>
+    <col min="13" max="13" width="17" customWidth="1"/>
+    <col min="14" max="14" width="13.83203125" customWidth="1"/>
+    <col min="15" max="15" width="17.83203125" customWidth="1"/>
+    <col min="16" max="16" width="14.1640625" customWidth="1"/>
+    <col min="17" max="17" width="13" customWidth="1"/>
+    <col min="19" max="20" width="19" customWidth="1"/>
+    <col min="21" max="21" width="12.1640625" customWidth="1"/>
+    <col min="22" max="22" width="255.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:23" ht="112" x14ac:dyDescent="0.2">
+      <c r="A1" s="22" t="s">
+        <v>292</v>
+      </c>
+      <c r="B1" s="22" t="s">
+        <v>293</v>
+      </c>
+      <c r="C1" s="22" t="s">
+        <v>132</v>
+      </c>
+      <c r="D1" s="22" t="s">
+        <v>294</v>
+      </c>
+      <c r="E1" s="22" t="s">
+        <v>295</v>
+      </c>
+      <c r="F1" s="22"/>
+      <c r="G1" s="167" t="s">
+        <v>296</v>
+      </c>
+      <c r="H1" s="167" t="s">
+        <v>297</v>
+      </c>
+      <c r="I1" s="168" t="s">
+        <v>298</v>
+      </c>
+      <c r="J1" s="168" t="s">
+        <v>299</v>
+      </c>
+      <c r="K1" s="168" t="s">
+        <v>300</v>
+      </c>
+      <c r="L1" s="169" t="s">
+        <v>301</v>
+      </c>
+      <c r="M1" s="22" t="s">
+        <v>302</v>
+      </c>
+      <c r="N1" s="169" t="s">
+        <v>303</v>
+      </c>
+      <c r="O1" s="170" t="s">
+        <v>304</v>
+      </c>
+      <c r="P1" s="22" t="s">
+        <v>305</v>
+      </c>
+      <c r="Q1" s="170" t="s">
+        <v>306</v>
+      </c>
+      <c r="R1" s="170" t="s">
+        <v>307</v>
+      </c>
+      <c r="S1" s="167" t="s">
+        <v>308</v>
+      </c>
+      <c r="T1" s="167" t="s">
+        <v>334</v>
+      </c>
+      <c r="U1" s="22" t="s">
+        <v>336</v>
+      </c>
+      <c r="V1" s="172" t="s">
+        <v>332</v>
+      </c>
+      <c r="W1" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="2" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="171" t="s">
+        <v>310</v>
+      </c>
+      <c r="B2" s="171" t="s">
+        <v>311</v>
+      </c>
+      <c r="C2" s="171" t="s">
+        <v>312</v>
+      </c>
+      <c r="D2" s="171" t="s">
+        <v>313</v>
+      </c>
+      <c r="E2" s="171" t="s">
+        <v>314</v>
+      </c>
+      <c r="F2" s="171" t="s">
+        <v>315</v>
+      </c>
+      <c r="G2" s="171" t="s">
+        <v>316</v>
+      </c>
+      <c r="H2" s="171" t="s">
+        <v>317</v>
+      </c>
+      <c r="I2" s="176" t="s">
+        <v>318</v>
+      </c>
+      <c r="J2" s="176" t="s">
+        <v>319</v>
+      </c>
+      <c r="K2" s="174" t="s">
+        <v>320</v>
+      </c>
+      <c r="L2" s="174" t="s">
+        <v>321</v>
+      </c>
+      <c r="M2" s="175" t="s">
+        <v>322</v>
+      </c>
+      <c r="N2" s="177" t="s">
+        <v>323</v>
+      </c>
+      <c r="O2" s="174" t="s">
+        <v>324</v>
+      </c>
+      <c r="P2" s="174" t="s">
+        <v>325</v>
+      </c>
+      <c r="Q2" s="174" t="s">
+        <v>326</v>
+      </c>
+      <c r="R2" s="174" t="s">
+        <v>327</v>
+      </c>
+      <c r="S2" s="174" t="s">
+        <v>328</v>
+      </c>
+      <c r="T2" s="174" t="s">
+        <v>335</v>
+      </c>
+      <c r="U2" s="174" t="s">
+        <v>329</v>
+      </c>
+      <c r="V2" s="173" t="s">
+        <v>330</v>
+      </c>
+      <c r="W2" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="W3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="A1:B1">
+    <cfRule type="expression" dxfId="10" priority="11">
+      <formula>AND(OR($I1&lt;&gt;"-",#REF!&lt;&gt;0,#REF!&lt;&gt;0,ISBLANK($M1)),ROW()&gt;2,$A1&lt;&gt;"")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:F2">
+    <cfRule type="expression" dxfId="9" priority="10" stopIfTrue="1">
+      <formula>$F2="x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:N2">
+    <cfRule type="expression" dxfId="8" priority="5">
+      <formula>$F2="x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2:K2">
+    <cfRule type="expression" dxfId="7" priority="6">
+      <formula>1=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L2">
+    <cfRule type="expression" dxfId="6" priority="8">
+      <formula>1=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N2">
+    <cfRule type="expression" dxfId="5" priority="7">
+      <formula>1=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O2">
+    <cfRule type="expression" dxfId="4" priority="9">
+      <formula>1=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O2:V2">
+    <cfRule type="expression" dxfId="3" priority="1">
+      <formula>$F2="x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q2:R2">
+    <cfRule type="expression" dxfId="2" priority="4">
+      <formula>1=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S2:T2">
+    <cfRule type="expression" dxfId="1" priority="3">
+      <formula>1=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="V2">
+    <cfRule type="expression" dxfId="0" priority="2">
+      <formula>1=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0AF7A98-8726-2B45-9E0D-08F39416C73F}">
   <sheetPr codeName="Feuil19"/>
   <dimension ref="L1:L19"/>
@@ -9423,7 +11410,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CDB0A74-92BE-614C-B933-4270BECA0D39}">
   <sheetPr codeName="Feuil12"/>
   <dimension ref="A1:M21"/>
@@ -9581,7 +11568,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40175DB0-40DB-6046-B965-F2F52476B1A1}">
   <sheetPr codeName="Feuil14">
     <pageSetUpPr fitToPage="1"/>
@@ -9688,7 +11675,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70C2B6A9-5FC7-3A43-BF37-0B81E3F33F51}">
   <sheetPr codeName="Feuil16">
     <tabColor rgb="FF01A94F"/>
@@ -11137,13 +13124,13 @@
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT A-JUST'!2:2,0)),{"Fonctionnaire CTECH placé ADD";"Fonctionnaire CTECH placé SUB"}))</f>
         <v>#N/A</v>
       </c>
-      <c r="I17" s="189" t="s">
+      <c r="I17" s="200" t="s">
         <v>119</v>
       </c>
-      <c r="J17" s="189"/>
-      <c r="K17" s="189"/>
-      <c r="L17" s="189"/>
-      <c r="M17" s="190"/>
+      <c r="J17" s="200"/>
+      <c r="K17" s="200"/>
+      <c r="L17" s="200"/>
+      <c r="M17" s="201"/>
       <c r="N17" s="73" t="e" cm="1">
         <f t="array" ref="N17">SUM(SUMIFS(
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("14. TOTAL INDISPONIBILITÉ",'ETPT A-JUST'!2:2,0)),
@@ -11158,1489 +13145,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{701921C7-025B-4F4F-A5C7-6D94075AC520}">
-  <sheetPr codeName="Feuil8">
-    <tabColor rgb="FFC00000"/>
-  </sheetPr>
-  <dimension ref="A1:AA17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="6" style="37" hidden="1" customWidth="1"/>
-    <col min="2" max="2" width="17.1640625" style="37" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="6.33203125" style="37" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="14.6640625" style="37" customWidth="1"/>
-    <col min="5" max="5" width="6.5" style="37" customWidth="1"/>
-    <col min="6" max="6" width="50" style="37" customWidth="1"/>
-    <col min="7" max="27" width="14" style="37" customWidth="1"/>
-    <col min="28" max="34" width="9.33203125" style="37" customWidth="1"/>
-    <col min="35" max="35" width="8.5" style="37" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="7.33203125" style="37" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14" style="37" customWidth="1"/>
-    <col min="38" max="58" width="9.33203125" style="37" customWidth="1"/>
-    <col min="59" max="59" width="4" style="37" customWidth="1"/>
-    <col min="60" max="16384" width="11" style="37"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:27" ht="87" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="E1" s="7"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
-      <c r="M1" s="7"/>
-      <c r="N1" s="7"/>
-      <c r="O1" s="7"/>
-      <c r="P1" s="7"/>
-      <c r="Q1" s="7"/>
-      <c r="R1" s="7"/>
-      <c r="S1" s="7"/>
-      <c r="T1" s="7"/>
-      <c r="U1" s="7"/>
-      <c r="V1" s="7"/>
-      <c r="W1" s="7"/>
-      <c r="X1" s="7"/>
-      <c r="Y1" s="7"/>
-      <c r="Z1" s="7"/>
-      <c r="AA1" s="7"/>
-    </row>
-    <row r="2" spans="1:27" ht="36" x14ac:dyDescent="0.2">
-      <c r="A2" s="44"/>
-      <c r="B2" s="43" t="s">
-        <v>75</v>
-      </c>
-      <c r="C2" s="43" t="s">
-        <v>74</v>
-      </c>
-      <c r="D2" s="43" t="s">
-        <v>32</v>
-      </c>
-      <c r="E2" s="95" t="s">
-        <v>73</v>
-      </c>
-      <c r="F2" s="95" t="s">
-        <v>72</v>
-      </c>
-      <c r="G2" s="99" t="s">
-        <v>71</v>
-      </c>
-      <c r="H2" s="100" t="s">
-        <v>81</v>
-      </c>
-      <c r="I2" s="99" t="s">
-        <v>70</v>
-      </c>
-      <c r="J2" s="99" t="s">
-        <v>273</v>
-      </c>
-      <c r="K2" s="99" t="s">
-        <v>68</v>
-      </c>
-      <c r="L2" s="99" t="s">
-        <v>274</v>
-      </c>
-      <c r="M2" s="99" t="s">
-        <v>110</v>
-      </c>
-      <c r="N2" s="99" t="s">
-        <v>67</v>
-      </c>
-      <c r="O2" s="100" t="s">
-        <v>80</v>
-      </c>
-      <c r="P2" s="99" t="s">
-        <v>275</v>
-      </c>
-      <c r="Q2" s="99" t="s">
-        <v>65</v>
-      </c>
-      <c r="R2" s="99" t="s">
-        <v>276</v>
-      </c>
-      <c r="S2" s="99" t="s">
-        <v>112</v>
-      </c>
-      <c r="T2" s="99" t="s">
-        <v>64</v>
-      </c>
-      <c r="U2" s="100" t="s">
-        <v>79</v>
-      </c>
-      <c r="V2" s="99" t="s">
-        <v>63</v>
-      </c>
-      <c r="W2" s="99" t="s">
-        <v>284</v>
-      </c>
-      <c r="X2" s="99" t="s">
-        <v>285</v>
-      </c>
-      <c r="Y2" s="99" t="s">
-        <v>61</v>
-      </c>
-      <c r="Z2" s="99" t="s">
-        <v>60</v>
-      </c>
-      <c r="AA2" s="100" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A3" s="42"/>
-      <c r="B3" s="41"/>
-      <c r="C3" s="41"/>
-      <c r="D3" s="150" t="s">
-        <v>266</v>
-      </c>
-      <c r="E3" s="96" t="s">
-        <v>59</v>
-      </c>
-      <c r="F3" s="96" t="s">
-        <v>58</v>
-      </c>
-      <c r="G3" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!G3),"",IF(ETPT_CA_JUR!G3=0,"",ETPT_CA_JUR!G3)))</f>
-        <v/>
-      </c>
-      <c r="H3" s="137">
-        <f>ETPT_CA_JUR!H3</f>
-        <v>0</v>
-      </c>
-      <c r="I3" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!I3),"",IF(ETPT_CA_JUR!I3=0,"",ETPT_CA_JUR!I3)))</f>
-        <v/>
-      </c>
-      <c r="J3" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!J3),"",IF(ETPT_CA_JUR!J3=0,"",ETPT_CA_JUR!J3)))</f>
-        <v/>
-      </c>
-      <c r="K3" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!K3),"",IF(ETPT_CA_JUR!K3=0,"",ETPT_CA_JUR!K3)))</f>
-        <v/>
-      </c>
-      <c r="L3" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!L3),"",IF(ETPT_CA_JUR!L3=0,"",ETPT_CA_JUR!L3)))</f>
-        <v/>
-      </c>
-      <c r="M3" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!M3),"",IF(ETPT_CA_JUR!M3=0,"",ETPT_CA_JUR!M3)))</f>
-        <v/>
-      </c>
-      <c r="N3" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!N3),"",IF(ETPT_CA_JUR!N3=0,"",ETPT_CA_JUR!N3)))</f>
-        <v/>
-      </c>
-      <c r="O3" s="137">
-        <f>ETPT_CA_JUR!O3</f>
-        <v>0</v>
-      </c>
-      <c r="P3" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!P3),"",IF(ETPT_CA_JUR!P3=0,"",ETPT_CA_JUR!P3)))</f>
-        <v/>
-      </c>
-      <c r="Q3" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Q3),"",IF(ETPT_CA_JUR!Q3=0,"",ETPT_CA_JUR!Q3)))</f>
-        <v/>
-      </c>
-      <c r="R3" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!R3),"",IF(ETPT_CA_JUR!R3=0,"",ETPT_CA_JUR!R3)))</f>
-        <v/>
-      </c>
-      <c r="S3" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!S3),"",IF(ETPT_CA_JUR!S3=0,"",ETPT_CA_JUR!S3)))</f>
-        <v/>
-      </c>
-      <c r="T3" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!T3),"",IF(ETPT_CA_JUR!T3=0,"",ETPT_CA_JUR!T3)))</f>
-        <v/>
-      </c>
-      <c r="U3" s="137">
-        <f>ETPT_CA_JUR!U3</f>
-        <v>0</v>
-      </c>
-      <c r="V3" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!V3),"",IF(ETPT_CA_JUR!V3=0,"",ETPT_CA_JUR!V3)))</f>
-        <v/>
-      </c>
-      <c r="W3" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!W3),"",IF(ETPT_CA_JUR!W3=0,"",ETPT_CA_JUR!W3)))</f>
-        <v/>
-      </c>
-      <c r="X3" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!X3),"",IF(ETPT_CA_JUR!X3=0,"",ETPT_CA_JUR!X3)))</f>
-        <v/>
-      </c>
-      <c r="Y3" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Y3),"",IF(ETPT_CA_JUR!Y3=0,"",ETPT_CA_JUR!Y3)))</f>
-        <v/>
-      </c>
-      <c r="Z3" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Z3),"",IF(ETPT_CA_JUR!Z3=0,"",ETPT_CA_JUR!Z3)))</f>
-        <v/>
-      </c>
-      <c r="AA3" s="137">
-        <f>ETPT_CA_JUR!AA3</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A4" s="42"/>
-      <c r="B4" s="41"/>
-      <c r="C4" s="41"/>
-      <c r="D4" s="38" t="str">
-        <f>IF(ISBLANK($D$3),"",$D$3)</f>
-        <v>A</v>
-      </c>
-      <c r="E4" s="96" t="s">
-        <v>57</v>
-      </c>
-      <c r="F4" s="96" t="s">
-        <v>56</v>
-      </c>
-      <c r="G4" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!G4),"",IF(ETPT_CA_JUR!G4=0,"",ETPT_CA_JUR!G4)))</f>
-        <v/>
-      </c>
-      <c r="H4" s="137">
-        <f>ETPT_CA_JUR!H4</f>
-        <v>0</v>
-      </c>
-      <c r="I4" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!I4),"",IF(ETPT_CA_JUR!I4=0,"",ETPT_CA_JUR!I4)))</f>
-        <v/>
-      </c>
-      <c r="J4" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!J4),"",IF(ETPT_CA_JUR!J4=0,"",ETPT_CA_JUR!J4)))</f>
-        <v/>
-      </c>
-      <c r="K4" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!K4),"",IF(ETPT_CA_JUR!K4=0,"",ETPT_CA_JUR!K4)))</f>
-        <v/>
-      </c>
-      <c r="L4" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!L4),"",IF(ETPT_CA_JUR!L4=0,"",ETPT_CA_JUR!L4)))</f>
-        <v/>
-      </c>
-      <c r="M4" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!M4),"",IF(ETPT_CA_JUR!M4=0,"",ETPT_CA_JUR!M4)))</f>
-        <v/>
-      </c>
-      <c r="N4" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!N4),"",IF(ETPT_CA_JUR!N4=0,"",ETPT_CA_JUR!N4)))</f>
-        <v/>
-      </c>
-      <c r="O4" s="137">
-        <f>ETPT_CA_JUR!O4</f>
-        <v>0</v>
-      </c>
-      <c r="P4" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!P4),"",IF(ETPT_CA_JUR!P4=0,"",ETPT_CA_JUR!P4)))</f>
-        <v/>
-      </c>
-      <c r="Q4" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Q4),"",IF(ETPT_CA_JUR!Q4=0,"",ETPT_CA_JUR!Q4)))</f>
-        <v/>
-      </c>
-      <c r="R4" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!R4),"",IF(ETPT_CA_JUR!R4=0,"",ETPT_CA_JUR!R4)))</f>
-        <v/>
-      </c>
-      <c r="S4" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!S4),"",IF(ETPT_CA_JUR!S4=0,"",ETPT_CA_JUR!S4)))</f>
-        <v/>
-      </c>
-      <c r="T4" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!T4),"",IF(ETPT_CA_JUR!T4=0,"",ETPT_CA_JUR!T4)))</f>
-        <v/>
-      </c>
-      <c r="U4" s="137">
-        <f>ETPT_CA_JUR!U4</f>
-        <v>0</v>
-      </c>
-      <c r="V4" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!V4),"",IF(ETPT_CA_JUR!V4=0,"",ETPT_CA_JUR!V4)))</f>
-        <v/>
-      </c>
-      <c r="W4" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!W4),"",IF(ETPT_CA_JUR!W4=0,"",ETPT_CA_JUR!W4)))</f>
-        <v/>
-      </c>
-      <c r="X4" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!X4),"",IF(ETPT_CA_JUR!X4=0,"",ETPT_CA_JUR!X4)))</f>
-        <v/>
-      </c>
-      <c r="Y4" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Y4),"",IF(ETPT_CA_JUR!Y4=0,"",ETPT_CA_JUR!Y4)))</f>
-        <v/>
-      </c>
-      <c r="Z4" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Z4),"",IF(ETPT_CA_JUR!Z4=0,"",ETPT_CA_JUR!Z4)))</f>
-        <v/>
-      </c>
-      <c r="AA4" s="137">
-        <f>ETPT_CA_JUR!AA4</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A5" s="42"/>
-      <c r="B5" s="41"/>
-      <c r="C5" s="41"/>
-      <c r="D5" s="38" t="str">
-        <f t="shared" ref="D5:D13" si="0">IF(ISBLANK($D$3),"",$D$3)</f>
-        <v>A</v>
-      </c>
-      <c r="E5" s="96" t="s">
-        <v>55</v>
-      </c>
-      <c r="F5" s="96" t="s">
-        <v>54</v>
-      </c>
-      <c r="G5" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!G5),"",IF(ETPT_CA_JUR!G5=0,"",ETPT_CA_JUR!G5)))</f>
-        <v/>
-      </c>
-      <c r="H5" s="137">
-        <f>ETPT_CA_JUR!H5</f>
-        <v>0</v>
-      </c>
-      <c r="I5" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!I5),"",IF(ETPT_CA_JUR!I5=0,"",ETPT_CA_JUR!I5)))</f>
-        <v/>
-      </c>
-      <c r="J5" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!J5),"",IF(ETPT_CA_JUR!J5=0,"",ETPT_CA_JUR!J5)))</f>
-        <v/>
-      </c>
-      <c r="K5" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!K5),"",IF(ETPT_CA_JUR!K5=0,"",ETPT_CA_JUR!K5)))</f>
-        <v/>
-      </c>
-      <c r="L5" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!L5),"",IF(ETPT_CA_JUR!L5=0,"",ETPT_CA_JUR!L5)))</f>
-        <v/>
-      </c>
-      <c r="M5" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!M5),"",IF(ETPT_CA_JUR!M5=0,"",ETPT_CA_JUR!M5)))</f>
-        <v/>
-      </c>
-      <c r="N5" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!N5),"",IF(ETPT_CA_JUR!N5=0,"",ETPT_CA_JUR!N5)))</f>
-        <v/>
-      </c>
-      <c r="O5" s="137">
-        <f>ETPT_CA_JUR!O5</f>
-        <v>0</v>
-      </c>
-      <c r="P5" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!P5),"",IF(ETPT_CA_JUR!P5=0,"",ETPT_CA_JUR!P5)))</f>
-        <v/>
-      </c>
-      <c r="Q5" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Q5),"",IF(ETPT_CA_JUR!Q5=0,"",ETPT_CA_JUR!Q5)))</f>
-        <v/>
-      </c>
-      <c r="R5" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!R5),"",IF(ETPT_CA_JUR!R5=0,"",ETPT_CA_JUR!R5)))</f>
-        <v/>
-      </c>
-      <c r="S5" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!S5),"",IF(ETPT_CA_JUR!S5=0,"",ETPT_CA_JUR!S5)))</f>
-        <v/>
-      </c>
-      <c r="T5" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!T5),"",IF(ETPT_CA_JUR!T5=0,"",ETPT_CA_JUR!T5)))</f>
-        <v/>
-      </c>
-      <c r="U5" s="137">
-        <f>ETPT_CA_JUR!U5</f>
-        <v>0</v>
-      </c>
-      <c r="V5" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!V5),"",IF(ETPT_CA_JUR!V5=0,"",ETPT_CA_JUR!V5)))</f>
-        <v/>
-      </c>
-      <c r="W5" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!W5),"",IF(ETPT_CA_JUR!W5=0,"",ETPT_CA_JUR!W5)))</f>
-        <v/>
-      </c>
-      <c r="X5" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!X5),"",IF(ETPT_CA_JUR!X5=0,"",ETPT_CA_JUR!X5)))</f>
-        <v/>
-      </c>
-      <c r="Y5" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Y5),"",IF(ETPT_CA_JUR!Y5=0,"",ETPT_CA_JUR!Y5)))</f>
-        <v/>
-      </c>
-      <c r="Z5" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Z5),"",IF(ETPT_CA_JUR!Z5=0,"",ETPT_CA_JUR!Z5)))</f>
-        <v/>
-      </c>
-      <c r="AA5" s="137">
-        <f>ETPT_CA_JUR!AA5</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A6" s="42"/>
-      <c r="B6" s="41"/>
-      <c r="C6" s="41"/>
-      <c r="D6" s="38" t="str">
-        <f t="shared" si="0"/>
-        <v>A</v>
-      </c>
-      <c r="E6" s="96" t="s">
-        <v>53</v>
-      </c>
-      <c r="F6" s="96" t="s">
-        <v>52</v>
-      </c>
-      <c r="G6" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!G6),"",IF(ETPT_CA_JUR!G6=0,"",ETPT_CA_JUR!G6)))</f>
-        <v/>
-      </c>
-      <c r="H6" s="137">
-        <f>ETPT_CA_JUR!H6</f>
-        <v>0</v>
-      </c>
-      <c r="I6" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!I6),"",IF(ETPT_CA_JUR!I6=0,"",ETPT_CA_JUR!I6)))</f>
-        <v/>
-      </c>
-      <c r="J6" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!J6),"",IF(ETPT_CA_JUR!J6=0,"",ETPT_CA_JUR!J6)))</f>
-        <v/>
-      </c>
-      <c r="K6" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!K6),"",IF(ETPT_CA_JUR!K6=0,"",ETPT_CA_JUR!K6)))</f>
-        <v/>
-      </c>
-      <c r="L6" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!L6),"",IF(ETPT_CA_JUR!L6=0,"",ETPT_CA_JUR!L6)))</f>
-        <v/>
-      </c>
-      <c r="M6" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!M6),"",IF(ETPT_CA_JUR!M6=0,"",ETPT_CA_JUR!M6)))</f>
-        <v/>
-      </c>
-      <c r="N6" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!N6),"",IF(ETPT_CA_JUR!N6=0,"",ETPT_CA_JUR!N6)))</f>
-        <v/>
-      </c>
-      <c r="O6" s="137">
-        <f>ETPT_CA_JUR!O6</f>
-        <v>0</v>
-      </c>
-      <c r="P6" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!P6),"",IF(ETPT_CA_JUR!P6=0,"",ETPT_CA_JUR!P6)))</f>
-        <v/>
-      </c>
-      <c r="Q6" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Q6),"",IF(ETPT_CA_JUR!Q6=0,"",ETPT_CA_JUR!Q6)))</f>
-        <v/>
-      </c>
-      <c r="R6" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!R6),"",IF(ETPT_CA_JUR!R6=0,"",ETPT_CA_JUR!R6)))</f>
-        <v/>
-      </c>
-      <c r="S6" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!S6),"",IF(ETPT_CA_JUR!S6=0,"",ETPT_CA_JUR!S6)))</f>
-        <v/>
-      </c>
-      <c r="T6" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!T6),"",IF(ETPT_CA_JUR!T6=0,"",ETPT_CA_JUR!T6)))</f>
-        <v/>
-      </c>
-      <c r="U6" s="137">
-        <f>ETPT_CA_JUR!U6</f>
-        <v>0</v>
-      </c>
-      <c r="V6" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!V6),"",IF(ETPT_CA_JUR!V6=0,"",ETPT_CA_JUR!V6)))</f>
-        <v/>
-      </c>
-      <c r="W6" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!W6),"",IF(ETPT_CA_JUR!W6=0,"",ETPT_CA_JUR!W6)))</f>
-        <v/>
-      </c>
-      <c r="X6" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!X6),"",IF(ETPT_CA_JUR!X6=0,"",ETPT_CA_JUR!X6)))</f>
-        <v/>
-      </c>
-      <c r="Y6" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Y6),"",IF(ETPT_CA_JUR!Y6=0,"",ETPT_CA_JUR!Y6)))</f>
-        <v/>
-      </c>
-      <c r="Z6" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Z6),"",IF(ETPT_CA_JUR!Z6=0,"",ETPT_CA_JUR!Z6)))</f>
-        <v/>
-      </c>
-      <c r="AA6" s="137">
-        <f>ETPT_CA_JUR!AA6</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A7" s="42"/>
-      <c r="B7" s="41"/>
-      <c r="C7" s="41"/>
-      <c r="D7" s="38" t="str">
-        <f t="shared" si="0"/>
-        <v>A</v>
-      </c>
-      <c r="E7" s="96" t="s">
-        <v>51</v>
-      </c>
-      <c r="F7" s="96" t="s">
-        <v>50</v>
-      </c>
-      <c r="G7" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!G7),"",IF(ETPT_CA_JUR!G7=0,"",ETPT_CA_JUR!G7)))</f>
-        <v/>
-      </c>
-      <c r="H7" s="137">
-        <f>ETPT_CA_JUR!H7</f>
-        <v>0</v>
-      </c>
-      <c r="I7" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!I7),"",IF(ETPT_CA_JUR!I7=0,"",ETPT_CA_JUR!I7)))</f>
-        <v/>
-      </c>
-      <c r="J7" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!J7),"",IF(ETPT_CA_JUR!J7=0,"",ETPT_CA_JUR!J7)))</f>
-        <v/>
-      </c>
-      <c r="K7" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!K7),"",IF(ETPT_CA_JUR!K7=0,"",ETPT_CA_JUR!K7)))</f>
-        <v/>
-      </c>
-      <c r="L7" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!L7),"",IF(ETPT_CA_JUR!L7=0,"",ETPT_CA_JUR!L7)))</f>
-        <v/>
-      </c>
-      <c r="M7" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!M7),"",IF(ETPT_CA_JUR!M7=0,"",ETPT_CA_JUR!M7)))</f>
-        <v/>
-      </c>
-      <c r="N7" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!N7),"",IF(ETPT_CA_JUR!N7=0,"",ETPT_CA_JUR!N7)))</f>
-        <v/>
-      </c>
-      <c r="O7" s="137">
-        <f>ETPT_CA_JUR!O7</f>
-        <v>0</v>
-      </c>
-      <c r="P7" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!P7),"",IF(ETPT_CA_JUR!P7=0,"",ETPT_CA_JUR!P7)))</f>
-        <v/>
-      </c>
-      <c r="Q7" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Q7),"",IF(ETPT_CA_JUR!Q7=0,"",ETPT_CA_JUR!Q7)))</f>
-        <v/>
-      </c>
-      <c r="R7" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!R7),"",IF(ETPT_CA_JUR!R7=0,"",ETPT_CA_JUR!R7)))</f>
-        <v/>
-      </c>
-      <c r="S7" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!S7),"",IF(ETPT_CA_JUR!S7=0,"",ETPT_CA_JUR!S7)))</f>
-        <v/>
-      </c>
-      <c r="T7" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!T7),"",IF(ETPT_CA_JUR!T7=0,"",ETPT_CA_JUR!T7)))</f>
-        <v/>
-      </c>
-      <c r="U7" s="137">
-        <f>ETPT_CA_JUR!U7</f>
-        <v>0</v>
-      </c>
-      <c r="V7" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!V7),"",IF(ETPT_CA_JUR!V7=0,"",ETPT_CA_JUR!V7)))</f>
-        <v/>
-      </c>
-      <c r="W7" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!W7),"",IF(ETPT_CA_JUR!W7=0,"",ETPT_CA_JUR!W7)))</f>
-        <v/>
-      </c>
-      <c r="X7" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!X7),"",IF(ETPT_CA_JUR!X7=0,"",ETPT_CA_JUR!X7)))</f>
-        <v/>
-      </c>
-      <c r="Y7" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Y7),"",IF(ETPT_CA_JUR!Y7=0,"",ETPT_CA_JUR!Y7)))</f>
-        <v/>
-      </c>
-      <c r="Z7" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Z7),"",IF(ETPT_CA_JUR!Z7=0,"",ETPT_CA_JUR!Z7)))</f>
-        <v/>
-      </c>
-      <c r="AA7" s="137">
-        <f>ETPT_CA_JUR!AA7</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A8" s="42"/>
-      <c r="B8" s="41"/>
-      <c r="C8" s="41"/>
-      <c r="D8" s="38" t="str">
-        <f t="shared" si="0"/>
-        <v>A</v>
-      </c>
-      <c r="E8" s="96" t="s">
-        <v>49</v>
-      </c>
-      <c r="F8" s="96" t="s">
-        <v>48</v>
-      </c>
-      <c r="G8" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!G8),"",IF(ETPT_CA_JUR!G8=0,"",ETPT_CA_JUR!G8)))</f>
-        <v/>
-      </c>
-      <c r="H8" s="137">
-        <f>ETPT_CA_JUR!H8</f>
-        <v>0</v>
-      </c>
-      <c r="I8" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!I8),"",IF(ETPT_CA_JUR!I8=0,"",ETPT_CA_JUR!I8)))</f>
-        <v/>
-      </c>
-      <c r="J8" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!J8),"",IF(ETPT_CA_JUR!J8=0,"",ETPT_CA_JUR!J8)))</f>
-        <v/>
-      </c>
-      <c r="K8" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!K8),"",IF(ETPT_CA_JUR!K8=0,"",ETPT_CA_JUR!K8)))</f>
-        <v/>
-      </c>
-      <c r="L8" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!L8),"",IF(ETPT_CA_JUR!L8=0,"",ETPT_CA_JUR!L8)))</f>
-        <v/>
-      </c>
-      <c r="M8" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!M8),"",IF(ETPT_CA_JUR!M8=0,"",ETPT_CA_JUR!M8)))</f>
-        <v/>
-      </c>
-      <c r="N8" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!N8),"",IF(ETPT_CA_JUR!N8=0,"",ETPT_CA_JUR!N8)))</f>
-        <v/>
-      </c>
-      <c r="O8" s="137">
-        <f>ETPT_CA_JUR!O8</f>
-        <v>0</v>
-      </c>
-      <c r="P8" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!P8),"",IF(ETPT_CA_JUR!P8=0,"",ETPT_CA_JUR!P8)))</f>
-        <v/>
-      </c>
-      <c r="Q8" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Q8),"",IF(ETPT_CA_JUR!Q8=0,"",ETPT_CA_JUR!Q8)))</f>
-        <v/>
-      </c>
-      <c r="R8" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!R8),"",IF(ETPT_CA_JUR!R8=0,"",ETPT_CA_JUR!R8)))</f>
-        <v/>
-      </c>
-      <c r="S8" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!S8),"",IF(ETPT_CA_JUR!S8=0,"",ETPT_CA_JUR!S8)))</f>
-        <v/>
-      </c>
-      <c r="T8" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!T8),"",IF(ETPT_CA_JUR!T8=0,"",ETPT_CA_JUR!T8)))</f>
-        <v/>
-      </c>
-      <c r="U8" s="137">
-        <f>ETPT_CA_JUR!U8</f>
-        <v>0</v>
-      </c>
-      <c r="V8" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!V8),"",IF(ETPT_CA_JUR!V8=0,"",ETPT_CA_JUR!V8)))</f>
-        <v/>
-      </c>
-      <c r="W8" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!W8),"",IF(ETPT_CA_JUR!W8=0,"",ETPT_CA_JUR!W8)))</f>
-        <v/>
-      </c>
-      <c r="X8" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!X8),"",IF(ETPT_CA_JUR!X8=0,"",ETPT_CA_JUR!X8)))</f>
-        <v/>
-      </c>
-      <c r="Y8" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Y8),"",IF(ETPT_CA_JUR!Y8=0,"",ETPT_CA_JUR!Y8)))</f>
-        <v/>
-      </c>
-      <c r="Z8" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Z8),"",IF(ETPT_CA_JUR!Z8=0,"",ETPT_CA_JUR!Z8)))</f>
-        <v/>
-      </c>
-      <c r="AA8" s="137">
-        <f>ETPT_CA_JUR!AA8</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A9" s="42"/>
-      <c r="B9" s="41"/>
-      <c r="C9" s="41"/>
-      <c r="D9" s="38" t="str">
-        <f t="shared" si="0"/>
-        <v>A</v>
-      </c>
-      <c r="E9" s="96" t="s">
-        <v>47</v>
-      </c>
-      <c r="F9" s="96" t="s">
-        <v>46</v>
-      </c>
-      <c r="G9" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!G9),"",IF(ETPT_CA_JUR!G9=0,"",ETPT_CA_JUR!G9)))</f>
-        <v/>
-      </c>
-      <c r="H9" s="137">
-        <f>ETPT_CA_JUR!H9</f>
-        <v>0</v>
-      </c>
-      <c r="I9" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!I9),"",IF(ETPT_CA_JUR!I9=0,"",ETPT_CA_JUR!I9)))</f>
-        <v/>
-      </c>
-      <c r="J9" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!J9),"",IF(ETPT_CA_JUR!J9=0,"",ETPT_CA_JUR!J9)))</f>
-        <v/>
-      </c>
-      <c r="K9" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!K9),"",IF(ETPT_CA_JUR!K9=0,"",ETPT_CA_JUR!K9)))</f>
-        <v/>
-      </c>
-      <c r="L9" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!L9),"",IF(ETPT_CA_JUR!L9=0,"",ETPT_CA_JUR!L9)))</f>
-        <v/>
-      </c>
-      <c r="M9" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!M9),"",IF(ETPT_CA_JUR!M9=0,"",ETPT_CA_JUR!M9)))</f>
-        <v/>
-      </c>
-      <c r="N9" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!N9),"",IF(ETPT_CA_JUR!N9=0,"",ETPT_CA_JUR!N9)))</f>
-        <v/>
-      </c>
-      <c r="O9" s="137">
-        <f>ETPT_CA_JUR!O9</f>
-        <v>0</v>
-      </c>
-      <c r="P9" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!P9),"",IF(ETPT_CA_JUR!P9=0,"",ETPT_CA_JUR!P9)))</f>
-        <v/>
-      </c>
-      <c r="Q9" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Q9),"",IF(ETPT_CA_JUR!Q9=0,"",ETPT_CA_JUR!Q9)))</f>
-        <v/>
-      </c>
-      <c r="R9" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!R9),"",IF(ETPT_CA_JUR!R9=0,"",ETPT_CA_JUR!R9)))</f>
-        <v/>
-      </c>
-      <c r="S9" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!S9),"",IF(ETPT_CA_JUR!S9=0,"",ETPT_CA_JUR!S9)))</f>
-        <v/>
-      </c>
-      <c r="T9" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!T9),"",IF(ETPT_CA_JUR!T9=0,"",ETPT_CA_JUR!T9)))</f>
-        <v/>
-      </c>
-      <c r="U9" s="137">
-        <f>ETPT_CA_JUR!U9</f>
-        <v>0</v>
-      </c>
-      <c r="V9" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!V9),"",IF(ETPT_CA_JUR!V9=0,"",ETPT_CA_JUR!V9)))</f>
-        <v/>
-      </c>
-      <c r="W9" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!W9),"",IF(ETPT_CA_JUR!W9=0,"",ETPT_CA_JUR!W9)))</f>
-        <v/>
-      </c>
-      <c r="X9" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!X9),"",IF(ETPT_CA_JUR!X9=0,"",ETPT_CA_JUR!X9)))</f>
-        <v/>
-      </c>
-      <c r="Y9" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Y9),"",IF(ETPT_CA_JUR!Y9=0,"",ETPT_CA_JUR!Y9)))</f>
-        <v/>
-      </c>
-      <c r="Z9" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Z9),"",IF(ETPT_CA_JUR!Z9=0,"",ETPT_CA_JUR!Z9)))</f>
-        <v/>
-      </c>
-      <c r="AA9" s="137">
-        <f>ETPT_CA_JUR!AA9</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A10" s="42"/>
-      <c r="B10" s="41"/>
-      <c r="C10" s="41"/>
-      <c r="D10" s="38" t="str">
-        <f t="shared" si="0"/>
-        <v>A</v>
-      </c>
-      <c r="E10" s="96" t="s">
-        <v>45</v>
-      </c>
-      <c r="F10" s="96" t="s">
-        <v>44</v>
-      </c>
-      <c r="G10" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!G10),"",IF(ETPT_CA_JUR!G10=0,"",ETPT_CA_JUR!G10)))</f>
-        <v/>
-      </c>
-      <c r="H10" s="137">
-        <f>ETPT_CA_JUR!H10</f>
-        <v>0</v>
-      </c>
-      <c r="I10" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!I10),"",IF(ETPT_CA_JUR!I10=0,"",ETPT_CA_JUR!I10)))</f>
-        <v/>
-      </c>
-      <c r="J10" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!J10),"",IF(ETPT_CA_JUR!J10=0,"",ETPT_CA_JUR!J10)))</f>
-        <v/>
-      </c>
-      <c r="K10" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!K10),"",IF(ETPT_CA_JUR!K10=0,"",ETPT_CA_JUR!K10)))</f>
-        <v/>
-      </c>
-      <c r="L10" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!L10),"",IF(ETPT_CA_JUR!L10=0,"",ETPT_CA_JUR!L10)))</f>
-        <v/>
-      </c>
-      <c r="M10" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!M10),"",IF(ETPT_CA_JUR!M10=0,"",ETPT_CA_JUR!M10)))</f>
-        <v/>
-      </c>
-      <c r="N10" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!N10),"",IF(ETPT_CA_JUR!N10=0,"",ETPT_CA_JUR!N10)))</f>
-        <v/>
-      </c>
-      <c r="O10" s="137">
-        <f>ETPT_CA_JUR!O10</f>
-        <v>0</v>
-      </c>
-      <c r="P10" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!P10),"",IF(ETPT_CA_JUR!P10=0,"",ETPT_CA_JUR!P10)))</f>
-        <v/>
-      </c>
-      <c r="Q10" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Q10),"",IF(ETPT_CA_JUR!Q10=0,"",ETPT_CA_JUR!Q10)))</f>
-        <v/>
-      </c>
-      <c r="R10" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!R10),"",IF(ETPT_CA_JUR!R10=0,"",ETPT_CA_JUR!R10)))</f>
-        <v/>
-      </c>
-      <c r="S10" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!S10),"",IF(ETPT_CA_JUR!S10=0,"",ETPT_CA_JUR!S10)))</f>
-        <v/>
-      </c>
-      <c r="T10" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!T10),"",IF(ETPT_CA_JUR!T10=0,"",ETPT_CA_JUR!T10)))</f>
-        <v/>
-      </c>
-      <c r="U10" s="137">
-        <f>ETPT_CA_JUR!U10</f>
-        <v>0</v>
-      </c>
-      <c r="V10" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!V10),"",IF(ETPT_CA_JUR!V10=0,"",ETPT_CA_JUR!V10)))</f>
-        <v/>
-      </c>
-      <c r="W10" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!W10),"",IF(ETPT_CA_JUR!W10=0,"",ETPT_CA_JUR!W10)))</f>
-        <v/>
-      </c>
-      <c r="X10" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!X10),"",IF(ETPT_CA_JUR!X10=0,"",ETPT_CA_JUR!X10)))</f>
-        <v/>
-      </c>
-      <c r="Y10" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Y10),"",IF(ETPT_CA_JUR!Y10=0,"",ETPT_CA_JUR!Y10)))</f>
-        <v/>
-      </c>
-      <c r="Z10" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Z10),"",IF(ETPT_CA_JUR!Z10=0,"",ETPT_CA_JUR!Z10)))</f>
-        <v/>
-      </c>
-      <c r="AA10" s="137">
-        <f>ETPT_CA_JUR!AA10</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A11" s="42"/>
-      <c r="B11" s="41"/>
-      <c r="C11" s="41"/>
-      <c r="D11" s="38" t="str">
-        <f t="shared" si="0"/>
-        <v>A</v>
-      </c>
-      <c r="E11" s="96" t="s">
-        <v>43</v>
-      </c>
-      <c r="F11" s="96" t="s">
-        <v>42</v>
-      </c>
-      <c r="G11" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!G11),"",IF(ETPT_CA_JUR!G11=0,"",ETPT_CA_JUR!G11)))</f>
-        <v/>
-      </c>
-      <c r="H11" s="137">
-        <f>ETPT_CA_JUR!H11</f>
-        <v>0</v>
-      </c>
-      <c r="I11" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!I11),"",IF(ETPT_CA_JUR!I11=0,"",ETPT_CA_JUR!I11)))</f>
-        <v/>
-      </c>
-      <c r="J11" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!J11),"",IF(ETPT_CA_JUR!J11=0,"",ETPT_CA_JUR!J11)))</f>
-        <v/>
-      </c>
-      <c r="K11" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!K11),"",IF(ETPT_CA_JUR!K11=0,"",ETPT_CA_JUR!K11)))</f>
-        <v/>
-      </c>
-      <c r="L11" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!L11),"",IF(ETPT_CA_JUR!L11=0,"",ETPT_CA_JUR!L11)))</f>
-        <v/>
-      </c>
-      <c r="M11" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!M11),"",IF(ETPT_CA_JUR!M11=0,"",ETPT_CA_JUR!M11)))</f>
-        <v/>
-      </c>
-      <c r="N11" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!N11),"",IF(ETPT_CA_JUR!N11=0,"",ETPT_CA_JUR!N11)))</f>
-        <v/>
-      </c>
-      <c r="O11" s="137">
-        <f>ETPT_CA_JUR!O11</f>
-        <v>0</v>
-      </c>
-      <c r="P11" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!P11),"",IF(ETPT_CA_JUR!P11=0,"",ETPT_CA_JUR!P11)))</f>
-        <v/>
-      </c>
-      <c r="Q11" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Q11),"",IF(ETPT_CA_JUR!Q11=0,"",ETPT_CA_JUR!Q11)))</f>
-        <v/>
-      </c>
-      <c r="R11" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!R11),"",IF(ETPT_CA_JUR!R11=0,"",ETPT_CA_JUR!R11)))</f>
-        <v/>
-      </c>
-      <c r="S11" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!S11),"",IF(ETPT_CA_JUR!S11=0,"",ETPT_CA_JUR!S11)))</f>
-        <v/>
-      </c>
-      <c r="T11" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!T11),"",IF(ETPT_CA_JUR!T11=0,"",ETPT_CA_JUR!T11)))</f>
-        <v/>
-      </c>
-      <c r="U11" s="137">
-        <f>ETPT_CA_JUR!U11</f>
-        <v>0</v>
-      </c>
-      <c r="V11" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!V11),"",IF(ETPT_CA_JUR!V11=0,"",ETPT_CA_JUR!V11)))</f>
-        <v/>
-      </c>
-      <c r="W11" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!W11),"",IF(ETPT_CA_JUR!W11=0,"",ETPT_CA_JUR!W11)))</f>
-        <v/>
-      </c>
-      <c r="X11" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!X11),"",IF(ETPT_CA_JUR!X11=0,"",ETPT_CA_JUR!X11)))</f>
-        <v/>
-      </c>
-      <c r="Y11" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Y11),"",IF(ETPT_CA_JUR!Y11=0,"",ETPT_CA_JUR!Y11)))</f>
-        <v/>
-      </c>
-      <c r="Z11" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Z11),"",IF(ETPT_CA_JUR!Z11=0,"",ETPT_CA_JUR!Z11)))</f>
-        <v/>
-      </c>
-      <c r="AA11" s="137">
-        <f>ETPT_CA_JUR!AA11</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A12" s="40"/>
-      <c r="B12" s="39"/>
-      <c r="C12" s="39"/>
-      <c r="D12" s="38" t="str">
-        <f t="shared" si="0"/>
-        <v>A</v>
-      </c>
-      <c r="E12" s="96" t="s">
-        <v>41</v>
-      </c>
-      <c r="F12" s="96" t="s">
-        <v>40</v>
-      </c>
-      <c r="G12" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!G12),"",IF(ETPT_CA_JUR!G12=0,"",ETPT_CA_JUR!G12)))</f>
-        <v/>
-      </c>
-      <c r="H12" s="137">
-        <f>ETPT_CA_JUR!H12</f>
-        <v>0</v>
-      </c>
-      <c r="I12" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!I12),"",IF(ETPT_CA_JUR!I12=0,"",ETPT_CA_JUR!I12)))</f>
-        <v/>
-      </c>
-      <c r="J12" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!J12),"",IF(ETPT_CA_JUR!J12=0,"",ETPT_CA_JUR!J12)))</f>
-        <v/>
-      </c>
-      <c r="K12" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!K12),"",IF(ETPT_CA_JUR!K12=0,"",ETPT_CA_JUR!K12)))</f>
-        <v/>
-      </c>
-      <c r="L12" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!L12),"",IF(ETPT_CA_JUR!L12=0,"",ETPT_CA_JUR!L12)))</f>
-        <v/>
-      </c>
-      <c r="M12" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!M12),"",IF(ETPT_CA_JUR!M12=0,"",ETPT_CA_JUR!M12)))</f>
-        <v/>
-      </c>
-      <c r="N12" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!N12),"",IF(ETPT_CA_JUR!N12=0,"",ETPT_CA_JUR!N12)))</f>
-        <v/>
-      </c>
-      <c r="O12" s="137">
-        <f>ETPT_CA_JUR!O12</f>
-        <v>0</v>
-      </c>
-      <c r="P12" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!P12),"",IF(ETPT_CA_JUR!P12=0,"",ETPT_CA_JUR!P12)))</f>
-        <v/>
-      </c>
-      <c r="Q12" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Q12),"",IF(ETPT_CA_JUR!Q12=0,"",ETPT_CA_JUR!Q12)))</f>
-        <v/>
-      </c>
-      <c r="R12" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!R12),"",IF(ETPT_CA_JUR!R12=0,"",ETPT_CA_JUR!R12)))</f>
-        <v/>
-      </c>
-      <c r="S12" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!S12),"",IF(ETPT_CA_JUR!S12=0,"",ETPT_CA_JUR!S12)))</f>
-        <v/>
-      </c>
-      <c r="T12" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!T12),"",IF(ETPT_CA_JUR!T12=0,"",ETPT_CA_JUR!T12)))</f>
-        <v/>
-      </c>
-      <c r="U12" s="137">
-        <f>ETPT_CA_JUR!U12</f>
-        <v>0</v>
-      </c>
-      <c r="V12" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!V12),"",IF(ETPT_CA_JUR!V12=0,"",ETPT_CA_JUR!V12)))</f>
-        <v/>
-      </c>
-      <c r="W12" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!W12),"",IF(ETPT_CA_JUR!W12=0,"",ETPT_CA_JUR!W12)))</f>
-        <v/>
-      </c>
-      <c r="X12" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!X12),"",IF(ETPT_CA_JUR!X12=0,"",ETPT_CA_JUR!X12)))</f>
-        <v/>
-      </c>
-      <c r="Y12" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Y12),"",IF(ETPT_CA_JUR!Y12=0,"",ETPT_CA_JUR!Y12)))</f>
-        <v/>
-      </c>
-      <c r="Z12" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Z12),"",IF(ETPT_CA_JUR!Z12=0,"",ETPT_CA_JUR!Z12)))</f>
-        <v/>
-      </c>
-      <c r="AA12" s="137">
-        <f>ETPT_CA_JUR!AA12</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="D13" s="38" t="str">
-        <f t="shared" si="0"/>
-        <v>A</v>
-      </c>
-      <c r="E13" s="96" t="s">
-        <v>114</v>
-      </c>
-      <c r="F13" s="96" t="s">
-        <v>115</v>
-      </c>
-      <c r="G13" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!G13),"",IF(ETPT_CA_JUR!G13=0,"",ETPT_CA_JUR!G13)))</f>
-        <v/>
-      </c>
-      <c r="H13" s="137">
-        <f>ETPT_CA_JUR!H13</f>
-        <v>0</v>
-      </c>
-      <c r="I13" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!I13),"",IF(ETPT_CA_JUR!I13=0,"",ETPT_CA_JUR!I13)))</f>
-        <v/>
-      </c>
-      <c r="J13" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!J13),"",IF(ETPT_CA_JUR!J13=0,"",ETPT_CA_JUR!J13)))</f>
-        <v/>
-      </c>
-      <c r="K13" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!K13),"",IF(ETPT_CA_JUR!K13=0,"",ETPT_CA_JUR!K13)))</f>
-        <v/>
-      </c>
-      <c r="L13" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!L13),"",IF(ETPT_CA_JUR!L13=0,"",ETPT_CA_JUR!L13)))</f>
-        <v/>
-      </c>
-      <c r="M13" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!M13),"",IF(ETPT_CA_JUR!M13=0,"",ETPT_CA_JUR!M13)))</f>
-        <v/>
-      </c>
-      <c r="N13" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!N13),"",IF(ETPT_CA_JUR!N13=0,"",ETPT_CA_JUR!N13)))</f>
-        <v/>
-      </c>
-      <c r="O13" s="137">
-        <f>ETPT_CA_JUR!O13</f>
-        <v>0</v>
-      </c>
-      <c r="P13" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!P13),"",IF(ETPT_CA_JUR!P13=0,"",ETPT_CA_JUR!P13)))</f>
-        <v/>
-      </c>
-      <c r="Q13" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Q13),"",IF(ETPT_CA_JUR!Q13=0,"",ETPT_CA_JUR!Q13)))</f>
-        <v/>
-      </c>
-      <c r="R13" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!R13),"",IF(ETPT_CA_JUR!R13=0,"",ETPT_CA_JUR!R13)))</f>
-        <v/>
-      </c>
-      <c r="S13" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!S13),"",IF(ETPT_CA_JUR!S13=0,"",ETPT_CA_JUR!S13)))</f>
-        <v/>
-      </c>
-      <c r="T13" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!T13),"",IF(ETPT_CA_JUR!T13=0,"",ETPT_CA_JUR!T13)))</f>
-        <v/>
-      </c>
-      <c r="U13" s="137">
-        <f>ETPT_CA_JUR!U13</f>
-        <v>0</v>
-      </c>
-      <c r="V13" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!V13),"",IF(ETPT_CA_JUR!V13=0,"",ETPT_CA_JUR!V13)))</f>
-        <v/>
-      </c>
-      <c r="W13" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!W13),"",IF(ETPT_CA_JUR!W13=0,"",ETPT_CA_JUR!W13)))</f>
-        <v/>
-      </c>
-      <c r="X13" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!X13),"",IF(ETPT_CA_JUR!X13=0,"",ETPT_CA_JUR!X13)))</f>
-        <v/>
-      </c>
-      <c r="Y13" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Y13),"",IF(ETPT_CA_JUR!Y13=0,"",ETPT_CA_JUR!Y13)))</f>
-        <v/>
-      </c>
-      <c r="Z13" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Z13),"",IF(ETPT_CA_JUR!Z13=0,"",ETPT_CA_JUR!Z13)))</f>
-        <v/>
-      </c>
-      <c r="AA13" s="137">
-        <f>ETPT_CA_JUR!AA13</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="D14" s="38" t="str">
-        <f>IF(ISBLANK($D$3),"",$D$3)</f>
-        <v>A</v>
-      </c>
-      <c r="E14" s="96" t="s">
-        <v>39</v>
-      </c>
-      <c r="F14" s="96" t="s">
-        <v>38</v>
-      </c>
-      <c r="G14" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!G14),"",IF(ETPT_CA_JUR!G14=0,"",ETPT_CA_JUR!G14)))</f>
-        <v/>
-      </c>
-      <c r="H14" s="137">
-        <f>ETPT_CA_JUR!H14</f>
-        <v>0</v>
-      </c>
-      <c r="I14" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!I14),"",IF(ETPT_CA_JUR!I14=0,"",ETPT_CA_JUR!I14)))</f>
-        <v/>
-      </c>
-      <c r="J14" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!J14),"",IF(ETPT_CA_JUR!J14=0,"",ETPT_CA_JUR!J14)))</f>
-        <v/>
-      </c>
-      <c r="K14" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!K14),"",IF(ETPT_CA_JUR!K14=0,"",ETPT_CA_JUR!K14)))</f>
-        <v/>
-      </c>
-      <c r="L14" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!L14),"",IF(ETPT_CA_JUR!L14=0,"",ETPT_CA_JUR!L14)))</f>
-        <v/>
-      </c>
-      <c r="M14" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!M14),"",IF(ETPT_CA_JUR!M14=0,"",ETPT_CA_JUR!M14)))</f>
-        <v/>
-      </c>
-      <c r="N14" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!N14),"",IF(ETPT_CA_JUR!N14=0,"",ETPT_CA_JUR!N14)))</f>
-        <v/>
-      </c>
-      <c r="O14" s="137">
-        <f>ETPT_CA_JUR!O14</f>
-        <v>0</v>
-      </c>
-      <c r="P14" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!P14),"",IF(ETPT_CA_JUR!P14=0,"",ETPT_CA_JUR!P14)))</f>
-        <v/>
-      </c>
-      <c r="Q14" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Q14),"",IF(ETPT_CA_JUR!Q14=0,"",ETPT_CA_JUR!Q14)))</f>
-        <v/>
-      </c>
-      <c r="R14" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!R14),"",IF(ETPT_CA_JUR!R14=0,"",ETPT_CA_JUR!R14)))</f>
-        <v/>
-      </c>
-      <c r="S14" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!S14),"",IF(ETPT_CA_JUR!S14=0,"",ETPT_CA_JUR!S14)))</f>
-        <v/>
-      </c>
-      <c r="T14" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!T14),"",IF(ETPT_CA_JUR!T14=0,"",ETPT_CA_JUR!T14)))</f>
-        <v/>
-      </c>
-      <c r="U14" s="137">
-        <f>ETPT_CA_JUR!U14</f>
-        <v>0</v>
-      </c>
-      <c r="V14" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!V14),"",IF(ETPT_CA_JUR!V14=0,"",ETPT_CA_JUR!V14)))</f>
-        <v/>
-      </c>
-      <c r="W14" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!W14),"",IF(ETPT_CA_JUR!W14=0,"",ETPT_CA_JUR!W14)))</f>
-        <v/>
-      </c>
-      <c r="X14" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!X14),"",IF(ETPT_CA_JUR!X14=0,"",ETPT_CA_JUR!X14)))</f>
-        <v/>
-      </c>
-      <c r="Y14" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Y14),"",IF(ETPT_CA_JUR!Y14=0,"",ETPT_CA_JUR!Y14)))</f>
-        <v/>
-      </c>
-      <c r="Z14" s="136" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!Z14),"",IF(ETPT_CA_JUR!Z14=0,"",ETPT_CA_JUR!Z14)))</f>
-        <v/>
-      </c>
-      <c r="AA14" s="137">
-        <f>ETPT_CA_JUR!AA14</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="D15" s="38"/>
-      <c r="E15" s="97"/>
-      <c r="F15" s="98" t="s">
-        <v>37</v>
-      </c>
-      <c r="G15" s="137">
-        <f>ETPT_CA_JUR!G15</f>
-        <v>0</v>
-      </c>
-      <c r="H15" s="137">
-        <f>ETPT_CA_JUR!H15</f>
-        <v>0</v>
-      </c>
-      <c r="I15" s="137">
-        <f>ETPT_CA_JUR!I15</f>
-        <v>0</v>
-      </c>
-      <c r="J15" s="137">
-        <f>ETPT_CA_JUR!J15</f>
-        <v>0</v>
-      </c>
-      <c r="K15" s="137">
-        <f>ETPT_CA_JUR!K15</f>
-        <v>0</v>
-      </c>
-      <c r="L15" s="137">
-        <f>ETPT_CA_JUR!L15</f>
-        <v>0</v>
-      </c>
-      <c r="M15" s="137">
-        <f>ETPT_CA_JUR!M15</f>
-        <v>0</v>
-      </c>
-      <c r="N15" s="137">
-        <f>ETPT_CA_JUR!N15</f>
-        <v>0</v>
-      </c>
-      <c r="O15" s="137">
-        <f>ETPT_CA_JUR!O15</f>
-        <v>0</v>
-      </c>
-      <c r="P15" s="137">
-        <f>ETPT_CA_JUR!P15</f>
-        <v>0</v>
-      </c>
-      <c r="Q15" s="137">
-        <f>ETPT_CA_JUR!Q15</f>
-        <v>0</v>
-      </c>
-      <c r="R15" s="137">
-        <f>ETPT_CA_JUR!R15</f>
-        <v>0</v>
-      </c>
-      <c r="S15" s="137">
-        <f>ETPT_CA_JUR!S15</f>
-        <v>0</v>
-      </c>
-      <c r="T15" s="137">
-        <f>ETPT_CA_JUR!T15</f>
-        <v>0</v>
-      </c>
-      <c r="U15" s="137">
-        <f>ETPT_CA_JUR!U15</f>
-        <v>0</v>
-      </c>
-      <c r="V15" s="137">
-        <f>ETPT_CA_JUR!V15</f>
-        <v>0</v>
-      </c>
-      <c r="W15" s="137">
-        <f>ETPT_CA_JUR!W15</f>
-        <v>0</v>
-      </c>
-      <c r="X15" s="137">
-        <f>ETPT_CA_JUR!X15</f>
-        <v>0</v>
-      </c>
-      <c r="Y15" s="137">
-        <f>ETPT_CA_JUR!Y15</f>
-        <v>0</v>
-      </c>
-      <c r="Z15" s="137">
-        <f>ETPT_CA_JUR!Z15</f>
-        <v>0</v>
-      </c>
-      <c r="AA15" s="137">
-        <f>ETPT_CA_JUR!AA15</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="D16" s="134"/>
-      <c r="E16" s="134"/>
-      <c r="F16" s="134"/>
-      <c r="G16" s="138"/>
-      <c r="H16" s="138"/>
-      <c r="I16" s="138"/>
-      <c r="J16" s="138"/>
-      <c r="K16" s="138"/>
-      <c r="L16" s="138"/>
-      <c r="M16" s="138"/>
-      <c r="N16" s="138"/>
-      <c r="O16" s="138"/>
-      <c r="P16" s="138"/>
-      <c r="Q16" s="138"/>
-      <c r="R16" s="138"/>
-      <c r="S16" s="138"/>
-      <c r="T16" s="138"/>
-      <c r="U16" s="138"/>
-      <c r="V16" s="138"/>
-      <c r="W16" s="138"/>
-      <c r="X16" s="138"/>
-      <c r="Y16" s="138"/>
-      <c r="Z16" s="138"/>
-      <c r="AA16" s="138"/>
-    </row>
-    <row r="17" spans="1:27" ht="24" x14ac:dyDescent="0.2">
-      <c r="A17" s="4"/>
-      <c r="B17"/>
-      <c r="C17"/>
-      <c r="D17" s="135"/>
-      <c r="E17" s="135"/>
-      <c r="F17" s="151" t="s">
-        <v>118</v>
-      </c>
-      <c r="G17" s="140" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!G17),"",IF(ETPT_CA_JUR!G17=0,"",ETPT_CA_JUR!G17)))</f>
-        <v/>
-      </c>
-      <c r="H17" s="139"/>
-      <c r="I17" s="191" t="s">
-        <v>119</v>
-      </c>
-      <c r="J17" s="192"/>
-      <c r="K17" s="192"/>
-      <c r="L17" s="192"/>
-      <c r="M17" s="193"/>
-      <c r="N17" s="140" t="str">
-        <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!N17),"",IF(ETPT_CA_JUR!N17=0,"",ETPT_CA_JUR!N17)))</f>
-        <v/>
-      </c>
-      <c r="O17" s="139"/>
-      <c r="P17" s="139"/>
-      <c r="Q17" s="139"/>
-      <c r="R17" s="139"/>
-      <c r="S17" s="139"/>
-      <c r="T17" s="139"/>
-      <c r="U17" s="139"/>
-      <c r="V17" s="139"/>
-      <c r="W17" s="139"/>
-      <c r="X17" s="139"/>
-      <c r="Y17" s="139"/>
-      <c r="Z17" s="139"/>
-      <c r="AA17" s="139"/>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="I17:M17"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Removed column attachés de justice pole social
</commit_message>
<xml_diff>
--- a/front/src/assets/template4CA.xlsx
+++ b/front/src/assets/template4CA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dinum-327809/Documents/a-just-dev/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05FF5B65-4CCB-0146-B631-893451DE7F7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D538FE4D-8930-3241-8D4E-243D5280FA96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="760" windowWidth="30240" windowHeight="17680" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
+    <workbookView xWindow="20" yWindow="760" windowWidth="30240" windowHeight="17680" activeTab="10" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
   <sheets>
     <sheet name="ACCUEIL" sheetId="33" r:id="rId1"/>
@@ -23,7 +23,7 @@
     <sheet name="Table_Fonctions" sheetId="19" state="hidden" r:id="rId8"/>
     <sheet name="ETPT_CA_ATTJ" sheetId="30" state="hidden" r:id="rId9"/>
     <sheet name="ETPT_CA_ATTJ_DDG" sheetId="25" r:id="rId10"/>
-    <sheet name="ETPT_ATTACHES_JUSTICE" sheetId="41" state="hidden" r:id="rId11"/>
+    <sheet name="ETPT_ATTACHES_JUSTICE" sheetId="41" r:id="rId11"/>
     <sheet name="ETPT_ATTACHES_JUSTICE_DDG" sheetId="42" r:id="rId12"/>
     <sheet name="ETPT_CA_JUR Corresp" sheetId="38" state="hidden" r:id="rId13"/>
     <sheet name="ETPT_ATTACHES_JUSTICE Corresp" sheetId="43" state="hidden" r:id="rId14"/>
@@ -76,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="341">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="603" uniqueCount="341">
   <si>
     <t>#! END_ROW</t>
   </si>
@@ -4829,16 +4829,6 @@
   </cellStyles>
   <dxfs count="23">
     <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill>
           <bgColor theme="9" tint="0.79998168889431442"/>
@@ -5032,6 +5022,16 @@
       <font>
         <color theme="0"/>
       </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -7605,15 +7605,15 @@
   <sheetPr>
     <tabColor rgb="FF0070C0"/>
   </sheetPr>
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:P11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="73.83203125" customWidth="1"/>
-    <col min="4" max="16" width="23.6640625" customWidth="1"/>
-    <col min="17" max="17" width="15.33203125" customWidth="1"/>
+    <col min="4" max="15" width="23.6640625" customWidth="1"/>
+    <col min="16" max="16" width="15.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="74" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" ht="74" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>120</v>
       </c>
@@ -7634,9 +7634,8 @@
       <c r="N1" s="7"/>
       <c r="O1" s="7"/>
       <c r="P1" s="7"/>
-      <c r="Q1" s="7"/>
-    </row>
-    <row r="2" spans="1:17" ht="71" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:16" ht="71" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="108" t="s">
         <v>32</v>
       </c>
@@ -7671,23 +7670,20 @@
         <v>334</v>
       </c>
       <c r="L2" s="99" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="M2" s="99" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="N2" s="99" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="O2" s="99" t="s">
-        <v>339</v>
-      </c>
-      <c r="P2" s="99" t="s">
         <v>335</v>
       </c>
-      <c r="Q2" s="128"/>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="P2" s="128"/>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" s="117" t="s">
         <v>129</v>
       </c>
@@ -7779,12 +7775,12 @@
       </c>
       <c r="J3" s="207"/>
       <c r="K3" s="207"/>
-      <c r="Q3" s="114">
-        <f>_xlfn.AGGREGATE(9,6,D3:P3)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="P3" s="114">
+        <f>_xlfn.AGGREGATE(9,6,D3:O3)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="117" t="s">
         <v>190</v>
       </c>
@@ -7864,12 +7860,12 @@
       </c>
       <c r="J4" s="207"/>
       <c r="K4" s="207"/>
-      <c r="Q4" s="114">
-        <f>_xlfn.AGGREGATE(9,6,D4:P4)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="P4" s="114">
+        <f>_xlfn.AGGREGATE(9,6,D4:O4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" s="117" t="s">
         <v>191</v>
       </c>
@@ -7907,12 +7903,12 @@
       </c>
       <c r="J5" s="207"/>
       <c r="K5" s="207"/>
-      <c r="Q5" s="114">
-        <f>_xlfn.AGGREGATE(9,6,D5:P5)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="P5" s="114">
+        <f>_xlfn.AGGREGATE(9,6,D5:O5)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" s="117" t="s">
         <v>192</v>
       </c>
@@ -8046,12 +8042,12 @@
       </c>
       <c r="J6" s="207"/>
       <c r="K6" s="207"/>
-      <c r="Q6" s="114">
-        <f>_xlfn.AGGREGATE(9,6,D6:P6)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="P6" s="114">
+        <f>_xlfn.AGGREGATE(9,6,D6:O6)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" s="117" t="s">
         <v>193</v>
       </c>
@@ -8089,12 +8085,12 @@
       </c>
       <c r="J7" s="207"/>
       <c r="K7" s="207"/>
-      <c r="Q7" s="114">
-        <f>_xlfn.AGGREGATE(9,6,D7:P7)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="P7" s="114">
+        <f>_xlfn.AGGREGATE(9,6,D7:O7)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" s="117" t="s">
         <v>194</v>
       </c>
@@ -8132,12 +8128,12 @@
       </c>
       <c r="J8" s="207"/>
       <c r="K8" s="207"/>
-      <c r="Q8" s="114">
-        <f>_xlfn.AGGREGATE(9,6,D8:P8)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="P8" s="114">
+        <f>_xlfn.AGGREGATE(9,6,D8:O8)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" s="117" t="s">
         <v>195</v>
       </c>
@@ -8187,12 +8183,12 @@
       </c>
       <c r="J9" s="207"/>
       <c r="K9" s="207"/>
-      <c r="Q9" s="114">
-        <f>_xlfn.AGGREGATE(9,6,D9:P9)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:17" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P9" s="114">
+        <f>_xlfn.AGGREGATE(9,6,D9:O9)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="117" t="s">
         <v>196</v>
       </c>
@@ -8230,12 +8226,12 @@
       </c>
       <c r="J10" s="207"/>
       <c r="K10" s="207"/>
-      <c r="Q10" s="114">
-        <f>_xlfn.AGGREGATE(9,6,D10:P10)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="P10" s="114">
+        <f>_xlfn.AGGREGATE(9,6,D10:O10)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="C11" s="115" t="s">
         <v>37</v>
       </c>
@@ -8244,7 +8240,7 @@
         <v>0</v>
       </c>
       <c r="E11" s="114">
-        <f t="shared" ref="E11:P11" si="0">_xlfn.AGGREGATE(9,6,E3:E10)</f>
+        <f t="shared" ref="E11:O11" si="0">_xlfn.AGGREGATE(9,6,E3:E10)</f>
         <v>0</v>
       </c>
       <c r="F11" s="114">
@@ -8288,11 +8284,7 @@
         <v>0</v>
       </c>
       <c r="P11" s="114">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="Q11" s="114">
-        <f>_xlfn.AGGREGATE(9,6,Q3:Q10)</f>
+        <f>_xlfn.AGGREGATE(9,6,P3:P10)</f>
         <v>0</v>
       </c>
     </row>
@@ -8313,7 +8305,9 @@
   <cols>
     <col min="1" max="1" width="14.1640625" customWidth="1"/>
     <col min="3" max="3" width="59.83203125" customWidth="1"/>
-    <col min="4" max="16" width="20.1640625" customWidth="1"/>
+    <col min="4" max="11" width="20.1640625" customWidth="1"/>
+    <col min="12" max="12" width="20.1640625" hidden="1" customWidth="1"/>
+    <col min="13" max="16" width="20.1640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="87" customHeight="1" x14ac:dyDescent="0.25">
@@ -8422,27 +8416,27 @@
       <c r="J3" s="135"/>
       <c r="K3" s="135"/>
       <c r="L3" s="135" t="str">
+        <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!#REF!),"",IF(ETPT_ATTACHES_JUSTICE!#REF!=0,"",ETPT_ATTACHES_JUSTICE!#REF!))</f>
+        <v/>
+      </c>
+      <c r="M3" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!L3),"",IF(ETPT_ATTACHES_JUSTICE!L3=0,"",ETPT_ATTACHES_JUSTICE!L3))</f>
         <v/>
       </c>
-      <c r="M3" s="135" t="str">
+      <c r="N3" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!M3),"",IF(ETPT_ATTACHES_JUSTICE!M3=0,"",ETPT_ATTACHES_JUSTICE!M3))</f>
         <v/>
       </c>
-      <c r="N3" s="135" t="str">
+      <c r="O3" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!N3),"",IF(ETPT_ATTACHES_JUSTICE!N3=0,"",ETPT_ATTACHES_JUSTICE!N3))</f>
         <v/>
       </c>
-      <c r="O3" s="135" t="str">
+      <c r="P3" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!O3),"",IF(ETPT_ATTACHES_JUSTICE!O3=0,"",ETPT_ATTACHES_JUSTICE!O3))</f>
         <v/>
       </c>
-      <c r="P3" s="135" t="str">
-        <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!P3),"",IF(ETPT_ATTACHES_JUSTICE!P3=0,"",ETPT_ATTACHES_JUSTICE!P3))</f>
-        <v/>
-      </c>
       <c r="Q3" s="141">
-        <f>ETPT_ATTACHES_JUSTICE!Q3</f>
+        <f>ETPT_ATTACHES_JUSTICE!P3</f>
         <v>0</v>
       </c>
     </row>
@@ -8478,27 +8472,27 @@
       <c r="J4" s="135"/>
       <c r="K4" s="135"/>
       <c r="L4" s="135" t="str">
+        <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!#REF!),"",IF(ETPT_ATTACHES_JUSTICE!#REF!=0,"",ETPT_ATTACHES_JUSTICE!#REF!))</f>
+        <v/>
+      </c>
+      <c r="M4" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!L4),"",IF(ETPT_ATTACHES_JUSTICE!L4=0,"",ETPT_ATTACHES_JUSTICE!L4))</f>
         <v/>
       </c>
-      <c r="M4" s="135" t="str">
+      <c r="N4" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!M4),"",IF(ETPT_ATTACHES_JUSTICE!M4=0,"",ETPT_ATTACHES_JUSTICE!M4))</f>
         <v/>
       </c>
-      <c r="N4" s="135" t="str">
+      <c r="O4" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!N4),"",IF(ETPT_ATTACHES_JUSTICE!N4=0,"",ETPT_ATTACHES_JUSTICE!N4))</f>
         <v/>
       </c>
-      <c r="O4" s="135" t="str">
+      <c r="P4" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!O4),"",IF(ETPT_ATTACHES_JUSTICE!O4=0,"",ETPT_ATTACHES_JUSTICE!O4))</f>
         <v/>
       </c>
-      <c r="P4" s="135" t="str">
-        <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!P4),"",IF(ETPT_ATTACHES_JUSTICE!P4=0,"",ETPT_ATTACHES_JUSTICE!P4))</f>
-        <v/>
-      </c>
       <c r="Q4" s="141">
-        <f>ETPT_ATTACHES_JUSTICE!Q4</f>
+        <f>ETPT_ATTACHES_JUSTICE!P4</f>
         <v>0</v>
       </c>
     </row>
@@ -8534,27 +8528,27 @@
       <c r="J5" s="135"/>
       <c r="K5" s="135"/>
       <c r="L5" s="135" t="str">
+        <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!#REF!),"",IF(ETPT_ATTACHES_JUSTICE!#REF!=0,"",ETPT_ATTACHES_JUSTICE!#REF!))</f>
+        <v/>
+      </c>
+      <c r="M5" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!L5),"",IF(ETPT_ATTACHES_JUSTICE!L5=0,"",ETPT_ATTACHES_JUSTICE!L5))</f>
         <v/>
       </c>
-      <c r="M5" s="135" t="str">
+      <c r="N5" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!M5),"",IF(ETPT_ATTACHES_JUSTICE!M5=0,"",ETPT_ATTACHES_JUSTICE!M5))</f>
         <v/>
       </c>
-      <c r="N5" s="135" t="str">
+      <c r="O5" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!N5),"",IF(ETPT_ATTACHES_JUSTICE!N5=0,"",ETPT_ATTACHES_JUSTICE!N5))</f>
         <v/>
       </c>
-      <c r="O5" s="135" t="str">
+      <c r="P5" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!O5),"",IF(ETPT_ATTACHES_JUSTICE!O5=0,"",ETPT_ATTACHES_JUSTICE!O5))</f>
         <v/>
       </c>
-      <c r="P5" s="135" t="str">
-        <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!P5),"",IF(ETPT_ATTACHES_JUSTICE!P5=0,"",ETPT_ATTACHES_JUSTICE!P5))</f>
-        <v/>
-      </c>
       <c r="Q5" s="141">
-        <f>ETPT_ATTACHES_JUSTICE!Q5</f>
+        <f>ETPT_ATTACHES_JUSTICE!P5</f>
         <v>0</v>
       </c>
     </row>
@@ -8590,27 +8584,27 @@
       <c r="J6" s="135"/>
       <c r="K6" s="135"/>
       <c r="L6" s="135" t="str">
+        <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!#REF!),"",IF(ETPT_ATTACHES_JUSTICE!#REF!=0,"",ETPT_ATTACHES_JUSTICE!#REF!))</f>
+        <v/>
+      </c>
+      <c r="M6" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!L6),"",IF(ETPT_ATTACHES_JUSTICE!L6=0,"",ETPT_ATTACHES_JUSTICE!L6))</f>
         <v/>
       </c>
-      <c r="M6" s="135" t="str">
+      <c r="N6" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!M6),"",IF(ETPT_ATTACHES_JUSTICE!M6=0,"",ETPT_ATTACHES_JUSTICE!M6))</f>
         <v/>
       </c>
-      <c r="N6" s="135" t="str">
+      <c r="O6" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!N6),"",IF(ETPT_ATTACHES_JUSTICE!N6=0,"",ETPT_ATTACHES_JUSTICE!N6))</f>
         <v/>
       </c>
-      <c r="O6" s="135" t="str">
+      <c r="P6" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!O6),"",IF(ETPT_ATTACHES_JUSTICE!O6=0,"",ETPT_ATTACHES_JUSTICE!O6))</f>
         <v/>
       </c>
-      <c r="P6" s="135" t="str">
-        <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!P6),"",IF(ETPT_ATTACHES_JUSTICE!P6=0,"",ETPT_ATTACHES_JUSTICE!P6))</f>
-        <v/>
-      </c>
       <c r="Q6" s="141">
-        <f>ETPT_ATTACHES_JUSTICE!Q6</f>
+        <f>ETPT_ATTACHES_JUSTICE!P6</f>
         <v>0</v>
       </c>
     </row>
@@ -8646,27 +8640,27 @@
       <c r="J7" s="135"/>
       <c r="K7" s="135"/>
       <c r="L7" s="135" t="str">
+        <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!#REF!),"",IF(ETPT_ATTACHES_JUSTICE!#REF!=0,"",ETPT_ATTACHES_JUSTICE!#REF!))</f>
+        <v/>
+      </c>
+      <c r="M7" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!L7),"",IF(ETPT_ATTACHES_JUSTICE!L7=0,"",ETPT_ATTACHES_JUSTICE!L7))</f>
         <v/>
       </c>
-      <c r="M7" s="135" t="str">
+      <c r="N7" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!M7),"",IF(ETPT_ATTACHES_JUSTICE!M7=0,"",ETPT_ATTACHES_JUSTICE!M7))</f>
         <v/>
       </c>
-      <c r="N7" s="135" t="str">
+      <c r="O7" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!N7),"",IF(ETPT_ATTACHES_JUSTICE!N7=0,"",ETPT_ATTACHES_JUSTICE!N7))</f>
         <v/>
       </c>
-      <c r="O7" s="135" t="str">
+      <c r="P7" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!O7),"",IF(ETPT_ATTACHES_JUSTICE!O7=0,"",ETPT_ATTACHES_JUSTICE!O7))</f>
         <v/>
       </c>
-      <c r="P7" s="135" t="str">
-        <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!P7),"",IF(ETPT_ATTACHES_JUSTICE!P7=0,"",ETPT_ATTACHES_JUSTICE!P7))</f>
-        <v/>
-      </c>
       <c r="Q7" s="141">
-        <f>ETPT_ATTACHES_JUSTICE!Q7</f>
+        <f>ETPT_ATTACHES_JUSTICE!P7</f>
         <v>0</v>
       </c>
     </row>
@@ -8702,27 +8696,27 @@
       <c r="J8" s="135"/>
       <c r="K8" s="135"/>
       <c r="L8" s="135" t="str">
+        <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!#REF!),"",IF(ETPT_ATTACHES_JUSTICE!#REF!=0,"",ETPT_ATTACHES_JUSTICE!#REF!))</f>
+        <v/>
+      </c>
+      <c r="M8" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!L8),"",IF(ETPT_ATTACHES_JUSTICE!L8=0,"",ETPT_ATTACHES_JUSTICE!L8))</f>
         <v/>
       </c>
-      <c r="M8" s="135" t="str">
+      <c r="N8" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!M8),"",IF(ETPT_ATTACHES_JUSTICE!M8=0,"",ETPT_ATTACHES_JUSTICE!M8))</f>
         <v/>
       </c>
-      <c r="N8" s="135" t="str">
+      <c r="O8" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!N8),"",IF(ETPT_ATTACHES_JUSTICE!N8=0,"",ETPT_ATTACHES_JUSTICE!N8))</f>
         <v/>
       </c>
-      <c r="O8" s="135" t="str">
+      <c r="P8" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!O8),"",IF(ETPT_ATTACHES_JUSTICE!O8=0,"",ETPT_ATTACHES_JUSTICE!O8))</f>
         <v/>
       </c>
-      <c r="P8" s="135" t="str">
-        <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!P8),"",IF(ETPT_ATTACHES_JUSTICE!P8=0,"",ETPT_ATTACHES_JUSTICE!P8))</f>
-        <v/>
-      </c>
       <c r="Q8" s="141">
-        <f>ETPT_ATTACHES_JUSTICE!Q8</f>
+        <f>ETPT_ATTACHES_JUSTICE!P8</f>
         <v>0</v>
       </c>
     </row>
@@ -8758,27 +8752,27 @@
       <c r="J9" s="135"/>
       <c r="K9" s="135"/>
       <c r="L9" s="135" t="str">
+        <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!#REF!),"",IF(ETPT_ATTACHES_JUSTICE!#REF!=0,"",ETPT_ATTACHES_JUSTICE!#REF!))</f>
+        <v/>
+      </c>
+      <c r="M9" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!L9),"",IF(ETPT_ATTACHES_JUSTICE!L9=0,"",ETPT_ATTACHES_JUSTICE!L9))</f>
         <v/>
       </c>
-      <c r="M9" s="135" t="str">
+      <c r="N9" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!M9),"",IF(ETPT_ATTACHES_JUSTICE!M9=0,"",ETPT_ATTACHES_JUSTICE!M9))</f>
         <v/>
       </c>
-      <c r="N9" s="135" t="str">
+      <c r="O9" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!N9),"",IF(ETPT_ATTACHES_JUSTICE!N9=0,"",ETPT_ATTACHES_JUSTICE!N9))</f>
         <v/>
       </c>
-      <c r="O9" s="135" t="str">
+      <c r="P9" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!O9),"",IF(ETPT_ATTACHES_JUSTICE!O9=0,"",ETPT_ATTACHES_JUSTICE!O9))</f>
         <v/>
       </c>
-      <c r="P9" s="135" t="str">
-        <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!P9),"",IF(ETPT_ATTACHES_JUSTICE!P9=0,"",ETPT_ATTACHES_JUSTICE!P9))</f>
-        <v/>
-      </c>
       <c r="Q9" s="141">
-        <f>ETPT_ATTACHES_JUSTICE!Q9</f>
+        <f>ETPT_ATTACHES_JUSTICE!P9</f>
         <v>0</v>
       </c>
     </row>
@@ -8814,27 +8808,27 @@
       <c r="J10" s="135"/>
       <c r="K10" s="135"/>
       <c r="L10" s="135" t="str">
+        <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!#REF!),"",IF(ETPT_ATTACHES_JUSTICE!#REF!=0,"",ETPT_ATTACHES_JUSTICE!#REF!))</f>
+        <v/>
+      </c>
+      <c r="M10" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!L10),"",IF(ETPT_ATTACHES_JUSTICE!L10=0,"",ETPT_ATTACHES_JUSTICE!L10))</f>
         <v/>
       </c>
-      <c r="M10" s="135" t="str">
+      <c r="N10" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!M10),"",IF(ETPT_ATTACHES_JUSTICE!M10=0,"",ETPT_ATTACHES_JUSTICE!M10))</f>
         <v/>
       </c>
-      <c r="N10" s="135" t="str">
+      <c r="O10" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!N10),"",IF(ETPT_ATTACHES_JUSTICE!N10=0,"",ETPT_ATTACHES_JUSTICE!N10))</f>
         <v/>
       </c>
-      <c r="O10" s="135" t="str">
+      <c r="P10" s="135" t="str">
         <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!O10),"",IF(ETPT_ATTACHES_JUSTICE!O10=0,"",ETPT_ATTACHES_JUSTICE!O10))</f>
         <v/>
       </c>
-      <c r="P10" s="135" t="str">
-        <f>IF(ISERROR(ETPT_ATTACHES_JUSTICE!P10),"",IF(ETPT_ATTACHES_JUSTICE!P10=0,"",ETPT_ATTACHES_JUSTICE!P10))</f>
-        <v/>
-      </c>
       <c r="Q10" s="141">
-        <f>ETPT_ATTACHES_JUSTICE!Q10</f>
+        <f>ETPT_ATTACHES_JUSTICE!P10</f>
         <v>0</v>
       </c>
     </row>
@@ -8876,28 +8870,28 @@
         <f>ETPT_ATTACHES_JUSTICE!K11</f>
         <v>0</v>
       </c>
-      <c r="L11" s="141">
+      <c r="L11" s="141" t="e">
+        <f>ETPT_ATTACHES_JUSTICE!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="M11" s="141">
         <f>ETPT_ATTACHES_JUSTICE!L11</f>
         <v>0</v>
       </c>
-      <c r="M11" s="141">
+      <c r="N11" s="141">
         <f>ETPT_ATTACHES_JUSTICE!M11</f>
         <v>0</v>
       </c>
-      <c r="N11" s="141">
+      <c r="O11" s="141">
         <f>ETPT_ATTACHES_JUSTICE!N11</f>
         <v>0</v>
       </c>
-      <c r="O11" s="141">
+      <c r="P11" s="141">
         <f>ETPT_ATTACHES_JUSTICE!O11</f>
         <v>0</v>
       </c>
-      <c r="P11" s="141">
+      <c r="Q11" s="141">
         <f>ETPT_ATTACHES_JUSTICE!P11</f>
-        <v>0</v>
-      </c>
-      <c r="Q11" s="141">
-        <f>ETPT_ATTACHES_JUSTICE!Q11</f>
         <v>0</v>
       </c>
     </row>
@@ -10750,7 +10744,7 @@
     <mergeCell ref="D1:Q1"/>
   </mergeCells>
   <conditionalFormatting sqref="A2:EZ2 A3:FB1048576">
-    <cfRule type="expression" dxfId="0" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="22" priority="2" stopIfTrue="1">
       <formula>OR(AND(OR($R1&lt;&gt;0,$S1&lt;&gt;0,$T1&lt;&gt;0,ISBLANK($P1)),ROW()&gt;2,$A1&lt;&gt;""),LEFT($I1,3)="JA ")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11063,57 +11057,57 @@
     <mergeCell ref="U4:V4"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:F4">
-    <cfRule type="expression" dxfId="22" priority="20">
+    <cfRule type="expression" dxfId="21" priority="20">
       <formula>IF(LEFT($A$3,2)&lt;&gt;"TJ",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:F6 C7:V151">
-    <cfRule type="expression" dxfId="21" priority="22">
+    <cfRule type="expression" dxfId="20" priority="22">
       <formula>AND(ISBLANK($C6)=FALSE,ISBLANK($E6)=TRUE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:F1048576">
-    <cfRule type="expression" dxfId="20" priority="19" stopIfTrue="1">
+    <cfRule type="expression" dxfId="19" priority="19" stopIfTrue="1">
       <formula>AND($D1="7. TOTAL CONTENTIEUX DES MINEURS",OR(ROUND(_xlfn.NUMBERVALUE($L1)-_xlfn.NUMBERVALUE($L2)-_xlfn.NUMBERVALUE($L3),3)&lt;&gt;0,ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3),3)&lt;&gt;0,ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3),3)&lt;&gt;0))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D7:F7">
-    <cfRule type="expression" dxfId="19" priority="17" stopIfTrue="1">
+    <cfRule type="expression" dxfId="18" priority="17" stopIfTrue="1">
       <formula>OR(_xlfn.NUMBERVALUE($L6)&lt;&gt;_xlfn.NUMBERVALUE($L7),_xlfn.NUMBERVALUE($S6)&lt;&gt;_xlfn.NUMBERVALUE($S7),_xlfn.NUMBERVALUE($U6)&lt;&gt;_xlfn.NUMBERVALUE($U7))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:M1048576">
-    <cfRule type="expression" dxfId="18" priority="6">
+    <cfRule type="expression" dxfId="17" priority="6">
       <formula>AND($D1="7. TOTAL CONTENTIEUX DES MINEURS",ROUND(_xlfn.NUMBERVALUE($L1)-_xlfn.NUMBERVALUE($L2)-_xlfn.NUMBERVALUE($L3),3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G7:M7">
-    <cfRule type="expression" dxfId="17" priority="14" stopIfTrue="1">
+    <cfRule type="expression" dxfId="16" priority="14" stopIfTrue="1">
       <formula>_xlfn.NUMBERVALUE($L7)&lt;&gt;_xlfn.NUMBERVALUE($L6)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G6:V6">
-    <cfRule type="expression" dxfId="16" priority="7">
+    <cfRule type="expression" dxfId="15" priority="7">
       <formula>AND(ISBLANK($C6)=FALSE,ISBLANK($E6)=TRUE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1:T1048576">
-    <cfRule type="expression" dxfId="15" priority="5">
+    <cfRule type="expression" dxfId="14" priority="5">
       <formula>AND($D1="7. TOTAL CONTENTIEUX DES MINEURS",ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3),3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N7:T7">
-    <cfRule type="expression" dxfId="14" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="13" priority="11" stopIfTrue="1">
       <formula>_xlfn.NUMBERVALUE($S7)&lt;&gt;_xlfn.NUMBERVALUE($S6)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U1:V1048576">
-    <cfRule type="expression" dxfId="13" priority="4">
+    <cfRule type="expression" dxfId="12" priority="4">
       <formula>AND($D1="7. TOTAL CONTENTIEUX DES MINEURS",ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3),3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U7:V7">
-    <cfRule type="expression" dxfId="12" priority="8">
+    <cfRule type="expression" dxfId="11" priority="8">
       <formula>_xlfn.NUMBERVALUE($U7)&lt;&gt;_xlfn.NUMBERVALUE($U6)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11293,57 +11287,57 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="expression" dxfId="11" priority="11">
+    <cfRule type="expression" dxfId="10" priority="11">
       <formula>AND(OR($I1&lt;&gt;"-",#REF!&lt;&gt;0,#REF!&lt;&gt;0,ISBLANK($M1)),ROW()&gt;2,$A1&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:F2">
-    <cfRule type="expression" dxfId="10" priority="10" stopIfTrue="1">
+    <cfRule type="expression" dxfId="9" priority="10" stopIfTrue="1">
       <formula>$F2="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:N2">
-    <cfRule type="expression" dxfId="9" priority="5">
+    <cfRule type="expression" dxfId="8" priority="5">
       <formula>$F2="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:K2">
-    <cfRule type="expression" dxfId="8" priority="6">
+    <cfRule type="expression" dxfId="7" priority="6">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L2">
-    <cfRule type="expression" dxfId="7" priority="8">
+    <cfRule type="expression" dxfId="6" priority="8">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N2">
-    <cfRule type="expression" dxfId="6" priority="7">
+    <cfRule type="expression" dxfId="5" priority="7">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2">
-    <cfRule type="expression" dxfId="5" priority="9">
+    <cfRule type="expression" dxfId="4" priority="9">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2:V2">
-    <cfRule type="expression" dxfId="4" priority="1">
+    <cfRule type="expression" dxfId="3" priority="1">
       <formula>$F2="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q2:R2">
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="2" priority="4">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S2:T2">
-    <cfRule type="expression" dxfId="2" priority="3">
+    <cfRule type="expression" dxfId="1" priority="3">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="V2">
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="0" priority="2">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
chore: update template4CA.xlsx with dropdown changes
</commit_message>
<xml_diff>
--- a/front/src/assets/template4CA.xlsx
+++ b/front/src/assets/template4CA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dinum-327809/Documents/a-just-dev/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C61E7D98-56A3-8046-80D8-C4C288796DE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ACA34D7-F6DA-E64A-8D56-65E7DB338BC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="760" windowWidth="30220" windowHeight="15320" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
+    <workbookView xWindow="20" yWindow="760" windowWidth="30220" windowHeight="15320" activeTab="11" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
   <sheets>
     <sheet name="ACCUEIL" sheetId="33" r:id="rId1"/>
@@ -76,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="602" uniqueCount="340">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="602" uniqueCount="339">
   <si>
     <t>#! END_ROW</t>
   </si>
@@ -2719,9 +2719,6 @@
   </si>
   <si>
     <t>Contractuels A J Prox et A VIF au Parquet</t>
-  </si>
-  <si>
-    <t>Juristes assistants au parquet</t>
   </si>
   <si>
     <t>A</t>
@@ -5992,10 +5989,10 @@
     <row r="7" spans="1:8" s="26" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="54"/>
       <c r="B7" s="163" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C7" s="63" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D7" s="63" t="s">
         <v>97</v>
@@ -6196,13 +6193,13 @@
         <v>70</v>
       </c>
       <c r="J2" s="99" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="K2" s="99" t="s">
         <v>68</v>
       </c>
       <c r="L2" s="99" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="M2" s="99" t="s">
         <v>110</v>
@@ -6214,13 +6211,13 @@
         <v>80</v>
       </c>
       <c r="P2" s="99" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="Q2" s="99" t="s">
         <v>65</v>
       </c>
       <c r="R2" s="99" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="S2" s="99" t="s">
         <v>112</v>
@@ -6235,10 +6232,10 @@
         <v>63</v>
       </c>
       <c r="W2" s="99" t="s">
+        <v>276</v>
+      </c>
+      <c r="X2" s="99" t="s">
         <v>277</v>
-      </c>
-      <c r="X2" s="99" t="s">
-        <v>278</v>
       </c>
       <c r="Y2" s="99" t="s">
         <v>61</v>
@@ -6255,7 +6252,7 @@
       <c r="B3" s="41"/>
       <c r="C3" s="41"/>
       <c r="D3" s="149" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E3" s="96" t="s">
         <v>59</v>
@@ -7619,7 +7616,7 @@
       <c r="D1" s="6"/>
       <c r="E1" s="7"/>
       <c r="F1" s="7" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="G1" s="7"/>
       <c r="H1" s="7"/>
@@ -7649,34 +7646,34 @@
         <v>257</v>
       </c>
       <c r="F2" s="99" t="s">
+        <v>329</v>
+      </c>
+      <c r="G2" s="99" t="s">
         <v>330</v>
       </c>
-      <c r="G2" s="99" t="s">
+      <c r="H2" s="99" t="s">
         <v>331</v>
       </c>
-      <c r="H2" s="99" t="s">
+      <c r="I2" s="99" t="s">
+        <v>338</v>
+      </c>
+      <c r="J2" s="99" t="s">
         <v>332</v>
       </c>
-      <c r="I2" s="99" t="s">
-        <v>339</v>
-      </c>
-      <c r="J2" s="99" t="s">
+      <c r="K2" s="99" t="s">
         <v>333</v>
       </c>
-      <c r="K2" s="99" t="s">
+      <c r="L2" s="99" t="s">
+        <v>335</v>
+      </c>
+      <c r="M2" s="99" t="s">
+        <v>336</v>
+      </c>
+      <c r="N2" s="99" t="s">
+        <v>337</v>
+      </c>
+      <c r="O2" s="99" t="s">
         <v>334</v>
-      </c>
-      <c r="L2" s="99" t="s">
-        <v>336</v>
-      </c>
-      <c r="M2" s="99" t="s">
-        <v>337</v>
-      </c>
-      <c r="N2" s="99" t="s">
-        <v>338</v>
-      </c>
-      <c r="O2" s="99" t="s">
-        <v>335</v>
       </c>
       <c r="P2" s="128"/>
     </row>
@@ -8342,34 +8339,34 @@
         <v>257</v>
       </c>
       <c r="F2" s="99" t="s">
+        <v>329</v>
+      </c>
+      <c r="G2" s="99" t="s">
         <v>330</v>
       </c>
-      <c r="G2" s="99" t="s">
+      <c r="H2" s="209" t="s">
         <v>331</v>
       </c>
-      <c r="H2" s="209" t="s">
+      <c r="I2" s="99" t="s">
+        <v>338</v>
+      </c>
+      <c r="J2" s="99" t="s">
         <v>332</v>
       </c>
-      <c r="I2" s="99" t="s">
-        <v>258</v>
-      </c>
-      <c r="J2" s="99" t="s">
+      <c r="K2" s="209" t="s">
         <v>333</v>
       </c>
-      <c r="K2" s="209" t="s">
+      <c r="L2" s="209" t="s">
+        <v>335</v>
+      </c>
+      <c r="M2" s="209" t="s">
+        <v>336</v>
+      </c>
+      <c r="N2" s="209" t="s">
+        <v>337</v>
+      </c>
+      <c r="O2" s="99" t="s">
         <v>334</v>
-      </c>
-      <c r="L2" s="209" t="s">
-        <v>336</v>
-      </c>
-      <c r="M2" s="209" t="s">
-        <v>337</v>
-      </c>
-      <c r="N2" s="209" t="s">
-        <v>338</v>
-      </c>
-      <c r="O2" s="99" t="s">
-        <v>335</v>
       </c>
       <c r="P2" s="129" t="s">
         <v>138</v>
@@ -8903,13 +8900,13 @@
         <v>70</v>
       </c>
       <c r="J2" s="72" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="K2" s="72" t="s">
         <v>68</v>
       </c>
       <c r="L2" s="72" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="M2" s="72" t="s">
         <v>110</v>
@@ -8919,13 +8916,13 @@
       </c>
       <c r="O2" s="151"/>
       <c r="P2" s="72" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="Q2" s="72" t="s">
         <v>65</v>
       </c>
       <c r="R2" s="72" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="S2" s="72" t="s">
         <v>112</v>
@@ -8949,7 +8946,7 @@
         <v>58</v>
       </c>
       <c r="G3" s="74" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="H3" s="71" t="e">
         <f>SUMIF(#REF!,#REF!,$G3:G3)</f>
@@ -8999,7 +8996,7 @@
         <v>56</v>
       </c>
       <c r="G4" s="74" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="H4" s="71" t="e">
         <f>SUMIF(#REF!,#REF!,$G4:G4)</f>
@@ -9017,7 +9014,7 @@
       </c>
       <c r="M4" s="154"/>
       <c r="N4" s="74" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="O4" s="71" t="e">
         <f>SUMIF(#REF!,#REF!,$G4:N4)</f>
@@ -9034,7 +9031,7 @@
       </c>
       <c r="S4" s="154"/>
       <c r="T4" s="74" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="U4" s="71" t="e">
         <f>SUMIF(#REF!,#REF!,$G4:T4)</f>
@@ -9381,7 +9378,7 @@
         <v>232</v>
       </c>
       <c r="N12" s="74" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="O12" s="71" t="e">
         <f>SUMIF(#REF!,#REF!,$G12:N12)</f>
@@ -9400,7 +9397,7 @@
         <v>236</v>
       </c>
       <c r="T12" s="74" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="U12" s="71" t="e">
         <f>SUMIF(#REF!,#REF!,$G12:T12)</f>
@@ -9444,7 +9441,7 @@
       <c r="R13" s="159"/>
       <c r="S13" s="159"/>
       <c r="T13" s="74" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="U13" s="71" t="e">
         <f>SUMIF(#REF!,#REF!,$G13:T13)</f>
@@ -9589,13 +9586,13 @@
         <v>118</v>
       </c>
       <c r="G17" s="74" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="M17" s="143" t="s">
         <v>119</v>
       </c>
       <c r="N17" s="74" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
   </sheetData>
@@ -9736,7 +9733,7 @@
         <v>150</v>
       </c>
       <c r="H4" s="108" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="I4" s="108" t="s">
         <v>148</v>
@@ -9745,19 +9742,19 @@
         <v>149</v>
       </c>
       <c r="K4" s="108" t="s">
+        <v>270</v>
+      </c>
+      <c r="L4" s="108" t="s">
         <v>271</v>
       </c>
-      <c r="L4" s="108" t="s">
+      <c r="M4" s="108" t="s">
         <v>272</v>
       </c>
-      <c r="M4" s="108" t="s">
+      <c r="N4" s="108" t="s">
         <v>273</v>
       </c>
-      <c r="N4" s="108" t="s">
+      <c r="O4" s="108" t="s">
         <v>274</v>
-      </c>
-      <c r="O4" s="108" t="s">
-        <v>275</v>
       </c>
       <c r="P4" s="206"/>
     </row>
@@ -10630,7 +10627,7 @@
       <c r="B1" s="130"/>
       <c r="C1" s="130"/>
       <c r="D1" s="192" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E1" s="192"/>
       <c r="F1" s="192"/>
@@ -10727,7 +10724,7 @@
         <v>96</v>
       </c>
       <c r="D1" s="61" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="E1" s="7"/>
       <c r="F1" s="7"/>
@@ -11085,142 +11082,142 @@
   <sheetData>
     <row r="1" spans="1:23" ht="112" x14ac:dyDescent="0.2">
       <c r="A1" s="22" t="s">
+        <v>284</v>
+      </c>
+      <c r="B1" s="22" t="s">
         <v>285</v>
-      </c>
-      <c r="B1" s="22" t="s">
-        <v>286</v>
       </c>
       <c r="C1" s="22" t="s">
         <v>132</v>
       </c>
       <c r="D1" s="22" t="s">
+        <v>286</v>
+      </c>
+      <c r="E1" s="22" t="s">
         <v>287</v>
-      </c>
-      <c r="E1" s="22" t="s">
-        <v>288</v>
       </c>
       <c r="F1" s="22"/>
       <c r="G1" s="166" t="s">
+        <v>288</v>
+      </c>
+      <c r="H1" s="166" t="s">
         <v>289</v>
       </c>
-      <c r="H1" s="166" t="s">
+      <c r="I1" s="167" t="s">
         <v>290</v>
       </c>
-      <c r="I1" s="167" t="s">
+      <c r="J1" s="167" t="s">
         <v>291</v>
       </c>
-      <c r="J1" s="167" t="s">
+      <c r="K1" s="167" t="s">
         <v>292</v>
       </c>
-      <c r="K1" s="167" t="s">
+      <c r="L1" s="168" t="s">
         <v>293</v>
       </c>
-      <c r="L1" s="168" t="s">
+      <c r="M1" s="22" t="s">
         <v>294</v>
       </c>
-      <c r="M1" s="22" t="s">
+      <c r="N1" s="168" t="s">
         <v>295</v>
       </c>
-      <c r="N1" s="168" t="s">
+      <c r="O1" s="169" t="s">
         <v>296</v>
       </c>
-      <c r="O1" s="169" t="s">
+      <c r="P1" s="22" t="s">
         <v>297</v>
       </c>
-      <c r="P1" s="22" t="s">
+      <c r="Q1" s="169" t="s">
         <v>298</v>
       </c>
-      <c r="Q1" s="169" t="s">
+      <c r="R1" s="169" t="s">
         <v>299</v>
       </c>
-      <c r="R1" s="169" t="s">
+      <c r="S1" s="166" t="s">
         <v>300</v>
       </c>
-      <c r="S1" s="166" t="s">
+      <c r="T1" s="166" t="s">
+        <v>326</v>
+      </c>
+      <c r="U1" s="22" t="s">
+        <v>328</v>
+      </c>
+      <c r="V1" s="171" t="s">
+        <v>324</v>
+      </c>
+      <c r="W1" t="s">
         <v>301</v>
-      </c>
-      <c r="T1" s="166" t="s">
-        <v>327</v>
-      </c>
-      <c r="U1" s="22" t="s">
-        <v>329</v>
-      </c>
-      <c r="V1" s="171" t="s">
-        <v>325</v>
-      </c>
-      <c r="W1" t="s">
-        <v>302</v>
       </c>
     </row>
     <row r="2" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="170" t="s">
+        <v>302</v>
+      </c>
+      <c r="B2" s="170" t="s">
         <v>303</v>
       </c>
-      <c r="B2" s="170" t="s">
+      <c r="C2" s="170" t="s">
         <v>304</v>
       </c>
-      <c r="C2" s="170" t="s">
+      <c r="D2" s="170" t="s">
         <v>305</v>
       </c>
-      <c r="D2" s="170" t="s">
+      <c r="E2" s="170" t="s">
         <v>306</v>
       </c>
-      <c r="E2" s="170" t="s">
+      <c r="F2" s="170" t="s">
         <v>307</v>
       </c>
-      <c r="F2" s="170" t="s">
+      <c r="G2" s="170" t="s">
         <v>308</v>
       </c>
-      <c r="G2" s="170" t="s">
+      <c r="H2" s="170" t="s">
         <v>309</v>
       </c>
-      <c r="H2" s="170" t="s">
+      <c r="I2" s="175" t="s">
         <v>310</v>
       </c>
-      <c r="I2" s="175" t="s">
+      <c r="J2" s="175" t="s">
         <v>311</v>
       </c>
-      <c r="J2" s="175" t="s">
+      <c r="K2" s="173" t="s">
         <v>312</v>
       </c>
-      <c r="K2" s="173" t="s">
+      <c r="L2" s="173" t="s">
         <v>313</v>
       </c>
-      <c r="L2" s="173" t="s">
+      <c r="M2" s="174" t="s">
         <v>314</v>
       </c>
-      <c r="M2" s="174" t="s">
+      <c r="N2" s="176" t="s">
         <v>315</v>
       </c>
-      <c r="N2" s="176" t="s">
+      <c r="O2" s="173" t="s">
         <v>316</v>
       </c>
-      <c r="O2" s="173" t="s">
+      <c r="P2" s="173" t="s">
         <v>317</v>
       </c>
-      <c r="P2" s="173" t="s">
+      <c r="Q2" s="173" t="s">
         <v>318</v>
       </c>
-      <c r="Q2" s="173" t="s">
+      <c r="R2" s="173" t="s">
         <v>319</v>
       </c>
-      <c r="R2" s="173" t="s">
+      <c r="S2" s="173" t="s">
         <v>320</v>
       </c>
-      <c r="S2" s="173" t="s">
+      <c r="T2" s="173" t="s">
+        <v>327</v>
+      </c>
+      <c r="U2" s="173" t="s">
         <v>321</v>
       </c>
-      <c r="T2" s="173" t="s">
-        <v>328</v>
-      </c>
-      <c r="U2" s="173" t="s">
+      <c r="V2" s="172" t="s">
         <v>322</v>
       </c>
-      <c r="V2" s="172" t="s">
+      <c r="W2" t="s">
         <v>323</v>
-      </c>
-      <c r="W2" t="s">
-        <v>324</v>
       </c>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.2">
@@ -11826,7 +11823,7 @@
       <c r="B3" s="41"/>
       <c r="C3" s="41"/>
       <c r="D3" s="45" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E3" s="96" t="s">
         <v>59</v>

</xml_diff>

<commit_message>
updated formulas per Andre's file
</commit_message>
<xml_diff>
--- a/front/src/assets/template4CA.xlsx
+++ b/front/src/assets/template4CA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dinum-327809/Documents/a-just-dev/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ACA34D7-F6DA-E64A-8D56-65E7DB338BC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73FD5277-E9E9-2D49-B0BE-7E1882C98C4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="760" windowWidth="30220" windowHeight="15320" activeTab="11" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
+    <workbookView xWindow="80" yWindow="760" windowWidth="30160" windowHeight="16060" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
   <sheets>
     <sheet name="ACCUEIL" sheetId="33" r:id="rId1"/>
@@ -4197,7 +4197,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="210">
+  <cellXfs count="209">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -4713,6 +4713,12 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="169" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
@@ -4801,15 +4807,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="8" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="11" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -5896,11 +5893,11 @@
       <c r="B1" s="48" t="s">
         <v>84</v>
       </c>
-      <c r="C1" s="179" t="s">
+      <c r="C1" s="181" t="s">
         <v>85</v>
       </c>
-      <c r="D1" s="179"/>
-      <c r="E1" s="179"/>
+      <c r="D1" s="181"/>
+      <c r="E1" s="181"/>
       <c r="F1" s="49"/>
       <c r="H1" s="26" t="s">
         <v>0</v>
@@ -5909,11 +5906,11 @@
     <row r="2" spans="1:8" s="53" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="50"/>
       <c r="B2" s="51"/>
-      <c r="C2" s="180" t="s">
+      <c r="C2" s="182" t="s">
         <v>106</v>
       </c>
-      <c r="D2" s="180"/>
-      <c r="E2" s="180"/>
+      <c r="D2" s="182"/>
+      <c r="E2" s="182"/>
       <c r="F2" s="52"/>
       <c r="H2" s="26" t="s">
         <v>0</v>
@@ -5937,10 +5934,10 @@
       <c r="D4" s="58" t="s">
         <v>88</v>
       </c>
-      <c r="E4" s="184" t="s">
+      <c r="E4" s="186" t="s">
         <v>89</v>
       </c>
-      <c r="F4" s="185"/>
+      <c r="F4" s="187"/>
       <c r="G4" s="65"/>
       <c r="H4" s="26" t="s">
         <v>0</v>
@@ -5957,10 +5954,10 @@
       <c r="D5" s="62" t="s">
         <v>92</v>
       </c>
-      <c r="E5" s="186" t="s">
+      <c r="E5" s="188" t="s">
         <v>100</v>
       </c>
-      <c r="F5" s="187"/>
+      <c r="F5" s="189"/>
       <c r="G5" s="64"/>
       <c r="H5" s="26" t="s">
         <v>0</v>
@@ -5977,10 +5974,10 @@
       <c r="D6" s="63" t="s">
         <v>95</v>
       </c>
-      <c r="E6" s="188" t="s">
+      <c r="E6" s="190" t="s">
         <v>101</v>
       </c>
-      <c r="F6" s="189"/>
+      <c r="F6" s="191"/>
       <c r="G6" s="64"/>
       <c r="H6" s="26" t="s">
         <v>0</v>
@@ -5997,10 +5994,10 @@
       <c r="D7" s="63" t="s">
         <v>97</v>
       </c>
-      <c r="E7" s="188" t="s">
+      <c r="E7" s="190" t="s">
         <v>100</v>
       </c>
-      <c r="F7" s="189"/>
+      <c r="F7" s="191"/>
       <c r="G7" s="64"/>
       <c r="H7" s="26" t="s">
         <v>0</v>
@@ -6011,16 +6008,16 @@
       <c r="B8" s="70" t="s">
         <v>255</v>
       </c>
-      <c r="C8" s="177" t="s">
+      <c r="C8" s="179" t="s">
         <v>254</v>
       </c>
-      <c r="D8" s="177" t="s">
+      <c r="D8" s="179" t="s">
         <v>98</v>
       </c>
-      <c r="E8" s="190" t="s">
+      <c r="E8" s="192" t="s">
         <v>102</v>
       </c>
-      <c r="F8" s="191"/>
+      <c r="F8" s="193"/>
       <c r="G8" s="64"/>
       <c r="H8" s="26" t="s">
         <v>0</v>
@@ -6031,10 +6028,10 @@
       <c r="B9" s="164" t="s">
         <v>253</v>
       </c>
-      <c r="C9" s="178"/>
-      <c r="D9" s="178"/>
-      <c r="E9" s="178"/>
-      <c r="F9" s="178"/>
+      <c r="C9" s="180"/>
+      <c r="D9" s="180"/>
+      <c r="E9" s="180"/>
+      <c r="F9" s="180"/>
       <c r="G9" s="64"/>
       <c r="H9" s="26" t="s">
         <v>0</v>
@@ -6054,11 +6051,11 @@
     <row r="11" spans="1:8" s="26" customFormat="1" ht="72" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="54"/>
       <c r="B11" s="66"/>
-      <c r="C11" s="183" t="s">
+      <c r="C11" s="185" t="s">
         <v>99</v>
       </c>
-      <c r="D11" s="183"/>
-      <c r="E11" s="183"/>
+      <c r="D11" s="185"/>
+      <c r="E11" s="185"/>
       <c r="F11" s="67"/>
       <c r="H11" s="26" t="s">
         <v>0</v>
@@ -6072,14 +6069,14 @@
       </c>
     </row>
     <row r="13" spans="1:8" s="26" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="181" t="s">
+      <c r="A13" s="183" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="181"/>
-      <c r="C13" s="181"/>
-      <c r="D13" s="181"/>
-      <c r="E13" s="181"/>
-      <c r="F13" s="182"/>
+      <c r="B13" s="183"/>
+      <c r="C13" s="183"/>
+      <c r="D13" s="183"/>
+      <c r="E13" s="183"/>
+      <c r="F13" s="184"/>
       <c r="H13" s="26" t="s">
         <v>0</v>
       </c>
@@ -7559,13 +7556,13 @@
         <v/>
       </c>
       <c r="H17" s="138"/>
-      <c r="I17" s="201" t="s">
+      <c r="I17" s="203" t="s">
         <v>119</v>
       </c>
-      <c r="J17" s="202"/>
-      <c r="K17" s="202"/>
-      <c r="L17" s="202"/>
-      <c r="M17" s="203"/>
+      <c r="J17" s="204"/>
+      <c r="K17" s="204"/>
+      <c r="L17" s="204"/>
+      <c r="M17" s="205"/>
       <c r="N17" s="139" t="str">
         <f>IF(ISBLANK($D$3),"",IF(ISERROR(ETPT_CA_JUR!N17),"",IF(ETPT_CA_JUR!N17=0,"",ETPT_CA_JUR!N17)))</f>
         <v/>
@@ -7729,48 +7726,48 @@
       <c r="F3" s="112" t="e" cm="1">
         <f t="array" ref="F3">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres"}))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("2. TOTAL CONTENTIEUX COMMERCIAL",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres"}))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3. TOTAL CONTENTIEUX DE LA FAMILLE",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres"}))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("4. TOTAL CONTENTIEUX DE LA PROTECTION",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres"}))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("5. TOTAL CONTENTIEUX CIVIL NON SPÉCIALISÉ",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres"}))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL ATTRIBUTIONS DU PP",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres"}))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. EXTRADITIONS ET MAE",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres"}))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.6. SAISIES ET CONFISCATIONS DES AVOIRS CRIMINELS",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres"}))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.9. AUTRES APPELS JLD",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres"}))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("7.1. ACTIVITÉ CIVILE",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres"}))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))</f>
         <v>#N/A</v>
       </c>
-      <c r="G3" s="208"/>
-      <c r="H3" s="208"/>
+      <c r="G3" s="160"/>
+      <c r="H3" s="160"/>
       <c r="I3" s="112" t="e" cm="1">
         <f t="array" ref="I3">SUM(SUMIFS(
 INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("13.9. FONCTIONNAIRES / JA AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),
-INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres"}))</f>
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))</f>
         <v>#N/A</v>
       </c>
-      <c r="J3" s="207"/>
-      <c r="K3" s="207"/>
+      <c r="J3" s="177"/>
+      <c r="K3" s="177"/>
       <c r="P3" s="114">
-        <f>_xlfn.AGGREGATE(9,6,D3:O3)</f>
+        <f t="shared" ref="P3:P10" si="0">_xlfn.AGGREGATE(9,6,D3:O3)</f>
         <v>0</v>
       </c>
     </row>
@@ -7820,42 +7817,55 @@
       <c r="F4" s="112" t="e" cm="1">
         <f t="array" ref="F4">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. EXTRADITIONS ET MAE",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres"}))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.6. SAISIES ET CONFISCATIONS DES AVOIRS CRIMINELS",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres"}))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.9. AUTRES APPELS JLD",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres"}))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("7.2. ACTIVITÉ PÉNALE",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres"}))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("8. TOTAL CORRECTIONNEL",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres"}))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("9. TOTAL INSTRUCTION ET ENTRAIDE",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres"}))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("10. TOTAL APPLICATION DES PEINES",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres"}))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11. TOTAL CONTENTIEUX CRIMINEL",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres"}))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))</f>
         <v>#N/A</v>
       </c>
-      <c r="G4" s="208"/>
-      <c r="H4" s="208"/>
+      <c r="G4" s="160" t="e" cm="1">
+        <f t="array" ref="G4">SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.1. ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))+
+SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.2 ASSISES JIRS",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H4" s="160" t="e" cm="1">
+        <f t="array" ref="H4">SUM(SUMIFS(
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("11.3. COUR CRIMINELLE DÉPARTEMENTALE",'ETPT Format DDG'!2:2,0)),
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))</f>
+        <v>#N/A</v>
+      </c>
       <c r="I4" s="112" t="e" cm="1">
         <f t="array" ref="I4">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.10. AUTRES FONCTIONNAIRES / JA AFFECTÉS AU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres"}))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))</f>
         <v>#N/A</v>
       </c>
-      <c r="J4" s="207"/>
-      <c r="K4" s="207"/>
+      <c r="J4" s="177"/>
+      <c r="K4" s="177"/>
       <c r="P4" s="114">
-        <f>_xlfn.AGGREGATE(9,6,D4:O4)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -7887,18 +7897,28 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))</f>
         <v>#N/A</v>
       </c>
-      <c r="G5" s="208"/>
-      <c r="H5" s="208"/>
+      <c r="G5" s="160" t="e">
+        <f>SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.8. ACCUEIL DU JUSTICIABLE",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège Assises"))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H5" s="160" t="e">
+        <f>SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.8. ACCUEIL DU JUSTICIABLE",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège CCD"))</f>
+        <v>#N/A</v>
+      </c>
       <c r="I5" s="112" t="e">
         <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.8. ACCUEIL DU JUSTICIABLE",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Parquet"))</f>
         <v>#N/A</v>
       </c>
-      <c r="J5" s="207"/>
-      <c r="K5" s="207"/>
+      <c r="J5" s="177"/>
+      <c r="K5" s="177"/>
       <c r="P5" s="114">
-        <f>_xlfn.AGGREGATE(9,6,D5:O5)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -8002,8 +8022,66 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))</f>
         <v>#N/A</v>
       </c>
-      <c r="G6" s="208"/>
-      <c r="H6" s="208"/>
+      <c r="G6" s="160" t="e">
+        <f>SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.11. ACTIVITÉS EXTÉRIEURES ET PARTENARIATS",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège Assises"))+
+SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.13. COMMUNICATION",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège Assises"))+
+SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.12. ÉQUIPEMENT",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))+
+SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.5. EXPERTISES (SUIVI ET LISTES)",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))+
+SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.2. FORMATIONS SUIVIES",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))+
+SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.6. MÉDIATION / CONCILIATION (SUIVI ET LISTES)",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))+
+SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.14. POLITIQUE ASSOCIATIVE ET AIDE AUX VICTIMES",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))+
+SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.1. SOUTIEN (AUTRES)",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))+
+SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.15. AUTRES ACTIVITÉS NON JURIDICTIONNELLES",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H6" s="160" t="e">
+        <f>SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.11. ACTIVITÉS EXTÉRIEURES ET PARTENARIATS",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège CCD"))+
+SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.13. COMMUNICATION",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège CCD"))+
+SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.12. ÉQUIPEMENT",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))+
+SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.5. EXPERTISES (SUIVI ET LISTES)",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))+
+SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.2. FORMATIONS SUIVIES",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))+
+SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.6. MÉDIATION / CONCILIATION (SUIVI ET LISTES)",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))+
+SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.14. POLITIQUE ASSOCIATIVE ET AIDE AUX VICTIMES",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))+
+SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.1. SOUTIEN (AUTRES)",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))+
+SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.15. AUTRES ACTIVITÉS NON JURIDICTIONNELLES",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))</f>
+        <v>#N/A</v>
+      </c>
       <c r="I6" s="112" t="e">
         <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.11. ACTIVITÉS EXTÉRIEURES ET PARTENARIATS",'ETPT Format DDG'!2:2,0)),
@@ -8034,10 +8112,10 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Parquet"))</f>
         <v>#N/A</v>
       </c>
-      <c r="J6" s="207"/>
-      <c r="K6" s="207"/>
+      <c r="J6" s="177"/>
+      <c r="K6" s="177"/>
       <c r="P6" s="114">
-        <f>_xlfn.AGGREGATE(9,6,D6:O6)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -8069,18 +8147,28 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))</f>
         <v>#N/A</v>
       </c>
-      <c r="G7" s="208"/>
-      <c r="H7" s="208"/>
+      <c r="G7" s="160" t="e">
+        <f>SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.3. FORMATIONS DISPENSÉES",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège Assises"))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H7" s="160" t="e">
+        <f>SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.3. FORMATIONS DISPENSÉES",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège Assises"))</f>
+        <v>#N/A</v>
+      </c>
       <c r="I7" s="112" t="e">
         <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.3. FORMATIONS DISPENSÉES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Parquet"))</f>
         <v>#N/A</v>
       </c>
-      <c r="J7" s="207"/>
-      <c r="K7" s="207"/>
+      <c r="J7" s="177"/>
+      <c r="K7" s="177"/>
       <c r="P7" s="114">
-        <f>_xlfn.AGGREGATE(9,6,D7:O7)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -8112,18 +8200,28 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))</f>
         <v>#N/A</v>
       </c>
-      <c r="G8" s="208"/>
-      <c r="H8" s="208"/>
+      <c r="G8" s="160" t="e">
+        <f>SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.7. ACCÈS AU DROIT ET À LA JUSTICE",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège Assises"))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H8" s="160" t="e">
+        <f>SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.7. ACCÈS AU DROIT ET À LA JUSTICE",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège CCD"))</f>
+        <v>#N/A</v>
+      </c>
       <c r="I8" s="112" t="e">
         <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.7. ACCÈS AU DROIT ET À LA JUSTICE",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Parquet"))</f>
         <v>#N/A</v>
       </c>
-      <c r="J8" s="207"/>
-      <c r="K8" s="207"/>
+      <c r="J8" s="177"/>
+      <c r="K8" s="177"/>
       <c r="P8" s="114">
-        <f>_xlfn.AGGREGATE(9,6,D8:O8)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -8164,8 +8262,24 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))</f>
         <v>#N/A</v>
       </c>
-      <c r="G9" s="208"/>
-      <c r="H9" s="208"/>
+      <c r="G9" s="160" t="e">
+        <f>SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("14. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège Assises"))-
+SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("14.9. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège Assises"))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H9" s="160" t="e">
+        <f>SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("14. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège CCD"))-
+SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("14.9. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège CCD"))</f>
+        <v>#N/A</v>
+      </c>
       <c r="I9" s="112" t="e">
         <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("14. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
@@ -8175,10 +8289,10 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Parquet"))</f>
         <v>#N/A</v>
       </c>
-      <c r="J9" s="207"/>
-      <c r="K9" s="207"/>
+      <c r="J9" s="177"/>
+      <c r="K9" s="177"/>
       <c r="P9" s="114">
-        <f>_xlfn.AGGREGATE(9,6,D9:O9)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -8210,18 +8324,28 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))</f>
         <v>#N/A</v>
       </c>
-      <c r="G10" s="208"/>
-      <c r="H10" s="208"/>
+      <c r="G10" s="160" t="e">
+        <f>SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("14.9. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège Assises"))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H10" s="160" t="e">
+        <f>SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("14.9. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège CCD"))</f>
+        <v>#N/A</v>
+      </c>
       <c r="I10" s="112" t="e">
         <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("14.9. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Parquet"))</f>
         <v>#N/A</v>
       </c>
-      <c r="J10" s="207"/>
-      <c r="K10" s="207"/>
+      <c r="J10" s="177"/>
+      <c r="K10" s="177"/>
       <c r="P10" s="114">
-        <f>_xlfn.AGGREGATE(9,6,D10:O10)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -8234,47 +8358,47 @@
         <v>0</v>
       </c>
       <c r="E11" s="114">
-        <f t="shared" ref="E11:O11" si="0">_xlfn.AGGREGATE(9,6,E3:E10)</f>
+        <f t="shared" ref="E11:O11" si="1">_xlfn.AGGREGATE(9,6,E3:E10)</f>
         <v>0</v>
       </c>
       <c r="F11" s="114">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="G11" s="114">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="H11" s="114">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I11" s="114">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J11" s="114">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K11" s="114">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="L11" s="114">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M11" s="114">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="N11" s="114">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O11" s="114">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="P11" s="114">
@@ -8344,7 +8468,7 @@
       <c r="G2" s="99" t="s">
         <v>330</v>
       </c>
-      <c r="H2" s="209" t="s">
+      <c r="H2" s="178" t="s">
         <v>331</v>
       </c>
       <c r="I2" s="99" t="s">
@@ -8353,16 +8477,16 @@
       <c r="J2" s="99" t="s">
         <v>332</v>
       </c>
-      <c r="K2" s="209" t="s">
+      <c r="K2" s="178" t="s">
         <v>333</v>
       </c>
-      <c r="L2" s="209" t="s">
+      <c r="L2" s="178" t="s">
         <v>335</v>
       </c>
-      <c r="M2" s="209" t="s">
+      <c r="M2" s="178" t="s">
         <v>336</v>
       </c>
-      <c r="N2" s="209" t="s">
+      <c r="N2" s="178" t="s">
         <v>337</v>
       </c>
       <c r="O2" s="99" t="s">
@@ -8851,13 +8975,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="56" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="204" t="s">
+      <c r="A1" s="206" t="s">
         <v>107</v>
       </c>
-      <c r="B1" s="204"/>
-      <c r="C1" s="204"/>
-      <c r="D1" s="204"/>
-      <c r="E1" s="204"/>
+      <c r="B1" s="206"/>
+      <c r="C1" s="206"/>
+      <c r="D1" s="206"/>
+      <c r="E1" s="206"/>
       <c r="F1" s="152"/>
       <c r="G1" s="153"/>
       <c r="H1" s="153"/>
@@ -9613,12 +9737,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="44" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="205" t="s">
+      <c r="A1" s="207" t="s">
         <v>250</v>
       </c>
-      <c r="B1" s="205"/>
-      <c r="C1" s="205"/>
-      <c r="D1" s="205"/>
+      <c r="B1" s="207"/>
+      <c r="C1" s="207"/>
+      <c r="D1" s="207"/>
       <c r="E1" s="119"/>
       <c r="F1" s="118"/>
       <c r="G1" s="118"/>
@@ -9668,7 +9792,7 @@
       <c r="O2" s="105" t="s">
         <v>36</v>
       </c>
-      <c r="P2" s="206" t="s">
+      <c r="P2" s="208" t="s">
         <v>138</v>
       </c>
     </row>
@@ -9708,7 +9832,7 @@
       <c r="O3" s="105" t="s">
         <v>145</v>
       </c>
-      <c r="P3" s="206"/>
+      <c r="P3" s="208"/>
     </row>
     <row r="4" spans="1:16" ht="28" x14ac:dyDescent="0.2">
       <c r="A4" s="106" t="s">
@@ -9756,7 +9880,7 @@
       <c r="O4" s="108" t="s">
         <v>274</v>
       </c>
-      <c r="P4" s="206"/>
+      <c r="P4" s="208"/>
     </row>
     <row r="5" spans="1:16" ht="252" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="109"/>
@@ -10626,22 +10750,22 @@
       <c r="A1" s="130"/>
       <c r="B1" s="130"/>
       <c r="C1" s="130"/>
-      <c r="D1" s="192" t="s">
+      <c r="D1" s="194" t="s">
         <v>278</v>
       </c>
-      <c r="E1" s="192"/>
-      <c r="F1" s="192"/>
-      <c r="G1" s="192"/>
-      <c r="H1" s="192"/>
-      <c r="I1" s="192"/>
-      <c r="J1" s="192"/>
-      <c r="K1" s="192"/>
-      <c r="L1" s="192"/>
-      <c r="M1" s="192"/>
-      <c r="N1" s="192"/>
-      <c r="O1" s="192"/>
-      <c r="P1" s="192"/>
-      <c r="Q1" s="192"/>
+      <c r="E1" s="194"/>
+      <c r="F1" s="194"/>
+      <c r="G1" s="194"/>
+      <c r="H1" s="194"/>
+      <c r="I1" s="194"/>
+      <c r="J1" s="194"/>
+      <c r="K1" s="194"/>
+      <c r="L1" s="194"/>
+      <c r="M1" s="194"/>
+      <c r="N1" s="194"/>
+      <c r="O1" s="194"/>
+      <c r="P1" s="194"/>
+      <c r="Q1" s="194"/>
       <c r="R1" s="131" t="s">
         <v>130</v>
       </c>
@@ -10778,28 +10902,28 @@
       <c r="D4" s="75"/>
       <c r="E4" s="75"/>
       <c r="F4" s="75"/>
-      <c r="G4" s="193" t="s">
+      <c r="G4" s="195" t="s">
         <v>26</v>
       </c>
-      <c r="H4" s="194"/>
-      <c r="I4" s="194"/>
-      <c r="J4" s="194"/>
-      <c r="K4" s="194"/>
-      <c r="L4" s="195"/>
-      <c r="M4" s="196"/>
-      <c r="N4" s="197" t="s">
+      <c r="H4" s="196"/>
+      <c r="I4" s="196"/>
+      <c r="J4" s="196"/>
+      <c r="K4" s="196"/>
+      <c r="L4" s="197"/>
+      <c r="M4" s="198"/>
+      <c r="N4" s="199" t="s">
         <v>27</v>
       </c>
-      <c r="O4" s="195"/>
-      <c r="P4" s="195"/>
-      <c r="Q4" s="195"/>
-      <c r="R4" s="195"/>
-      <c r="S4" s="195"/>
-      <c r="T4" s="198"/>
-      <c r="U4" s="193" t="s">
+      <c r="O4" s="197"/>
+      <c r="P4" s="197"/>
+      <c r="Q4" s="197"/>
+      <c r="R4" s="197"/>
+      <c r="S4" s="197"/>
+      <c r="T4" s="200"/>
+      <c r="U4" s="195" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="196"/>
+      <c r="V4" s="198"/>
       <c r="W4" s="82"/>
       <c r="X4" t="s">
         <v>0</v>
@@ -13105,13 +13229,13 @@
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT A-JUST'!2:2,0)),{"Fonctionnaire CTECH placé ADD";"Fonctionnaire CTECH placé SUB"}))</f>
         <v>#N/A</v>
       </c>
-      <c r="I17" s="199" t="s">
+      <c r="I17" s="201" t="s">
         <v>119</v>
       </c>
-      <c r="J17" s="199"/>
-      <c r="K17" s="199"/>
-      <c r="L17" s="199"/>
-      <c r="M17" s="200"/>
+      <c r="J17" s="201"/>
+      <c r="K17" s="201"/>
+      <c r="L17" s="201"/>
+      <c r="M17" s="202"/>
       <c r="N17" s="73" t="e" cm="1">
         <f t="array" ref="N17">SUM(SUMIFS(
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("14. TOTAL INDISPONIBILITÉ",'ETPT A-JUST'!2:2,0)),

</xml_diff>

<commit_message>
fix: correct CA documentation URLs and update template4CA
</commit_message>
<xml_diff>
--- a/front/src/assets/template4CA.xlsx
+++ b/front/src/assets/template4CA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dinum-327809/Documents/a-just-dev/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73FD5277-E9E9-2D49-B0BE-7E1882C98C4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80E205C7-0047-1C48-9645-15B0FDB2E0BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="80" yWindow="760" windowWidth="30160" windowHeight="16060" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
+    <workbookView xWindow="100" yWindow="780" windowWidth="30160" windowHeight="17660" activeTab="11" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
   <sheets>
     <sheet name="ACCUEIL" sheetId="33" r:id="rId1"/>
@@ -23,7 +23,7 @@
     <sheet name="Table_Fonctions" sheetId="19" state="hidden" r:id="rId8"/>
     <sheet name="ETPT_CA_JUR" sheetId="30" state="hidden" r:id="rId9"/>
     <sheet name="ETPT_CA_JUR_DDG" sheetId="25" r:id="rId10"/>
-    <sheet name="ETPT_CA_ATTJ" sheetId="41" state="hidden" r:id="rId11"/>
+    <sheet name="ETPT_CA_ATTJ" sheetId="41" r:id="rId11"/>
     <sheet name="ETPT_CA_ATTJ_DDG" sheetId="42" r:id="rId12"/>
     <sheet name="ETPT_CA_JUR Corresp" sheetId="38" state="hidden" r:id="rId13"/>
     <sheet name="ETPT_ATTACHES_JUSTICE Corresp" sheetId="43" state="hidden" r:id="rId14"/>
@@ -7719,7 +7719,7 @@
       </c>
       <c r="E3" s="113" t="e" cm="1">
         <f t="array" ref="E3">SUM(SUMIFS(
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.9. FONCTIONNAIRES / JA AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.9. FONCTIONNAIRES / AJ AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"CONT A VIF Parquet";"CONT A VIF Siège";"CONT A JP Parquet";"CONT A JP Siège"}))</f>
         <v>#N/A</v>
       </c>
@@ -7760,7 +7760,7 @@
       <c r="H3" s="160"/>
       <c r="I3" s="112" t="e" cm="1">
         <f t="array" ref="I3">SUM(SUMIFS(
-INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("13.9. FONCTIONNAIRES / JA AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("13.9. FONCTIONNAIRES / AJ AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),
 INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))</f>
         <v>#N/A</v>
       </c>
@@ -8519,8 +8519,14 @@
         <f>IF(ISERROR(ETPT_CA_ATTJ!F3),"",IF(ETPT_CA_ATTJ!F3=0,"",ETPT_CA_ATTJ!F3))</f>
         <v/>
       </c>
-      <c r="G3" s="135"/>
-      <c r="H3" s="135"/>
+      <c r="G3" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!G3),"",IF(ETPT_CA_ATTJ!G3=0,"",ETPT_CA_ATTJ!G3))</f>
+        <v/>
+      </c>
+      <c r="H3" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!H3),"",IF(ETPT_CA_ATTJ!H3=0,"",ETPT_CA_ATTJ!H3))</f>
+        <v/>
+      </c>
       <c r="I3" s="135" t="str">
         <f>IF(ISERROR(ETPT_CA_ATTJ!I3),"",IF(ETPT_CA_ATTJ!I3=0,"",ETPT_CA_ATTJ!I3))</f>
         <v/>
@@ -8571,8 +8577,14 @@
         <f>IF(ISERROR(ETPT_CA_ATTJ!F4),"",IF(ETPT_CA_ATTJ!F4=0,"",ETPT_CA_ATTJ!F4))</f>
         <v/>
       </c>
-      <c r="G4" s="135"/>
-      <c r="H4" s="135"/>
+      <c r="G4" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!G4),"",IF(ETPT_CA_ATTJ!G4=0,"",ETPT_CA_ATTJ!G4))</f>
+        <v/>
+      </c>
+      <c r="H4" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!H4),"",IF(ETPT_CA_ATTJ!H4=0,"",ETPT_CA_ATTJ!H4))</f>
+        <v/>
+      </c>
       <c r="I4" s="135" t="str">
         <f>IF(ISERROR(ETPT_CA_ATTJ!I4),"",IF(ETPT_CA_ATTJ!I4=0,"",ETPT_CA_ATTJ!I4))</f>
         <v/>
@@ -8623,8 +8635,14 @@
         <f>IF(ISERROR(ETPT_CA_ATTJ!F5),"",IF(ETPT_CA_ATTJ!F5=0,"",ETPT_CA_ATTJ!F5))</f>
         <v/>
       </c>
-      <c r="G5" s="135"/>
-      <c r="H5" s="135"/>
+      <c r="G5" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!G5),"",IF(ETPT_CA_ATTJ!G5=0,"",ETPT_CA_ATTJ!G5))</f>
+        <v/>
+      </c>
+      <c r="H5" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!H5),"",IF(ETPT_CA_ATTJ!H5=0,"",ETPT_CA_ATTJ!H5))</f>
+        <v/>
+      </c>
       <c r="I5" s="135" t="str">
         <f>IF(ISERROR(ETPT_CA_ATTJ!I5),"",IF(ETPT_CA_ATTJ!I5=0,"",ETPT_CA_ATTJ!I5))</f>
         <v/>
@@ -8675,8 +8693,14 @@
         <f>IF(ISERROR(ETPT_CA_ATTJ!F6),"",IF(ETPT_CA_ATTJ!F6=0,"",ETPT_CA_ATTJ!F6))</f>
         <v/>
       </c>
-      <c r="G6" s="135"/>
-      <c r="H6" s="135"/>
+      <c r="G6" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!G6),"",IF(ETPT_CA_ATTJ!G6=0,"",ETPT_CA_ATTJ!G6))</f>
+        <v/>
+      </c>
+      <c r="H6" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!H6),"",IF(ETPT_CA_ATTJ!H6=0,"",ETPT_CA_ATTJ!H6))</f>
+        <v/>
+      </c>
       <c r="I6" s="135" t="str">
         <f>IF(ISERROR(ETPT_CA_ATTJ!I6),"",IF(ETPT_CA_ATTJ!I6=0,"",ETPT_CA_ATTJ!I6))</f>
         <v/>
@@ -8727,8 +8751,14 @@
         <f>IF(ISERROR(ETPT_CA_ATTJ!F7),"",IF(ETPT_CA_ATTJ!F7=0,"",ETPT_CA_ATTJ!F7))</f>
         <v/>
       </c>
-      <c r="G7" s="135"/>
-      <c r="H7" s="135"/>
+      <c r="G7" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!G7),"",IF(ETPT_CA_ATTJ!G7=0,"",ETPT_CA_ATTJ!G7))</f>
+        <v/>
+      </c>
+      <c r="H7" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!H7),"",IF(ETPT_CA_ATTJ!H7=0,"",ETPT_CA_ATTJ!H7))</f>
+        <v/>
+      </c>
       <c r="I7" s="135" t="str">
         <f>IF(ISERROR(ETPT_CA_ATTJ!I7),"",IF(ETPT_CA_ATTJ!I7=0,"",ETPT_CA_ATTJ!I7))</f>
         <v/>
@@ -8779,8 +8809,14 @@
         <f>IF(ISERROR(ETPT_CA_ATTJ!F8),"",IF(ETPT_CA_ATTJ!F8=0,"",ETPT_CA_ATTJ!F8))</f>
         <v/>
       </c>
-      <c r="G8" s="135"/>
-      <c r="H8" s="135"/>
+      <c r="G8" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!G8),"",IF(ETPT_CA_ATTJ!G8=0,"",ETPT_CA_ATTJ!G8))</f>
+        <v/>
+      </c>
+      <c r="H8" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!H8),"",IF(ETPT_CA_ATTJ!H8=0,"",ETPT_CA_ATTJ!H8))</f>
+        <v/>
+      </c>
       <c r="I8" s="135" t="str">
         <f>IF(ISERROR(ETPT_CA_ATTJ!I8),"",IF(ETPT_CA_ATTJ!I8=0,"",ETPT_CA_ATTJ!I8))</f>
         <v/>
@@ -8831,8 +8867,14 @@
         <f>IF(ISERROR(ETPT_CA_ATTJ!F9),"",IF(ETPT_CA_ATTJ!F9=0,"",ETPT_CA_ATTJ!F9))</f>
         <v/>
       </c>
-      <c r="G9" s="135"/>
-      <c r="H9" s="135"/>
+      <c r="G9" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!G9),"",IF(ETPT_CA_ATTJ!G9=0,"",ETPT_CA_ATTJ!G9))</f>
+        <v/>
+      </c>
+      <c r="H9" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!H9),"",IF(ETPT_CA_ATTJ!H9=0,"",ETPT_CA_ATTJ!H9))</f>
+        <v/>
+      </c>
       <c r="I9" s="135" t="str">
         <f>IF(ISERROR(ETPT_CA_ATTJ!I9),"",IF(ETPT_CA_ATTJ!I9=0,"",ETPT_CA_ATTJ!I9))</f>
         <v/>
@@ -8883,8 +8925,14 @@
         <f>IF(ISERROR(ETPT_CA_ATTJ!F10),"",IF(ETPT_CA_ATTJ!F10=0,"",ETPT_CA_ATTJ!F10))</f>
         <v/>
       </c>
-      <c r="G10" s="135"/>
-      <c r="H10" s="135"/>
+      <c r="G10" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!G10),"",IF(ETPT_CA_ATTJ!G10=0,"",ETPT_CA_ATTJ!G10))</f>
+        <v/>
+      </c>
+      <c r="H10" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!H10),"",IF(ETPT_CA_ATTJ!H10=0,"",ETPT_CA_ATTJ!H10))</f>
+        <v/>
+      </c>
       <c r="I10" s="135" t="str">
         <f>IF(ISERROR(ETPT_CA_ATTJ!I10),"",IF(ETPT_CA_ATTJ!I10=0,"",ETPT_CA_ATTJ!I10))</f>
         <v/>
@@ -8930,8 +8978,14 @@
         <f>ETPT_CA_ATTJ!F11</f>
         <v>0</v>
       </c>
-      <c r="G11" s="141"/>
-      <c r="H11" s="141"/>
+      <c r="G11" s="141">
+        <f>ETPT_CA_ATTJ!G11</f>
+        <v>0</v>
+      </c>
+      <c r="H11" s="141">
+        <f>ETPT_CA_ATTJ!H11</f>
+        <v>0</v>
+      </c>
       <c r="I11" s="141">
         <f>ETPT_CA_ATTJ!I11</f>
         <v>0</v>

</xml_diff>

<commit_message>
fix: correct CA documentation URLs and update template4CA (#469)
Co-authored-by: Joseph Dureau <dinum-327809@MacBook-Pro-de-DINUM-327809.local>
</commit_message>
<xml_diff>
--- a/front/src/assets/template4CA.xlsx
+++ b/front/src/assets/template4CA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dinum-327809/Documents/a-just-dev/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73FD5277-E9E9-2D49-B0BE-7E1882C98C4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80E205C7-0047-1C48-9645-15B0FDB2E0BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="80" yWindow="760" windowWidth="30160" windowHeight="16060" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
+    <workbookView xWindow="100" yWindow="780" windowWidth="30160" windowHeight="17660" activeTab="11" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
   <sheets>
     <sheet name="ACCUEIL" sheetId="33" r:id="rId1"/>
@@ -23,7 +23,7 @@
     <sheet name="Table_Fonctions" sheetId="19" state="hidden" r:id="rId8"/>
     <sheet name="ETPT_CA_JUR" sheetId="30" state="hidden" r:id="rId9"/>
     <sheet name="ETPT_CA_JUR_DDG" sheetId="25" r:id="rId10"/>
-    <sheet name="ETPT_CA_ATTJ" sheetId="41" state="hidden" r:id="rId11"/>
+    <sheet name="ETPT_CA_ATTJ" sheetId="41" r:id="rId11"/>
     <sheet name="ETPT_CA_ATTJ_DDG" sheetId="42" r:id="rId12"/>
     <sheet name="ETPT_CA_JUR Corresp" sheetId="38" state="hidden" r:id="rId13"/>
     <sheet name="ETPT_ATTACHES_JUSTICE Corresp" sheetId="43" state="hidden" r:id="rId14"/>
@@ -7719,7 +7719,7 @@
       </c>
       <c r="E3" s="113" t="e" cm="1">
         <f t="array" ref="E3">SUM(SUMIFS(
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.9. FONCTIONNAIRES / JA AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.9. FONCTIONNAIRES / AJ AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"CONT A VIF Parquet";"CONT A VIF Siège";"CONT A JP Parquet";"CONT A JP Siège"}))</f>
         <v>#N/A</v>
       </c>
@@ -7760,7 +7760,7 @@
       <c r="H3" s="160"/>
       <c r="I3" s="112" t="e" cm="1">
         <f t="array" ref="I3">SUM(SUMIFS(
-INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("13.9. FONCTIONNAIRES / JA AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("13.9. FONCTIONNAIRES / AJ AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),
 INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))</f>
         <v>#N/A</v>
       </c>
@@ -8519,8 +8519,14 @@
         <f>IF(ISERROR(ETPT_CA_ATTJ!F3),"",IF(ETPT_CA_ATTJ!F3=0,"",ETPT_CA_ATTJ!F3))</f>
         <v/>
       </c>
-      <c r="G3" s="135"/>
-      <c r="H3" s="135"/>
+      <c r="G3" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!G3),"",IF(ETPT_CA_ATTJ!G3=0,"",ETPT_CA_ATTJ!G3))</f>
+        <v/>
+      </c>
+      <c r="H3" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!H3),"",IF(ETPT_CA_ATTJ!H3=0,"",ETPT_CA_ATTJ!H3))</f>
+        <v/>
+      </c>
       <c r="I3" s="135" t="str">
         <f>IF(ISERROR(ETPT_CA_ATTJ!I3),"",IF(ETPT_CA_ATTJ!I3=0,"",ETPT_CA_ATTJ!I3))</f>
         <v/>
@@ -8571,8 +8577,14 @@
         <f>IF(ISERROR(ETPT_CA_ATTJ!F4),"",IF(ETPT_CA_ATTJ!F4=0,"",ETPT_CA_ATTJ!F4))</f>
         <v/>
       </c>
-      <c r="G4" s="135"/>
-      <c r="H4" s="135"/>
+      <c r="G4" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!G4),"",IF(ETPT_CA_ATTJ!G4=0,"",ETPT_CA_ATTJ!G4))</f>
+        <v/>
+      </c>
+      <c r="H4" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!H4),"",IF(ETPT_CA_ATTJ!H4=0,"",ETPT_CA_ATTJ!H4))</f>
+        <v/>
+      </c>
       <c r="I4" s="135" t="str">
         <f>IF(ISERROR(ETPT_CA_ATTJ!I4),"",IF(ETPT_CA_ATTJ!I4=0,"",ETPT_CA_ATTJ!I4))</f>
         <v/>
@@ -8623,8 +8635,14 @@
         <f>IF(ISERROR(ETPT_CA_ATTJ!F5),"",IF(ETPT_CA_ATTJ!F5=0,"",ETPT_CA_ATTJ!F5))</f>
         <v/>
       </c>
-      <c r="G5" s="135"/>
-      <c r="H5" s="135"/>
+      <c r="G5" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!G5),"",IF(ETPT_CA_ATTJ!G5=0,"",ETPT_CA_ATTJ!G5))</f>
+        <v/>
+      </c>
+      <c r="H5" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!H5),"",IF(ETPT_CA_ATTJ!H5=0,"",ETPT_CA_ATTJ!H5))</f>
+        <v/>
+      </c>
       <c r="I5" s="135" t="str">
         <f>IF(ISERROR(ETPT_CA_ATTJ!I5),"",IF(ETPT_CA_ATTJ!I5=0,"",ETPT_CA_ATTJ!I5))</f>
         <v/>
@@ -8675,8 +8693,14 @@
         <f>IF(ISERROR(ETPT_CA_ATTJ!F6),"",IF(ETPT_CA_ATTJ!F6=0,"",ETPT_CA_ATTJ!F6))</f>
         <v/>
       </c>
-      <c r="G6" s="135"/>
-      <c r="H6" s="135"/>
+      <c r="G6" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!G6),"",IF(ETPT_CA_ATTJ!G6=0,"",ETPT_CA_ATTJ!G6))</f>
+        <v/>
+      </c>
+      <c r="H6" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!H6),"",IF(ETPT_CA_ATTJ!H6=0,"",ETPT_CA_ATTJ!H6))</f>
+        <v/>
+      </c>
       <c r="I6" s="135" t="str">
         <f>IF(ISERROR(ETPT_CA_ATTJ!I6),"",IF(ETPT_CA_ATTJ!I6=0,"",ETPT_CA_ATTJ!I6))</f>
         <v/>
@@ -8727,8 +8751,14 @@
         <f>IF(ISERROR(ETPT_CA_ATTJ!F7),"",IF(ETPT_CA_ATTJ!F7=0,"",ETPT_CA_ATTJ!F7))</f>
         <v/>
       </c>
-      <c r="G7" s="135"/>
-      <c r="H7" s="135"/>
+      <c r="G7" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!G7),"",IF(ETPT_CA_ATTJ!G7=0,"",ETPT_CA_ATTJ!G7))</f>
+        <v/>
+      </c>
+      <c r="H7" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!H7),"",IF(ETPT_CA_ATTJ!H7=0,"",ETPT_CA_ATTJ!H7))</f>
+        <v/>
+      </c>
       <c r="I7" s="135" t="str">
         <f>IF(ISERROR(ETPT_CA_ATTJ!I7),"",IF(ETPT_CA_ATTJ!I7=0,"",ETPT_CA_ATTJ!I7))</f>
         <v/>
@@ -8779,8 +8809,14 @@
         <f>IF(ISERROR(ETPT_CA_ATTJ!F8),"",IF(ETPT_CA_ATTJ!F8=0,"",ETPT_CA_ATTJ!F8))</f>
         <v/>
       </c>
-      <c r="G8" s="135"/>
-      <c r="H8" s="135"/>
+      <c r="G8" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!G8),"",IF(ETPT_CA_ATTJ!G8=0,"",ETPT_CA_ATTJ!G8))</f>
+        <v/>
+      </c>
+      <c r="H8" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!H8),"",IF(ETPT_CA_ATTJ!H8=0,"",ETPT_CA_ATTJ!H8))</f>
+        <v/>
+      </c>
       <c r="I8" s="135" t="str">
         <f>IF(ISERROR(ETPT_CA_ATTJ!I8),"",IF(ETPT_CA_ATTJ!I8=0,"",ETPT_CA_ATTJ!I8))</f>
         <v/>
@@ -8831,8 +8867,14 @@
         <f>IF(ISERROR(ETPT_CA_ATTJ!F9),"",IF(ETPT_CA_ATTJ!F9=0,"",ETPT_CA_ATTJ!F9))</f>
         <v/>
       </c>
-      <c r="G9" s="135"/>
-      <c r="H9" s="135"/>
+      <c r="G9" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!G9),"",IF(ETPT_CA_ATTJ!G9=0,"",ETPT_CA_ATTJ!G9))</f>
+        <v/>
+      </c>
+      <c r="H9" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!H9),"",IF(ETPT_CA_ATTJ!H9=0,"",ETPT_CA_ATTJ!H9))</f>
+        <v/>
+      </c>
       <c r="I9" s="135" t="str">
         <f>IF(ISERROR(ETPT_CA_ATTJ!I9),"",IF(ETPT_CA_ATTJ!I9=0,"",ETPT_CA_ATTJ!I9))</f>
         <v/>
@@ -8883,8 +8925,14 @@
         <f>IF(ISERROR(ETPT_CA_ATTJ!F10),"",IF(ETPT_CA_ATTJ!F10=0,"",ETPT_CA_ATTJ!F10))</f>
         <v/>
       </c>
-      <c r="G10" s="135"/>
-      <c r="H10" s="135"/>
+      <c r="G10" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!G10),"",IF(ETPT_CA_ATTJ!G10=0,"",ETPT_CA_ATTJ!G10))</f>
+        <v/>
+      </c>
+      <c r="H10" s="135" t="str">
+        <f>IF(ISERROR(ETPT_CA_ATTJ!H10),"",IF(ETPT_CA_ATTJ!H10=0,"",ETPT_CA_ATTJ!H10))</f>
+        <v/>
+      </c>
       <c r="I10" s="135" t="str">
         <f>IF(ISERROR(ETPT_CA_ATTJ!I10),"",IF(ETPT_CA_ATTJ!I10=0,"",ETPT_CA_ATTJ!I10))</f>
         <v/>
@@ -8930,8 +8978,14 @@
         <f>ETPT_CA_ATTJ!F11</f>
         <v>0</v>
       </c>
-      <c r="G11" s="141"/>
-      <c r="H11" s="141"/>
+      <c r="G11" s="141">
+        <f>ETPT_CA_ATTJ!G11</f>
+        <v>0</v>
+      </c>
+      <c r="H11" s="141">
+        <f>ETPT_CA_ATTJ!H11</f>
+        <v>0</v>
+      </c>
       <c r="I11" s="141">
         <f>ETPT_CA_ATTJ!I11</f>
         <v>0</v>

</xml_diff>

<commit_message>
Feat/extracteur ca v3 (#471)
* fix: correct CA documentation URLs in async polling path

* fix: correct CA documentation URLs and update template4CA

---------

Co-authored-by: Joseph Dureau <dinum-327809@MacBook-Pro-de-DINUM-327809.local>
</commit_message>
<xml_diff>
--- a/front/src/assets/template4CA.xlsx
+++ b/front/src/assets/template4CA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dinum-327809/Documents/a-just-dev/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80E205C7-0047-1C48-9645-15B0FDB2E0BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C06C8C46-6865-3447-AD79-D84B63EE4F8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="100" yWindow="780" windowWidth="30160" windowHeight="17660" activeTab="11" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
+    <workbookView xWindow="100" yWindow="780" windowWidth="30160" windowHeight="17660" activeTab="10" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
   <sheets>
     <sheet name="ACCUEIL" sheetId="33" r:id="rId1"/>
@@ -7810,7 +7810,7 @@
       </c>
       <c r="E4" s="113" t="e" cm="1">
         <f t="array" ref="E4">SUM(SUMIFS(
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.10. AUTRES FONCTIONNAIRES / JA AFFECTÉS AU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.10. AUTRES FONCTIONNAIRES / AJ AFFECTÉS AU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"CONT A VIF Parquet";"CONT A VIF Siège";"CONT A JP Parquet";"CONT A JP Siège"}))</f>
         <v>#N/A</v>
       </c>
@@ -7858,7 +7858,7 @@
       </c>
       <c r="I4" s="112" t="e" cm="1">
         <f t="array" ref="I4">SUM(SUMIFS(
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.10. AUTRES FONCTIONNAIRES / JA AFFECTÉS AU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.10. AUTRES FONCTIONNAIRES / AJ AFFECTÉS AU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))</f>
         <v>#N/A</v>
       </c>

</xml_diff>

<commit_message>
chore: update template4CA (#472)
Co-authored-by: Joseph Dureau <dinum-327809@MacBook-Pro-de-DINUM-327809.local>
</commit_message>
<xml_diff>
--- a/front/src/assets/template4CA.xlsx
+++ b/front/src/assets/template4CA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dinum-327809/Documents/a-just-dev/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C06C8C46-6865-3447-AD79-D84B63EE4F8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A10A64C9-D6CD-F949-89B0-13F353138135}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="100" yWindow="780" windowWidth="30160" windowHeight="17660" activeTab="10" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
+    <workbookView xWindow="100" yWindow="780" windowWidth="30160" windowHeight="17660" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
   <sheets>
     <sheet name="ACCUEIL" sheetId="33" r:id="rId1"/>
@@ -23,7 +23,7 @@
     <sheet name="Table_Fonctions" sheetId="19" state="hidden" r:id="rId8"/>
     <sheet name="ETPT_CA_JUR" sheetId="30" state="hidden" r:id="rId9"/>
     <sheet name="ETPT_CA_JUR_DDG" sheetId="25" r:id="rId10"/>
-    <sheet name="ETPT_CA_ATTJ" sheetId="41" r:id="rId11"/>
+    <sheet name="ETPT_CA_ATTJ" sheetId="41" state="hidden" r:id="rId11"/>
     <sheet name="ETPT_CA_ATTJ_DDG" sheetId="42" r:id="rId12"/>
     <sheet name="ETPT_CA_JUR Corresp" sheetId="38" state="hidden" r:id="rId13"/>
     <sheet name="ETPT_ATTACHES_JUSTICE Corresp" sheetId="43" state="hidden" r:id="rId14"/>

</xml_diff>

<commit_message>
chore: update template4CA (#481)
Co-authored-by: Joseph Dureau <dinum-327809@MacBook-Pro-de-DINUM-327809.local>
</commit_message>
<xml_diff>
--- a/front/src/assets/template4CA.xlsx
+++ b/front/src/assets/template4CA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dinum-327809/Documents/a-just-dev/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80B326FC-4D0B-9640-8AAC-39F5ED11396D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FA17441-E878-754A-8EE7-0EAC73BF83A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="100" yWindow="780" windowWidth="30160" windowHeight="17660" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -8031,25 +8031,25 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège Assises"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.12. ÉQUIPEMENT",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège Assises"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.5. EXPERTISES (SUIVI ET LISTES)",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège Assises"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.2. FORMATIONS SUIVIES",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège Assises"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.6. MÉDIATION / CONCILIATION (SUIVI ET LISTES)",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège Assises"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.14. POLITIQUE ASSOCIATIVE ET AIDE AUX VICTIMES",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège Assises"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.1. SOUTIEN (AUTRES)",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège Assises"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.15. AUTRES ACTIVITÉS NON JURIDICTIONNELLES",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège Assises"))</f>
         <v>#N/A</v>
       </c>
       <c r="H6" s="160" t="e">
@@ -8061,25 +8061,25 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège CCD"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.12. ÉQUIPEMENT",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège CCD"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.5. EXPERTISES (SUIVI ET LISTES)",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège CCD"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.2. FORMATIONS SUIVIES",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège CCD"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.6. MÉDIATION / CONCILIATION (SUIVI ET LISTES)",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège CCD"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.14. POLITIQUE ASSOCIATIVE ET AIDE AUX VICTIMES",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège CCD"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.1. SOUTIEN (AUTRES)",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège CCD"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.15. AUTRES ACTIVITÉS NON JURIDICTIONNELLES",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres"))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège CCD"))</f>
         <v>#N/A</v>
       </c>
       <c r="I6" s="112" t="e">
@@ -8156,7 +8156,7 @@
       <c r="H7" s="160" t="e">
         <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.3. FORMATIONS DISPENSÉES",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège Assises"))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège CCD"))</f>
         <v>#N/A</v>
       </c>
       <c r="I7" s="112" t="e">

</xml_diff>

<commit_message>
fix: correct recodedFunction for Assises and CCD with accent on Siège
</commit_message>
<xml_diff>
--- a/front/src/assets/template4CA.xlsx
+++ b/front/src/assets/template4CA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dinum-327809/Documents/a-just-dev/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FA17441-E878-754A-8EE7-0EAC73BF83A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E1F4294-F08B-3C45-805F-C79E554A6C9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="100" yWindow="780" windowWidth="30160" windowHeight="17660" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -7816,29 +7816,49 @@
       </c>
       <c r="F4" s="112" t="e" cm="1">
         <f t="array" ref="F4">SUM(SUMIFS(
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. EXTRADITIONS ET MAE",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))+
-SUM(SUMIFS(
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.6. SAISIES ET CONFISCATIONS DES AVOIRS CRIMINELS",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))+
-SUM(SUMIFS(
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.9. AUTRES APPELS JLD",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))+
-SUM(SUMIFS(
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("7.2. ACTIVITÉ PÉNALE",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))+
-SUM(SUMIFS(
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("8. TOTAL CORRECTIONNEL",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))+
-SUM(SUMIFS(
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("9. TOTAL INSTRUCTION ET ENTRAIDE",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))+
-SUM(SUMIFS(
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("10. TOTAL APPLICATION DES PEINES",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))+
-SUM(SUMIFS(
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11. TOTAL CONTENTIEUX CRIMINEL",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))</f>
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. EXTRADITIONS ET MAE",'ETPT Format DDG'!2:2,0)),
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),
+{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))
++SUM(SUMIFS(
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("12.6. SAISIES ET CONFISCATIONS DES AVOIRS CRIMINELS",'ETPT Format DDG'!2:2,0)),
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),
+{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))
++SUM(SUMIFS(
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("12.9. AUTRES APPELS JLD",'ETPT Format DDG'!2:2,0)),
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),
+{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))
++SUM(SUMIFS(
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("7.2. ACTIVITÉ PÉNALE",'ETPT Format DDG'!2:2,0)),
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),
+{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))
++SUM(SUMIFS(
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("8. TOTAL CORRECTIONNEL",'ETPT Format DDG'!2:2,0)),
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),
+{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))
++SUM(SUMIFS(
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("9. TOTAL INSTRUCTION ET ENTRAIDE",'ETPT Format DDG'!2:2,0)),
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),
+{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))
++SUM(SUMIFS(
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("10. TOTAL APPLICATION DES PEINES",'ETPT Format DDG'!2:2,0)),
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),
+{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))
++SUM(SUMIFS(
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("11. TOTAL CONTENTIEUX CRIMINEL",'ETPT Format DDG'!2:2,0)),
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),
+{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))
+-SUM(SUMIFS(
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("11.1. ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),
+{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))
+-SUM(SUMIFS(
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("11.2 ASSISES JIRS",'ETPT Format DDG'!2:2,0)),
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),
+{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))
+-SUM(SUMIFS(
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("11.3. COUR CRIMINELLE DÉPARTEMENTALE",'ETPT Format DDG'!2:2,0)),
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),
+{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))</f>
         <v>#N/A</v>
       </c>
       <c r="G4" s="160" t="e" cm="1">

</xml_diff>

<commit_message>
fix: correct recodedFunction for Assises and CCD with accent on Siège (#482)
Co-authored-by: Joseph Dureau <dinum-327809@MacBook-Pro-de-DINUM-327809.local>
</commit_message>
<xml_diff>
--- a/front/src/assets/template4CA.xlsx
+++ b/front/src/assets/template4CA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dinum-327809/Documents/a-just-dev/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FA17441-E878-754A-8EE7-0EAC73BF83A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E1F4294-F08B-3C45-805F-C79E554A6C9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="100" yWindow="780" windowWidth="30160" windowHeight="17660" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -7816,29 +7816,49 @@
       </c>
       <c r="F4" s="112" t="e" cm="1">
         <f t="array" ref="F4">SUM(SUMIFS(
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. EXTRADITIONS ET MAE",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))+
-SUM(SUMIFS(
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.6. SAISIES ET CONFISCATIONS DES AVOIRS CRIMINELS",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))+
-SUM(SUMIFS(
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.9. AUTRES APPELS JLD",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))+
-SUM(SUMIFS(
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("7.2. ACTIVITÉ PÉNALE",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))+
-SUM(SUMIFS(
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("8. TOTAL CORRECTIONNEL",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))+
-SUM(SUMIFS(
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("9. TOTAL INSTRUCTION ET ENTRAIDE",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))+
-SUM(SUMIFS(
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("10. TOTAL APPLICATION DES PEINES",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))+
-SUM(SUMIFS(
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11. TOTAL CONTENTIEUX CRIMINEL",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))</f>
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. EXTRADITIONS ET MAE",'ETPT Format DDG'!2:2,0)),
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),
+{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))
++SUM(SUMIFS(
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("12.6. SAISIES ET CONFISCATIONS DES AVOIRS CRIMINELS",'ETPT Format DDG'!2:2,0)),
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),
+{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))
++SUM(SUMIFS(
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("12.9. AUTRES APPELS JLD",'ETPT Format DDG'!2:2,0)),
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),
+{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))
++SUM(SUMIFS(
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("7.2. ACTIVITÉ PÉNALE",'ETPT Format DDG'!2:2,0)),
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),
+{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))
++SUM(SUMIFS(
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("8. TOTAL CORRECTIONNEL",'ETPT Format DDG'!2:2,0)),
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),
+{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))
++SUM(SUMIFS(
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("9. TOTAL INSTRUCTION ET ENTRAIDE",'ETPT Format DDG'!2:2,0)),
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),
+{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))
++SUM(SUMIFS(
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("10. TOTAL APPLICATION DES PEINES",'ETPT Format DDG'!2:2,0)),
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),
+{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))
++SUM(SUMIFS(
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("11. TOTAL CONTENTIEUX CRIMINEL",'ETPT Format DDG'!2:2,0)),
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),
+{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))
+-SUM(SUMIFS(
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("11.1. ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),
+{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))
+-SUM(SUMIFS(
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("11.2 ASSISES JIRS",'ETPT Format DDG'!2:2,0)),
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),
+{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))
+-SUM(SUMIFS(
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("11.3. COUR CRIMINELLE DÉPARTEMENTALE",'ETPT Format DDG'!2:2,0)),
+INDEX('ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),
+{"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siège Assises";"JA/AttJ Siège CCD"}))</f>
         <v>#N/A</v>
       </c>
       <c r="G4" s="160" t="e" cm="1">

</xml_diff>

<commit_message>
chore: update template4CA (#484)
Co-authored-by: Joseph Dureau <dinum-327809@mac-1.home>
</commit_message>
<xml_diff>
--- a/front/src/assets/template4CA.xlsx
+++ b/front/src/assets/template4CA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dinum-327809/Documents/a-just-dev/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E1F4294-F08B-3C45-805F-C79E554A6C9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2C3AC54-7268-204E-93BC-32BB714E9DEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="100" yWindow="780" windowWidth="30160" windowHeight="17660" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
+    <workbookView xWindow="100" yWindow="780" windowWidth="30160" windowHeight="17660" activeTab="8" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
   <sheets>
     <sheet name="ACCUEIL" sheetId="33" r:id="rId1"/>
@@ -21,7 +21,7 @@
     <sheet name="codage tribunal" sheetId="12" state="hidden" r:id="rId6"/>
     <sheet name="Juridictions" sheetId="17" state="hidden" r:id="rId7"/>
     <sheet name="Table_Fonctions" sheetId="19" state="hidden" r:id="rId8"/>
-    <sheet name="ETPT_CA_JUR" sheetId="30" state="hidden" r:id="rId9"/>
+    <sheet name="ETPT_CA_JUR" sheetId="30" r:id="rId9"/>
     <sheet name="ETPT_CA_JUR_DDG" sheetId="25" r:id="rId10"/>
     <sheet name="ETPT_CA_ATTJ" sheetId="41" state="hidden" r:id="rId11"/>
     <sheet name="ETPT_CA_ATTJ_DDG" sheetId="42" r:id="rId12"/>
@@ -12061,7 +12061,7 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("7.1. ACTIVITÉ CIVILE",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire CTECH"))+
 SUM(SUMIFS(
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.9. FONCTIONNAIRES / JA AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.9. FONCTIONNAIRES / AJ AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire CTECH"))</f>
         <v>#N/A</v>
       </c>
@@ -12071,7 +12071,7 @@
       </c>
       <c r="I3" s="142" t="e">
         <f>SUM(SUMIFS(
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.9. FONCTIONNAIRES / JA AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.9. FONCTIONNAIRES / AJ AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR"))</f>
         <v>#N/A</v>
       </c>
@@ -12903,7 +12903,7 @@
       </c>
       <c r="I12" s="135" t="e">
         <f>SUM(SUMIFS(
-INDEX('ETPT A-JUST'!$A:$ZZ,,MATCH("13.9. FONCTIONNAIRES / JA AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT A-JUST'!2:2,0)),
+INDEX('ETPT A-JUST'!$A:$ZZ,,MATCH("13.9. FONCTIONNAIRES / AJ AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT A-JUST'!2:2,0)),
 INDEX('ETPT A-JUST'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT A-JUST'!2:2,0)),"Fonctionnaire A-B-CBUR placé ADD"))</f>
         <v>#N/A</v>
       </c>
@@ -13087,7 +13087,7 @@
       </c>
       <c r="I14" s="135" t="e">
         <f>SUM(SUMIFS(
-INDEX('ETPT A-JUST'!$A:$ZZ,,MATCH("13.9. FONCTIONNAIRES / JA AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT A-JUST'!2:2,0)),
+INDEX('ETPT A-JUST'!$A:$ZZ,,MATCH("13.9. FONCTIONNAIRES / AJ AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET GÉNÉRAL",'ETPT A-JUST'!2:2,0)),
 INDEX('ETPT A-JUST'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT A-JUST'!2:2,0)),"Fonctionnaire A-B-CBUR placé SUB"))</f>
         <v>#N/A</v>
       </c>

</xml_diff>

<commit_message>
chore: update template4CA (#485)
Co-authored-by: Joseph Dureau <dinum-327809@mac-1.home>
</commit_message>
<xml_diff>
--- a/front/src/assets/template4CA.xlsx
+++ b/front/src/assets/template4CA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dinum-327809/Documents/a-just-dev/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2C3AC54-7268-204E-93BC-32BB714E9DEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B40D2F7-3B7F-C042-A959-F34694F23E4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="100" yWindow="780" windowWidth="30160" windowHeight="17660" activeTab="8" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -12211,7 +12211,7 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11. TOTAL CONTENTIEUX CRIMINEL",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire CTECH"))+
 SUM(SUMIFS(
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.10. AUTRES FONCTIONNAIRES / JA AFFECTÉS AU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.10. AUTRES FONCTIONNAIRES / AJ AFFECTÉS AU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire CTECH"))</f>
         <v>#N/A</v>
       </c>
@@ -12280,7 +12280,7 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11. TOTAL CONTENTIEUX CRIMINEL",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR"))+
 SUM(SUMIFS(
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.10. AUTRES FONCTIONNAIRES / JA AFFECTÉS AU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13.10. AUTRES FONCTIONNAIRES / AJ AFFECTÉS AU PARQUET GÉNÉRAL",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR"))-
 SUM(I4:M4)</f>
         <v>#N/A</v>

</xml_diff>

<commit_message>
chore: update template4CA (#486)
Co-authored-by: Joseph Dureau <dinum-327809@MacBook-Pro-de-DINUM-327809.local>
</commit_message>
<xml_diff>
--- a/front/src/assets/template4CA.xlsx
+++ b/front/src/assets/template4CA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dinum-327809/Documents/a-just-dev/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B40D2F7-3B7F-C042-A959-F34694F23E4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C157242-DAA6-7E4F-86EE-CB1B1EEF8BFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="100" yWindow="780" windowWidth="30160" windowHeight="17660" activeTab="8" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
+    <workbookView xWindow="100" yWindow="780" windowWidth="30160" windowHeight="17660" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
   <sheets>
     <sheet name="ACCUEIL" sheetId="33" r:id="rId1"/>
@@ -21,7 +21,7 @@
     <sheet name="codage tribunal" sheetId="12" state="hidden" r:id="rId6"/>
     <sheet name="Juridictions" sheetId="17" state="hidden" r:id="rId7"/>
     <sheet name="Table_Fonctions" sheetId="19" state="hidden" r:id="rId8"/>
-    <sheet name="ETPT_CA_JUR" sheetId="30" r:id="rId9"/>
+    <sheet name="ETPT_CA_JUR" sheetId="30" state="hidden" r:id="rId9"/>
     <sheet name="ETPT_CA_JUR_DDG" sheetId="25" r:id="rId10"/>
     <sheet name="ETPT_CA_ATTJ" sheetId="41" state="hidden" r:id="rId11"/>
     <sheet name="ETPT_CA_ATTJ_DDG" sheetId="42" r:id="rId12"/>

</xml_diff>

<commit_message>
chore: update template4CA (#487)
Co-authored-by: Joseph Dureau <dinum-327809@mac-1.home>
</commit_message>
<xml_diff>
--- a/front/src/assets/template4CA.xlsx
+++ b/front/src/assets/template4CA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dinum-327809/Documents/a-just-dev/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C157242-DAA6-7E4F-86EE-CB1B1EEF8BFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA9F2146-4D56-9644-B279-B105CACAC41E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="100" yWindow="780" windowWidth="30160" windowHeight="17660" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
+    <workbookView xWindow="100" yWindow="780" windowWidth="30160" windowHeight="17660" activeTab="1" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
   <sheets>
     <sheet name="ACCUEIL" sheetId="33" r:id="rId1"/>
@@ -10488,9 +10488,9 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26.1640625" customWidth="1"/>
-    <col min="2" max="2" width="22.1640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="7.6640625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="12" style="2" customWidth="1"/>
+    <col min="2" max="2" width="22.5" style="1" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="18.6640625" style="2" customWidth="1"/>
     <col min="5" max="5" width="11.83203125" style="2" customWidth="1"/>
     <col min="6" max="6" width="60.1640625" customWidth="1"/>
     <col min="7" max="7" width="5.1640625" customWidth="1"/>
@@ -10790,7 +10790,7 @@
       <c r="C8" s="2"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1" sort="0" autoFilter="0"/>
+  <sheetProtection sort="0" autoFilter="0"/>
   <autoFilter ref="A2:DN2" xr:uid="{F3674A8A-13E9-4EDB-B294-D1FF8F18362C}"/>
   <dataConsolidate/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>